<commit_message>
Auto update scanner reports (2026-09-14 09:00 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -1884,10 +1884,10 @@
         <v>1969</v>
       </c>
       <c r="Z2" t="n">
-        <v>2277186</v>
+        <v>2277375</v>
       </c>
       <c r="AA2" t="n">
-        <v>3578266</v>
+        <v>3578275</v>
       </c>
       <c r="AB2" t="n">
         <v>0.64</v>
@@ -2085,7 +2085,7 @@
         <v>76.27</v>
       </c>
       <c r="CO2" t="n">
-        <v>38.6</v>
+        <v>38.59</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2258,7 +2258,7 @@
         <v>12.2787</v>
       </c>
       <c r="ET2" t="n">
-        <v>41.381</v>
+        <v>41.377</v>
       </c>
       <c r="EU2" t="n">
         <v>1.312</v>
@@ -2296,7 +2296,7 @@
         <v>69.735</v>
       </c>
       <c r="FF2" t="n">
-        <v>37.465</v>
+        <v>37.46</v>
       </c>
       <c r="FG2" t="n">
         <v>21.9167</v>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260911_195359</t>
+          <t>20260914_143055</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46276.82916529106</v>
+        <v>46279.60481297351</v>
       </c>
     </row>
   </sheetData>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46276.82915509259</v>
+        <v>46279.60480324074</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2682,7 +2682,7 @@
         <v>1969</v>
       </c>
       <c r="P2" t="n">
-        <v>2277186</v>
+        <v>2277375</v>
       </c>
       <c r="Q2" t="n">
         <v>1969</v>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02057924365393107</v>
+        <v>0.02057924387964351</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3266853652686347</v>
+        <v>0.3266853688517086</v>
       </c>
     </row>
     <row r="7">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266353895739713</v>
+        <v>0.04266353542026954</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869493934347615</v>
       </c>
     </row>
     <row r="14">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-11 19:53:59.909622+05:30</t>
+          <t>2026-09-14 14:30:55.876688+05:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-14 16:21 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -2020,7 +2020,7 @@
         <v>0.246</v>
       </c>
       <c r="BT2" t="n">
-        <v>1480.7</v>
+        <v>1480.71</v>
       </c>
       <c r="BU2" t="n">
         <v>-13.83</v>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260914_143055</t>
+          <t>20260914_215132</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46279.60481297351</v>
+        <v>46279.91079213945</v>
       </c>
     </row>
   </sheetData>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46279.60480324074</v>
+        <v>46279.91078703704</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02057924387964351</v>
+        <v>0.02057924428704479</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3266853688517086</v>
+        <v>0.3266853753190034</v>
       </c>
     </row>
     <row r="7">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266353542026954</v>
+        <v>0.04266353042005967</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347615</v>
+        <v>0.1869492979645462</v>
       </c>
     </row>
     <row r="14">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-14 14:30:55.876688+05:30</t>
+          <t>2026-09-14 21:51:32.481840+05:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-15 08:45 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1816,14 +1816,14 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46276</v>
+        <v>46280</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46276</v>
+        <v>46280</v>
       </c>
       <c r="H2" t="n">
         <v>8.699999999999999</v>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>STRONG BUY</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1862,56 +1862,56 @@
         <v>11.77</v>
       </c>
       <c r="R2" t="n">
-        <v>49.13</v>
+        <v>48.99</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="n">
-        <v>1943</v>
+        <v>1975</v>
       </c>
       <c r="V2" t="n">
-        <v>1981.8</v>
+        <v>1981</v>
       </c>
       <c r="W2" t="n">
-        <v>1918.1</v>
+        <v>1931.8</v>
       </c>
       <c r="X2" t="n">
-        <v>1969</v>
+        <v>1931.9</v>
       </c>
       <c r="Y2" t="n">
-        <v>1969</v>
+        <v>1931.9</v>
       </c>
       <c r="Z2" t="n">
-        <v>2277375</v>
+        <v>1082455</v>
       </c>
       <c r="AA2" t="n">
-        <v>3578275</v>
+        <v>3553330</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.64</v>
+        <v>0.3</v>
       </c>
       <c r="AC2" t="n">
-        <v>1.23</v>
+        <v>-1.88</v>
       </c>
       <c r="AD2" t="n">
-        <v>-0.1</v>
+        <v>0.3</v>
       </c>
       <c r="AE2" t="n">
-        <v>63.7</v>
+        <v>49.2</v>
       </c>
       <c r="AF2" t="n">
-        <v>3.24</v>
+        <v>2.55</v>
       </c>
       <c r="AG2" t="n">
-        <v>48.82</v>
+        <v>48.85</v>
       </c>
       <c r="AH2" t="n">
-        <v>48.82</v>
+        <v>48.85</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.48</v>
+        <v>2.53</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,50 +1920,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>5.27</v>
+        <v>2.89</v>
       </c>
       <c r="AM2" t="n">
-        <v>12.43</v>
+        <v>9.82</v>
       </c>
       <c r="AN2" t="n">
-        <v>52.57</v>
+        <v>49.15</v>
       </c>
       <c r="AO2" t="n">
-        <v>67.81</v>
+        <v>61.03</v>
       </c>
       <c r="AP2" t="n">
-        <v>2.05</v>
+        <v>-0.34</v>
       </c>
       <c r="AQ2" t="n">
-        <v>41.75</v>
+        <v>40.36</v>
       </c>
       <c r="AR2" t="n">
-        <v>1969</v>
+        <v>1931.9</v>
       </c>
       <c r="AS2" t="n">
-        <v>2164.3</v>
+        <v>2127.3</v>
       </c>
       <c r="AT2" t="n">
-        <v>1871.35</v>
+        <v>1834.2</v>
       </c>
       <c r="AU2" t="n">
-        <v>1969</v>
+        <v>1931.900024414062</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.92</v>
+        <v>10.11</v>
       </c>
       <c r="AY2" t="n">
-        <v>195.3</v>
+        <v>195.4</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.96</v>
+        <v>5.06</v>
       </c>
       <c r="BA2" t="n">
-        <v>97.65000000000001</v>
+        <v>97.7</v>
       </c>
       <c r="BB2" t="n">
         <v>2.05</v>
@@ -2082,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>76.27</v>
+        <v>79.36</v>
       </c>
       <c r="CO2" t="n">
-        <v>38.59</v>
+        <v>37.71</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2106,19 +2106,19 @@
         <v>95.45454545454545</v>
       </c>
       <c r="CV2" t="n">
-        <v>84.09090909090909</v>
+        <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
         <v>68.18181818181817</v>
       </c>
       <c r="CX2" t="n">
-        <v>59.09090909090909</v>
+        <v>54.54545454545454</v>
       </c>
       <c r="CY2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.918699999999999</v>
+        <v>10.1144</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,31 +2127,31 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6613</v>
+        <v>0.674</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3307</v>
+        <v>0.3373</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0992</v>
+        <v>0.1011</v>
       </c>
       <c r="DF2" t="n">
-        <v>2</v>
+        <v>1.998</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1676</v>
+        <v>1.1899</v>
       </c>
       <c r="DH2" t="n">
-        <v>4</v>
+        <v>3.996</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.9594</v>
+        <v>5.0572</v>
       </c>
       <c r="DJ2" t="n">
-        <v>42.73</v>
+        <v>43.58</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.9594</v>
+        <v>5.0572</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
@@ -2160,25 +2160,25 @@
         <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>4</v>
+        <v>3.996</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9997</v>
+        <v>1.9982</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8065</v>
+        <v>0.7897</v>
       </c>
       <c r="DQ2" t="n">
-        <v>97.65000000000001</v>
+        <v>97.7</v>
       </c>
       <c r="DR2" t="n">
-        <v>54.26</v>
+        <v>54.93</v>
       </c>
       <c r="DS2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="DT2" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,49 +2187,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.8266</v>
+        <v>-0.1344</v>
       </c>
       <c r="DX2" t="n">
-        <v>80.47499999999999</v>
+        <v>97.425</v>
       </c>
       <c r="DY2" t="n">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="DZ2" t="n">
-        <v>82.943</v>
+        <v>80.483</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
       </c>
       <c r="EB2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>72.83</v>
+        <v>66.65000000000001</v>
       </c>
       <c r="ED2" t="n">
-        <v>82.55</v>
+        <v>99.70999999999999</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.8266</v>
+        <v>-0.1344</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.64</v>
+        <v>0.3</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.2413</v>
+        <v>-0.04</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9995</v>
+        <v>3.9978</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0284</v>
+        <v>-0.0047</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6711</v>
+        <v>0.6597</v>
       </c>
       <c r="EK2" t="n">
-        <v>63.2</v>
+        <v>64.22</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2240,37 +2240,37 @@
         <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>22.44</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="EP2" t="n">
-        <v>2.6412</v>
+        <v>1.0946</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.07530000000000001</v>
+        <v>0.0353</v>
       </c>
       <c r="ER2" t="n">
-        <v>15.5</v>
+        <v>33.7</v>
       </c>
       <c r="ES2" t="n">
-        <v>12.2787</v>
+        <v>12.3456</v>
       </c>
       <c r="ET2" t="n">
-        <v>41.377</v>
+        <v>37.083</v>
       </c>
       <c r="EU2" t="n">
-        <v>1.312</v>
+        <v>-0.102</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.5122</v>
+        <v>1.9462</v>
       </c>
       <c r="EW2" t="n">
-        <v>17.115</v>
+        <v>7.3805</v>
       </c>
       <c r="EX2" t="n">
-        <v>36.33</v>
+        <v>31.73</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2278,37 +2278,37 @@
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="FA2" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="FB2" t="n">
         <v>64.03</v>
       </c>
       <c r="FC2" t="n">
-        <v>36.03</v>
+        <v>36.23</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.33</v>
+        <v>73.3</v>
       </c>
       <c r="FE2" t="n">
-        <v>69.735</v>
+        <v>71.79000000000001</v>
       </c>
       <c r="FF2" t="n">
-        <v>37.46</v>
+        <v>34.72</v>
       </c>
       <c r="FG2" t="n">
-        <v>21.9167</v>
+        <v>22.4816</v>
       </c>
       <c r="FH2" t="n">
-        <v>62.162</v>
+        <v>62.169</v>
       </c>
       <c r="FI2" t="n">
-        <v>48.495</v>
+        <v>49.255</v>
       </c>
       <c r="FJ2" t="n">
-        <v>67.25</v>
+        <v>67.98999999999999</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,22 +2322,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>72.92</v>
+        <v>70.70999999999999</v>
       </c>
       <c r="FO2" t="n">
-        <v>63.64</v>
+        <v>65.56999999999999</v>
       </c>
       <c r="FP2" t="n">
-        <v>62.01</v>
+        <v>54.02</v>
       </c>
       <c r="FQ2" t="n">
-        <v>74.93000000000001</v>
+        <v>71.92</v>
       </c>
       <c r="FR2" t="n">
-        <v>84.38</v>
+        <v>77.19</v>
       </c>
       <c r="FS2" t="n">
-        <v>100</v>
+        <v>95.4545</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2347,11 +2347,11 @@
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>70.1885</v>
+        <v>66.9695</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260914_215132</t>
+          <t>20260915_141527</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46279.91079213945</v>
+        <v>46280.5940680392</v>
       </c>
     </row>
   </sheetData>
@@ -2458,7 +2458,7 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
     <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46279.91078703704</v>
+        <v>46280.5940625</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2667,43 +2667,43 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>1969</v>
+        <v>1931.9</v>
       </c>
       <c r="L2" t="n">
-        <v>1943</v>
+        <v>1975</v>
       </c>
       <c r="M2" t="n">
-        <v>1981.8</v>
+        <v>1981</v>
       </c>
       <c r="N2" t="n">
-        <v>1918.1</v>
+        <v>1931.8</v>
       </c>
       <c r="O2" t="n">
-        <v>1969</v>
+        <v>1931.9</v>
       </c>
       <c r="P2" t="n">
-        <v>2277375</v>
+        <v>1082455</v>
       </c>
       <c r="Q2" t="n">
-        <v>1969</v>
+        <v>1931.9</v>
       </c>
       <c r="R2" t="n">
-        <v>2164.3</v>
+        <v>2127.3</v>
       </c>
       <c r="S2" t="n">
-        <v>1871.35</v>
+        <v>1834.2</v>
       </c>
       <c r="T2" t="n">
-        <v>9.918740477399703</v>
+        <v>10.11439515502873</v>
       </c>
       <c r="U2" t="n">
-        <v>195.3000000000002</v>
+        <v>195.4000000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>4.959370238699852</v>
+        <v>5.057197577514366</v>
       </c>
       <c r="W2" t="n">
-        <v>97.65000000000009</v>
+        <v>97.70000000000005</v>
       </c>
       <c r="X2" t="n">
         <v>2</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.918740477399703</v>
+        <v>10.11439515502873</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.959370238699852</v>
+        <v>5.057197577514366</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02057924428704479</v>
+        <v>0.02058054488607412</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3266853753190034</v>
+        <v>0.3267060216885256</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909829344476882</v>
+        <v>0.02909818349534118</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266353042005967</v>
+        <v>0.0426635390556001</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645462</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.87</v>
+        <v>38.86</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-14 21:51:32.481840+05:30</t>
+          <t>2026-09-15 14:15:27.518505+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.918740477399703, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.114395155028733, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-15 14:58 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -1847,7 +1847,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1862,7 +1862,7 @@
         <v>11.77</v>
       </c>
       <c r="R2" t="n">
-        <v>48.99</v>
+        <v>49.05</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,43 +1875,43 @@
         <v>1981</v>
       </c>
       <c r="W2" t="n">
-        <v>1931.8</v>
+        <v>1915.6</v>
       </c>
       <c r="X2" t="n">
-        <v>1931.9</v>
+        <v>1926.9</v>
       </c>
       <c r="Y2" t="n">
-        <v>1931.9</v>
+        <v>1926.9</v>
       </c>
       <c r="Z2" t="n">
-        <v>1082455</v>
+        <v>1536709</v>
       </c>
       <c r="AA2" t="n">
-        <v>3553330</v>
+        <v>3576043</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.3</v>
+        <v>0.43</v>
       </c>
       <c r="AC2" t="n">
-        <v>-1.88</v>
+        <v>-2.14</v>
       </c>
       <c r="AD2" t="n">
         <v>0.3</v>
       </c>
       <c r="AE2" t="n">
-        <v>49.2</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.55</v>
+        <v>3.39</v>
       </c>
       <c r="AG2" t="n">
-        <v>48.85</v>
+        <v>50.01</v>
       </c>
       <c r="AH2" t="n">
-        <v>48.85</v>
+        <v>50.01</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.53</v>
+        <v>2.6</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,50 +1920,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>2.89</v>
+        <v>2.64</v>
       </c>
       <c r="AM2" t="n">
-        <v>9.82</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="AN2" t="n">
-        <v>49.15</v>
+        <v>48.77</v>
       </c>
       <c r="AO2" t="n">
-        <v>61.03</v>
+        <v>60.22</v>
       </c>
       <c r="AP2" t="n">
-        <v>-0.34</v>
+        <v>-0.6</v>
       </c>
       <c r="AQ2" t="n">
-        <v>40.36</v>
+        <v>40</v>
       </c>
       <c r="AR2" t="n">
-        <v>1931.9</v>
+        <v>1926.9</v>
       </c>
       <c r="AS2" t="n">
-        <v>2127.3</v>
+        <v>2126.93</v>
       </c>
       <c r="AT2" t="n">
-        <v>1834.2</v>
+        <v>1826.88</v>
       </c>
       <c r="AU2" t="n">
-        <v>1931.900024414062</v>
+        <v>1926.900024414062</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>10.11</v>
+        <v>10.38</v>
       </c>
       <c r="AY2" t="n">
-        <v>195.4</v>
+        <v>200.03</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.06</v>
+        <v>5.19</v>
       </c>
       <c r="BA2" t="n">
-        <v>97.7</v>
+        <v>100.02</v>
       </c>
       <c r="BB2" t="n">
         <v>2.05</v>
@@ -2020,7 +2020,7 @@
         <v>0.246</v>
       </c>
       <c r="BT2" t="n">
-        <v>1480.71</v>
+        <v>1480.7</v>
       </c>
       <c r="BU2" t="n">
         <v>-13.83</v>
@@ -2032,7 +2032,7 @@
         <v>2.05</v>
       </c>
       <c r="BX2" t="n">
-        <v>2</v>
+        <v>1.9999</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2082,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>79.36</v>
+        <v>83.14</v>
       </c>
       <c r="CO2" t="n">
-        <v>37.71</v>
+        <v>35.79</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2118,7 +2118,7 @@
         <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>10.1144</v>
+        <v>10.3809</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,58 +2127,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.674</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3373</v>
+        <v>0.346</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1011</v>
+        <v>0.1038</v>
       </c>
       <c r="DF2" t="n">
-        <v>1.998</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1899</v>
+        <v>1.2217</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.996</v>
+        <v>3.9923</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.0572</v>
+        <v>5.1907</v>
       </c>
       <c r="DJ2" t="n">
-        <v>43.58</v>
+        <v>45.05</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.0572</v>
+        <v>5.1907</v>
       </c>
       <c r="DL2" t="n">
+        <v>1.9999</v>
+      </c>
+      <c r="DM2" t="n">
+        <v>1.9962</v>
+      </c>
+      <c r="DN2" t="n">
+        <v>3.9923</v>
+      </c>
+      <c r="DO2" t="n">
         <v>2</v>
       </c>
-      <c r="DM2" t="n">
-        <v>2</v>
-      </c>
-      <c r="DN2" t="n">
-        <v>3.996</v>
-      </c>
-      <c r="DO2" t="n">
-        <v>1.9982</v>
-      </c>
       <c r="DP2" t="n">
-        <v>0.7897</v>
+        <v>0.7692</v>
       </c>
       <c r="DQ2" t="n">
-        <v>97.7</v>
+        <v>100.02</v>
       </c>
       <c r="DR2" t="n">
-        <v>54.93</v>
+        <v>56.54</v>
       </c>
       <c r="DS2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,49 +2187,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>-0.1344</v>
+        <v>-0.2308</v>
       </c>
       <c r="DX2" t="n">
-        <v>97.425</v>
+        <v>99.45</v>
       </c>
       <c r="DY2" t="n">
-        <v>15</v>
+        <v>21.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>80.483</v>
+        <v>81.099</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
       </c>
       <c r="EB2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>66.65000000000001</v>
+        <v>67.64</v>
       </c>
       <c r="ED2" t="n">
-        <v>99.70999999999999</v>
+        <v>100</v>
       </c>
       <c r="EE2" t="n">
-        <v>-0.1344</v>
+        <v>-0.2308</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.3</v>
+        <v>0.43</v>
       </c>
       <c r="EG2" t="n">
-        <v>-0.04</v>
+        <v>-0.0706</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9978</v>
+        <v>3.9927</v>
       </c>
       <c r="EI2" t="n">
-        <v>-0.0047</v>
+        <v>-0.0083</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6597</v>
+        <v>0.645</v>
       </c>
       <c r="EK2" t="n">
-        <v>64.22</v>
+        <v>63.22</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2240,37 +2240,37 @@
         <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>9.300000000000001</v>
+        <v>10.17</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.0946</v>
+        <v>1.197</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0353</v>
+        <v>0.0506</v>
       </c>
       <c r="ER2" t="n">
-        <v>33.7</v>
+        <v>24.1395</v>
       </c>
       <c r="ES2" t="n">
-        <v>12.3456</v>
+        <v>12.5139</v>
       </c>
       <c r="ET2" t="n">
-        <v>37.083</v>
+        <v>36.576</v>
       </c>
       <c r="EU2" t="n">
-        <v>-0.102</v>
+        <v>-0.258</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.9462</v>
+        <v>1.8182</v>
       </c>
       <c r="EW2" t="n">
-        <v>7.3805</v>
+        <v>8.455299999999999</v>
       </c>
       <c r="EX2" t="n">
-        <v>31.73</v>
+        <v>31.36</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2287,28 +2287,28 @@
         <v>64.03</v>
       </c>
       <c r="FC2" t="n">
-        <v>36.23</v>
+        <v>37.95</v>
       </c>
       <c r="FD2" t="n">
         <v>73.3</v>
       </c>
       <c r="FE2" t="n">
-        <v>71.79000000000001</v>
+        <v>73.18000000000001</v>
       </c>
       <c r="FF2" t="n">
-        <v>34.72</v>
+        <v>33.575</v>
       </c>
       <c r="FG2" t="n">
-        <v>22.4816</v>
+        <v>23.0944</v>
       </c>
       <c r="FH2" t="n">
-        <v>62.169</v>
+        <v>63.229</v>
       </c>
       <c r="FI2" t="n">
-        <v>49.255</v>
+        <v>50.795</v>
       </c>
       <c r="FJ2" t="n">
-        <v>67.98999999999999</v>
+        <v>67.48</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,19 +2322,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>70.70999999999999</v>
+        <v>71.44</v>
       </c>
       <c r="FO2" t="n">
-        <v>65.56999999999999</v>
+        <v>62.83</v>
       </c>
       <c r="FP2" t="n">
-        <v>54.02</v>
+        <v>57.35</v>
       </c>
       <c r="FQ2" t="n">
-        <v>71.92</v>
+        <v>76.08</v>
       </c>
       <c r="FR2" t="n">
-        <v>77.19</v>
+        <v>81.89</v>
       </c>
       <c r="FS2" t="n">
         <v>95.4545</v>
@@ -2347,11 +2347,11 @@
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>66.9695</v>
+        <v>69.6795</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260915_141527</t>
+          <t>20260915_202807</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46280.5940680392</v>
+        <v>46280.85286487779</v>
       </c>
     </row>
   </sheetData>
@@ -2458,9 +2458,9 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
-    <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46280.5940625</v>
+        <v>46280.85285879629</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2667,7 +2667,7 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>1931.9</v>
+        <v>1926.9</v>
       </c>
       <c r="L2" t="n">
         <v>1975</v>
@@ -2676,37 +2676,37 @@
         <v>1981</v>
       </c>
       <c r="N2" t="n">
-        <v>1931.8</v>
+        <v>1915.6</v>
       </c>
       <c r="O2" t="n">
-        <v>1931.9</v>
+        <v>1926.9</v>
       </c>
       <c r="P2" t="n">
-        <v>1082455</v>
+        <v>1536709</v>
       </c>
       <c r="Q2" t="n">
-        <v>1931.9</v>
+        <v>1926.9</v>
       </c>
       <c r="R2" t="n">
-        <v>2127.3</v>
+        <v>2126.93</v>
       </c>
       <c r="S2" t="n">
-        <v>1834.2</v>
+        <v>1826.88</v>
       </c>
       <c r="T2" t="n">
-        <v>10.11439515502873</v>
+        <v>10.38092272562145</v>
       </c>
       <c r="U2" t="n">
-        <v>195.4000000000001</v>
+        <v>200.0299999999997</v>
       </c>
       <c r="V2" t="n">
-        <v>5.057197577514366</v>
+        <v>5.19072084695625</v>
       </c>
       <c r="W2" t="n">
-        <v>97.70000000000005</v>
+        <v>100.02</v>
       </c>
       <c r="X2" t="n">
-        <v>2</v>
+        <v>1.999900019995999</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>10.11439515502873</v>
+        <v>10.38092272562145</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.057197577514366</v>
+        <v>5.19072084695625</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02058054488607412</v>
+        <v>0.02058460939821866</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3267060216885256</v>
+        <v>0.3267705438185371</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909818349534118</v>
+        <v>0.02909823423828552</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.0426635390556001</v>
+        <v>0.04266353895739713</v>
       </c>
     </row>
     <row r="13">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-15 14:15:27.518505+05:30</t>
+          <t>2026-09-15 20:28:07.561355+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.114395155028733, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.380922725621451, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9999000199959986}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-16 08:39 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="20" customWidth="1" min="47" max="47"/>
+    <col width="19" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="17" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,14 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46280</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
+        <v>46281</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>46281</v>
+      </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H2" t="n">
         <v>8.699999999999999</v>
@@ -1847,71 +1849,75 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>STRONG BUY</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="P2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.77</v>
+        <v>11.69</v>
       </c>
       <c r="R2" t="n">
-        <v>49.05</v>
+        <v>49.15</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
       </c>
-      <c r="T2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>UPTREND</t>
+        </is>
+      </c>
       <c r="U2" t="n">
-        <v>1975</v>
+        <v>1924.6</v>
       </c>
       <c r="V2" t="n">
-        <v>1981</v>
+        <v>1940.4</v>
       </c>
       <c r="W2" t="n">
-        <v>1915.6</v>
+        <v>1863.5</v>
       </c>
       <c r="X2" t="n">
-        <v>1926.9</v>
+        <v>1897.2</v>
       </c>
       <c r="Y2" t="n">
-        <v>1926.9</v>
+        <v>1897.2</v>
       </c>
       <c r="Z2" t="n">
-        <v>1536709</v>
+        <v>2442260</v>
       </c>
       <c r="AA2" t="n">
-        <v>3576043</v>
+        <v>3552050</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.43</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="AC2" t="n">
-        <v>-2.14</v>
+        <v>-1.54</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.3</v>
+        <v>-0.12</v>
       </c>
       <c r="AE2" t="n">
-        <v>65.40000000000001</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="AF2" t="n">
-        <v>3.39</v>
+        <v>4.05</v>
       </c>
       <c r="AG2" t="n">
-        <v>50.01</v>
+        <v>48.92</v>
       </c>
       <c r="AH2" t="n">
-        <v>50.01</v>
+        <v>48.92</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.6</v>
+        <v>2.58</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,50 +1926,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>2.64</v>
+        <v>0.4</v>
       </c>
       <c r="AM2" t="n">
-        <v>9.539999999999999</v>
+        <v>6.81</v>
       </c>
       <c r="AN2" t="n">
-        <v>48.77</v>
+        <v>45.44</v>
       </c>
       <c r="AO2" t="n">
-        <v>60.22</v>
+        <v>54.73</v>
       </c>
       <c r="AP2" t="n">
-        <v>-0.6</v>
+        <v>1.91</v>
       </c>
       <c r="AQ2" t="n">
-        <v>40</v>
+        <v>38.6</v>
       </c>
       <c r="AR2" t="n">
-        <v>1926.9</v>
+        <v>1897.2</v>
       </c>
       <c r="AS2" t="n">
-        <v>2126.93</v>
+        <v>2092.89</v>
       </c>
       <c r="AT2" t="n">
-        <v>1826.88</v>
+        <v>1799.36</v>
       </c>
       <c r="AU2" t="n">
-        <v>1926.900024414062</v>
+        <v>1897.199951171875</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>10.38</v>
+        <v>10.31</v>
       </c>
       <c r="AY2" t="n">
-        <v>200.03</v>
+        <v>195.69</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.19</v>
+        <v>5.16</v>
       </c>
       <c r="BA2" t="n">
-        <v>100.02</v>
+        <v>97.84</v>
       </c>
       <c r="BB2" t="n">
         <v>2.05</v>
@@ -1978,7 +1984,7 @@
         <v>326</v>
       </c>
       <c r="BF2" t="n">
-        <v>49.4</v>
+        <v>49.3</v>
       </c>
       <c r="BG2" t="n">
         <v>120</v>
@@ -1987,22 +1993,22 @@
         <v>18.2</v>
       </c>
       <c r="BI2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BM2" t="n">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="BN2" t="n">
-        <v>50</v>
+        <v>49.9</v>
       </c>
       <c r="BO2" t="n">
         <v>2.24</v>
@@ -2017,13 +2023,13 @@
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.246</v>
+        <v>0.245</v>
       </c>
       <c r="BT2" t="n">
-        <v>1480.7</v>
+        <v>1479.09</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.83</v>
+        <v>-13.93</v>
       </c>
       <c r="BV2" t="n">
         <v>2.05</v>
@@ -2032,7 +2038,7 @@
         <v>2.05</v>
       </c>
       <c r="BX2" t="n">
-        <v>1.9999</v>
+        <v>2.0001</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2041,7 +2047,7 @@
         <v>8</v>
       </c>
       <c r="CA2" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="CB2" t="n">
         <v>0</v>
@@ -2061,7 +2067,7 @@
         <v>68.3</v>
       </c>
       <c r="CG2" t="n">
-        <v>71.40000000000001</v>
+        <v>71.3</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2082,43 +2088,43 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>83.14</v>
+        <v>75.27</v>
       </c>
       <c r="CO2" t="n">
-        <v>35.79</v>
+        <v>46.8</v>
       </c>
       <c r="CP2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CQ2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CR2" t="n">
-        <v>86.36363636363636</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="CS2" t="n">
         <v>100</v>
       </c>
       <c r="CT2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CU2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CV2" t="n">
-        <v>86.36363636363636</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="CW2" t="n">
-        <v>68.18181818181817</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="CX2" t="n">
-        <v>54.54545454545454</v>
+        <v>57.14285714285714</v>
       </c>
       <c r="CY2" t="n">
         <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>10.3809</v>
+        <v>10.3147</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6919999999999999</v>
+        <v>0.6873</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.346</v>
+        <v>0.344</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1038</v>
+        <v>0.1031</v>
       </c>
       <c r="DF2" t="n">
+        <v>1.9981</v>
+      </c>
+      <c r="DG2" t="n">
+        <v>1.2052</v>
+      </c>
+      <c r="DH2" t="n">
+        <v>3.9961</v>
+      </c>
+      <c r="DI2" t="n">
+        <v>5.1571</v>
+      </c>
+      <c r="DJ2" t="n">
+        <v>57</v>
+      </c>
+      <c r="DK2" t="n">
+        <v>5.1571</v>
+      </c>
+      <c r="DL2" t="n">
+        <v>2.0001</v>
+      </c>
+      <c r="DM2" t="n">
         <v>2</v>
       </c>
-      <c r="DG2" t="n">
-        <v>1.2217</v>
-      </c>
-      <c r="DH2" t="n">
-        <v>3.9923</v>
-      </c>
-      <c r="DI2" t="n">
-        <v>5.1907</v>
-      </c>
-      <c r="DJ2" t="n">
-        <v>45.05</v>
-      </c>
-      <c r="DK2" t="n">
-        <v>5.1907</v>
-      </c>
-      <c r="DL2" t="n">
-        <v>1.9999</v>
-      </c>
-      <c r="DM2" t="n">
-        <v>1.9962</v>
-      </c>
       <c r="DN2" t="n">
-        <v>3.9923</v>
+        <v>3.9961</v>
       </c>
       <c r="DO2" t="n">
-        <v>2</v>
+        <v>1.998</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.7692</v>
+        <v>0.7744</v>
       </c>
       <c r="DQ2" t="n">
-        <v>100.02</v>
+        <v>97.84</v>
       </c>
       <c r="DR2" t="n">
-        <v>56.54</v>
+        <v>48.43</v>
       </c>
       <c r="DS2" t="n">
+        <v>3</v>
+      </c>
+      <c r="DT2" t="n">
         <v>5</v>
-      </c>
-      <c r="DT2" t="n">
-        <v>9</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>-0.2308</v>
+        <v>0.7403</v>
       </c>
       <c r="DX2" t="n">
-        <v>99.45</v>
+        <v>86.82499999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>21.5</v>
+        <v>34.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>81.099</v>
+        <v>78.658</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2205,31 +2211,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>67.64</v>
+        <v>69.04000000000001</v>
       </c>
       <c r="ED2" t="n">
-        <v>100</v>
+        <v>93.16</v>
       </c>
       <c r="EE2" t="n">
-        <v>-0.2308</v>
+        <v>0.7403</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.43</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="EG2" t="n">
-        <v>-0.0706</v>
+        <v>0.2233</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9927</v>
+        <v>3.9979</v>
       </c>
       <c r="EI2" t="n">
-        <v>-0.0083</v>
+        <v>0.0261</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.645</v>
+        <v>0.649</v>
       </c>
       <c r="EK2" t="n">
-        <v>63.22</v>
+        <v>60.5</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2243,34 +2249,34 @@
         <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>10.17</v>
+        <v>19.84</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.197</v>
+        <v>2.3193</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0506</v>
+        <v>0.08069999999999999</v>
       </c>
       <c r="ER2" t="n">
-        <v>24.1395</v>
+        <v>14.942</v>
       </c>
       <c r="ES2" t="n">
-        <v>12.5139</v>
+        <v>15.9218</v>
       </c>
       <c r="ET2" t="n">
-        <v>36.576</v>
+        <v>43.68</v>
       </c>
       <c r="EU2" t="n">
-        <v>-0.258</v>
+        <v>1.3179</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.8182</v>
+        <v>1.5266</v>
       </c>
       <c r="EW2" t="n">
-        <v>8.455299999999999</v>
+        <v>14.9336</v>
       </c>
       <c r="EX2" t="n">
-        <v>31.36</v>
+        <v>39.9</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2278,37 +2284,37 @@
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="FA2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="FB2" t="n">
-        <v>64.03</v>
+        <v>63.36</v>
       </c>
       <c r="FC2" t="n">
-        <v>37.95</v>
+        <v>48.14</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.3</v>
+        <v>73.31</v>
       </c>
       <c r="FE2" t="n">
-        <v>73.18000000000001</v>
+        <v>67.88500000000001</v>
       </c>
       <c r="FF2" t="n">
-        <v>33.575</v>
+        <v>43.35</v>
       </c>
       <c r="FG2" t="n">
-        <v>23.0944</v>
+        <v>21.0251</v>
       </c>
       <c r="FH2" t="n">
-        <v>63.229</v>
+        <v>62.241</v>
       </c>
       <c r="FI2" t="n">
-        <v>50.795</v>
+        <v>52.715</v>
       </c>
       <c r="FJ2" t="n">
-        <v>67.48</v>
+        <v>68.95999999999999</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>71.44</v>
+        <v>68.45</v>
       </c>
       <c r="FO2" t="n">
-        <v>62.83</v>
+        <v>66.43000000000001</v>
       </c>
       <c r="FP2" t="n">
-        <v>57.35</v>
+        <v>55.83</v>
       </c>
       <c r="FQ2" t="n">
-        <v>76.08</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="FR2" t="n">
-        <v>81.89</v>
+        <v>77.33</v>
       </c>
       <c r="FS2" t="n">
-        <v>95.4545</v>
+        <v>95.2381</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2347,11 +2353,11 @@
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>69.6795</v>
+        <v>68.2715</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260915_202807</t>
+          <t>20260916_140941</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46280.85286487779</v>
+        <v>46281.59006720836</v>
       </c>
     </row>
   </sheetData>
@@ -2438,8 +2444,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -2458,8 +2464,8 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
-    <col width="20" customWidth="1" min="23" max="23"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
@@ -2641,10 +2647,14 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46280.85285879629</v>
-      </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
+        <v>46281.59005787037</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>46296</v>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>LAURUSLABS</t>
@@ -2663,50 +2673,54 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.77</v>
-      </c>
-      <c r="J2" t="inlineStr"/>
+        <v>11.69</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>UPTREND</t>
+        </is>
+      </c>
       <c r="K2" t="n">
-        <v>1926.9</v>
+        <v>1897.2</v>
       </c>
       <c r="L2" t="n">
-        <v>1975</v>
+        <v>1924.6</v>
       </c>
       <c r="M2" t="n">
-        <v>1981</v>
+        <v>1940.4</v>
       </c>
       <c r="N2" t="n">
-        <v>1915.6</v>
+        <v>1863.5</v>
       </c>
       <c r="O2" t="n">
-        <v>1926.9</v>
+        <v>1897.2</v>
       </c>
       <c r="P2" t="n">
-        <v>1536709</v>
+        <v>2442260</v>
       </c>
       <c r="Q2" t="n">
-        <v>1926.9</v>
+        <v>1897.2</v>
       </c>
       <c r="R2" t="n">
-        <v>2126.93</v>
+        <v>2092.89</v>
       </c>
       <c r="S2" t="n">
-        <v>1826.88</v>
+        <v>1799.36</v>
       </c>
       <c r="T2" t="n">
-        <v>10.38092272562145</v>
+        <v>10.31467425679948</v>
       </c>
       <c r="U2" t="n">
-        <v>200.0299999999997</v>
+        <v>195.6899999999998</v>
       </c>
       <c r="V2" t="n">
-        <v>5.19072084695625</v>
+        <v>5.157073582121028</v>
       </c>
       <c r="W2" t="n">
-        <v>100.02</v>
+        <v>97.84000000000015</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999900019995999</v>
+        <v>2.000102207686013</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2727,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>10.38092272562145</v>
+        <v>10.31467425679948</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.19072084695625</v>
+        <v>5.157073582121028</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02058460939821866</v>
+        <v>0.02057577448759861</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3267705438185371</v>
+        <v>0.3266302939604003</v>
       </c>
     </row>
     <row r="7">
@@ -2875,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266353895739713</v>
+        <v>0.04266353098562824</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869492979645464</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.86</v>
+        <v>38.87</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-15 20:28:07.561355+05:30</t>
+          <t>2026-09-16 14:09:41.844895+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.380922725621451, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9999000199959986}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.314674256799485, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001022076860133}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-16 14:56 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="19" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="17" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1864,7 +1864,7 @@
         <v>11.69</v>
       </c>
       <c r="R2" t="n">
-        <v>49.15</v>
+        <v>49.2</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1884,22 +1884,22 @@
         <v>1863.5</v>
       </c>
       <c r="X2" t="n">
-        <v>1897.2</v>
+        <v>1905.5</v>
       </c>
       <c r="Y2" t="n">
-        <v>1897.2</v>
+        <v>1905.5</v>
       </c>
       <c r="Z2" t="n">
-        <v>2442260</v>
+        <v>2870749</v>
       </c>
       <c r="AA2" t="n">
-        <v>3552050</v>
+        <v>3573474</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.8</v>
       </c>
       <c r="AC2" t="n">
-        <v>-1.54</v>
+        <v>-1.11</v>
       </c>
       <c r="AD2" t="n">
         <v>-0.12</v>
@@ -1908,7 +1908,7 @@
         <v>76.90000000000001</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.05</v>
+        <v>4.04</v>
       </c>
       <c r="AG2" t="n">
         <v>48.92</v>
@@ -1917,7 +1917,7 @@
         <v>48.92</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.58</v>
+        <v>2.57</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,47 +1926,47 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>0.4</v>
+        <v>0.82</v>
       </c>
       <c r="AM2" t="n">
-        <v>6.81</v>
+        <v>7.27</v>
       </c>
       <c r="AN2" t="n">
-        <v>45.44</v>
+        <v>46.08</v>
       </c>
       <c r="AO2" t="n">
-        <v>54.73</v>
+        <v>56.04</v>
       </c>
       <c r="AP2" t="n">
-        <v>1.91</v>
+        <v>2.36</v>
       </c>
       <c r="AQ2" t="n">
-        <v>38.6</v>
+        <v>39.21</v>
       </c>
       <c r="AR2" t="n">
-        <v>1897.2</v>
+        <v>1905.5</v>
       </c>
       <c r="AS2" t="n">
-        <v>2092.89</v>
+        <v>2101.19</v>
       </c>
       <c r="AT2" t="n">
-        <v>1799.36</v>
+        <v>1807.66</v>
       </c>
       <c r="AU2" t="n">
-        <v>1897.199951171875</v>
+        <v>1905.5</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>10.31</v>
+        <v>10.27</v>
       </c>
       <c r="AY2" t="n">
         <v>195.69</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.16</v>
+        <v>5.13</v>
       </c>
       <c r="BA2" t="n">
         <v>97.84</v>
@@ -2017,7 +2017,7 @@
         <v>8.77</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.28</v>
+        <v>-4.27</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
@@ -2026,10 +2026,10 @@
         <v>0.245</v>
       </c>
       <c r="BT2" t="n">
-        <v>1479.09</v>
+        <v>1479.51</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.93</v>
+        <v>-13.88</v>
       </c>
       <c r="BV2" t="n">
         <v>2.05</v>
@@ -2088,43 +2088,43 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>75.27</v>
+        <v>75.05</v>
       </c>
       <c r="CO2" t="n">
-        <v>46.8</v>
+        <v>44.23</v>
       </c>
       <c r="CP2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CQ2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CR2" t="n">
-        <v>85.71428571428571</v>
+        <v>86.36363636363636</v>
       </c>
       <c r="CS2" t="n">
         <v>100</v>
       </c>
       <c r="CT2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CU2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CV2" t="n">
-        <v>85.71428571428571</v>
+        <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>66.66666666666666</v>
+        <v>68.18181818181817</v>
       </c>
       <c r="CX2" t="n">
-        <v>57.14285714285714</v>
+        <v>54.54545454545454</v>
       </c>
       <c r="CY2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>10.3147</v>
+        <v>10.2697</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6873</v>
+        <v>0.6847</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.344</v>
+        <v>0.342</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1031</v>
+        <v>0.1027</v>
       </c>
       <c r="DF2" t="n">
-        <v>1.9981</v>
+        <v>2.0019</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.2052</v>
+        <v>1.2006</v>
       </c>
       <c r="DH2" t="n">
         <v>3.9961</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.1571</v>
+        <v>5.1346</v>
       </c>
       <c r="DJ2" t="n">
-        <v>57</v>
+        <v>55.31</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.1571</v>
+        <v>5.1346</v>
       </c>
       <c r="DL2" t="n">
         <v>2.0001</v>
       </c>
       <c r="DM2" t="n">
-        <v>2</v>
+        <v>1.9961</v>
       </c>
       <c r="DN2" t="n">
         <v>3.9961</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.998</v>
+        <v>2.002</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.7744</v>
+        <v>0.779</v>
       </c>
       <c r="DQ2" t="n">
         <v>97.84</v>
       </c>
       <c r="DR2" t="n">
-        <v>48.43</v>
+        <v>69.31</v>
       </c>
       <c r="DS2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.7403</v>
+        <v>0.9183</v>
       </c>
       <c r="DX2" t="n">
-        <v>86.82499999999999</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>34.5</v>
+        <v>40</v>
       </c>
       <c r="DZ2" t="n">
-        <v>78.658</v>
+        <v>78.928</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>69.04000000000001</v>
+        <v>68.04000000000001</v>
       </c>
       <c r="ED2" t="n">
-        <v>93.16</v>
+        <v>96.16</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.7403</v>
+        <v>0.9183</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.8</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.2233</v>
+        <v>0.2759</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9979</v>
+        <v>3.996</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0261</v>
+        <v>0.0323</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.649</v>
+        <v>0.6519</v>
       </c>
       <c r="EK2" t="n">
-        <v>60.5</v>
+        <v>60.63</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2249,34 @@
         <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>19.84</v>
+        <v>20.18</v>
       </c>
       <c r="EP2" t="n">
-        <v>2.3193</v>
+        <v>2.359</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.08069999999999999</v>
+        <v>0.0935</v>
       </c>
       <c r="ER2" t="n">
-        <v>14.942</v>
+        <v>12.8375</v>
       </c>
       <c r="ES2" t="n">
-        <v>15.9218</v>
+        <v>15.493</v>
       </c>
       <c r="ET2" t="n">
-        <v>43.68</v>
+        <v>42.841</v>
       </c>
       <c r="EU2" t="n">
-        <v>1.3179</v>
+        <v>1.888</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.5266</v>
+        <v>1.4278</v>
       </c>
       <c r="EW2" t="n">
-        <v>14.9336</v>
+        <v>15.1451</v>
       </c>
       <c r="EX2" t="n">
-        <v>39.9</v>
+        <v>38.01</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2290,31 @@
         <v>9</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.36</v>
+        <v>63.65</v>
       </c>
       <c r="FC2" t="n">
-        <v>48.14</v>
+        <v>46.61</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.31</v>
+        <v>73.41</v>
       </c>
       <c r="FE2" t="n">
-        <v>67.88500000000001</v>
+        <v>67.84</v>
       </c>
       <c r="FF2" t="n">
-        <v>43.35</v>
+        <v>41.12</v>
       </c>
       <c r="FG2" t="n">
-        <v>21.0251</v>
+        <v>21.0224</v>
       </c>
       <c r="FH2" t="n">
-        <v>62.241</v>
+        <v>61.942</v>
       </c>
       <c r="FI2" t="n">
-        <v>52.715</v>
+        <v>62.31</v>
       </c>
       <c r="FJ2" t="n">
-        <v>68.95999999999999</v>
+        <v>69.65000000000001</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>68.45</v>
+        <v>76.88</v>
       </c>
       <c r="FO2" t="n">
         <v>66.43000000000001</v>
       </c>
       <c r="FP2" t="n">
-        <v>55.83</v>
+        <v>67.51000000000001</v>
       </c>
       <c r="FQ2" t="n">
-        <v>70.40000000000001</v>
+        <v>82.73</v>
       </c>
       <c r="FR2" t="n">
-        <v>77.33</v>
+        <v>85.09</v>
       </c>
       <c r="FS2" t="n">
-        <v>95.2381</v>
+        <v>100</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2353,11 +2353,11 @@
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>68.2715</v>
+        <v>75.16800000000001</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260916_140941</t>
+          <t>20260916_202634</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46281.59006720836</v>
+        <v>46281.85179397242</v>
       </c>
     </row>
   </sheetData>
@@ -2464,7 +2464,7 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46281.59005787037</v>
+        <v>46281.85179398148</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46281</v>
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1897.2</v>
+        <v>1905.5</v>
       </c>
       <c r="L2" t="n">
         <v>1924.6</v>
@@ -2693,34 +2693,34 @@
         <v>1863.5</v>
       </c>
       <c r="O2" t="n">
-        <v>1897.2</v>
+        <v>1905.5</v>
       </c>
       <c r="P2" t="n">
-        <v>2442260</v>
+        <v>2870749</v>
       </c>
       <c r="Q2" t="n">
-        <v>1897.2</v>
+        <v>1905.5</v>
       </c>
       <c r="R2" t="n">
-        <v>2092.89</v>
+        <v>2101.19</v>
       </c>
       <c r="S2" t="n">
-        <v>1799.36</v>
+        <v>1807.66</v>
       </c>
       <c r="T2" t="n">
-        <v>10.31467425679948</v>
+        <v>10.26974547362897</v>
       </c>
       <c r="U2" t="n">
-        <v>195.6899999999998</v>
+        <v>195.6900000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>5.157073582121028</v>
+        <v>5.13461033849383</v>
       </c>
       <c r="W2" t="n">
-        <v>97.84000000000015</v>
+        <v>97.83999999999992</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000102207686013</v>
+        <v>2.00010220768602</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>10.31467425679948</v>
+        <v>10.26974547362897</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.157073582121028</v>
+        <v>5.13461033849383</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02057577448759861</v>
+        <v>0.02057628779489107</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3266302939604003</v>
+        <v>0.3266384424610523</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909823423828552</v>
+        <v>0.02909817503180223</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266353098562824</v>
+        <v>0.04266353728064191</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869493934347614</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-16 14:09:41.844895+05:30</t>
+          <t>2026-09-16 20:26:35.040214+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.314674256799485, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001022076860133}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.269745473628971, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001022076860204}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-17 08:43 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="19" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="17" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H2" t="n">
         <v>8.699999999999999</v>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.69</v>
+        <v>11.81</v>
       </c>
       <c r="R2" t="n">
-        <v>49.2</v>
+        <v>48.99</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1924.6</v>
+        <v>1898</v>
       </c>
       <c r="V2" t="n">
-        <v>1940.4</v>
+        <v>1964.5</v>
       </c>
       <c r="W2" t="n">
-        <v>1863.5</v>
+        <v>1894.8</v>
       </c>
       <c r="X2" t="n">
-        <v>1905.5</v>
+        <v>1952.2</v>
       </c>
       <c r="Y2" t="n">
-        <v>1905.5</v>
+        <v>1952.2</v>
       </c>
       <c r="Z2" t="n">
-        <v>2870749</v>
+        <v>1153851</v>
       </c>
       <c r="AA2" t="n">
-        <v>3573474</v>
+        <v>3559881</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.8</v>
+        <v>0.32</v>
       </c>
       <c r="AC2" t="n">
-        <v>-1.11</v>
+        <v>2.45</v>
       </c>
       <c r="AD2" t="n">
-        <v>-0.12</v>
+        <v>-0.39</v>
       </c>
       <c r="AE2" t="n">
-        <v>76.90000000000001</v>
+        <v>69.7</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.04</v>
+        <v>3.57</v>
       </c>
       <c r="AG2" t="n">
-        <v>48.92</v>
+        <v>50.41</v>
       </c>
       <c r="AH2" t="n">
-        <v>48.92</v>
+        <v>50.41</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.57</v>
+        <v>2.58</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,119 +1926,119 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>0.82</v>
+        <v>2.88</v>
       </c>
       <c r="AM2" t="n">
-        <v>7.27</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="AN2" t="n">
-        <v>46.08</v>
+        <v>49.13</v>
       </c>
       <c r="AO2" t="n">
-        <v>56.04</v>
+        <v>61.58</v>
       </c>
       <c r="AP2" t="n">
-        <v>2.36</v>
+        <v>4.73</v>
       </c>
       <c r="AQ2" t="n">
-        <v>39.21</v>
+        <v>38.17</v>
       </c>
       <c r="AR2" t="n">
-        <v>1905.5</v>
+        <v>1952.2</v>
       </c>
       <c r="AS2" t="n">
-        <v>2101.19</v>
+        <v>2153.82</v>
       </c>
       <c r="AT2" t="n">
-        <v>1807.66</v>
+        <v>1851.39</v>
       </c>
       <c r="AU2" t="n">
-        <v>1905.5</v>
+        <v>1952.199951171875</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>10.27</v>
+        <v>10.33</v>
       </c>
       <c r="AY2" t="n">
-        <v>195.69</v>
+        <v>201.62</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.13</v>
+        <v>5.16</v>
       </c>
       <c r="BA2" t="n">
-        <v>97.84</v>
+        <v>100.81</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.05</v>
+        <v>2.04</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
       </c>
       <c r="BD2" t="n">
-        <v>32.4</v>
+        <v>32.3</v>
       </c>
       <c r="BE2" t="n">
         <v>326</v>
       </c>
       <c r="BF2" t="n">
-        <v>49.3</v>
+        <v>49.2</v>
       </c>
       <c r="BG2" t="n">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.2</v>
+        <v>18.4</v>
       </c>
       <c r="BI2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BM2" t="n">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="BN2" t="n">
-        <v>49.9</v>
+        <v>50.2</v>
       </c>
       <c r="BO2" t="n">
         <v>2.24</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.77</v>
+        <v>8.73</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.27</v>
+        <v>-4.28</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.245</v>
+        <v>0.246</v>
       </c>
       <c r="BT2" t="n">
-        <v>1479.51</v>
+        <v>1483.82</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.88</v>
+        <v>-13.43</v>
       </c>
       <c r="BV2" t="n">
         <v>2.05</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.05</v>
+        <v>2.04</v>
       </c>
       <c r="BX2" t="n">
-        <v>2.0001</v>
+        <v>2</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2047,7 +2047,7 @@
         <v>8</v>
       </c>
       <c r="CA2" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="CB2" t="n">
         <v>0</v>
@@ -2064,10 +2064,10 @@
         <v>52.5</v>
       </c>
       <c r="CF2" t="n">
-        <v>68.3</v>
+        <v>68</v>
       </c>
       <c r="CG2" t="n">
-        <v>71.3</v>
+        <v>71.7</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>75.05</v>
+        <v>81.48</v>
       </c>
       <c r="CO2" t="n">
-        <v>44.23</v>
+        <v>46.43</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2124,7 +2124,7 @@
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>10.2697</v>
+        <v>10.3278</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,52 +2133,52 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6847</v>
+        <v>0.6887</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.342</v>
+        <v>0.344</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1027</v>
+        <v>0.1033</v>
       </c>
       <c r="DF2" t="n">
         <v>2.0019</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.2006</v>
+        <v>1.22</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9961</v>
+        <v>4.0039</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.1346</v>
+        <v>5.1639</v>
       </c>
       <c r="DJ2" t="n">
-        <v>55.31</v>
+        <v>57.91</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.1346</v>
+        <v>5.1639</v>
       </c>
       <c r="DL2" t="n">
-        <v>2.0001</v>
+        <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>1.9961</v>
+        <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9961</v>
+        <v>4.0039</v>
       </c>
       <c r="DO2" t="n">
         <v>2.002</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.779</v>
+        <v>0.7759</v>
       </c>
       <c r="DQ2" t="n">
-        <v>97.84</v>
+        <v>100.81</v>
       </c>
       <c r="DR2" t="n">
-        <v>69.31</v>
+        <v>59.12</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2193,49 +2193,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.9183</v>
+        <v>1.8333</v>
       </c>
       <c r="DX2" t="n">
-        <v>90.09999999999999</v>
+        <v>96.05000000000001</v>
       </c>
       <c r="DY2" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="DZ2" t="n">
-        <v>78.928</v>
+        <v>85.313</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
       </c>
       <c r="EB2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>68.04000000000001</v>
+        <v>80.97</v>
       </c>
       <c r="ED2" t="n">
-        <v>96.16</v>
+        <v>98.98</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.9183</v>
+        <v>1.8333</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.8</v>
+        <v>0.32</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.2759</v>
+        <v>0.5586</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.996</v>
+        <v>4.003</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0323</v>
+        <v>0.066</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6519</v>
+        <v>0.6498</v>
       </c>
       <c r="EK2" t="n">
-        <v>60.63</v>
+        <v>71.73</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2246,37 +2246,37 @@
         <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>20.18</v>
+        <v>10.22</v>
       </c>
       <c r="EP2" t="n">
-        <v>2.359</v>
+        <v>1.207</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0935</v>
+        <v>0.0378</v>
       </c>
       <c r="ER2" t="n">
-        <v>12.8375</v>
+        <v>32.2812</v>
       </c>
       <c r="ES2" t="n">
-        <v>15.493</v>
+        <v>16.176</v>
       </c>
       <c r="ET2" t="n">
-        <v>42.841</v>
+        <v>40.904</v>
       </c>
       <c r="EU2" t="n">
-        <v>1.888</v>
+        <v>1.5136</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.4278</v>
+        <v>1.9545</v>
       </c>
       <c r="EW2" t="n">
-        <v>15.1451</v>
+        <v>8.327299999999999</v>
       </c>
       <c r="EX2" t="n">
-        <v>38.01</v>
+        <v>35.03</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2290,31 @@
         <v>9</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.65</v>
+        <v>64.22</v>
       </c>
       <c r="FC2" t="n">
-        <v>46.61</v>
+        <v>47.11</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.41</v>
+        <v>72.88</v>
       </c>
       <c r="FE2" t="n">
-        <v>67.84</v>
+        <v>76.605</v>
       </c>
       <c r="FF2" t="n">
-        <v>41.12</v>
+        <v>40.73</v>
       </c>
       <c r="FG2" t="n">
-        <v>21.0224</v>
+        <v>22.7598</v>
       </c>
       <c r="FH2" t="n">
-        <v>61.942</v>
+        <v>63.56</v>
       </c>
       <c r="FI2" t="n">
-        <v>62.31</v>
+        <v>58.515</v>
       </c>
       <c r="FJ2" t="n">
-        <v>69.65000000000001</v>
+        <v>71.88</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>76.88</v>
+        <v>81.03</v>
       </c>
       <c r="FO2" t="n">
-        <v>66.43000000000001</v>
+        <v>75.45</v>
       </c>
       <c r="FP2" t="n">
-        <v>67.51000000000001</v>
+        <v>64.84999999999999</v>
       </c>
       <c r="FQ2" t="n">
-        <v>82.73</v>
+        <v>83.22</v>
       </c>
       <c r="FR2" t="n">
-        <v>85.09</v>
+        <v>88.92</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>75.16800000000001</v>
+        <v>76.3905</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260916_202634</t>
+          <t>20260917_141324</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46281.85179397242</v>
+        <v>46282.59264688721</v>
       </c>
     </row>
   </sheetData>
@@ -2464,9 +2464,9 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
-    <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="23" max="23"/>
+    <col width="19" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46281.85179398148</v>
+        <v>46282.59263888889</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.69</v>
+        <v>11.81</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1905.5</v>
+        <v>1952.2</v>
       </c>
       <c r="L2" t="n">
-        <v>1924.6</v>
+        <v>1898</v>
       </c>
       <c r="M2" t="n">
-        <v>1940.4</v>
+        <v>1964.5</v>
       </c>
       <c r="N2" t="n">
-        <v>1863.5</v>
+        <v>1894.8</v>
       </c>
       <c r="O2" t="n">
-        <v>1905.5</v>
+        <v>1952.2</v>
       </c>
       <c r="P2" t="n">
-        <v>2870749</v>
+        <v>1153851</v>
       </c>
       <c r="Q2" t="n">
-        <v>1905.5</v>
+        <v>1952.2</v>
       </c>
       <c r="R2" t="n">
-        <v>2101.19</v>
+        <v>2153.82</v>
       </c>
       <c r="S2" t="n">
-        <v>1807.66</v>
+        <v>1851.39</v>
       </c>
       <c r="T2" t="n">
-        <v>10.26974547362897</v>
+        <v>10.32783526278046</v>
       </c>
       <c r="U2" t="n">
-        <v>195.6900000000001</v>
+        <v>201.6200000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>5.13461033849383</v>
+        <v>5.163917631390223</v>
       </c>
       <c r="W2" t="n">
-        <v>97.83999999999992</v>
+        <v>100.8099999999999</v>
       </c>
       <c r="X2" t="n">
-        <v>2.00010220768602</v>
+        <v>2.000000000000002</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>10.26974547362897</v>
+        <v>10.32783526278046</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.13461033849383</v>
+        <v>5.163917631390223</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02057628779489107</v>
+        <v>0.02058657306202866</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3266384424610523</v>
+        <v>0.3268017160151358</v>
       </c>
     </row>
     <row r="7">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266353728064191</v>
+        <v>0.04266353057055038</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347614</v>
+        <v>0.1869492979645464</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.87</v>
+        <v>38.86</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-16 20:26:35.040214+05:30</t>
+          <t>2026-09-17 14:13:24.724444+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.269745473628971, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001022076860204}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.327835262780459, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000000000000002}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-17 14:58 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="19" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="17" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1864,7 +1864,7 @@
         <v>11.81</v>
       </c>
       <c r="R2" t="n">
-        <v>48.99</v>
+        <v>49.05</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1884,22 +1884,22 @@
         <v>1894.8</v>
       </c>
       <c r="X2" t="n">
-        <v>1952.2</v>
+        <v>1948.1</v>
       </c>
       <c r="Y2" t="n">
-        <v>1952.2</v>
+        <v>1948.1</v>
       </c>
       <c r="Z2" t="n">
-        <v>1153851</v>
+        <v>1645038</v>
       </c>
       <c r="AA2" t="n">
-        <v>3559881</v>
+        <v>3584440</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.32</v>
+        <v>0.46</v>
       </c>
       <c r="AC2" t="n">
-        <v>2.45</v>
+        <v>2.24</v>
       </c>
       <c r="AD2" t="n">
         <v>-0.39</v>
@@ -1908,7 +1908,7 @@
         <v>69.7</v>
       </c>
       <c r="AF2" t="n">
-        <v>3.57</v>
+        <v>3.58</v>
       </c>
       <c r="AG2" t="n">
         <v>50.41</v>
@@ -1917,7 +1917,7 @@
         <v>50.41</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.58</v>
+        <v>2.59</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,47 +1926,47 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>2.88</v>
+        <v>2.68</v>
       </c>
       <c r="AM2" t="n">
-        <v>9.300000000000001</v>
+        <v>9.08</v>
       </c>
       <c r="AN2" t="n">
-        <v>49.13</v>
+        <v>48.82</v>
       </c>
       <c r="AO2" t="n">
-        <v>61.58</v>
+        <v>61.15</v>
       </c>
       <c r="AP2" t="n">
-        <v>4.73</v>
+        <v>4.51</v>
       </c>
       <c r="AQ2" t="n">
-        <v>38.17</v>
+        <v>37.88</v>
       </c>
       <c r="AR2" t="n">
-        <v>1952.2</v>
+        <v>1948.1</v>
       </c>
       <c r="AS2" t="n">
-        <v>2153.82</v>
+        <v>2149.72</v>
       </c>
       <c r="AT2" t="n">
-        <v>1851.39</v>
+        <v>1847.29</v>
       </c>
       <c r="AU2" t="n">
-        <v>1952.199951171875</v>
+        <v>1948.099975585938</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>10.33</v>
+        <v>10.35</v>
       </c>
       <c r="AY2" t="n">
         <v>201.62</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.16</v>
+        <v>5.17</v>
       </c>
       <c r="BA2" t="n">
         <v>100.81</v>
@@ -2026,10 +2026,10 @@
         <v>0.246</v>
       </c>
       <c r="BT2" t="n">
-        <v>1483.82</v>
+        <v>1483.48</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.43</v>
+        <v>-13.47</v>
       </c>
       <c r="BV2" t="n">
         <v>2.05</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>81.48</v>
+        <v>82.97</v>
       </c>
       <c r="CO2" t="n">
-        <v>46.43</v>
+        <v>48.83</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2124,7 +2124,7 @@
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>10.3278</v>
+        <v>10.3496</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,52 +2133,52 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6887</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.344</v>
+        <v>0.3447</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1033</v>
+        <v>0.1035</v>
       </c>
       <c r="DF2" t="n">
         <v>2.0019</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.22</v>
+        <v>1.2223</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0039</v>
+        <v>3.9961</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.1639</v>
+        <v>5.1748</v>
       </c>
       <c r="DJ2" t="n">
-        <v>57.91</v>
+        <v>58.15</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.1639</v>
+        <v>5.1748</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>2</v>
+        <v>1.9961</v>
       </c>
       <c r="DN2" t="n">
-        <v>4.0039</v>
+        <v>3.9961</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.002</v>
+        <v>2.0017</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.7759</v>
+        <v>0.7729</v>
       </c>
       <c r="DQ2" t="n">
         <v>100.81</v>
       </c>
       <c r="DR2" t="n">
-        <v>59.12</v>
+        <v>65</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.8333</v>
+        <v>1.7413</v>
       </c>
       <c r="DX2" t="n">
-        <v>96.05000000000001</v>
+        <v>97.125</v>
       </c>
       <c r="DY2" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="DZ2" t="n">
-        <v>85.313</v>
+        <v>85.446</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>80.97</v>
+        <v>81.17</v>
       </c>
       <c r="ED2" t="n">
-        <v>98.98</v>
+        <v>100</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.8333</v>
+        <v>1.7413</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.32</v>
+        <v>0.46</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.5586</v>
+        <v>0.5326</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.003</v>
+        <v>3.996</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.066</v>
+        <v>0.0629</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6498</v>
+        <v>0.6476</v>
       </c>
       <c r="EK2" t="n">
-        <v>71.73</v>
+        <v>68.66</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2249,34 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>10.22</v>
+        <v>11.19</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.207</v>
+        <v>1.3215</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0378</v>
+        <v>0.0543</v>
       </c>
       <c r="ER2" t="n">
-        <v>32.2812</v>
+        <v>22.5</v>
       </c>
       <c r="ES2" t="n">
-        <v>16.176</v>
+        <v>16.1978</v>
       </c>
       <c r="ET2" t="n">
-        <v>40.904</v>
+        <v>42.155</v>
       </c>
       <c r="EU2" t="n">
-        <v>1.5136</v>
+        <v>2.0746</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.9545</v>
+        <v>1.774</v>
       </c>
       <c r="EW2" t="n">
-        <v>8.327299999999999</v>
+        <v>9.2843</v>
       </c>
       <c r="EX2" t="n">
-        <v>35.03</v>
+        <v>37.43</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2293,28 +2293,28 @@
         <v>64.22</v>
       </c>
       <c r="FC2" t="n">
-        <v>47.11</v>
+        <v>47.68</v>
       </c>
       <c r="FD2" t="n">
-        <v>72.88</v>
+        <v>72.98999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>76.605</v>
+        <v>75.815</v>
       </c>
       <c r="FF2" t="n">
-        <v>40.73</v>
+        <v>43.13</v>
       </c>
       <c r="FG2" t="n">
-        <v>22.7598</v>
+        <v>23.1114</v>
       </c>
       <c r="FH2" t="n">
-        <v>63.56</v>
+        <v>64.48699999999999</v>
       </c>
       <c r="FI2" t="n">
-        <v>58.515</v>
+        <v>61.575</v>
       </c>
       <c r="FJ2" t="n">
-        <v>71.88</v>
+        <v>72.29000000000001</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>81.03</v>
+        <v>82.17</v>
       </c>
       <c r="FO2" t="n">
-        <v>75.45</v>
+        <v>75</v>
       </c>
       <c r="FP2" t="n">
-        <v>64.84999999999999</v>
+        <v>67.79000000000001</v>
       </c>
       <c r="FQ2" t="n">
-        <v>83.22</v>
+        <v>85.31</v>
       </c>
       <c r="FR2" t="n">
-        <v>88.92</v>
+        <v>89.39</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>76.3905</v>
+        <v>77.6255</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260917_141324</t>
+          <t>20260917_202807</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46282.59264688721</v>
+        <v>46282.85286566643</v>
       </c>
     </row>
   </sheetData>
@@ -2466,7 +2466,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="20" customWidth="1" min="23" max="23"/>
-    <col width="19" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46282.59263888889</v>
+        <v>46282.85285879629</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46282</v>
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1952.2</v>
+        <v>1948.1</v>
       </c>
       <c r="L2" t="n">
         <v>1898</v>
@@ -2693,34 +2693,34 @@
         <v>1894.8</v>
       </c>
       <c r="O2" t="n">
-        <v>1952.2</v>
+        <v>1948.1</v>
       </c>
       <c r="P2" t="n">
-        <v>1153851</v>
+        <v>1645038</v>
       </c>
       <c r="Q2" t="n">
-        <v>1952.2</v>
+        <v>1948.1</v>
       </c>
       <c r="R2" t="n">
-        <v>2153.82</v>
+        <v>2149.72</v>
       </c>
       <c r="S2" t="n">
-        <v>1851.39</v>
+        <v>1847.29</v>
       </c>
       <c r="T2" t="n">
-        <v>10.32783526278046</v>
+        <v>10.34957137723936</v>
       </c>
       <c r="U2" t="n">
-        <v>201.6200000000001</v>
+        <v>201.6199999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>5.163917631390223</v>
+        <v>5.174785688619679</v>
       </c>
       <c r="W2" t="n">
         <v>100.8099999999999</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000000000000002</v>
+        <v>2</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>10.32783526278046</v>
+        <v>10.34957137723936</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.163917631390223</v>
+        <v>5.174785688619679</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02058657306202866</v>
+        <v>0.02057513998721375</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3268017160151358</v>
+        <v>0.3266202215790496</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909817503180223</v>
+        <v>0.02909811582531894</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266353057055038</v>
+        <v>0.04266352966163063</v>
       </c>
     </row>
     <row r="13">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.86</v>
+        <v>38.87</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-17 14:13:24.724444+05:30</t>
+          <t>2026-09-17 20:28:07.617694+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.327835262780459, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000000000000002}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.349571377239357, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-18 08:19 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="20" customWidth="1" min="47" max="47"/>
+    <col width="19" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="17" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H2" t="n">
         <v>8.699999999999999</v>
@@ -1864,7 +1864,7 @@
         <v>11.81</v>
       </c>
       <c r="R2" t="n">
-        <v>49.05</v>
+        <v>49.06</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,46 +1875,46 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1898</v>
+        <v>1962</v>
       </c>
       <c r="V2" t="n">
-        <v>1964.5</v>
+        <v>1982</v>
       </c>
       <c r="W2" t="n">
-        <v>1894.8</v>
+        <v>1955.3</v>
       </c>
       <c r="X2" t="n">
-        <v>1948.1</v>
+        <v>1968.2</v>
       </c>
       <c r="Y2" t="n">
-        <v>1948.1</v>
+        <v>1968.2</v>
       </c>
       <c r="Z2" t="n">
-        <v>1645038</v>
+        <v>1695948</v>
       </c>
       <c r="AA2" t="n">
-        <v>3584440</v>
+        <v>3586986</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.46</v>
+        <v>0.47</v>
       </c>
       <c r="AC2" t="n">
-        <v>2.24</v>
+        <v>3.29</v>
       </c>
       <c r="AD2" t="n">
-        <v>-0.39</v>
+        <v>2.97</v>
       </c>
       <c r="AE2" t="n">
-        <v>69.7</v>
+        <v>26.7</v>
       </c>
       <c r="AF2" t="n">
-        <v>3.58</v>
+        <v>1.36</v>
       </c>
       <c r="AG2" t="n">
-        <v>50.41</v>
+        <v>50.89</v>
       </c>
       <c r="AH2" t="n">
-        <v>50.41</v>
+        <v>50.89</v>
       </c>
       <c r="AI2" t="n">
         <v>2.59</v>
@@ -1926,50 +1926,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>2.68</v>
+        <v>3.68</v>
       </c>
       <c r="AM2" t="n">
-        <v>9.08</v>
+        <v>10.18</v>
       </c>
       <c r="AN2" t="n">
-        <v>48.82</v>
+        <v>50.34</v>
       </c>
       <c r="AO2" t="n">
-        <v>61.15</v>
+        <v>63.17</v>
       </c>
       <c r="AP2" t="n">
-        <v>4.51</v>
+        <v>5.59</v>
       </c>
       <c r="AQ2" t="n">
-        <v>37.88</v>
+        <v>39.3</v>
       </c>
       <c r="AR2" t="n">
-        <v>1948.1</v>
+        <v>1968.2</v>
       </c>
       <c r="AS2" t="n">
-        <v>2149.72</v>
+        <v>2171.77</v>
       </c>
       <c r="AT2" t="n">
-        <v>1847.29</v>
+        <v>1866.42</v>
       </c>
       <c r="AU2" t="n">
-        <v>1948.099975585938</v>
+        <v>1968.199951171875</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>10.35</v>
+        <v>10.34</v>
       </c>
       <c r="AY2" t="n">
-        <v>201.62</v>
+        <v>203.57</v>
       </c>
       <c r="AZ2" t="n">
         <v>5.17</v>
       </c>
       <c r="BA2" t="n">
-        <v>100.81</v>
+        <v>101.78</v>
       </c>
       <c r="BB2" t="n">
         <v>2.04</v>
@@ -2014,7 +2014,7 @@
         <v>2.24</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.73</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="BQ2" t="n">
         <v>-4.28</v>
@@ -2026,10 +2026,10 @@
         <v>0.246</v>
       </c>
       <c r="BT2" t="n">
-        <v>1483.48</v>
+        <v>1482.44</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.47</v>
+        <v>-13.57</v>
       </c>
       <c r="BV2" t="n">
         <v>2.05</v>
@@ -2038,7 +2038,7 @@
         <v>2.04</v>
       </c>
       <c r="BX2" t="n">
-        <v>2</v>
+        <v>2.0001</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>82.97</v>
+        <v>88.25</v>
       </c>
       <c r="CO2" t="n">
-        <v>48.83</v>
+        <v>53.52</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2124,7 +2124,7 @@
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>10.3496</v>
+        <v>10.343</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.6893</v>
       </c>
       <c r="DD2" t="n">
         <v>0.3447</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1035</v>
+        <v>0.1034</v>
       </c>
       <c r="DF2" t="n">
-        <v>2.0019</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.2223</v>
+        <v>1.2212</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9961</v>
+        <v>3.9923</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.1748</v>
+        <v>5.1712</v>
       </c>
       <c r="DJ2" t="n">
-        <v>58.15</v>
+        <v>60.95</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.1748</v>
+        <v>5.1712</v>
       </c>
       <c r="DL2" t="n">
-        <v>2</v>
+        <v>2.0001</v>
       </c>
       <c r="DM2" t="n">
         <v>1.9961</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9961</v>
+        <v>3.9923</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0017</v>
+        <v>1.9997</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.7729</v>
+        <v>0.7722</v>
       </c>
       <c r="DQ2" t="n">
-        <v>100.81</v>
+        <v>101.78</v>
       </c>
       <c r="DR2" t="n">
-        <v>65</v>
+        <v>43.94</v>
       </c>
       <c r="DS2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="DT2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,49 +2193,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.7413</v>
+        <v>2.1583</v>
       </c>
       <c r="DX2" t="n">
-        <v>97.125</v>
+        <v>92.07499999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>23</v>
+        <v>23.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>85.446</v>
+        <v>86.40600000000001</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
       </c>
       <c r="EB2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>81.17</v>
+        <v>81.2</v>
       </c>
       <c r="ED2" t="n">
-        <v>100</v>
+        <v>89.22</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.7413</v>
+        <v>2.1583</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.46</v>
+        <v>0.47</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.5326</v>
+        <v>0.6602</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.996</v>
+        <v>3.9934</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0629</v>
+        <v>0.078</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6476</v>
+        <v>0.6472</v>
       </c>
       <c r="EK2" t="n">
-        <v>68.66</v>
+        <v>66.73999999999999</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2246,37 +2246,37 @@
         <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>11.19</v>
+        <v>24.28</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.3215</v>
+        <v>2.8675</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0543</v>
+        <v>0.0555</v>
       </c>
       <c r="ER2" t="n">
-        <v>22.5</v>
+        <v>22</v>
       </c>
       <c r="ES2" t="n">
-        <v>16.1978</v>
+        <v>16.9777</v>
       </c>
       <c r="ET2" t="n">
-        <v>42.155</v>
+        <v>47.958</v>
       </c>
       <c r="EU2" t="n">
-        <v>2.0746</v>
+        <v>2.6273</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.774</v>
+        <v>1.7619</v>
       </c>
       <c r="EW2" t="n">
-        <v>9.2843</v>
+        <v>21.4271</v>
       </c>
       <c r="EX2" t="n">
-        <v>37.43</v>
+        <v>37</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2287,34 +2287,34 @@
         <v>5</v>
       </c>
       <c r="FA2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="FB2" t="n">
         <v>64.22</v>
       </c>
       <c r="FC2" t="n">
-        <v>47.68</v>
+        <v>51.24</v>
       </c>
       <c r="FD2" t="n">
-        <v>72.98999999999999</v>
+        <v>72.73</v>
       </c>
       <c r="FE2" t="n">
-        <v>75.815</v>
+        <v>77.495</v>
       </c>
       <c r="FF2" t="n">
-        <v>43.13</v>
+        <v>45.26</v>
       </c>
       <c r="FG2" t="n">
-        <v>23.1114</v>
+        <v>24.5822</v>
       </c>
       <c r="FH2" t="n">
-        <v>64.48699999999999</v>
+        <v>65.985</v>
       </c>
       <c r="FI2" t="n">
-        <v>61.575</v>
+        <v>52.445</v>
       </c>
       <c r="FJ2" t="n">
-        <v>72.29000000000001</v>
+        <v>73.45</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>82.17</v>
+        <v>74.73</v>
       </c>
       <c r="FO2" t="n">
-        <v>75</v>
+        <v>78.65000000000001</v>
       </c>
       <c r="FP2" t="n">
-        <v>67.79000000000001</v>
+        <v>53.19</v>
       </c>
       <c r="FQ2" t="n">
-        <v>85.31</v>
+        <v>72.88</v>
       </c>
       <c r="FR2" t="n">
-        <v>89.39</v>
+        <v>85.77</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>77.6255</v>
+        <v>73.3085</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260917_202807</t>
+          <t>20260918_134908</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46282.85286566643</v>
+        <v>46283.57579704429</v>
       </c>
     </row>
   </sheetData>
@@ -2466,7 +2466,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="20" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="19" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46282.85285879629</v>
+        <v>46283.57578703704</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1948.1</v>
+        <v>1968.2</v>
       </c>
       <c r="L2" t="n">
-        <v>1898</v>
+        <v>1962</v>
       </c>
       <c r="M2" t="n">
-        <v>1964.5</v>
+        <v>1982</v>
       </c>
       <c r="N2" t="n">
-        <v>1894.8</v>
+        <v>1955.3</v>
       </c>
       <c r="O2" t="n">
-        <v>1948.1</v>
+        <v>1968.2</v>
       </c>
       <c r="P2" t="n">
-        <v>1645038</v>
+        <v>1695948</v>
       </c>
       <c r="Q2" t="n">
-        <v>1948.1</v>
+        <v>1968.2</v>
       </c>
       <c r="R2" t="n">
-        <v>2149.72</v>
+        <v>2171.77</v>
       </c>
       <c r="S2" t="n">
-        <v>1847.29</v>
+        <v>1866.42</v>
       </c>
       <c r="T2" t="n">
-        <v>10.34957137723936</v>
+        <v>10.34295295193578</v>
       </c>
       <c r="U2" t="n">
-        <v>201.6199999999999</v>
+        <v>203.5699999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>5.174785688619679</v>
+        <v>5.171222436744232</v>
       </c>
       <c r="W2" t="n">
-        <v>100.8099999999999</v>
+        <v>101.78</v>
       </c>
       <c r="X2" t="n">
-        <v>2</v>
+        <v>2.000098251129888</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>10.34957137723936</v>
+        <v>10.34295295193578</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.174785688619679</v>
+        <v>5.171222436744232</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02057513998721375</v>
+        <v>0.02057905073368083</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3266202215790496</v>
+        <v>0.3266823027546046</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909811582531894</v>
+        <v>0.02909805661883564</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266352966163063</v>
+        <v>0.0426635290707733</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869493934347615</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-17 20:28:07.617694+05:30</t>
+          <t>2026-09-18 13:49:08.903374+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.349571377239357, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.342952951935775, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000098251129888}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-18 14:28 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="19" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="17" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>STRONG BUY</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.81</v>
+        <v>11.7</v>
       </c>
       <c r="R2" t="n">
-        <v>49.06</v>
+        <v>49.07</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1881,43 +1881,43 @@
         <v>1982</v>
       </c>
       <c r="W2" t="n">
-        <v>1955.3</v>
+        <v>1954</v>
       </c>
       <c r="X2" t="n">
-        <v>1968.2</v>
+        <v>1954</v>
       </c>
       <c r="Y2" t="n">
-        <v>1968.2</v>
+        <v>1954</v>
       </c>
       <c r="Z2" t="n">
-        <v>1695948</v>
+        <v>2655873</v>
       </c>
       <c r="AA2" t="n">
-        <v>3586986</v>
+        <v>3626662</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.47</v>
+        <v>0.73</v>
       </c>
       <c r="AC2" t="n">
-        <v>3.29</v>
+        <v>2.55</v>
       </c>
       <c r="AD2" t="n">
         <v>2.97</v>
       </c>
       <c r="AE2" t="n">
-        <v>26.7</v>
+        <v>28</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.36</v>
+        <v>1.43</v>
       </c>
       <c r="AG2" t="n">
-        <v>50.89</v>
+        <v>49.88</v>
       </c>
       <c r="AH2" t="n">
-        <v>50.89</v>
+        <v>49.88</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.59</v>
+        <v>2.55</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>3.68</v>
+        <v>2.83</v>
       </c>
       <c r="AM2" t="n">
-        <v>10.18</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="AN2" t="n">
-        <v>50.34</v>
+        <v>48.78</v>
       </c>
       <c r="AO2" t="n">
-        <v>63.17</v>
+        <v>61.86</v>
       </c>
       <c r="AP2" t="n">
-        <v>5.59</v>
+        <v>4.58</v>
       </c>
       <c r="AQ2" t="n">
-        <v>39.3</v>
+        <v>36.08</v>
       </c>
       <c r="AR2" t="n">
-        <v>1968.2</v>
+        <v>1954</v>
       </c>
       <c r="AS2" t="n">
-        <v>2171.77</v>
+        <v>2153.51</v>
       </c>
       <c r="AT2" t="n">
-        <v>1866.42</v>
+        <v>1854.24</v>
       </c>
       <c r="AU2" t="n">
-        <v>1968.199951171875</v>
+        <v>1954</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>10.34</v>
+        <v>10.21</v>
       </c>
       <c r="AY2" t="n">
-        <v>203.57</v>
+        <v>199.51</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.17</v>
+        <v>5.11</v>
       </c>
       <c r="BA2" t="n">
-        <v>101.78</v>
+        <v>99.76000000000001</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.04</v>
+        <v>2.05</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
@@ -1981,64 +1981,64 @@
         <v>32.3</v>
       </c>
       <c r="BE2" t="n">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="BF2" t="n">
-        <v>49.2</v>
+        <v>49.3</v>
       </c>
       <c r="BG2" t="n">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.4</v>
+        <v>18.3</v>
       </c>
       <c r="BI2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BM2" t="n">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="BN2" t="n">
-        <v>50.2</v>
+        <v>49.9</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.24</v>
+        <v>2.23</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.720000000000001</v>
+        <v>8.75</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.28</v>
+        <v>-4.27</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.246</v>
+        <v>0.245</v>
       </c>
       <c r="BT2" t="n">
-        <v>1482.44</v>
+        <v>1476.8</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.57</v>
+        <v>-14.17</v>
       </c>
       <c r="BV2" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="BW2" t="n">
         <v>2.05</v>
       </c>
-      <c r="BW2" t="n">
-        <v>2.04</v>
-      </c>
       <c r="BX2" t="n">
-        <v>2.0001</v>
+        <v>1.9999</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2047,7 +2047,7 @@
         <v>8</v>
       </c>
       <c r="CA2" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="CB2" t="n">
         <v>0</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>44.8</v>
+        <v>44.6</v>
       </c>
       <c r="CE2" t="n">
-        <v>52.5</v>
+        <v>52</v>
       </c>
       <c r="CF2" t="n">
-        <v>68</v>
+        <v>68.3</v>
       </c>
       <c r="CG2" t="n">
-        <v>71.7</v>
+        <v>71.3</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>88.25</v>
+        <v>82.06</v>
       </c>
       <c r="CO2" t="n">
-        <v>53.52</v>
+        <v>37.56</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2112,7 +2112,7 @@
         <v>95.45454545454545</v>
       </c>
       <c r="CV2" t="n">
-        <v>86.36363636363636</v>
+        <v>81.81818181818183</v>
       </c>
       <c r="CW2" t="n">
         <v>68.18181818181817</v>
@@ -2124,7 +2124,7 @@
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>10.343</v>
+        <v>10.2103</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6893</v>
+        <v>0.6807</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3447</v>
+        <v>0.3407</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1034</v>
+        <v>0.1021</v>
       </c>
       <c r="DF2" t="n">
-        <v>2</v>
+        <v>1.998</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.2212</v>
+        <v>1.1946</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9923</v>
+        <v>4.0039</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.1712</v>
+        <v>5.1054</v>
       </c>
       <c r="DJ2" t="n">
-        <v>60.95</v>
+        <v>57.86</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.1712</v>
+        <v>5.1054</v>
       </c>
       <c r="DL2" t="n">
-        <v>2.0001</v>
+        <v>1.9999</v>
       </c>
       <c r="DM2" t="n">
-        <v>1.9961</v>
+        <v>2.0039</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9923</v>
+        <v>4.0039</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9997</v>
+        <v>1.9979</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.7722</v>
+        <v>0.7835</v>
       </c>
       <c r="DQ2" t="n">
-        <v>101.78</v>
+        <v>99.76000000000001</v>
       </c>
       <c r="DR2" t="n">
-        <v>43.94</v>
+        <v>38.54</v>
       </c>
       <c r="DS2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="DT2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>2.1583</v>
+        <v>1.7961</v>
       </c>
       <c r="DX2" t="n">
-        <v>92.07499999999999</v>
+        <v>95.34999999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>23.5</v>
+        <v>36.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>86.40600000000001</v>
+        <v>79.491</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>81.2</v>
+        <v>72.13</v>
       </c>
       <c r="ED2" t="n">
-        <v>89.22</v>
+        <v>94.98999999999999</v>
       </c>
       <c r="EE2" t="n">
-        <v>2.1583</v>
+        <v>1.7961</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.47</v>
+        <v>0.73</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.6602</v>
+        <v>0.5359</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9934</v>
+        <v>4.004</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.078</v>
+        <v>0.06270000000000001</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6472</v>
+        <v>0.6553</v>
       </c>
       <c r="EK2" t="n">
-        <v>66.73999999999999</v>
+        <v>70.45</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2246,37 +2246,37 @@
         <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>24.28</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="EP2" t="n">
-        <v>2.8675</v>
+        <v>0.9407</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0555</v>
+        <v>0.0854</v>
       </c>
       <c r="ER2" t="n">
-        <v>22</v>
+        <v>13.9863</v>
       </c>
       <c r="ES2" t="n">
-        <v>16.9777</v>
+        <v>16.2986</v>
       </c>
       <c r="ET2" t="n">
-        <v>47.958</v>
+        <v>36.504</v>
       </c>
       <c r="EU2" t="n">
-        <v>2.6273</v>
+        <v>3.3434</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.7619</v>
+        <v>1.474</v>
       </c>
       <c r="EW2" t="n">
-        <v>21.4271</v>
+        <v>6.5976</v>
       </c>
       <c r="EX2" t="n">
-        <v>37</v>
+        <v>30.2</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2284,37 +2284,37 @@
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="FA2" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="FB2" t="n">
-        <v>64.22</v>
+        <v>63.56</v>
       </c>
       <c r="FC2" t="n">
-        <v>51.24</v>
+        <v>47.05</v>
       </c>
       <c r="FD2" t="n">
-        <v>72.73</v>
+        <v>73.27</v>
       </c>
       <c r="FE2" t="n">
-        <v>77.495</v>
+        <v>76.255</v>
       </c>
       <c r="FF2" t="n">
-        <v>45.26</v>
+        <v>33.88</v>
       </c>
       <c r="FG2" t="n">
-        <v>24.5822</v>
+        <v>23.1155</v>
       </c>
       <c r="FH2" t="n">
-        <v>65.985</v>
+        <v>62.438</v>
       </c>
       <c r="FI2" t="n">
-        <v>52.445</v>
+        <v>48.2</v>
       </c>
       <c r="FJ2" t="n">
-        <v>73.45</v>
+        <v>71.42</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>74.73</v>
+        <v>71.33</v>
       </c>
       <c r="FO2" t="n">
-        <v>78.65000000000001</v>
+        <v>77.84</v>
       </c>
       <c r="FP2" t="n">
-        <v>53.19</v>
+        <v>44.98</v>
       </c>
       <c r="FQ2" t="n">
-        <v>72.88</v>
+        <v>67.7</v>
       </c>
       <c r="FR2" t="n">
-        <v>85.77</v>
+        <v>82.18000000000001</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>73.3085</v>
+        <v>69.834</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260918_134908</t>
+          <t>20260918_195842</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46283.57579704429</v>
+        <v>46283.83243661495</v>
       </c>
     </row>
   </sheetData>
@@ -2464,9 +2464,9 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="20" customWidth="1" min="23" max="23"/>
-    <col width="19" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46283.57578703704</v>
+        <v>46283.83243055556</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46283</v>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.81</v>
+        <v>11.7</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1968.2</v>
+        <v>1954</v>
       </c>
       <c r="L2" t="n">
         <v>1962</v>
@@ -2690,37 +2690,37 @@
         <v>1982</v>
       </c>
       <c r="N2" t="n">
-        <v>1955.3</v>
+        <v>1954</v>
       </c>
       <c r="O2" t="n">
-        <v>1968.2</v>
+        <v>1954</v>
       </c>
       <c r="P2" t="n">
-        <v>1695948</v>
+        <v>2655873</v>
       </c>
       <c r="Q2" t="n">
-        <v>1968.2</v>
+        <v>1954</v>
       </c>
       <c r="R2" t="n">
-        <v>2171.77</v>
+        <v>2153.51</v>
       </c>
       <c r="S2" t="n">
-        <v>1866.42</v>
+        <v>1854.24</v>
       </c>
       <c r="T2" t="n">
-        <v>10.34295295193578</v>
+        <v>10.21033776867964</v>
       </c>
       <c r="U2" t="n">
-        <v>203.5699999999999</v>
+        <v>199.5100000000002</v>
       </c>
       <c r="V2" t="n">
-        <v>5.171222436744232</v>
+        <v>5.105424769703172</v>
       </c>
       <c r="W2" t="n">
-        <v>101.78</v>
+        <v>99.75999999999999</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000098251129888</v>
+        <v>1.999899759422617</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>10.34295295193578</v>
+        <v>10.21033776867964</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.171222436744232</v>
+        <v>5.105424769703172</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02057905073368083</v>
+        <v>0.02049518580591932</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3266823027546046</v>
+        <v>0.3253509882991407</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909805661883564</v>
+        <v>0.02909799741235235</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.0426635290707733</v>
+        <v>0.04266353403342596</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347615</v>
+        <v>0.1869492979645463</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.87</v>
+        <v>38.97</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-18 13:49:08.903374+05:30</t>
+          <t>2026-09-18 19:58:42.561272+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.342952951935775, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000098251129888}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.210337768679642, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998997594226167}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-21 09:02 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="17" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46283</v>
+        <v>46286</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46283</v>
+        <v>46286</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46283</v>
+        <v>46286</v>
       </c>
       <c r="H2" t="n">
         <v>8.699999999999999</v>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.7</v>
+        <v>11.82</v>
       </c>
       <c r="R2" t="n">
-        <v>49.07</v>
+        <v>49.04</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1962</v>
+        <v>1966.6</v>
       </c>
       <c r="V2" t="n">
-        <v>1982</v>
+        <v>2023.5</v>
       </c>
       <c r="W2" t="n">
-        <v>1954</v>
+        <v>1963.8</v>
       </c>
       <c r="X2" t="n">
-        <v>1954</v>
+        <v>2015.5</v>
       </c>
       <c r="Y2" t="n">
-        <v>1954</v>
+        <v>2015.5</v>
       </c>
       <c r="Z2" t="n">
-        <v>2655873</v>
+        <v>1857943</v>
       </c>
       <c r="AA2" t="n">
-        <v>3626662</v>
+        <v>3649459</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.73</v>
+        <v>0.51</v>
       </c>
       <c r="AC2" t="n">
-        <v>2.55</v>
+        <v>3.15</v>
       </c>
       <c r="AD2" t="n">
-        <v>2.97</v>
+        <v>0.64</v>
       </c>
       <c r="AE2" t="n">
-        <v>28</v>
+        <v>59.7</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.43</v>
+        <v>2.96</v>
       </c>
       <c r="AG2" t="n">
-        <v>49.88</v>
+        <v>51.28</v>
       </c>
       <c r="AH2" t="n">
-        <v>49.88</v>
+        <v>51.28</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.55</v>
+        <v>2.54</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,119 +1926,119 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>2.83</v>
+        <v>5.48</v>
       </c>
       <c r="AM2" t="n">
-        <v>8.949999999999999</v>
+        <v>11.78</v>
       </c>
       <c r="AN2" t="n">
-        <v>48.78</v>
+        <v>52.88</v>
       </c>
       <c r="AO2" t="n">
-        <v>61.86</v>
+        <v>67.81999999999999</v>
       </c>
       <c r="AP2" t="n">
-        <v>4.58</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="AQ2" t="n">
-        <v>36.08</v>
+        <v>36.09</v>
       </c>
       <c r="AR2" t="n">
-        <v>1954</v>
+        <v>2015.5</v>
       </c>
       <c r="AS2" t="n">
-        <v>2153.51</v>
+        <v>2220.62</v>
       </c>
       <c r="AT2" t="n">
-        <v>1854.24</v>
+        <v>1912.94</v>
       </c>
       <c r="AU2" t="n">
-        <v>1954</v>
+        <v>2015.5</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>10.21</v>
+        <v>10.18</v>
       </c>
       <c r="AY2" t="n">
-        <v>199.51</v>
+        <v>205.12</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.11</v>
+        <v>5.09</v>
       </c>
       <c r="BA2" t="n">
-        <v>99.76000000000001</v>
+        <v>102.56</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.05</v>
+        <v>2.04</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
       </c>
       <c r="BD2" t="n">
-        <v>32.3</v>
+        <v>32.2</v>
       </c>
       <c r="BE2" t="n">
         <v>327</v>
       </c>
       <c r="BF2" t="n">
-        <v>49.3</v>
+        <v>49.2</v>
       </c>
       <c r="BG2" t="n">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.3</v>
+        <v>18.5</v>
       </c>
       <c r="BI2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BM2" t="n">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="BN2" t="n">
-        <v>49.9</v>
+        <v>50.2</v>
       </c>
       <c r="BO2" t="n">
         <v>2.23</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.75</v>
+        <v>8.710000000000001</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.27</v>
+        <v>-4.28</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.245</v>
+        <v>0.246</v>
       </c>
       <c r="BT2" t="n">
-        <v>1476.8</v>
+        <v>1483.82</v>
       </c>
       <c r="BU2" t="n">
-        <v>-14.17</v>
+        <v>-13.64</v>
       </c>
       <c r="BV2" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="BW2" t="n">
         <v>2.04</v>
       </c>
-      <c r="BW2" t="n">
-        <v>2.05</v>
-      </c>
       <c r="BX2" t="n">
-        <v>1.9999</v>
+        <v>2</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2061,13 +2061,13 @@
         <v>44.6</v>
       </c>
       <c r="CE2" t="n">
-        <v>52</v>
+        <v>52.5</v>
       </c>
       <c r="CF2" t="n">
-        <v>68.3</v>
+        <v>68</v>
       </c>
       <c r="CG2" t="n">
-        <v>71.3</v>
+        <v>71.7</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>82.06</v>
+        <v>90.64</v>
       </c>
       <c r="CO2" t="n">
-        <v>37.56</v>
+        <v>49.65</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2112,7 +2112,7 @@
         <v>95.45454545454545</v>
       </c>
       <c r="CV2" t="n">
-        <v>81.81818181818183</v>
+        <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
         <v>68.18181818181817</v>
@@ -2124,7 +2124,7 @@
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>10.2103</v>
+        <v>10.1771</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6807</v>
+        <v>0.6787</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3407</v>
+        <v>0.3393</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1021</v>
+        <v>0.1018</v>
       </c>
       <c r="DF2" t="n">
-        <v>1.998</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1946</v>
+        <v>1.2033</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0039</v>
+        <v>4.0079</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.1054</v>
+        <v>5.0886</v>
       </c>
       <c r="DJ2" t="n">
-        <v>57.86</v>
+        <v>57.38</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.1054</v>
+        <v>5.0886</v>
       </c>
       <c r="DL2" t="n">
-        <v>1.9999</v>
+        <v>2</v>
       </c>
       <c r="DM2" t="n">
         <v>2.0039</v>
       </c>
       <c r="DN2" t="n">
-        <v>4.0039</v>
+        <v>4.0079</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9979</v>
+        <v>2.0003</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.7835</v>
+        <v>0.7874</v>
       </c>
       <c r="DQ2" t="n">
-        <v>99.76000000000001</v>
+        <v>102.56</v>
       </c>
       <c r="DR2" t="n">
-        <v>38.54</v>
+        <v>55.59</v>
       </c>
       <c r="DS2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.7961</v>
+        <v>3.7559</v>
       </c>
       <c r="DX2" t="n">
-        <v>95.34999999999999</v>
+        <v>80.45000000000002</v>
       </c>
       <c r="DY2" t="n">
-        <v>36.5</v>
+        <v>25.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>79.491</v>
+        <v>93.169</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>72.13</v>
+        <v>100</v>
       </c>
       <c r="ED2" t="n">
-        <v>94.98999999999999</v>
+        <v>71.83</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.7961</v>
+        <v>3.7559</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.73</v>
+        <v>0.51</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.5359</v>
+        <v>1.1276</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.004</v>
+        <v>4.0067</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.06270000000000001</v>
+        <v>0.1333</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6553</v>
+        <v>0.6579</v>
       </c>
       <c r="EK2" t="n">
-        <v>70.45</v>
+        <v>78.17</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2249,34 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>8.039999999999999</v>
+        <v>31.69</v>
       </c>
       <c r="EP2" t="n">
-        <v>0.9407</v>
+        <v>3.7458</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0854</v>
+        <v>0.0603</v>
       </c>
       <c r="ER2" t="n">
-        <v>13.9863</v>
+        <v>19.9608</v>
       </c>
       <c r="ES2" t="n">
-        <v>16.2986</v>
+        <v>16.209</v>
       </c>
       <c r="ET2" t="n">
-        <v>36.504</v>
+        <v>48.678</v>
       </c>
       <c r="EU2" t="n">
-        <v>3.3434</v>
+        <v>4.8654</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.474</v>
+        <v>1.6821</v>
       </c>
       <c r="EW2" t="n">
-        <v>6.5976</v>
+        <v>28.7238</v>
       </c>
       <c r="EX2" t="n">
-        <v>30.2</v>
+        <v>36.7</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2284,37 +2284,37 @@
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="FA2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.56</v>
+        <v>64.37</v>
       </c>
       <c r="FC2" t="n">
-        <v>47.05</v>
+        <v>46.36</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.27</v>
+        <v>72.2</v>
       </c>
       <c r="FE2" t="n">
-        <v>76.255</v>
+        <v>84.405</v>
       </c>
       <c r="FF2" t="n">
-        <v>33.88</v>
+        <v>43.175</v>
       </c>
       <c r="FG2" t="n">
-        <v>23.1155</v>
+        <v>25.6045</v>
       </c>
       <c r="FH2" t="n">
-        <v>62.438</v>
+        <v>66.717</v>
       </c>
       <c r="FI2" t="n">
-        <v>48.2</v>
+        <v>56.485</v>
       </c>
       <c r="FJ2" t="n">
-        <v>71.42</v>
+        <v>74.91</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>71.33</v>
+        <v>79.64</v>
       </c>
       <c r="FO2" t="n">
-        <v>77.84</v>
+        <v>78.8</v>
       </c>
       <c r="FP2" t="n">
-        <v>44.98</v>
+        <v>60.74</v>
       </c>
       <c r="FQ2" t="n">
-        <v>67.7</v>
+        <v>78.15000000000001</v>
       </c>
       <c r="FR2" t="n">
-        <v>82.18000000000001</v>
+        <v>88.76000000000001</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>69.834</v>
+        <v>76.3075</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260918_195842</t>
+          <t>20260921_143231</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46283.83243661495</v>
+        <v>46286.60591625832</v>
       </c>
     </row>
   </sheetData>
@@ -2464,9 +2464,9 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
-    <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46283.83243055556</v>
+        <v>46286.60591435185</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46283</v>
+        <v>46286</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.7</v>
+        <v>11.82</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1954</v>
+        <v>2015.5</v>
       </c>
       <c r="L2" t="n">
-        <v>1962</v>
+        <v>1966.6</v>
       </c>
       <c r="M2" t="n">
-        <v>1982</v>
+        <v>2023.5</v>
       </c>
       <c r="N2" t="n">
-        <v>1954</v>
+        <v>1963.8</v>
       </c>
       <c r="O2" t="n">
-        <v>1954</v>
+        <v>2015.5</v>
       </c>
       <c r="P2" t="n">
-        <v>2655873</v>
+        <v>1857943</v>
       </c>
       <c r="Q2" t="n">
-        <v>1954</v>
+        <v>2015.5</v>
       </c>
       <c r="R2" t="n">
-        <v>2153.51</v>
+        <v>2220.62</v>
       </c>
       <c r="S2" t="n">
-        <v>1854.24</v>
+        <v>1912.94</v>
       </c>
       <c r="T2" t="n">
-        <v>10.21033776867964</v>
+        <v>10.17712726370627</v>
       </c>
       <c r="U2" t="n">
-        <v>199.5100000000002</v>
+        <v>205.1199999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>5.105424769703172</v>
+        <v>5.088563631853135</v>
       </c>
       <c r="W2" t="n">
-        <v>99.75999999999999</v>
+        <v>102.5599999999999</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999899759422617</v>
+        <v>2</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>10.21033776867964</v>
+        <v>10.17712726370627</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.105424769703172</v>
+        <v>5.088563631853135</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02049518580591932</v>
+        <v>0.02050614683876245</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3253509882991407</v>
+        <v>0.3255249893012326</v>
       </c>
     </row>
     <row r="7">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266353403342596</v>
+        <v>0.04266354143766427</v>
       </c>
     </row>
     <row r="13">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.97</v>
+        <v>38.96</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-18 19:58:42.561272+05:30</t>
+          <t>2026-09-21 14:32:31.184863+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.210337768679642, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998997594226167}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.17712726370627, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-21 16:27 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>STRONG BUY</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.82</v>
+        <v>11.86</v>
       </c>
       <c r="R2" t="n">
-        <v>49.04</v>
+        <v>49.08</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1884,22 +1884,22 @@
         <v>1963.8</v>
       </c>
       <c r="X2" t="n">
-        <v>2015.5</v>
+        <v>2017.5</v>
       </c>
       <c r="Y2" t="n">
-        <v>2015.5</v>
+        <v>2017.5</v>
       </c>
       <c r="Z2" t="n">
-        <v>1857943</v>
+        <v>2170267</v>
       </c>
       <c r="AA2" t="n">
-        <v>3649459</v>
+        <v>3602619</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.51</v>
+        <v>0.6</v>
       </c>
       <c r="AC2" t="n">
-        <v>3.15</v>
+        <v>3.25</v>
       </c>
       <c r="AD2" t="n">
         <v>0.64</v>
@@ -1911,13 +1911,13 @@
         <v>2.96</v>
       </c>
       <c r="AG2" t="n">
-        <v>51.28</v>
+        <v>49.8</v>
       </c>
       <c r="AH2" t="n">
-        <v>51.28</v>
+        <v>49.8</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.54</v>
+        <v>2.47</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>5.48</v>
+        <v>5.17</v>
       </c>
       <c r="AM2" t="n">
-        <v>11.78</v>
+        <v>11.41</v>
       </c>
       <c r="AN2" t="n">
-        <v>52.88</v>
+        <v>52.49</v>
       </c>
       <c r="AO2" t="n">
-        <v>67.81999999999999</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="AP2" t="n">
-        <v>9.539999999999999</v>
+        <v>7.5</v>
       </c>
       <c r="AQ2" t="n">
-        <v>36.09</v>
+        <v>38.74</v>
       </c>
       <c r="AR2" t="n">
-        <v>2015.5</v>
+        <v>2017.5</v>
       </c>
       <c r="AS2" t="n">
-        <v>2220.62</v>
+        <v>2216.71</v>
       </c>
       <c r="AT2" t="n">
-        <v>1912.94</v>
+        <v>1917.9</v>
       </c>
       <c r="AU2" t="n">
-        <v>2015.5</v>
+        <v>2017.5</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>10.18</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="AY2" t="n">
-        <v>205.12</v>
+        <v>199.21</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.09</v>
+        <v>4.94</v>
       </c>
       <c r="BA2" t="n">
-        <v>102.56</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.04</v>
+        <v>2.03</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
@@ -1987,10 +1987,10 @@
         <v>49.2</v>
       </c>
       <c r="BG2" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.5</v>
+        <v>18.6</v>
       </c>
       <c r="BI2" t="n">
         <v>0</v>
@@ -2005,16 +2005,16 @@
         <v>0</v>
       </c>
       <c r="BM2" t="n">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="BN2" t="n">
         <v>50.2</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.23</v>
+        <v>2.24</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.710000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="BQ2" t="n">
         <v>-4.28</v>
@@ -2023,22 +2023,22 @@
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.246</v>
+        <v>0.247</v>
       </c>
       <c r="BT2" t="n">
-        <v>1483.82</v>
+        <v>1488.93</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.64</v>
+        <v>-13.63</v>
       </c>
       <c r="BV2" t="n">
         <v>2.05</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.04</v>
+        <v>2.03</v>
       </c>
       <c r="BX2" t="n">
-        <v>2</v>
+        <v>2.0001</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2058,13 +2058,13 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>44.6</v>
+        <v>44.8</v>
       </c>
       <c r="CE2" t="n">
         <v>52.5</v>
       </c>
       <c r="CF2" t="n">
-        <v>68</v>
+        <v>67.7</v>
       </c>
       <c r="CG2" t="n">
         <v>71.7</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>90.64</v>
+        <v>89.98999999999999</v>
       </c>
       <c r="CO2" t="n">
-        <v>49.65</v>
+        <v>47.48</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2121,10 +2121,10 @@
         <v>54.54545454545454</v>
       </c>
       <c r="CY2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CZ2" t="n">
-        <v>10.1771</v>
+        <v>9.8741</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6787</v>
+        <v>0.658</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3393</v>
+        <v>0.3293</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1018</v>
+        <v>0.0987</v>
       </c>
       <c r="DF2" t="n">
+        <v>1.998</v>
+      </c>
+      <c r="DG2" t="n">
+        <v>1.1706</v>
+      </c>
+      <c r="DH2" t="n">
+        <v>3.996</v>
+      </c>
+      <c r="DI2" t="n">
+        <v>4.9368</v>
+      </c>
+      <c r="DJ2" t="n">
+        <v>51.29</v>
+      </c>
+      <c r="DK2" t="n">
+        <v>4.9368</v>
+      </c>
+      <c r="DL2" t="n">
+        <v>2.0001</v>
+      </c>
+      <c r="DM2" t="n">
         <v>2</v>
       </c>
-      <c r="DG2" t="n">
-        <v>1.2033</v>
-      </c>
-      <c r="DH2" t="n">
-        <v>4.0079</v>
-      </c>
-      <c r="DI2" t="n">
-        <v>5.0886</v>
-      </c>
-      <c r="DJ2" t="n">
-        <v>57.38</v>
-      </c>
-      <c r="DK2" t="n">
-        <v>5.0886</v>
-      </c>
-      <c r="DL2" t="n">
-        <v>2</v>
-      </c>
-      <c r="DM2" t="n">
-        <v>2.0039</v>
-      </c>
       <c r="DN2" t="n">
-        <v>4.0079</v>
+        <v>3.996</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0003</v>
+        <v>1.9982</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.7874</v>
+        <v>0.8089</v>
       </c>
       <c r="DQ2" t="n">
-        <v>102.56</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="DR2" t="n">
-        <v>55.59</v>
+        <v>44.46</v>
       </c>
       <c r="DS2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="DT2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>3.7559</v>
+        <v>3.0364</v>
       </c>
       <c r="DX2" t="n">
-        <v>80.45000000000002</v>
+        <v>78.99999999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>25.5</v>
+        <v>30</v>
       </c>
       <c r="DZ2" t="n">
-        <v>93.169</v>
+        <v>90.572</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>100</v>
+        <v>92.81999999999999</v>
       </c>
       <c r="ED2" t="n">
-        <v>71.83</v>
+        <v>69.55</v>
       </c>
       <c r="EE2" t="n">
-        <v>3.7559</v>
+        <v>3.0364</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.51</v>
+        <v>0.6</v>
       </c>
       <c r="EG2" t="n">
-        <v>1.1276</v>
+        <v>0.8895</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0067</v>
+        <v>3.9976</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.1333</v>
+        <v>0.1055</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6579</v>
+        <v>0.673</v>
       </c>
       <c r="EK2" t="n">
-        <v>78.17</v>
+        <v>70.77</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2249,34 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>31.69</v>
+        <v>27.26</v>
       </c>
       <c r="EP2" t="n">
-        <v>3.7458</v>
+        <v>3.233</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0603</v>
+        <v>0.0712</v>
       </c>
       <c r="ER2" t="n">
-        <v>19.9608</v>
+        <v>16.45</v>
       </c>
       <c r="ES2" t="n">
-        <v>16.209</v>
+        <v>14.781</v>
       </c>
       <c r="ET2" t="n">
-        <v>48.678</v>
+        <v>46.538</v>
       </c>
       <c r="EU2" t="n">
-        <v>4.8654</v>
+        <v>4.5</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.6821</v>
+        <v>1.5438</v>
       </c>
       <c r="EW2" t="n">
-        <v>28.7238</v>
+        <v>24.5313</v>
       </c>
       <c r="EX2" t="n">
-        <v>36.7</v>
+        <v>35.43</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2290,31 @@
         <v>9</v>
       </c>
       <c r="FB2" t="n">
-        <v>64.37</v>
+        <v>64.56</v>
       </c>
       <c r="FC2" t="n">
-        <v>46.36</v>
+        <v>40.97</v>
       </c>
       <c r="FD2" t="n">
-        <v>72.2</v>
+        <v>71.66</v>
       </c>
       <c r="FE2" t="n">
-        <v>84.405</v>
+        <v>80.38</v>
       </c>
       <c r="FF2" t="n">
-        <v>43.175</v>
+        <v>41.455</v>
       </c>
       <c r="FG2" t="n">
-        <v>25.6045</v>
+        <v>25.9337</v>
       </c>
       <c r="FH2" t="n">
-        <v>66.717</v>
+        <v>66.363</v>
       </c>
       <c r="FI2" t="n">
-        <v>56.485</v>
+        <v>47.875</v>
       </c>
       <c r="FJ2" t="n">
-        <v>74.91</v>
+        <v>71.77</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>79.64</v>
+        <v>70.81</v>
       </c>
       <c r="FO2" t="n">
-        <v>78.8</v>
+        <v>71.77</v>
       </c>
       <c r="FP2" t="n">
-        <v>60.74</v>
+        <v>52.62</v>
       </c>
       <c r="FQ2" t="n">
-        <v>78.15000000000001</v>
+        <v>68.78</v>
       </c>
       <c r="FR2" t="n">
-        <v>88.76000000000001</v>
+        <v>78.44</v>
       </c>
       <c r="FS2" t="n">
-        <v>100</v>
+        <v>90.9091</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2353,11 +2353,11 @@
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>76.3075</v>
+        <v>67.9365</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260921_143231</t>
+          <t>20260921_215750</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46286.60591625832</v>
+        <v>46286.9151656508</v>
       </c>
     </row>
   </sheetData>
@@ -2465,8 +2465,8 @@
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="20" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="19" customWidth="1" min="23" max="23"/>
+    <col width="19" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46286.60591435185</v>
+        <v>46286.91516203704</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46286</v>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.82</v>
+        <v>11.86</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>2015.5</v>
+        <v>2017.5</v>
       </c>
       <c r="L2" t="n">
         <v>1966.6</v>
@@ -2693,34 +2693,34 @@
         <v>1963.8</v>
       </c>
       <c r="O2" t="n">
-        <v>2015.5</v>
+        <v>2017.5</v>
       </c>
       <c r="P2" t="n">
-        <v>1857943</v>
+        <v>2170267</v>
       </c>
       <c r="Q2" t="n">
-        <v>2015.5</v>
+        <v>2017.5</v>
       </c>
       <c r="R2" t="n">
-        <v>2220.62</v>
+        <v>2216.71</v>
       </c>
       <c r="S2" t="n">
-        <v>1912.94</v>
+        <v>1917.9</v>
       </c>
       <c r="T2" t="n">
-        <v>10.17712726370627</v>
+        <v>9.874101610904587</v>
       </c>
       <c r="U2" t="n">
-        <v>205.1199999999999</v>
+        <v>199.21</v>
       </c>
       <c r="V2" t="n">
-        <v>5.088563631853135</v>
+        <v>4.936802973977691</v>
       </c>
       <c r="W2" t="n">
-        <v>102.5599999999999</v>
+        <v>99.59999999999991</v>
       </c>
       <c r="X2" t="n">
-        <v>2</v>
+        <v>2.000100401606428</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>10.17712726370627</v>
+        <v>9.874101610904587</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.088563631853135</v>
+        <v>4.936802973977691</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02050614683876245</v>
+        <v>0.02049241041929946</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3255249893012326</v>
+        <v>0.3253069304024114</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909799741235235</v>
+        <v>0.02909787899938576</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266354143766427</v>
+        <v>0.04266353163762541</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645463</v>
+        <v>0.1869492979645464</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.96</v>
+        <v>38.98</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-21 14:32:31.184863+05:30</t>
+          <t>2026-09-21 21:57:50.352289+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.17712726370627, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.874101610904587, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000100401606428}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-22 08:37 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="19" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H2" t="n">
         <v>8.699999999999999</v>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.86</v>
+        <v>11.82</v>
       </c>
       <c r="R2" t="n">
-        <v>49.08</v>
+        <v>48.96</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1966.6</v>
+        <v>2018</v>
       </c>
       <c r="V2" t="n">
-        <v>2023.5</v>
+        <v>2032.8</v>
       </c>
       <c r="W2" t="n">
-        <v>1963.8</v>
+        <v>2003</v>
       </c>
       <c r="X2" t="n">
-        <v>2017.5</v>
+        <v>2007.7</v>
       </c>
       <c r="Y2" t="n">
-        <v>2017.5</v>
+        <v>2007.7</v>
       </c>
       <c r="Z2" t="n">
-        <v>2170267</v>
+        <v>1091733</v>
       </c>
       <c r="AA2" t="n">
-        <v>3602619</v>
+        <v>3479658</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.6</v>
+        <v>0.31</v>
       </c>
       <c r="AC2" t="n">
-        <v>3.25</v>
+        <v>-0.49</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.64</v>
+        <v>0.02</v>
       </c>
       <c r="AE2" t="n">
-        <v>59.7</v>
+        <v>29.8</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.96</v>
+        <v>1.48</v>
       </c>
       <c r="AG2" t="n">
-        <v>49.8</v>
+        <v>48.37</v>
       </c>
       <c r="AH2" t="n">
-        <v>49.8</v>
+        <v>48.37</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.47</v>
+        <v>2.41</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,65 +1926,65 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>5.17</v>
+        <v>4.28</v>
       </c>
       <c r="AM2" t="n">
-        <v>11.41</v>
+        <v>10.32</v>
       </c>
       <c r="AN2" t="n">
-        <v>52.49</v>
+        <v>51.19</v>
       </c>
       <c r="AO2" t="n">
-        <v>68.40000000000001</v>
+        <v>66.52</v>
       </c>
       <c r="AP2" t="n">
-        <v>7.5</v>
+        <v>3.12</v>
       </c>
       <c r="AQ2" t="n">
-        <v>38.74</v>
+        <v>38.46</v>
       </c>
       <c r="AR2" t="n">
-        <v>2017.5</v>
+        <v>2007.7</v>
       </c>
       <c r="AS2" t="n">
-        <v>2216.71</v>
+        <v>2201.19</v>
       </c>
       <c r="AT2" t="n">
-        <v>1917.9</v>
+        <v>1910.95</v>
       </c>
       <c r="AU2" t="n">
-        <v>2017.5</v>
+        <v>2007.699951171875</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.869999999999999</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="AY2" t="n">
-        <v>199.21</v>
+        <v>193.49</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.94</v>
+        <v>4.82</v>
       </c>
       <c r="BA2" t="n">
-        <v>99.59999999999999</v>
+        <v>96.75</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.03</v>
+        <v>2.04</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
       </c>
       <c r="BD2" t="n">
-        <v>32.2</v>
+        <v>32.1</v>
       </c>
       <c r="BE2" t="n">
         <v>327</v>
       </c>
       <c r="BF2" t="n">
-        <v>49.2</v>
+        <v>49.1</v>
       </c>
       <c r="BG2" t="n">
         <v>124</v>
@@ -1993,52 +1993,52 @@
         <v>18.6</v>
       </c>
       <c r="BI2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BM2" t="n">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="BN2" t="n">
         <v>50.2</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.24</v>
+        <v>2.23</v>
       </c>
       <c r="BP2" t="n">
         <v>8.699999999999999</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.28</v>
+        <v>-4.27</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.247</v>
+        <v>0.246</v>
       </c>
       <c r="BT2" t="n">
-        <v>1488.93</v>
+        <v>1486.59</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.63</v>
+        <v>-13.93</v>
       </c>
       <c r="BV2" t="n">
         <v>2.05</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.03</v>
+        <v>2.04</v>
       </c>
       <c r="BX2" t="n">
-        <v>2.0001</v>
+        <v>1.9999</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2058,13 +2058,13 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>44.8</v>
+        <v>44.6</v>
       </c>
       <c r="CE2" t="n">
         <v>52.5</v>
       </c>
       <c r="CF2" t="n">
-        <v>67.7</v>
+        <v>68</v>
       </c>
       <c r="CG2" t="n">
         <v>71.7</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>89.98999999999999</v>
+        <v>76.98999999999999</v>
       </c>
       <c r="CO2" t="n">
-        <v>47.48</v>
+        <v>37.56</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2121,10 +2121,10 @@
         <v>54.54545454545454</v>
       </c>
       <c r="CY2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.8741</v>
+        <v>9.6374</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.658</v>
+        <v>0.6427</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3293</v>
+        <v>0.3213</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0987</v>
+        <v>0.0964</v>
       </c>
       <c r="DF2" t="n">
-        <v>1.998</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1706</v>
+        <v>1.1394</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.996</v>
+        <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.9368</v>
+        <v>4.8189</v>
       </c>
       <c r="DJ2" t="n">
-        <v>51.29</v>
+        <v>51.34</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.9368</v>
+        <v>4.8189</v>
       </c>
       <c r="DL2" t="n">
-        <v>2.0001</v>
+        <v>1.9999</v>
       </c>
       <c r="DM2" t="n">
         <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.996</v>
+        <v>4</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9982</v>
+        <v>2.0003</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8089</v>
+        <v>0.8299</v>
       </c>
       <c r="DQ2" t="n">
-        <v>99.59999999999999</v>
+        <v>96.75</v>
       </c>
       <c r="DR2" t="n">
-        <v>44.46</v>
+        <v>47.19</v>
       </c>
       <c r="DS2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,90 +2193,90 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>3.0364</v>
+        <v>1.2946</v>
       </c>
       <c r="DX2" t="n">
-        <v>78.99999999999999</v>
+        <v>83.70000000000002</v>
       </c>
       <c r="DY2" t="n">
-        <v>30</v>
+        <v>15.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>90.572</v>
+        <v>79.48</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
       </c>
       <c r="EB2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>92.81999999999999</v>
+        <v>67.58</v>
       </c>
       <c r="ED2" t="n">
-        <v>69.55</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="EE2" t="n">
-        <v>3.0364</v>
+        <v>1.2946</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.6</v>
+        <v>0.31</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.8895</v>
+        <v>0.3688</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9976</v>
+        <v>3.9989</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.1055</v>
+        <v>0.0436</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.673</v>
+        <v>0.6871</v>
       </c>
       <c r="EK2" t="n">
-        <v>70.77</v>
+        <v>58.46</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="EM2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="EN2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="EO2" t="n">
-        <v>27.26</v>
+        <v>7.76</v>
       </c>
       <c r="EP2" t="n">
-        <v>3.233</v>
+        <v>0.9172</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0712</v>
+        <v>0.0366</v>
       </c>
       <c r="ER2" t="n">
-        <v>16.45</v>
+        <v>31.0968</v>
       </c>
       <c r="ES2" t="n">
-        <v>14.781</v>
+        <v>15.0557</v>
       </c>
       <c r="ET2" t="n">
-        <v>46.538</v>
+        <v>36.663</v>
       </c>
       <c r="EU2" t="n">
-        <v>4.5</v>
+        <v>0.9671999999999999</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.5438</v>
+        <v>1.8397</v>
       </c>
       <c r="EW2" t="n">
-        <v>24.5313</v>
+        <v>5.9744</v>
       </c>
       <c r="EX2" t="n">
-        <v>35.43</v>
+        <v>30.93</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2284,37 +2284,37 @@
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="FA2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="FB2" t="n">
-        <v>64.56</v>
+        <v>64.37</v>
       </c>
       <c r="FC2" t="n">
-        <v>40.97</v>
+        <v>41.72</v>
       </c>
       <c r="FD2" t="n">
-        <v>71.66</v>
+        <v>72.34999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>80.38</v>
+        <v>67.72499999999999</v>
       </c>
       <c r="FF2" t="n">
-        <v>41.455</v>
+        <v>34.245</v>
       </c>
       <c r="FG2" t="n">
-        <v>25.9337</v>
+        <v>22.5777</v>
       </c>
       <c r="FH2" t="n">
-        <v>66.363</v>
+        <v>61.468</v>
       </c>
       <c r="FI2" t="n">
-        <v>47.875</v>
+        <v>49.265</v>
       </c>
       <c r="FJ2" t="n">
-        <v>71.77</v>
+        <v>67.45999999999999</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>70.81</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="FO2" t="n">
-        <v>71.77</v>
+        <v>65.02</v>
       </c>
       <c r="FP2" t="n">
-        <v>52.62</v>
+        <v>52.52</v>
       </c>
       <c r="FQ2" t="n">
-        <v>68.78</v>
+        <v>71.67</v>
       </c>
       <c r="FR2" t="n">
-        <v>78.44</v>
+        <v>79.15000000000001</v>
       </c>
       <c r="FS2" t="n">
-        <v>90.9091</v>
+        <v>95.4545</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>67.9365</v>
+        <v>67.84650000000001</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260921_215750</t>
+          <t>20260922_140715</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46286.9151656508</v>
+        <v>46287.58837222776</v>
       </c>
     </row>
   </sheetData>
@@ -2465,8 +2465,8 @@
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="19" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46286.91516203704</v>
+        <v>46287.58836805556</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.86</v>
+        <v>11.82</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>2017.5</v>
+        <v>2007.7</v>
       </c>
       <c r="L2" t="n">
-        <v>1966.6</v>
+        <v>2018</v>
       </c>
       <c r="M2" t="n">
-        <v>2023.5</v>
+        <v>2032.8</v>
       </c>
       <c r="N2" t="n">
-        <v>1963.8</v>
+        <v>2003</v>
       </c>
       <c r="O2" t="n">
-        <v>2017.5</v>
+        <v>2007.7</v>
       </c>
       <c r="P2" t="n">
-        <v>2170267</v>
+        <v>1091733</v>
       </c>
       <c r="Q2" t="n">
-        <v>2017.5</v>
+        <v>2007.7</v>
       </c>
       <c r="R2" t="n">
-        <v>2216.71</v>
+        <v>2201.19</v>
       </c>
       <c r="S2" t="n">
-        <v>1917.9</v>
+        <v>1910.95</v>
       </c>
       <c r="T2" t="n">
-        <v>9.874101610904587</v>
+        <v>9.637396025302586</v>
       </c>
       <c r="U2" t="n">
-        <v>199.21</v>
+        <v>193.49</v>
       </c>
       <c r="V2" t="n">
-        <v>4.936802973977691</v>
+        <v>4.818947053842706</v>
       </c>
       <c r="W2" t="n">
-        <v>99.59999999999991</v>
+        <v>96.75</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000100401606428</v>
+        <v>1.999896640826873</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.874101610904587</v>
+        <v>9.637396025302586</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.936802973977691</v>
+        <v>4.818947053842706</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02049241041929946</v>
+        <v>0.02047965433756102</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3253069304024114</v>
+        <v>0.3251044338825103</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909787899938576</v>
+        <v>0.02909781979290247</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266353163762541</v>
+        <v>0.04266353895739713</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.98</v>
+        <v>38.99</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-21 21:57:50.352289+05:30</t>
+          <t>2026-09-22 14:07:15.398458+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.874101610904587, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000100401606428}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.637396025302586, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998966408268735}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-22 14:49 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="19" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1864,7 +1864,7 @@
         <v>11.82</v>
       </c>
       <c r="R2" t="n">
-        <v>48.96</v>
+        <v>49</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1881,40 +1881,40 @@
         <v>2032.8</v>
       </c>
       <c r="W2" t="n">
-        <v>2003</v>
+        <v>2002.2</v>
       </c>
       <c r="X2" t="n">
-        <v>2007.7</v>
+        <v>2006.5</v>
       </c>
       <c r="Y2" t="n">
-        <v>2007.7</v>
+        <v>2006.5</v>
       </c>
       <c r="Z2" t="n">
-        <v>1091733</v>
+        <v>1485458</v>
       </c>
       <c r="AA2" t="n">
-        <v>3479658</v>
+        <v>3499344</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.31</v>
+        <v>0.42</v>
       </c>
       <c r="AC2" t="n">
-        <v>-0.49</v>
+        <v>-0.55</v>
       </c>
       <c r="AD2" t="n">
         <v>0.02</v>
       </c>
       <c r="AE2" t="n">
-        <v>29.8</v>
+        <v>30.6</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.48</v>
+        <v>1.53</v>
       </c>
       <c r="AG2" t="n">
-        <v>48.37</v>
+        <v>48.43</v>
       </c>
       <c r="AH2" t="n">
-        <v>48.37</v>
+        <v>48.43</v>
       </c>
       <c r="AI2" t="n">
         <v>2.41</v>
@@ -1926,50 +1926,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>4.28</v>
+        <v>4.22</v>
       </c>
       <c r="AM2" t="n">
-        <v>10.32</v>
+        <v>10.26</v>
       </c>
       <c r="AN2" t="n">
-        <v>51.19</v>
+        <v>51.1</v>
       </c>
       <c r="AO2" t="n">
-        <v>66.52</v>
+        <v>66.3</v>
       </c>
       <c r="AP2" t="n">
-        <v>3.12</v>
+        <v>3.06</v>
       </c>
       <c r="AQ2" t="n">
-        <v>38.46</v>
+        <v>38.38</v>
       </c>
       <c r="AR2" t="n">
-        <v>2007.7</v>
+        <v>2006.5</v>
       </c>
       <c r="AS2" t="n">
-        <v>2201.19</v>
+        <v>2200.22</v>
       </c>
       <c r="AT2" t="n">
-        <v>1910.95</v>
+        <v>1909.64</v>
       </c>
       <c r="AU2" t="n">
-        <v>2007.699951171875</v>
+        <v>2006.5</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.640000000000001</v>
+        <v>9.65</v>
       </c>
       <c r="AY2" t="n">
-        <v>193.49</v>
+        <v>193.72</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.82</v>
+        <v>4.83</v>
       </c>
       <c r="BA2" t="n">
-        <v>96.75</v>
+        <v>96.86</v>
       </c>
       <c r="BB2" t="n">
         <v>2.04</v>
@@ -2026,10 +2026,10 @@
         <v>0.246</v>
       </c>
       <c r="BT2" t="n">
-        <v>1486.59</v>
+        <v>1486.34</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.93</v>
+        <v>-13.95</v>
       </c>
       <c r="BV2" t="n">
         <v>2.05</v>
@@ -2038,7 +2038,7 @@
         <v>2.04</v>
       </c>
       <c r="BX2" t="n">
-        <v>1.9999</v>
+        <v>2</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>76.98999999999999</v>
+        <v>76.08</v>
       </c>
       <c r="CO2" t="n">
-        <v>37.56</v>
+        <v>38.24</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2124,7 +2124,7 @@
         <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.6374</v>
+        <v>9.6546</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6427</v>
+        <v>0.6433</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3213</v>
+        <v>0.322</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0964</v>
+        <v>0.0965</v>
       </c>
       <c r="DF2" t="n">
+        <v>1.9979</v>
+      </c>
+      <c r="DG2" t="n">
+        <v>1.1406</v>
+      </c>
+      <c r="DH2" t="n">
+        <v>4.0041</v>
+      </c>
+      <c r="DI2" t="n">
+        <v>4.8273</v>
+      </c>
+      <c r="DJ2" t="n">
+        <v>49.77</v>
+      </c>
+      <c r="DK2" t="n">
+        <v>4.8273</v>
+      </c>
+      <c r="DL2" t="n">
         <v>2</v>
       </c>
-      <c r="DG2" t="n">
-        <v>1.1394</v>
-      </c>
-      <c r="DH2" t="n">
+      <c r="DM2" t="n">
+        <v>2.0041</v>
+      </c>
+      <c r="DN2" t="n">
+        <v>4.0041</v>
+      </c>
+      <c r="DO2" t="n">
+        <v>1.9978</v>
+      </c>
+      <c r="DP2" t="n">
+        <v>0.829</v>
+      </c>
+      <c r="DQ2" t="n">
+        <v>96.86</v>
+      </c>
+      <c r="DR2" t="n">
+        <v>41.27</v>
+      </c>
+      <c r="DS2" t="n">
         <v>4</v>
       </c>
-      <c r="DI2" t="n">
-        <v>4.8189</v>
-      </c>
-      <c r="DJ2" t="n">
-        <v>51.34</v>
-      </c>
-      <c r="DK2" t="n">
-        <v>4.8189</v>
-      </c>
-      <c r="DL2" t="n">
-        <v>1.9999</v>
-      </c>
-      <c r="DM2" t="n">
-        <v>2</v>
-      </c>
-      <c r="DN2" t="n">
-        <v>4</v>
-      </c>
-      <c r="DO2" t="n">
-        <v>2.0003</v>
-      </c>
-      <c r="DP2" t="n">
-        <v>0.8299</v>
-      </c>
-      <c r="DQ2" t="n">
-        <v>96.75</v>
-      </c>
-      <c r="DR2" t="n">
-        <v>47.19</v>
-      </c>
-      <c r="DS2" t="n">
-        <v>5</v>
-      </c>
       <c r="DT2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.2946</v>
+        <v>1.2697</v>
       </c>
       <c r="DX2" t="n">
-        <v>83.70000000000002</v>
+        <v>84.25000000000001</v>
       </c>
       <c r="DY2" t="n">
-        <v>15.5</v>
+        <v>21</v>
       </c>
       <c r="DZ2" t="n">
-        <v>79.48</v>
+        <v>77.89700000000001</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,72 +2211,72 @@
         <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>67.58</v>
+        <v>64.68000000000001</v>
       </c>
       <c r="ED2" t="n">
-        <v>77.45999999999999</v>
+        <v>79.8</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.2946</v>
+        <v>1.2697</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.31</v>
+        <v>0.42</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.3688</v>
+        <v>0.3617</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9989</v>
+        <v>4.0061</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0436</v>
+        <v>0.0428</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6871</v>
+        <v>0.6872</v>
       </c>
       <c r="EK2" t="n">
-        <v>58.46</v>
+        <v>63.88</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Strong</t>
         </is>
       </c>
       <c r="EM2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>7.76</v>
+        <v>7.65</v>
       </c>
       <c r="EP2" t="n">
-        <v>0.9172</v>
+        <v>0.9042</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0366</v>
+        <v>0.0496</v>
       </c>
       <c r="ER2" t="n">
-        <v>31.0968</v>
+        <v>22.9762</v>
       </c>
       <c r="ES2" t="n">
-        <v>15.0557</v>
+        <v>14.5953</v>
       </c>
       <c r="ET2" t="n">
-        <v>36.663</v>
+        <v>36.902</v>
       </c>
       <c r="EU2" t="n">
-        <v>0.9671999999999999</v>
+        <v>1.2852</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.8397</v>
+        <v>1.6972</v>
       </c>
       <c r="EW2" t="n">
-        <v>5.9744</v>
+        <v>5.8201</v>
       </c>
       <c r="EX2" t="n">
-        <v>30.93</v>
+        <v>31.48</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2287,34 +2287,34 @@
         <v>4</v>
       </c>
       <c r="FA2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="FB2" t="n">
         <v>64.37</v>
       </c>
       <c r="FC2" t="n">
-        <v>41.72</v>
+        <v>41.6</v>
       </c>
       <c r="FD2" t="n">
-        <v>72.34999999999999</v>
+        <v>72.11</v>
       </c>
       <c r="FE2" t="n">
-        <v>67.72499999999999</v>
+        <v>69.98</v>
       </c>
       <c r="FF2" t="n">
-        <v>34.245</v>
+        <v>34.86</v>
       </c>
       <c r="FG2" t="n">
-        <v>22.5777</v>
+        <v>22.3109</v>
       </c>
       <c r="FH2" t="n">
-        <v>61.468</v>
+        <v>61.305</v>
       </c>
       <c r="FI2" t="n">
-        <v>49.265</v>
+        <v>45.52</v>
       </c>
       <c r="FJ2" t="n">
-        <v>67.45999999999999</v>
+        <v>67.69</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>68.40000000000001</v>
+        <v>67</v>
       </c>
       <c r="FO2" t="n">
-        <v>65.02</v>
+        <v>66.23999999999999</v>
       </c>
       <c r="FP2" t="n">
-        <v>52.52</v>
+        <v>49.2</v>
       </c>
       <c r="FQ2" t="n">
-        <v>71.67</v>
+        <v>67.86</v>
       </c>
       <c r="FR2" t="n">
-        <v>79.15000000000001</v>
+        <v>76.67</v>
       </c>
       <c r="FS2" t="n">
         <v>95.4545</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>67.84650000000001</v>
+        <v>65.529</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260922_140715</t>
+          <t>20260922_201904</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46287.58837222776</v>
+        <v>46287.84658097686</v>
       </c>
     </row>
   </sheetData>
@@ -2465,8 +2465,8 @@
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="13" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46287.58836805556</v>
+        <v>46287.84657407407</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46287</v>
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>2007.7</v>
+        <v>2006.5</v>
       </c>
       <c r="L2" t="n">
         <v>2018</v>
@@ -2690,37 +2690,37 @@
         <v>2032.8</v>
       </c>
       <c r="N2" t="n">
-        <v>2003</v>
+        <v>2002.2</v>
       </c>
       <c r="O2" t="n">
-        <v>2007.7</v>
+        <v>2006.5</v>
       </c>
       <c r="P2" t="n">
-        <v>1091733</v>
+        <v>1485458</v>
       </c>
       <c r="Q2" t="n">
-        <v>2007.7</v>
+        <v>2006.5</v>
       </c>
       <c r="R2" t="n">
-        <v>2201.19</v>
+        <v>2200.22</v>
       </c>
       <c r="S2" t="n">
-        <v>1910.95</v>
+        <v>1909.64</v>
       </c>
       <c r="T2" t="n">
-        <v>9.637396025302586</v>
+        <v>9.654622476949903</v>
       </c>
       <c r="U2" t="n">
-        <v>193.49</v>
+        <v>193.7199999999998</v>
       </c>
       <c r="V2" t="n">
-        <v>4.818947053842706</v>
+        <v>4.827311238474952</v>
       </c>
       <c r="W2" t="n">
-        <v>96.75</v>
+        <v>96.8599999999999</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999896640826873</v>
+        <v>2</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.637396025302586</v>
+        <v>9.654622476949903</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.818947053842706</v>
+        <v>4.827311238474952</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02047965433756102</v>
+        <v>0.0204799778532972</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3251044338825103</v>
+        <v>0.325109569535609</v>
       </c>
     </row>
     <row r="7">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266353895739713</v>
+        <v>0.04266353403342596</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869492979645463</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-22 14:07:15.398458+05:30</t>
+          <t>2026-09-22 20:19:04.623932+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.637396025302586, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998966408268735}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.654622476949903, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-23 08:39 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H2" t="n">
         <v>8.699999999999999</v>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.82</v>
+        <v>11.91</v>
       </c>
       <c r="R2" t="n">
-        <v>49</v>
+        <v>48.93</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>2018</v>
+        <v>2009.5</v>
       </c>
       <c r="V2" t="n">
-        <v>2032.8</v>
+        <v>2029</v>
       </c>
       <c r="W2" t="n">
-        <v>2002.2</v>
+        <v>1999.7</v>
       </c>
       <c r="X2" t="n">
-        <v>2006.5</v>
+        <v>2026.5</v>
       </c>
       <c r="Y2" t="n">
-        <v>2006.5</v>
+        <v>2026.5</v>
       </c>
       <c r="Z2" t="n">
-        <v>1485458</v>
+        <v>864623</v>
       </c>
       <c r="AA2" t="n">
-        <v>3499344</v>
+        <v>3375946</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.42</v>
+        <v>0.26</v>
       </c>
       <c r="AC2" t="n">
-        <v>-0.55</v>
+        <v>1</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.02</v>
+        <v>0.15</v>
       </c>
       <c r="AE2" t="n">
-        <v>30.6</v>
+        <v>29.3</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.53</v>
+        <v>1.45</v>
       </c>
       <c r="AG2" t="n">
-        <v>48.43</v>
+        <v>47.06</v>
       </c>
       <c r="AH2" t="n">
-        <v>48.43</v>
+        <v>47.06</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.41</v>
+        <v>2.32</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>4.22</v>
+        <v>4.88</v>
       </c>
       <c r="AM2" t="n">
-        <v>10.26</v>
+        <v>10.78</v>
       </c>
       <c r="AN2" t="n">
-        <v>51.1</v>
+        <v>52.02</v>
       </c>
       <c r="AO2" t="n">
-        <v>66.3</v>
+        <v>68.20999999999999</v>
       </c>
       <c r="AP2" t="n">
-        <v>3.06</v>
+        <v>4.62</v>
       </c>
       <c r="AQ2" t="n">
-        <v>38.38</v>
+        <v>39.76</v>
       </c>
       <c r="AR2" t="n">
-        <v>2006.5</v>
+        <v>2026.5</v>
       </c>
       <c r="AS2" t="n">
-        <v>2200.22</v>
+        <v>2214.75</v>
       </c>
       <c r="AT2" t="n">
-        <v>1909.64</v>
+        <v>1932.37</v>
       </c>
       <c r="AU2" t="n">
-        <v>2006.5</v>
+        <v>2026.5</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.65</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="AY2" t="n">
-        <v>193.72</v>
+        <v>188.25</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.83</v>
+        <v>4.64</v>
       </c>
       <c r="BA2" t="n">
-        <v>96.86</v>
+        <v>94.13</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.04</v>
+        <v>2.02</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
@@ -1984,61 +1984,61 @@
         <v>327</v>
       </c>
       <c r="BF2" t="n">
-        <v>49.1</v>
+        <v>49</v>
       </c>
       <c r="BG2" t="n">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.6</v>
+        <v>18.9</v>
       </c>
       <c r="BI2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BM2" t="n">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="BN2" t="n">
-        <v>50.2</v>
+        <v>50.4</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.23</v>
+        <v>2.24</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.699999999999999</v>
+        <v>8.66</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.27</v>
+        <v>-4.28</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.246</v>
+        <v>0.247</v>
       </c>
       <c r="BT2" t="n">
-        <v>1486.34</v>
+        <v>1491.14</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.95</v>
+        <v>-13.72</v>
       </c>
       <c r="BV2" t="n">
         <v>2.05</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.04</v>
+        <v>2.02</v>
       </c>
       <c r="BX2" t="n">
-        <v>2</v>
+        <v>1.9999</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>44.6</v>
+        <v>44.8</v>
       </c>
       <c r="CE2" t="n">
         <v>52.5</v>
       </c>
       <c r="CF2" t="n">
-        <v>68</v>
+        <v>67.3</v>
       </c>
       <c r="CG2" t="n">
-        <v>71.7</v>
+        <v>72</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>76.08</v>
+        <v>75.09</v>
       </c>
       <c r="CO2" t="n">
-        <v>38.24</v>
+        <v>36.54</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2124,7 +2124,7 @@
         <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.6546</v>
+        <v>9.289400000000001</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6433</v>
+        <v>0.6193</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.322</v>
+        <v>0.3093</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0965</v>
+        <v>0.0929</v>
       </c>
       <c r="DF2" t="n">
-        <v>1.9979</v>
+        <v>2.0022</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1406</v>
+        <v>1.1064</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0041</v>
+        <v>4.0043</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.8273</v>
+        <v>4.645</v>
       </c>
       <c r="DJ2" t="n">
-        <v>49.77</v>
+        <v>47.16</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.8273</v>
+        <v>4.645</v>
       </c>
       <c r="DL2" t="n">
+        <v>1.9999</v>
+      </c>
+      <c r="DM2" t="n">
         <v>2</v>
       </c>
-      <c r="DM2" t="n">
-        <v>2.0041</v>
-      </c>
       <c r="DN2" t="n">
-        <v>4.0041</v>
+        <v>4.0043</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9978</v>
+        <v>2.0023</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.829</v>
+        <v>0.863</v>
       </c>
       <c r="DQ2" t="n">
-        <v>96.86</v>
+        <v>94.13</v>
       </c>
       <c r="DR2" t="n">
-        <v>41.27</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="DS2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.2697</v>
+        <v>1.9914</v>
       </c>
       <c r="DX2" t="n">
-        <v>84.25000000000001</v>
+        <v>79.47500000000002</v>
       </c>
       <c r="DY2" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="DZ2" t="n">
-        <v>77.89700000000001</v>
+        <v>82.54900000000001</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>64.68000000000001</v>
+        <v>79.19</v>
       </c>
       <c r="ED2" t="n">
-        <v>79.8</v>
+        <v>73.69</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.2697</v>
+        <v>1.9914</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.42</v>
+        <v>0.26</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.3617</v>
+        <v>0.5502</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0061</v>
+        <v>4.0041</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0428</v>
+        <v>0.0655</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6872</v>
+        <v>0.7099</v>
       </c>
       <c r="EK2" t="n">
-        <v>63.88</v>
+        <v>63.93</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2246,37 +2246,37 @@
         <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>7.65</v>
+        <v>4</v>
       </c>
       <c r="EP2" t="n">
-        <v>0.9042</v>
+        <v>0.4764</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0496</v>
+        <v>0.031</v>
       </c>
       <c r="ER2" t="n">
-        <v>22.9762</v>
+        <v>35.7308</v>
       </c>
       <c r="ES2" t="n">
-        <v>14.5953</v>
+        <v>14.2048</v>
       </c>
       <c r="ET2" t="n">
-        <v>36.902</v>
+        <v>35.256</v>
       </c>
       <c r="EU2" t="n">
-        <v>1.2852</v>
+        <v>1.2012</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.6972</v>
+        <v>1.8413</v>
       </c>
       <c r="EW2" t="n">
-        <v>5.8201</v>
+        <v>3.0036</v>
       </c>
       <c r="EX2" t="n">
-        <v>31.48</v>
+        <v>28.8</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2287,34 +2287,34 @@
         <v>4</v>
       </c>
       <c r="FA2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="FB2" t="n">
-        <v>64.37</v>
+        <v>64.8</v>
       </c>
       <c r="FC2" t="n">
-        <v>41.6</v>
+        <v>36.26</v>
       </c>
       <c r="FD2" t="n">
-        <v>72.11</v>
+        <v>71.04000000000001</v>
       </c>
       <c r="FE2" t="n">
-        <v>69.98</v>
+        <v>69.51000000000001</v>
       </c>
       <c r="FF2" t="n">
-        <v>34.86</v>
+        <v>32.67</v>
       </c>
       <c r="FG2" t="n">
-        <v>22.3109</v>
+        <v>22.6175</v>
       </c>
       <c r="FH2" t="n">
-        <v>61.305</v>
+        <v>60.687</v>
       </c>
       <c r="FI2" t="n">
-        <v>45.52</v>
+        <v>59.53</v>
       </c>
       <c r="FJ2" t="n">
-        <v>67.69</v>
+        <v>66.69</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>67</v>
+        <v>73.87</v>
       </c>
       <c r="FO2" t="n">
-        <v>66.23999999999999</v>
+        <v>64.23</v>
       </c>
       <c r="FP2" t="n">
-        <v>49.2</v>
+        <v>55.43</v>
       </c>
       <c r="FQ2" t="n">
-        <v>67.86</v>
+        <v>80.73999999999999</v>
       </c>
       <c r="FR2" t="n">
-        <v>76.67</v>
+        <v>83.44</v>
       </c>
       <c r="FS2" t="n">
         <v>95.4545</v>
@@ -2353,11 +2353,11 @@
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>65.529</v>
+        <v>72.917</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260922_201904</t>
+          <t>20260923_140908</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46287.84658097686</v>
+        <v>46288.58968385548</v>
       </c>
     </row>
   </sheetData>
@@ -2464,9 +2464,9 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="18" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46287.84657407407</v>
+        <v>46288.58967592593</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.82</v>
+        <v>11.91</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>2006.5</v>
+        <v>2026.5</v>
       </c>
       <c r="L2" t="n">
-        <v>2018</v>
+        <v>2009.5</v>
       </c>
       <c r="M2" t="n">
-        <v>2032.8</v>
+        <v>2029</v>
       </c>
       <c r="N2" t="n">
-        <v>2002.2</v>
+        <v>1999.7</v>
       </c>
       <c r="O2" t="n">
-        <v>2006.5</v>
+        <v>2026.5</v>
       </c>
       <c r="P2" t="n">
-        <v>1485458</v>
+        <v>864623</v>
       </c>
       <c r="Q2" t="n">
-        <v>2006.5</v>
+        <v>2026.5</v>
       </c>
       <c r="R2" t="n">
-        <v>2200.22</v>
+        <v>2214.75</v>
       </c>
       <c r="S2" t="n">
-        <v>1909.64</v>
+        <v>1932.37</v>
       </c>
       <c r="T2" t="n">
-        <v>9.654622476949903</v>
+        <v>9.28941524796447</v>
       </c>
       <c r="U2" t="n">
-        <v>193.7199999999998</v>
+        <v>188.25</v>
       </c>
       <c r="V2" t="n">
-        <v>4.827311238474952</v>
+        <v>4.64495435479892</v>
       </c>
       <c r="W2" t="n">
-        <v>96.8599999999999</v>
+        <v>94.13000000000011</v>
       </c>
       <c r="X2" t="n">
-        <v>2</v>
+        <v>1.99989376394348</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.654622476949903</v>
+        <v>9.28941524796447</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.827311238474952</v>
+        <v>4.64495435479892</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2767,7 +2767,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0204799778532972</v>
+        <v>0.02047956570771352</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.325109569535609</v>
+        <v>0.3251030269272989</v>
       </c>
     </row>
     <row r="7">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266353403342596</v>
+        <v>0.04266352740440432</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645463</v>
+        <v>0.1869492979645464</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-22 20:19:04.623932+05:30</t>
+          <t>2026-09-23 14:09:08.723564+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.654622476949903, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.28941524796447, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998937639434802}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-23 14:59 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>STRONG BUY</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1864,7 +1864,7 @@
         <v>11.91</v>
       </c>
       <c r="R2" t="n">
-        <v>48.93</v>
+        <v>48.99</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1878,46 +1878,46 @@
         <v>2009.5</v>
       </c>
       <c r="V2" t="n">
-        <v>2029</v>
+        <v>2037.2</v>
       </c>
       <c r="W2" t="n">
         <v>1999.7</v>
       </c>
       <c r="X2" t="n">
-        <v>2026.5</v>
+        <v>2034</v>
       </c>
       <c r="Y2" t="n">
-        <v>2026.5</v>
+        <v>2034</v>
       </c>
       <c r="Z2" t="n">
-        <v>864623</v>
+        <v>1360444</v>
       </c>
       <c r="AA2" t="n">
-        <v>3375946</v>
+        <v>3400737</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.26</v>
+        <v>0.4</v>
       </c>
       <c r="AC2" t="n">
-        <v>1</v>
+        <v>1.37</v>
       </c>
       <c r="AD2" t="n">
         <v>0.15</v>
       </c>
       <c r="AE2" t="n">
-        <v>29.3</v>
+        <v>37.5</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.45</v>
+        <v>1.84</v>
       </c>
       <c r="AG2" t="n">
-        <v>47.06</v>
+        <v>47.65</v>
       </c>
       <c r="AH2" t="n">
-        <v>47.06</v>
+        <v>47.65</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.32</v>
+        <v>2.34</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,50 +1926,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>4.88</v>
+        <v>5.24</v>
       </c>
       <c r="AM2" t="n">
-        <v>10.78</v>
+        <v>11.18</v>
       </c>
       <c r="AN2" t="n">
-        <v>52.02</v>
+        <v>52.57</v>
       </c>
       <c r="AO2" t="n">
-        <v>68.20999999999999</v>
+        <v>68.88</v>
       </c>
       <c r="AP2" t="n">
-        <v>4.62</v>
+        <v>5.01</v>
       </c>
       <c r="AQ2" t="n">
-        <v>39.76</v>
+        <v>40.28</v>
       </c>
       <c r="AR2" t="n">
-        <v>2026.5</v>
+        <v>2034</v>
       </c>
       <c r="AS2" t="n">
-        <v>2214.75</v>
+        <v>2224.6</v>
       </c>
       <c r="AT2" t="n">
-        <v>1932.37</v>
+        <v>1938.7</v>
       </c>
       <c r="AU2" t="n">
-        <v>2026.5</v>
+        <v>2034</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.289999999999999</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="AY2" t="n">
-        <v>188.25</v>
+        <v>190.6</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.64</v>
+        <v>4.69</v>
       </c>
       <c r="BA2" t="n">
-        <v>94.13</v>
+        <v>95.3</v>
       </c>
       <c r="BB2" t="n">
         <v>2.02</v>
@@ -2026,10 +2026,10 @@
         <v>0.247</v>
       </c>
       <c r="BT2" t="n">
-        <v>1491.14</v>
+        <v>1492.96</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.72</v>
+        <v>-13.66</v>
       </c>
       <c r="BV2" t="n">
         <v>2.05</v>
@@ -2038,7 +2038,7 @@
         <v>2.02</v>
       </c>
       <c r="BX2" t="n">
-        <v>1.9999</v>
+        <v>2</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>75.09</v>
+        <v>77.15000000000001</v>
       </c>
       <c r="CO2" t="n">
-        <v>36.54</v>
+        <v>36.58</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2121,10 +2121,10 @@
         <v>54.54545454545454</v>
       </c>
       <c r="CY2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.289400000000001</v>
+        <v>9.370699999999999</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6193</v>
+        <v>0.6247</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3093</v>
+        <v>0.3127</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0929</v>
+        <v>0.09370000000000001</v>
       </c>
       <c r="DF2" t="n">
-        <v>2.0022</v>
+        <v>1.9979</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1064</v>
+        <v>1.116</v>
       </c>
       <c r="DH2" t="n">
         <v>4.0043</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.645</v>
+        <v>4.6853</v>
       </c>
       <c r="DJ2" t="n">
-        <v>47.16</v>
+        <v>48.43</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.645</v>
+        <v>4.6853</v>
       </c>
       <c r="DL2" t="n">
-        <v>1.9999</v>
+        <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>2</v>
+        <v>2.0043</v>
       </c>
       <c r="DN2" t="n">
         <v>4.0043</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0023</v>
+        <v>1.9978</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.863</v>
+        <v>0.8538</v>
       </c>
       <c r="DQ2" t="n">
-        <v>94.13</v>
+        <v>95.3</v>
       </c>
       <c r="DR2" t="n">
-        <v>71.90000000000001</v>
+        <v>60.59</v>
       </c>
       <c r="DS2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="DT2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.9914</v>
+        <v>2.141</v>
       </c>
       <c r="DX2" t="n">
-        <v>79.47500000000002</v>
+        <v>77.80000000000001</v>
       </c>
       <c r="DY2" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="DZ2" t="n">
-        <v>82.54900000000001</v>
+        <v>84.48099999999999</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>79.19</v>
+        <v>83.65000000000001</v>
       </c>
       <c r="ED2" t="n">
-        <v>73.69</v>
+        <v>73.81</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.9914</v>
+        <v>2.141</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.26</v>
+        <v>0.4</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.5502</v>
+        <v>0.5967</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0041</v>
+        <v>4.0046</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0655</v>
+        <v>0.0711</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7099</v>
+        <v>0.7038</v>
       </c>
       <c r="EK2" t="n">
-        <v>63.93</v>
+        <v>64.89</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2246,37 +2246,37 @@
         <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>4</v>
+        <v>6.6</v>
       </c>
       <c r="EP2" t="n">
-        <v>0.4764</v>
+        <v>0.7861</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.031</v>
+        <v>0.0476</v>
       </c>
       <c r="ER2" t="n">
-        <v>35.7308</v>
+        <v>23.425</v>
       </c>
       <c r="ES2" t="n">
-        <v>14.2048</v>
+        <v>14.5</v>
       </c>
       <c r="ET2" t="n">
-        <v>35.256</v>
+        <v>36.052</v>
       </c>
       <c r="EU2" t="n">
-        <v>1.2012</v>
+        <v>2.004</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.8413</v>
+        <v>1.6714</v>
       </c>
       <c r="EW2" t="n">
-        <v>3.0036</v>
+        <v>5.0919</v>
       </c>
       <c r="EX2" t="n">
-        <v>28.8</v>
+        <v>30.57</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2284,37 +2284,37 @@
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="FA2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="FB2" t="n">
         <v>64.8</v>
       </c>
       <c r="FC2" t="n">
-        <v>36.26</v>
+        <v>37.56</v>
       </c>
       <c r="FD2" t="n">
         <v>71.04000000000001</v>
       </c>
       <c r="FE2" t="n">
-        <v>69.51000000000001</v>
+        <v>71.02</v>
       </c>
       <c r="FF2" t="n">
-        <v>32.67</v>
+        <v>33.575</v>
       </c>
       <c r="FG2" t="n">
-        <v>22.6175</v>
+        <v>23.0988</v>
       </c>
       <c r="FH2" t="n">
-        <v>60.687</v>
+        <v>61.659</v>
       </c>
       <c r="FI2" t="n">
-        <v>59.53</v>
+        <v>54.51</v>
       </c>
       <c r="FJ2" t="n">
-        <v>66.69</v>
+        <v>65.92</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>73.87</v>
+        <v>68.22</v>
       </c>
       <c r="FO2" t="n">
-        <v>64.23</v>
+        <v>64.20999999999999</v>
       </c>
       <c r="FP2" t="n">
-        <v>55.43</v>
+        <v>49.27</v>
       </c>
       <c r="FQ2" t="n">
-        <v>80.73999999999999</v>
+        <v>71.98</v>
       </c>
       <c r="FR2" t="n">
-        <v>83.44</v>
+        <v>77.47</v>
       </c>
       <c r="FS2" t="n">
-        <v>95.4545</v>
+        <v>90.9091</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2353,11 +2353,11 @@
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>72.917</v>
+        <v>68.27200000000001</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260923_140908</t>
+          <t>20260923_202927</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46288.58968385548</v>
+        <v>46288.85379257143</v>
       </c>
     </row>
   </sheetData>
@@ -2464,9 +2464,9 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46288.58967592593</v>
+        <v>46288.85378472223</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46288</v>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>2026.5</v>
+        <v>2034</v>
       </c>
       <c r="L2" t="n">
         <v>2009.5</v>
       </c>
       <c r="M2" t="n">
-        <v>2029</v>
+        <v>2037.2</v>
       </c>
       <c r="N2" t="n">
         <v>1999.7</v>
       </c>
       <c r="O2" t="n">
-        <v>2026.5</v>
+        <v>2034</v>
       </c>
       <c r="P2" t="n">
-        <v>864623</v>
+        <v>1360444</v>
       </c>
       <c r="Q2" t="n">
-        <v>2026.5</v>
+        <v>2034</v>
       </c>
       <c r="R2" t="n">
-        <v>2214.75</v>
+        <v>2224.6</v>
       </c>
       <c r="S2" t="n">
-        <v>1932.37</v>
+        <v>1938.7</v>
       </c>
       <c r="T2" t="n">
-        <v>9.28941524796447</v>
+        <v>9.370698131760074</v>
       </c>
       <c r="U2" t="n">
-        <v>188.25</v>
+        <v>190.5999999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.64495435479892</v>
+        <v>4.685349065880037</v>
       </c>
       <c r="W2" t="n">
-        <v>94.13000000000011</v>
+        <v>95.29999999999995</v>
       </c>
       <c r="X2" t="n">
-        <v>1.99989376394348</v>
+        <v>2</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.28941524796447</v>
+        <v>9.370698131760074</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.64495435479892</v>
+        <v>4.685349065880037</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2767,7 +2767,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02047956570771352</v>
+        <v>0.02046957760840529</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3251030269272989</v>
+        <v>0.3249444707662601</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909781979290247</v>
+        <v>0.02909776058641917</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266352740440432</v>
+        <v>0.04266353535286108</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869492979645465</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.99</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-23 14:09:08.723564+05:30</t>
+          <t>2026-09-23 20:29:27.716985+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.28941524796447, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998937639434802}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.370698131760074, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-24 08:31 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="17" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H2" t="n">
         <v>8.699999999999999</v>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1864,7 +1864,7 @@
         <v>11.91</v>
       </c>
       <c r="R2" t="n">
-        <v>48.99</v>
+        <v>48.95</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>2009.5</v>
+        <v>2021.1</v>
       </c>
       <c r="V2" t="n">
-        <v>2037.2</v>
+        <v>2055.3</v>
       </c>
       <c r="W2" t="n">
-        <v>1999.7</v>
+        <v>2020</v>
       </c>
       <c r="X2" t="n">
-        <v>2034</v>
+        <v>2040.1</v>
       </c>
       <c r="Y2" t="n">
-        <v>2034</v>
+        <v>2040.1</v>
       </c>
       <c r="Z2" t="n">
-        <v>1360444</v>
+        <v>1005121</v>
       </c>
       <c r="AA2" t="n">
-        <v>3400737</v>
+        <v>3238676</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.4</v>
+        <v>0.31</v>
       </c>
       <c r="AC2" t="n">
-        <v>1.37</v>
+        <v>0.3</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.15</v>
+        <v>-0.63</v>
       </c>
       <c r="AE2" t="n">
-        <v>37.5</v>
+        <v>35.3</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.84</v>
+        <v>1.73</v>
       </c>
       <c r="AG2" t="n">
-        <v>47.65</v>
+        <v>46.77</v>
       </c>
       <c r="AH2" t="n">
-        <v>47.65</v>
+        <v>46.77</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.34</v>
+        <v>2.29</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,50 +1926,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>5.24</v>
+        <v>5.26</v>
       </c>
       <c r="AM2" t="n">
-        <v>11.18</v>
+        <v>10.93</v>
       </c>
       <c r="AN2" t="n">
-        <v>52.57</v>
+        <v>52.45</v>
       </c>
       <c r="AO2" t="n">
-        <v>68.88</v>
+        <v>69.44</v>
       </c>
       <c r="AP2" t="n">
-        <v>5.01</v>
+        <v>4.89</v>
       </c>
       <c r="AQ2" t="n">
-        <v>40.28</v>
+        <v>35.98</v>
       </c>
       <c r="AR2" t="n">
-        <v>2034</v>
+        <v>2040.1</v>
       </c>
       <c r="AS2" t="n">
-        <v>2224.6</v>
+        <v>2227.17</v>
       </c>
       <c r="AT2" t="n">
-        <v>1938.7</v>
+        <v>1946.57</v>
       </c>
       <c r="AU2" t="n">
-        <v>2034</v>
+        <v>2040.099975585938</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.369999999999999</v>
+        <v>9.17</v>
       </c>
       <c r="AY2" t="n">
-        <v>190.6</v>
+        <v>187.07</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.69</v>
+        <v>4.58</v>
       </c>
       <c r="BA2" t="n">
-        <v>95.3</v>
+        <v>93.53</v>
       </c>
       <c r="BB2" t="n">
         <v>2.02</v>
@@ -1978,7 +1978,7 @@
         <v>214</v>
       </c>
       <c r="BD2" t="n">
-        <v>32.1</v>
+        <v>32</v>
       </c>
       <c r="BE2" t="n">
         <v>327</v>
@@ -1987,10 +1987,10 @@
         <v>49</v>
       </c>
       <c r="BG2" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.9</v>
+        <v>19</v>
       </c>
       <c r="BI2" t="n">
         <v>0</v>
@@ -2005,7 +2005,7 @@
         <v>0</v>
       </c>
       <c r="BM2" t="n">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="BN2" t="n">
         <v>50.4</v>
@@ -2014,7 +2014,7 @@
         <v>2.24</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.66</v>
+        <v>8.640000000000001</v>
       </c>
       <c r="BQ2" t="n">
         <v>-4.28</v>
@@ -2026,7 +2026,7 @@
         <v>0.247</v>
       </c>
       <c r="BT2" t="n">
-        <v>1492.96</v>
+        <v>1495.03</v>
       </c>
       <c r="BU2" t="n">
         <v>-13.66</v>
@@ -2038,7 +2038,7 @@
         <v>2.02</v>
       </c>
       <c r="BX2" t="n">
-        <v>2</v>
+        <v>2.0001</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>77.15000000000001</v>
+        <v>82.73</v>
       </c>
       <c r="CO2" t="n">
-        <v>36.58</v>
+        <v>36.68</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2121,10 +2121,10 @@
         <v>54.54545454545454</v>
       </c>
       <c r="CY2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.370699999999999</v>
+        <v>9.169600000000001</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6247</v>
+        <v>0.6113</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3127</v>
+        <v>0.3053</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.09370000000000001</v>
+        <v>0.0917</v>
       </c>
       <c r="DF2" t="n">
-        <v>1.9979</v>
+        <v>2.0022</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.116</v>
+        <v>1.0921</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0043</v>
+        <v>4.0044</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.6853</v>
+        <v>4.5846</v>
       </c>
       <c r="DJ2" t="n">
-        <v>48.43</v>
+        <v>41.43</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.6853</v>
+        <v>4.5846</v>
       </c>
       <c r="DL2" t="n">
+        <v>2.0001</v>
+      </c>
+      <c r="DM2" t="n">
         <v>2</v>
       </c>
-      <c r="DM2" t="n">
-        <v>2.0043</v>
-      </c>
       <c r="DN2" t="n">
-        <v>4.0043</v>
+        <v>4.0044</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9978</v>
+        <v>2.0023</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8538</v>
+        <v>0.8743</v>
       </c>
       <c r="DQ2" t="n">
-        <v>95.3</v>
+        <v>93.53</v>
       </c>
       <c r="DR2" t="n">
-        <v>60.59</v>
+        <v>71.23999999999999</v>
       </c>
       <c r="DS2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>2.141</v>
+        <v>2.1354</v>
       </c>
       <c r="DX2" t="n">
-        <v>77.80000000000001</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="DY2" t="n">
-        <v>20</v>
+        <v>15.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>84.48099999999999</v>
+        <v>89.953</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>83.65000000000001</v>
+        <v>98.8</v>
       </c>
       <c r="ED2" t="n">
-        <v>73.81</v>
+        <v>79.09</v>
       </c>
       <c r="EE2" t="n">
-        <v>2.141</v>
+        <v>2.1354</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.4</v>
+        <v>0.31</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.5967</v>
+        <v>0.5824</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0046</v>
+        <v>4.0042</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0711</v>
+        <v>0.0694</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7038</v>
+        <v>0.7176</v>
       </c>
       <c r="EK2" t="n">
-        <v>64.89</v>
+        <v>74.33</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2249,34 @@
         <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>6.6</v>
+        <v>3.13</v>
       </c>
       <c r="EP2" t="n">
-        <v>0.7861</v>
+        <v>0.3728</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0476</v>
+        <v>0.0369</v>
       </c>
       <c r="ER2" t="n">
-        <v>23.425</v>
+        <v>29.5806</v>
       </c>
       <c r="ES2" t="n">
-        <v>14.5</v>
+        <v>12.5927</v>
       </c>
       <c r="ET2" t="n">
-        <v>36.052</v>
+        <v>35.084</v>
       </c>
       <c r="EU2" t="n">
-        <v>2.004</v>
+        <v>1.5159</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.6714</v>
+        <v>1.7481</v>
       </c>
       <c r="EW2" t="n">
-        <v>5.0919</v>
+        <v>2.5894</v>
       </c>
       <c r="EX2" t="n">
-        <v>30.57</v>
+        <v>30.83</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2284,37 +2284,37 @@
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="FA2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="FB2" t="n">
-        <v>64.8</v>
+        <v>64.91</v>
       </c>
       <c r="FC2" t="n">
-        <v>37.56</v>
+        <v>30.93</v>
       </c>
       <c r="FD2" t="n">
-        <v>71.04000000000001</v>
+        <v>71.70999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>71.02</v>
+        <v>78.53</v>
       </c>
       <c r="FF2" t="n">
-        <v>33.575</v>
+        <v>33.755</v>
       </c>
       <c r="FG2" t="n">
-        <v>23.0988</v>
+        <v>25.1459</v>
       </c>
       <c r="FH2" t="n">
-        <v>61.659</v>
+        <v>63.44</v>
       </c>
       <c r="FI2" t="n">
-        <v>54.51</v>
+        <v>56.335</v>
       </c>
       <c r="FJ2" t="n">
-        <v>65.92</v>
+        <v>66.79000000000001</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>68.22</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="FO2" t="n">
-        <v>64.20999999999999</v>
+        <v>65.18000000000001</v>
       </c>
       <c r="FP2" t="n">
-        <v>49.27</v>
+        <v>52.72</v>
       </c>
       <c r="FQ2" t="n">
-        <v>71.98</v>
+        <v>75.83</v>
       </c>
       <c r="FR2" t="n">
-        <v>77.47</v>
+        <v>82.28</v>
       </c>
       <c r="FS2" t="n">
-        <v>90.9091</v>
+        <v>95.4545</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2353,11 +2353,11 @@
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>68.27200000000001</v>
+        <v>71.3985</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260923_202927</t>
+          <t>20260924_140156</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46288.85379257143</v>
+        <v>46289.58468325198</v>
       </c>
     </row>
   </sheetData>
@@ -2464,9 +2464,9 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46288.85378472223</v>
+        <v>46289.58467592593</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>2034</v>
+        <v>2040.1</v>
       </c>
       <c r="L2" t="n">
-        <v>2009.5</v>
+        <v>2021.1</v>
       </c>
       <c r="M2" t="n">
-        <v>2037.2</v>
+        <v>2055.3</v>
       </c>
       <c r="N2" t="n">
-        <v>1999.7</v>
+        <v>2020</v>
       </c>
       <c r="O2" t="n">
-        <v>2034</v>
+        <v>2040.1</v>
       </c>
       <c r="P2" t="n">
-        <v>1360444</v>
+        <v>1005121</v>
       </c>
       <c r="Q2" t="n">
-        <v>2034</v>
+        <v>2040.1</v>
       </c>
       <c r="R2" t="n">
-        <v>2224.6</v>
+        <v>2227.17</v>
       </c>
       <c r="S2" t="n">
-        <v>1938.7</v>
+        <v>1946.57</v>
       </c>
       <c r="T2" t="n">
-        <v>9.370698131760074</v>
+        <v>9.169648546639879</v>
       </c>
       <c r="U2" t="n">
-        <v>190.5999999999999</v>
+        <v>187.0700000000002</v>
       </c>
       <c r="V2" t="n">
-        <v>4.685349065880037</v>
+        <v>4.584579187294739</v>
       </c>
       <c r="W2" t="n">
-        <v>95.29999999999995</v>
+        <v>93.52999999999997</v>
       </c>
       <c r="X2" t="n">
-        <v>2</v>
+        <v>2.000106917566558</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.370698131760074</v>
+        <v>9.169648546639879</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.685349065880037</v>
+        <v>4.584579187294739</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02046957760840529</v>
+        <v>0.0204652854735177</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3249444707662601</v>
+        <v>0.3248763352372235</v>
       </c>
     </row>
     <row r="7">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266353535286108</v>
+        <v>0.04266352473774886</v>
       </c>
     </row>
     <row r="13">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39</v>
+        <v>39.01</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-23 20:29:27.716985+05:30</t>
+          <t>2026-09-24 14:01:56.673040+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.370698131760074, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.169648546639879, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001069175665585}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-24 15:01 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="20" customWidth="1" min="47" max="47"/>
+    <col width="19" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>STRONG BUY</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.91</v>
+        <v>11.87</v>
       </c>
       <c r="R2" t="n">
-        <v>48.95</v>
+        <v>48.97</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1884,22 +1884,22 @@
         <v>2020</v>
       </c>
       <c r="X2" t="n">
-        <v>2040.1</v>
+        <v>2026.2</v>
       </c>
       <c r="Y2" t="n">
-        <v>2040.1</v>
+        <v>2026.2</v>
       </c>
       <c r="Z2" t="n">
-        <v>1005121</v>
+        <v>1387808</v>
       </c>
       <c r="AA2" t="n">
-        <v>3238676</v>
+        <v>3257811</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.31</v>
+        <v>0.43</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.3</v>
+        <v>-0.38</v>
       </c>
       <c r="AD2" t="n">
         <v>-0.63</v>
@@ -1908,7 +1908,7 @@
         <v>35.3</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.73</v>
+        <v>1.74</v>
       </c>
       <c r="AG2" t="n">
         <v>46.77</v>
@@ -1917,7 +1917,7 @@
         <v>46.77</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.29</v>
+        <v>2.31</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,47 +1926,47 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>5.26</v>
+        <v>4.58</v>
       </c>
       <c r="AM2" t="n">
-        <v>10.93</v>
+        <v>10.19</v>
       </c>
       <c r="AN2" t="n">
-        <v>52.45</v>
+        <v>51.42</v>
       </c>
       <c r="AO2" t="n">
-        <v>69.44</v>
+        <v>67.3</v>
       </c>
       <c r="AP2" t="n">
-        <v>4.89</v>
+        <v>4.17</v>
       </c>
       <c r="AQ2" t="n">
-        <v>35.98</v>
+        <v>35.05</v>
       </c>
       <c r="AR2" t="n">
-        <v>2040.1</v>
+        <v>2026.2</v>
       </c>
       <c r="AS2" t="n">
-        <v>2227.17</v>
+        <v>2213.27</v>
       </c>
       <c r="AT2" t="n">
-        <v>1946.57</v>
+        <v>1932.67</v>
       </c>
       <c r="AU2" t="n">
-        <v>2040.099975585938</v>
+        <v>2026.199951171875</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.17</v>
+        <v>9.23</v>
       </c>
       <c r="AY2" t="n">
         <v>187.07</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.58</v>
+        <v>4.62</v>
       </c>
       <c r="BA2" t="n">
         <v>93.53</v>
@@ -2011,10 +2011,10 @@
         <v>50.4</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.24</v>
+        <v>2.23</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.640000000000001</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="BQ2" t="n">
         <v>-4.28</v>
@@ -2023,13 +2023,13 @@
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.247</v>
+        <v>0.246</v>
       </c>
       <c r="BT2" t="n">
-        <v>1495.03</v>
+        <v>1491.07</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.66</v>
+        <v>-13.77</v>
       </c>
       <c r="BV2" t="n">
         <v>2.05</v>
@@ -2058,7 +2058,7 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>44.8</v>
+        <v>44.6</v>
       </c>
       <c r="CE2" t="n">
         <v>52.5</v>
@@ -2088,43 +2088,43 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>82.73</v>
+        <v>82.84</v>
       </c>
       <c r="CO2" t="n">
-        <v>36.68</v>
+        <v>37.37</v>
       </c>
       <c r="CP2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CQ2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CR2" t="n">
-        <v>86.36363636363636</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="CS2" t="n">
         <v>100</v>
       </c>
       <c r="CT2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CU2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CV2" t="n">
-        <v>86.36363636363636</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="CW2" t="n">
-        <v>68.18181818181817</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="CX2" t="n">
-        <v>54.54545454545454</v>
+        <v>57.14285714285714</v>
       </c>
       <c r="CY2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.169600000000001</v>
+        <v>9.2326</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,31 +2133,31 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6113</v>
+        <v>0.6153</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3053</v>
+        <v>0.308</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0917</v>
+        <v>0.09229999999999999</v>
       </c>
       <c r="DF2" t="n">
-        <v>2.0022</v>
+        <v>1.9978</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.0921</v>
+        <v>1.0956</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0044</v>
+        <v>3.9957</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.5846</v>
+        <v>4.616</v>
       </c>
       <c r="DJ2" t="n">
-        <v>41.43</v>
+        <v>42.22</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.5846</v>
+        <v>4.616</v>
       </c>
       <c r="DL2" t="n">
         <v>2.0001</v>
@@ -2166,25 +2166,25 @@
         <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>4.0044</v>
+        <v>3.9957</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0023</v>
+        <v>1.9977</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8743</v>
+        <v>0.8649</v>
       </c>
       <c r="DQ2" t="n">
         <v>93.53</v>
       </c>
       <c r="DR2" t="n">
-        <v>71.23999999999999</v>
+        <v>45.52</v>
       </c>
       <c r="DS2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="DT2" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>2.1354</v>
+        <v>1.8052</v>
       </c>
       <c r="DX2" t="n">
-        <v>76.40000000000001</v>
+        <v>81.75</v>
       </c>
       <c r="DY2" t="n">
-        <v>15.5</v>
+        <v>21.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>89.953</v>
+        <v>88.66500000000001</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>98.8</v>
+        <v>94.38</v>
       </c>
       <c r="ED2" t="n">
-        <v>79.09</v>
+        <v>84.17</v>
       </c>
       <c r="EE2" t="n">
-        <v>2.1354</v>
+        <v>1.8052</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.31</v>
+        <v>0.43</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.5824</v>
+        <v>0.495</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0042</v>
+        <v>3.9968</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0694</v>
+        <v>0.0588</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7176</v>
+        <v>0.7112000000000001</v>
       </c>
       <c r="EK2" t="n">
-        <v>74.33</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2249,34 @@
         <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>3.13</v>
+        <v>3.51</v>
       </c>
       <c r="EP2" t="n">
-        <v>0.3728</v>
+        <v>0.4166</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0369</v>
+        <v>0.051</v>
       </c>
       <c r="ER2" t="n">
-        <v>29.5806</v>
+        <v>21.4651</v>
       </c>
       <c r="ES2" t="n">
-        <v>12.5927</v>
+        <v>12.7553</v>
       </c>
       <c r="ET2" t="n">
-        <v>35.084</v>
+        <v>35.33</v>
       </c>
       <c r="EU2" t="n">
-        <v>1.5159</v>
+        <v>1.7931</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.7481</v>
+        <v>1.6154</v>
       </c>
       <c r="EW2" t="n">
-        <v>2.5894</v>
+        <v>2.9077</v>
       </c>
       <c r="EX2" t="n">
-        <v>30.83</v>
+        <v>32.14</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2290,31 @@
         <v>8</v>
       </c>
       <c r="FB2" t="n">
-        <v>64.91</v>
+        <v>64.43000000000001</v>
       </c>
       <c r="FC2" t="n">
-        <v>30.93</v>
+        <v>31.49</v>
       </c>
       <c r="FD2" t="n">
-        <v>71.70999999999999</v>
+        <v>71.61</v>
       </c>
       <c r="FE2" t="n">
-        <v>78.53</v>
+        <v>75.72</v>
       </c>
       <c r="FF2" t="n">
-        <v>33.755</v>
+        <v>34.755</v>
       </c>
       <c r="FG2" t="n">
-        <v>25.1459</v>
+        <v>25.0272</v>
       </c>
       <c r="FH2" t="n">
-        <v>63.44</v>
+        <v>63.495</v>
       </c>
       <c r="FI2" t="n">
-        <v>56.335</v>
+        <v>43.87</v>
       </c>
       <c r="FJ2" t="n">
-        <v>66.79000000000001</v>
+        <v>66.27</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>72.90000000000001</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="FO2" t="n">
-        <v>65.18000000000001</v>
+        <v>64.02</v>
       </c>
       <c r="FP2" t="n">
-        <v>52.72</v>
+        <v>41.33</v>
       </c>
       <c r="FQ2" t="n">
-        <v>75.83</v>
+        <v>63.93</v>
       </c>
       <c r="FR2" t="n">
-        <v>82.28</v>
+        <v>73.87</v>
       </c>
       <c r="FS2" t="n">
-        <v>95.4545</v>
+        <v>90.47620000000001</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2353,11 +2353,11 @@
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>71.3985</v>
+        <v>63.35</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260924_140156</t>
+          <t>20260924_203140</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46289.58468325198</v>
+        <v>46289.85533341491</v>
       </c>
     </row>
   </sheetData>
@@ -2464,7 +2464,7 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46289.58467592593</v>
+        <v>46289.85532407407</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46289</v>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.91</v>
+        <v>11.87</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>2040.1</v>
+        <v>2026.2</v>
       </c>
       <c r="L2" t="n">
         <v>2021.1</v>
@@ -2693,34 +2693,34 @@
         <v>2020</v>
       </c>
       <c r="O2" t="n">
-        <v>2040.1</v>
+        <v>2026.2</v>
       </c>
       <c r="P2" t="n">
-        <v>1005121</v>
+        <v>1387808</v>
       </c>
       <c r="Q2" t="n">
-        <v>2040.1</v>
+        <v>2026.2</v>
       </c>
       <c r="R2" t="n">
-        <v>2227.17</v>
+        <v>2213.27</v>
       </c>
       <c r="S2" t="n">
-        <v>1946.57</v>
+        <v>1932.67</v>
       </c>
       <c r="T2" t="n">
-        <v>9.169648546639879</v>
+        <v>9.232553548514458</v>
       </c>
       <c r="U2" t="n">
-        <v>187.0700000000002</v>
+        <v>187.0699999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.584579187294739</v>
+        <v>4.616030006909484</v>
       </c>
       <c r="W2" t="n">
         <v>93.52999999999997</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000106917566558</v>
+        <v>2.000106917566556</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.169648546639879</v>
+        <v>9.232553548514458</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.584579187294739</v>
+        <v>4.616030006909484</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0204652854735177</v>
+        <v>0.02045637796684109</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3248763352372235</v>
+        <v>0.3247349329524157</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909776058641917</v>
+        <v>0.02909770137993588</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266352473774886</v>
+        <v>0.04266353730326321</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645465</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.01</v>
+        <v>39.02</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-24 14:01:56.673040+05:30</t>
+          <t>2026-09-24 20:31:40.837056+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.169648546639879, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001069175665585}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.232553548514458, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001069175665562}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-25 08:53 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="17" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,16 +1816,14 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46289</v>
-      </c>
-      <c r="E2" s="1" t="n">
-        <v>46289</v>
-      </c>
+        <v>46290</v>
+      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H2" t="n">
         <v>8.699999999999999</v>
@@ -1854,70 +1852,66 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="P2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.87</v>
+        <v>11.65</v>
       </c>
       <c r="R2" t="n">
-        <v>48.97</v>
+        <v>48.83</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
       </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>UPTREND</t>
-        </is>
-      </c>
+      <c r="T2" t="inlineStr"/>
       <c r="U2" t="n">
-        <v>2021.1</v>
+        <v>2026</v>
       </c>
       <c r="V2" t="n">
-        <v>2055.3</v>
+        <v>2040</v>
       </c>
       <c r="W2" t="n">
-        <v>2020</v>
+        <v>1979.2</v>
       </c>
       <c r="X2" t="n">
-        <v>2026.2</v>
+        <v>1995.7</v>
       </c>
       <c r="Y2" t="n">
-        <v>2026.2</v>
+        <v>1995.7</v>
       </c>
       <c r="Z2" t="n">
-        <v>1387808</v>
+        <v>1188082</v>
       </c>
       <c r="AA2" t="n">
-        <v>3257811</v>
+        <v>3205653</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.43</v>
+        <v>0.37</v>
       </c>
       <c r="AC2" t="n">
-        <v>-0.38</v>
+        <v>-1.51</v>
       </c>
       <c r="AD2" t="n">
-        <v>-0.63</v>
+        <v>-0.01</v>
       </c>
       <c r="AE2" t="n">
-        <v>35.3</v>
+        <v>60.8</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.74</v>
+        <v>3.05</v>
       </c>
       <c r="AG2" t="n">
-        <v>46.77</v>
+        <v>47.77</v>
       </c>
       <c r="AH2" t="n">
-        <v>46.77</v>
+        <v>47.77</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.31</v>
+        <v>2.39</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,53 +1920,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>4.58</v>
+        <v>2.85</v>
       </c>
       <c r="AM2" t="n">
-        <v>10.19</v>
+        <v>7.99</v>
       </c>
       <c r="AN2" t="n">
-        <v>51.42</v>
+        <v>48.6</v>
       </c>
       <c r="AO2" t="n">
-        <v>67.3</v>
+        <v>61.39</v>
       </c>
       <c r="AP2" t="n">
-        <v>4.17</v>
+        <v>1.36</v>
       </c>
       <c r="AQ2" t="n">
-        <v>35.05</v>
+        <v>31.52</v>
       </c>
       <c r="AR2" t="n">
-        <v>2026.2</v>
+        <v>1995.7</v>
       </c>
       <c r="AS2" t="n">
-        <v>2213.27</v>
+        <v>2186.78</v>
       </c>
       <c r="AT2" t="n">
-        <v>1932.67</v>
+        <v>1900.16</v>
       </c>
       <c r="AU2" t="n">
-        <v>2026.199951171875</v>
+        <v>1995.699951171875</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.23</v>
+        <v>9.57</v>
       </c>
       <c r="AY2" t="n">
-        <v>187.07</v>
+        <v>191.08</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.62</v>
+        <v>4.79</v>
       </c>
       <c r="BA2" t="n">
-        <v>93.53</v>
+        <v>95.54000000000001</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.02</v>
+        <v>2.04</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
@@ -1984,61 +1978,61 @@
         <v>327</v>
       </c>
       <c r="BF2" t="n">
-        <v>49</v>
+        <v>48.9</v>
       </c>
       <c r="BG2" t="n">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="BH2" t="n">
-        <v>19</v>
+        <v>18.5</v>
       </c>
       <c r="BI2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="BM2" t="n">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="BN2" t="n">
-        <v>50.4</v>
+        <v>49.9</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.23</v>
+        <v>2.21</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.630000000000001</v>
+        <v>8.69</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.28</v>
+        <v>-4.25</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.246</v>
+        <v>0.244</v>
       </c>
       <c r="BT2" t="n">
-        <v>1491.07</v>
+        <v>1479.98</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.77</v>
+        <v>-14.07</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.05</v>
+        <v>2.04</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.02</v>
+        <v>2.04</v>
       </c>
       <c r="BX2" t="n">
-        <v>2.0001</v>
+        <v>2</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2058,16 +2052,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>44.6</v>
+        <v>44.2</v>
       </c>
       <c r="CE2" t="n">
-        <v>52.5</v>
+        <v>52</v>
       </c>
       <c r="CF2" t="n">
-        <v>67.3</v>
+        <v>68</v>
       </c>
       <c r="CG2" t="n">
-        <v>72</v>
+        <v>71.3</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,43 +2082,43 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>82.84</v>
+        <v>79.65000000000001</v>
       </c>
       <c r="CO2" t="n">
-        <v>37.37</v>
+        <v>46.06</v>
       </c>
       <c r="CP2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CQ2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CR2" t="n">
-        <v>85.71428571428571</v>
+        <v>86.36363636363636</v>
       </c>
       <c r="CS2" t="n">
         <v>100</v>
       </c>
       <c r="CT2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CU2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CV2" t="n">
-        <v>85.71428571428571</v>
+        <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>66.66666666666666</v>
+        <v>68.18181818181817</v>
       </c>
       <c r="CX2" t="n">
-        <v>57.14285714285714</v>
+        <v>54.54545454545454</v>
       </c>
       <c r="CY2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.2326</v>
+        <v>9.5746</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2127,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6153</v>
+        <v>0.638</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.308</v>
+        <v>0.3193</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.09229999999999999</v>
+        <v>0.09569999999999999</v>
       </c>
       <c r="DF2" t="n">
-        <v>1.9978</v>
+        <v>1.9979</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.0956</v>
+        <v>1.1149</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9957</v>
+        <v>4.0042</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.616</v>
+        <v>4.7873</v>
       </c>
       <c r="DJ2" t="n">
-        <v>42.22</v>
+        <v>42.62</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.616</v>
+        <v>4.7873</v>
       </c>
       <c r="DL2" t="n">
-        <v>2.0001</v>
+        <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>2</v>
+        <v>2.0042</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9957</v>
+        <v>4.0042</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9977</v>
+        <v>1.9981</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8649</v>
+        <v>0.8359</v>
       </c>
       <c r="DQ2" t="n">
-        <v>93.53</v>
+        <v>95.54000000000001</v>
       </c>
       <c r="DR2" t="n">
-        <v>45.52</v>
+        <v>47.55</v>
       </c>
       <c r="DS2" t="n">
         <v>3</v>
       </c>
       <c r="DT2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2187,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.8052</v>
+        <v>0.569</v>
       </c>
       <c r="DX2" t="n">
-        <v>81.75</v>
+        <v>96.52499999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>21.5</v>
+        <v>18.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>88.66500000000001</v>
+        <v>82.322</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2205,31 @@
         <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>94.38</v>
+        <v>72.01000000000001</v>
       </c>
       <c r="ED2" t="n">
-        <v>84.17</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.8052</v>
+        <v>0.569</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.43</v>
+        <v>0.37</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.495</v>
+        <v>0.1584</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9968</v>
+        <v>4.0061</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0588</v>
+        <v>0.0185</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7112000000000001</v>
+        <v>0.6919</v>
       </c>
       <c r="EK2" t="n">
-        <v>68.59999999999999</v>
+        <v>70.02</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,72 +2243,72 @@
         <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>3.51</v>
+        <v>7.19</v>
       </c>
       <c r="EP2" t="n">
-        <v>0.4166</v>
+        <v>0.8376</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.051</v>
+        <v>0.0431</v>
       </c>
       <c r="ER2" t="n">
-        <v>21.4651</v>
+        <v>25.8649</v>
       </c>
       <c r="ES2" t="n">
-        <v>12.7553</v>
+        <v>12.5723</v>
       </c>
       <c r="ET2" t="n">
-        <v>35.33</v>
+        <v>39.685</v>
       </c>
       <c r="EU2" t="n">
-        <v>1.7931</v>
+        <v>0.5032</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.6154</v>
+        <v>1.7445</v>
       </c>
       <c r="EW2" t="n">
-        <v>2.9077</v>
+        <v>5.7268</v>
       </c>
       <c r="EX2" t="n">
-        <v>32.14</v>
+        <v>45.43</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="FA2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="FB2" t="n">
-        <v>64.43000000000001</v>
+        <v>63.68</v>
       </c>
       <c r="FC2" t="n">
-        <v>31.49</v>
+        <v>33.32</v>
       </c>
       <c r="FD2" t="n">
-        <v>71.61</v>
+        <v>72.77</v>
       </c>
       <c r="FE2" t="n">
-        <v>75.72</v>
+        <v>74.83499999999999</v>
       </c>
       <c r="FF2" t="n">
-        <v>34.755</v>
+        <v>45.745</v>
       </c>
       <c r="FG2" t="n">
-        <v>25.0272</v>
+        <v>23.4956</v>
       </c>
       <c r="FH2" t="n">
-        <v>63.495</v>
+        <v>64.821</v>
       </c>
       <c r="FI2" t="n">
-        <v>43.87</v>
+        <v>45.085</v>
       </c>
       <c r="FJ2" t="n">
-        <v>66.27</v>
+        <v>66.65000000000001</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2322,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>64.09999999999999</v>
+        <v>65.31999999999999</v>
       </c>
       <c r="FO2" t="n">
-        <v>64.02</v>
+        <v>64.09</v>
       </c>
       <c r="FP2" t="n">
-        <v>41.33</v>
+        <v>52.31</v>
       </c>
       <c r="FQ2" t="n">
-        <v>63.93</v>
+        <v>62</v>
       </c>
       <c r="FR2" t="n">
-        <v>73.87</v>
+        <v>74.34</v>
       </c>
       <c r="FS2" t="n">
-        <v>90.47620000000001</v>
+        <v>95.4545</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2357,7 +2351,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>63.35</v>
+        <v>64.02549999999999</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260924_203140</t>
+          <t>20260925_142345</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46289.85533341491</v>
+        <v>46290.59983286201</v>
       </c>
     </row>
   </sheetData>
@@ -2444,8 +2438,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -2466,7 +2460,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="19" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,14 +2641,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46289.85532407407</v>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>46289</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>46304</v>
-      </c>
+        <v>46290.59982638889</v>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>LAURUSLABS</t>
@@ -2673,54 +2663,50 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.87</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>UPTREND</t>
-        </is>
-      </c>
+        <v>11.65</v>
+      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>2026.2</v>
+        <v>1995.7</v>
       </c>
       <c r="L2" t="n">
-        <v>2021.1</v>
+        <v>2026</v>
       </c>
       <c r="M2" t="n">
-        <v>2055.3</v>
+        <v>2040</v>
       </c>
       <c r="N2" t="n">
-        <v>2020</v>
+        <v>1979.2</v>
       </c>
       <c r="O2" t="n">
-        <v>2026.2</v>
+        <v>1995.7</v>
       </c>
       <c r="P2" t="n">
-        <v>1387808</v>
+        <v>1188082</v>
       </c>
       <c r="Q2" t="n">
-        <v>2026.2</v>
+        <v>1995.7</v>
       </c>
       <c r="R2" t="n">
-        <v>2213.27</v>
+        <v>2186.78</v>
       </c>
       <c r="S2" t="n">
-        <v>1932.67</v>
+        <v>1900.16</v>
       </c>
       <c r="T2" t="n">
-        <v>9.232553548514458</v>
+        <v>9.574585358520828</v>
       </c>
       <c r="U2" t="n">
-        <v>187.0699999999999</v>
+        <v>191.0800000000002</v>
       </c>
       <c r="V2" t="n">
-        <v>4.616030006909484</v>
+        <v>4.787292679260409</v>
       </c>
       <c r="W2" t="n">
-        <v>93.52999999999997</v>
+        <v>95.53999999999996</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000106917566556</v>
+        <v>2.000000000000002</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.232553548514458</v>
+        <v>9.574585358520828</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.616030006909484</v>
+        <v>4.787292679260409</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02045637796684109</v>
+        <v>0.02045266715794346</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3247349329524157</v>
+        <v>0.3246760256873797</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909770137993588</v>
+        <v>0.02909764217345259</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266353730326321</v>
+        <v>0.04266353310149015</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869492979645464</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.02</v>
+        <v>39.03</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-24 20:31:40.837056+05:30</t>
+          <t>2026-09-25 14:23:45.595600+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.232553548514458, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001069175665562}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.574585358520828, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000000000000002}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-25 15:13 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="19" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="17" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1859,10 +1859,10 @@
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.65</v>
+        <v>11.7</v>
       </c>
       <c r="R2" t="n">
-        <v>48.83</v>
+        <v>48.92</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1878,22 +1878,22 @@
         <v>1979.2</v>
       </c>
       <c r="X2" t="n">
-        <v>1995.7</v>
+        <v>2007</v>
       </c>
       <c r="Y2" t="n">
-        <v>1995.7</v>
+        <v>2007</v>
       </c>
       <c r="Z2" t="n">
-        <v>1188082</v>
+        <v>1438852</v>
       </c>
       <c r="AA2" t="n">
-        <v>3205653</v>
+        <v>3218191</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.37</v>
+        <v>0.45</v>
       </c>
       <c r="AC2" t="n">
-        <v>-1.51</v>
+        <v>-0.95</v>
       </c>
       <c r="AD2" t="n">
         <v>-0.01</v>
@@ -1902,7 +1902,7 @@
         <v>60.8</v>
       </c>
       <c r="AF2" t="n">
-        <v>3.05</v>
+        <v>3.03</v>
       </c>
       <c r="AG2" t="n">
         <v>47.77</v>
@@ -1911,7 +1911,7 @@
         <v>47.77</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.39</v>
+        <v>2.38</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,53 +1920,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>2.85</v>
+        <v>3.4</v>
       </c>
       <c r="AM2" t="n">
-        <v>7.99</v>
+        <v>8.59</v>
       </c>
       <c r="AN2" t="n">
-        <v>48.6</v>
+        <v>49.43</v>
       </c>
       <c r="AO2" t="n">
-        <v>61.39</v>
+        <v>63.46</v>
       </c>
       <c r="AP2" t="n">
-        <v>1.36</v>
+        <v>1.93</v>
       </c>
       <c r="AQ2" t="n">
-        <v>31.52</v>
+        <v>32.27</v>
       </c>
       <c r="AR2" t="n">
-        <v>1995.7</v>
+        <v>2007</v>
       </c>
       <c r="AS2" t="n">
-        <v>2186.78</v>
+        <v>2198.08</v>
       </c>
       <c r="AT2" t="n">
-        <v>1900.16</v>
+        <v>1911.46</v>
       </c>
       <c r="AU2" t="n">
-        <v>1995.699951171875</v>
+        <v>2007</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.57</v>
+        <v>9.52</v>
       </c>
       <c r="AY2" t="n">
         <v>191.08</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.79</v>
+        <v>4.76</v>
       </c>
       <c r="BA2" t="n">
         <v>95.54000000000001</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.04</v>
+        <v>2.05</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
@@ -2005,31 +2005,31 @@
         <v>49.9</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.21</v>
+        <v>2.22</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.69</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.25</v>
+        <v>-4.24</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.244</v>
+        <v>0.245</v>
       </c>
       <c r="BT2" t="n">
-        <v>1479.98</v>
+        <v>1484.08</v>
       </c>
       <c r="BU2" t="n">
-        <v>-14.07</v>
+        <v>-13.97</v>
       </c>
       <c r="BV2" t="n">
         <v>2.04</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.04</v>
+        <v>2.05</v>
       </c>
       <c r="BX2" t="n">
         <v>2</v>
@@ -2052,13 +2052,13 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>44.2</v>
+        <v>44.4</v>
       </c>
       <c r="CE2" t="n">
         <v>52</v>
       </c>
       <c r="CF2" t="n">
-        <v>68</v>
+        <v>68.3</v>
       </c>
       <c r="CG2" t="n">
         <v>71.3</v>
@@ -2082,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>79.65000000000001</v>
+        <v>81.41</v>
       </c>
       <c r="CO2" t="n">
-        <v>46.06</v>
+        <v>43.72</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2118,7 +2118,7 @@
         <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.5746</v>
+        <v>9.5207</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,58 +2127,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.638</v>
+        <v>0.6347</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3193</v>
+        <v>0.3173</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.09569999999999999</v>
+        <v>0.09520000000000001</v>
       </c>
       <c r="DF2" t="n">
-        <v>1.9979</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1149</v>
+        <v>1.1138</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0042</v>
+        <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.7873</v>
+        <v>4.7603</v>
       </c>
       <c r="DJ2" t="n">
-        <v>42.62</v>
+        <v>41.71</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.7873</v>
+        <v>4.7603</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>2.0042</v>
+        <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>4.0042</v>
+        <v>4</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9981</v>
+        <v>2.0003</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8359</v>
+        <v>0.8403</v>
       </c>
       <c r="DQ2" t="n">
         <v>95.54000000000001</v>
       </c>
       <c r="DR2" t="n">
-        <v>47.55</v>
+        <v>61.82</v>
       </c>
       <c r="DS2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,16 +2187,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.569</v>
+        <v>0.8109</v>
       </c>
       <c r="DX2" t="n">
-        <v>96.52499999999999</v>
+        <v>91.34999999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>18.5</v>
+        <v>22.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>82.322</v>
+        <v>84.16500000000001</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2205,31 +2205,31 @@
         <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>72.01000000000001</v>
+        <v>78.52</v>
       </c>
       <c r="ED2" t="n">
-        <v>96.59999999999999</v>
+        <v>91.31999999999999</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.569</v>
+        <v>0.8109</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.37</v>
+        <v>0.45</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.1584</v>
+        <v>0.2258</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0061</v>
+        <v>4.0003</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0185</v>
+        <v>0.0264</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6919</v>
+        <v>0.6945</v>
       </c>
       <c r="EK2" t="n">
-        <v>70.02</v>
+        <v>69.77</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2243,34 +2243,34 @@
         <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>7.19</v>
+        <v>6.09</v>
       </c>
       <c r="EP2" t="n">
-        <v>0.8376</v>
+        <v>0.7125</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0431</v>
+        <v>0.0526</v>
       </c>
       <c r="ER2" t="n">
-        <v>25.8649</v>
+        <v>21.1556</v>
       </c>
       <c r="ES2" t="n">
-        <v>12.5723</v>
+        <v>12.3402</v>
       </c>
       <c r="ET2" t="n">
-        <v>39.685</v>
+        <v>38.491</v>
       </c>
       <c r="EU2" t="n">
-        <v>0.5032</v>
+        <v>0.8685</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.7445</v>
+        <v>1.6414</v>
       </c>
       <c r="EW2" t="n">
-        <v>5.7268</v>
+        <v>4.9579</v>
       </c>
       <c r="EX2" t="n">
-        <v>45.43</v>
+        <v>44.45</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2284,31 +2284,31 @@
         <v>9</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.68</v>
+        <v>63.92</v>
       </c>
       <c r="FC2" t="n">
-        <v>33.32</v>
+        <v>32.25</v>
       </c>
       <c r="FD2" t="n">
-        <v>72.77</v>
+        <v>73.3</v>
       </c>
       <c r="FE2" t="n">
-        <v>74.83499999999999</v>
+        <v>75.59</v>
       </c>
       <c r="FF2" t="n">
-        <v>45.745</v>
+        <v>44.085</v>
       </c>
       <c r="FG2" t="n">
-        <v>23.4956</v>
+        <v>24.0858</v>
       </c>
       <c r="FH2" t="n">
-        <v>64.821</v>
+        <v>65.273</v>
       </c>
       <c r="FI2" t="n">
-        <v>45.085</v>
+        <v>51.765</v>
       </c>
       <c r="FJ2" t="n">
-        <v>66.65000000000001</v>
+        <v>67.26000000000001</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,19 +2322,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>65.31999999999999</v>
+        <v>72.09</v>
       </c>
       <c r="FO2" t="n">
-        <v>64.09</v>
+        <v>63.91</v>
       </c>
       <c r="FP2" t="n">
-        <v>52.31</v>
+        <v>60.76</v>
       </c>
       <c r="FQ2" t="n">
-        <v>62</v>
+        <v>72.78</v>
       </c>
       <c r="FR2" t="n">
-        <v>74.34</v>
+        <v>82.79000000000001</v>
       </c>
       <c r="FS2" t="n">
         <v>95.4545</v>
@@ -2347,11 +2347,11 @@
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>64.02549999999999</v>
+        <v>70.37649999999999</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260925_142345</t>
+          <t>20260925_204343</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46290.59983286201</v>
+        <v>46290.86370059318</v>
       </c>
     </row>
   </sheetData>
@@ -2460,7 +2460,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="19" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46290.59982638889</v>
+        <v>46290.86369212963</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2663,11 +2663,11 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.65</v>
+        <v>11.7</v>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>1995.7</v>
+        <v>2007</v>
       </c>
       <c r="L2" t="n">
         <v>2026</v>
@@ -2679,34 +2679,34 @@
         <v>1979.2</v>
       </c>
       <c r="O2" t="n">
-        <v>1995.7</v>
+        <v>2007</v>
       </c>
       <c r="P2" t="n">
-        <v>1188082</v>
+        <v>1438852</v>
       </c>
       <c r="Q2" t="n">
-        <v>1995.7</v>
+        <v>2007</v>
       </c>
       <c r="R2" t="n">
-        <v>2186.78</v>
+        <v>2198.08</v>
       </c>
       <c r="S2" t="n">
-        <v>1900.16</v>
+        <v>1911.46</v>
       </c>
       <c r="T2" t="n">
-        <v>9.574585358520828</v>
+        <v>9.520677628300943</v>
       </c>
       <c r="U2" t="n">
-        <v>191.0800000000002</v>
+        <v>191.0799999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.787292679260409</v>
+        <v>4.760338814150471</v>
       </c>
       <c r="W2" t="n">
         <v>95.53999999999996</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000000000000002</v>
+        <v>2</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.574585358520828</v>
+        <v>9.520677628300943</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.787292679260409</v>
+        <v>4.760338814150471</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02045266715794346</v>
+        <v>0.02044686195612276</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3246760256873797</v>
+        <v>0.324583870965411</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909764217345259</v>
+        <v>0.02909753504945897</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266353310149015</v>
+        <v>0.04266353304091999</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-25 14:23:45.595600+05:30</t>
+          <t>2026-09-25 20:43:43.770596+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.574585358520828, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000000000000002}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.520677628300943, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-28 09:53 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -1816,14 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46290</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
+        <v>46293</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>46293</v>
+      </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46290</v>
+        <v>46293</v>
       </c>
       <c r="H2" t="n">
         <v>8.699999999999999</v>
@@ -1852,66 +1854,70 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="P2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q2" t="n">
         <v>11.7</v>
       </c>
       <c r="R2" t="n">
-        <v>48.92</v>
+        <v>49.02</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
       </c>
-      <c r="T2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>UPTREND</t>
+        </is>
+      </c>
       <c r="U2" t="n">
-        <v>2026</v>
+        <v>2000</v>
       </c>
       <c r="V2" t="n">
-        <v>2040</v>
+        <v>2012.3</v>
       </c>
       <c r="W2" t="n">
-        <v>1979.2</v>
+        <v>1984.8</v>
       </c>
       <c r="X2" t="n">
-        <v>2007</v>
+        <v>2010</v>
       </c>
       <c r="Y2" t="n">
-        <v>2007</v>
+        <v>2010</v>
       </c>
       <c r="Z2" t="n">
-        <v>1438852</v>
+        <v>926358</v>
       </c>
       <c r="AA2" t="n">
-        <v>3218191</v>
+        <v>1714906</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.45</v>
+        <v>0.54</v>
       </c>
       <c r="AC2" t="n">
-        <v>-0.95</v>
+        <v>0.15</v>
       </c>
       <c r="AD2" t="n">
-        <v>-0.01</v>
+        <v>-0.35</v>
       </c>
       <c r="AE2" t="n">
-        <v>60.8</v>
+        <v>27.5</v>
       </c>
       <c r="AF2" t="n">
-        <v>3.03</v>
+        <v>1.37</v>
       </c>
       <c r="AG2" t="n">
-        <v>47.77</v>
+        <v>46.32</v>
       </c>
       <c r="AH2" t="n">
-        <v>47.77</v>
+        <v>46.32</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.38</v>
+        <v>2.3</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,50 +1926,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>3.4</v>
+        <v>3.31</v>
       </c>
       <c r="AM2" t="n">
-        <v>8.59</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="AN2" t="n">
-        <v>49.43</v>
+        <v>49.1</v>
       </c>
       <c r="AO2" t="n">
-        <v>63.46</v>
+        <v>63.8</v>
       </c>
       <c r="AP2" t="n">
-        <v>1.93</v>
+        <v>2.08</v>
       </c>
       <c r="AQ2" t="n">
-        <v>32.27</v>
+        <v>34.6</v>
       </c>
       <c r="AR2" t="n">
-        <v>2007</v>
+        <v>2010</v>
       </c>
       <c r="AS2" t="n">
-        <v>2198.08</v>
+        <v>2195.29</v>
       </c>
       <c r="AT2" t="n">
-        <v>1911.46</v>
+        <v>1917.36</v>
       </c>
       <c r="AU2" t="n">
-        <v>2007</v>
+        <v>2010</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.52</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="AY2" t="n">
-        <v>191.08</v>
+        <v>185.29</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.76</v>
+        <v>4.61</v>
       </c>
       <c r="BA2" t="n">
-        <v>95.54000000000001</v>
+        <v>92.64</v>
       </c>
       <c r="BB2" t="n">
         <v>2.05</v>
@@ -1981,22 +1987,22 @@
         <v>48.9</v>
       </c>
       <c r="BG2" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.5</v>
+        <v>18.7</v>
       </c>
       <c r="BI2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="BM2" t="n">
         <v>669</v>
@@ -2020,19 +2026,19 @@
         <v>0.245</v>
       </c>
       <c r="BT2" t="n">
-        <v>1484.08</v>
+        <v>1485.18</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.97</v>
+        <v>-13.83</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.04</v>
+        <v>2.05</v>
       </c>
       <c r="BW2" t="n">
         <v>2.05</v>
       </c>
       <c r="BX2" t="n">
-        <v>2</v>
+        <v>2.0001</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2041,7 +2047,7 @@
         <v>8</v>
       </c>
       <c r="CA2" t="n">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="CB2" t="n">
         <v>0</v>
@@ -2055,7 +2061,7 @@
         <v>44.4</v>
       </c>
       <c r="CE2" t="n">
-        <v>52</v>
+        <v>52.5</v>
       </c>
       <c r="CF2" t="n">
         <v>68.3</v>
@@ -2082,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>81.41</v>
+        <v>89.45</v>
       </c>
       <c r="CO2" t="n">
-        <v>43.72</v>
+        <v>35.06</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2115,10 +2121,10 @@
         <v>54.54545454545454</v>
       </c>
       <c r="CY2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.5207</v>
+        <v>9.218400000000001</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6347</v>
+        <v>0.6147</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3173</v>
+        <v>0.3073</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.09520000000000001</v>
+        <v>0.0922</v>
       </c>
       <c r="DF2" t="n">
         <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1138</v>
+        <v>1.0787</v>
       </c>
       <c r="DH2" t="n">
-        <v>4</v>
+        <v>4.0087</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.7603</v>
+        <v>4.609</v>
       </c>
       <c r="DJ2" t="n">
-        <v>41.71</v>
+        <v>32.57</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.7603</v>
+        <v>4.609</v>
       </c>
       <c r="DL2" t="n">
-        <v>2</v>
+        <v>2.0001</v>
       </c>
       <c r="DM2" t="n">
-        <v>2</v>
+        <v>2.0043</v>
       </c>
       <c r="DN2" t="n">
-        <v>4</v>
+        <v>4.0087</v>
       </c>
       <c r="DO2" t="n">
         <v>2.0003</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8403</v>
+        <v>0.8696</v>
       </c>
       <c r="DQ2" t="n">
-        <v>95.54000000000001</v>
+        <v>92.64</v>
       </c>
       <c r="DR2" t="n">
-        <v>61.82</v>
+        <v>74.08</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,90 +2193,90 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.8109</v>
+        <v>0.9043</v>
       </c>
       <c r="DX2" t="n">
-        <v>91.34999999999999</v>
+        <v>90.5</v>
       </c>
       <c r="DY2" t="n">
-        <v>22.5</v>
+        <v>27</v>
       </c>
       <c r="DZ2" t="n">
-        <v>84.16500000000001</v>
+        <v>88.426</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
       </c>
       <c r="EB2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>78.52</v>
+        <v>92.77</v>
       </c>
       <c r="ED2" t="n">
-        <v>91.31999999999999</v>
+        <v>99.98</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.8109</v>
+        <v>0.9043</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.45</v>
+        <v>0.54</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.2258</v>
+        <v>0.2434</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0003</v>
+        <v>4.008</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0264</v>
+        <v>0.0285</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6945</v>
+        <v>0.7144</v>
       </c>
       <c r="EK2" t="n">
-        <v>69.77</v>
+        <v>85.68000000000001</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Excellent</t>
         </is>
       </c>
       <c r="EM2" t="n">
         <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>6.09</v>
+        <v>5.95</v>
       </c>
       <c r="EP2" t="n">
-        <v>0.7125</v>
+        <v>0.6961000000000001</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0526</v>
+        <v>0.06320000000000001</v>
       </c>
       <c r="ER2" t="n">
-        <v>21.1556</v>
+        <v>17.0741</v>
       </c>
       <c r="ES2" t="n">
-        <v>12.3402</v>
+        <v>9.8697</v>
       </c>
       <c r="ET2" t="n">
-        <v>38.491</v>
+        <v>34.985</v>
       </c>
       <c r="EU2" t="n">
-        <v>0.8685</v>
+        <v>1.1232</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.6414</v>
+        <v>1.4935</v>
       </c>
       <c r="EW2" t="n">
-        <v>4.9579</v>
+        <v>5.3223</v>
       </c>
       <c r="EX2" t="n">
-        <v>44.45</v>
+        <v>43.12</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2278,37 +2284,37 @@
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="FA2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="FB2" t="n">
         <v>63.92</v>
       </c>
       <c r="FC2" t="n">
-        <v>32.25</v>
+        <v>23.42</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.3</v>
+        <v>73.19</v>
       </c>
       <c r="FE2" t="n">
-        <v>75.59</v>
+        <v>87.565</v>
       </c>
       <c r="FF2" t="n">
-        <v>44.085</v>
+        <v>39.09</v>
       </c>
       <c r="FG2" t="n">
-        <v>24.0858</v>
+        <v>27.1061</v>
       </c>
       <c r="FH2" t="n">
-        <v>65.273</v>
+        <v>67.419</v>
       </c>
       <c r="FI2" t="n">
-        <v>51.765</v>
+        <v>53.325</v>
       </c>
       <c r="FJ2" t="n">
-        <v>67.26000000000001</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>72.09</v>
+        <v>76.47</v>
       </c>
       <c r="FO2" t="n">
-        <v>63.91</v>
+        <v>64.73999999999999</v>
       </c>
       <c r="FP2" t="n">
-        <v>60.76</v>
+        <v>63.59</v>
       </c>
       <c r="FQ2" t="n">
-        <v>72.78</v>
+        <v>75.56</v>
       </c>
       <c r="FR2" t="n">
-        <v>82.79000000000001</v>
+        <v>86.31999999999999</v>
       </c>
       <c r="FS2" t="n">
-        <v>95.4545</v>
+        <v>100</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2351,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>70.37649999999999</v>
+        <v>72.58750000000001</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260925_204343</t>
+          <t>20260928_152300</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46290.86370059318</v>
+        <v>46293.64098367205</v>
       </c>
     </row>
   </sheetData>
@@ -2438,8 +2444,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -2459,8 +2465,8 @@
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2641,10 +2647,14 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46290.86369212963</v>
-      </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
+        <v>46293.64097222222</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>46308</v>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>LAURUSLABS</t>
@@ -2665,48 +2675,52 @@
       <c r="I2" t="n">
         <v>11.7</v>
       </c>
-      <c r="J2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>UPTREND</t>
+        </is>
+      </c>
       <c r="K2" t="n">
-        <v>2007</v>
+        <v>2010</v>
       </c>
       <c r="L2" t="n">
-        <v>2026</v>
+        <v>2000</v>
       </c>
       <c r="M2" t="n">
-        <v>2040</v>
+        <v>2012.3</v>
       </c>
       <c r="N2" t="n">
-        <v>1979.2</v>
+        <v>1984.8</v>
       </c>
       <c r="O2" t="n">
-        <v>2007</v>
+        <v>2010</v>
       </c>
       <c r="P2" t="n">
-        <v>1438852</v>
+        <v>926358</v>
       </c>
       <c r="Q2" t="n">
-        <v>2007</v>
+        <v>2010</v>
       </c>
       <c r="R2" t="n">
-        <v>2198.08</v>
+        <v>2195.29</v>
       </c>
       <c r="S2" t="n">
-        <v>1911.46</v>
+        <v>1917.36</v>
       </c>
       <c r="T2" t="n">
-        <v>9.520677628300943</v>
+        <v>9.218407960199002</v>
       </c>
       <c r="U2" t="n">
-        <v>191.0799999999999</v>
+        <v>185.29</v>
       </c>
       <c r="V2" t="n">
-        <v>4.760338814150471</v>
+        <v>4.608955223880602</v>
       </c>
       <c r="W2" t="n">
-        <v>95.53999999999996</v>
+        <v>92.6400000000001</v>
       </c>
       <c r="X2" t="n">
-        <v>2</v>
+        <v>2.000107944732294</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2727,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.520677628300943</v>
+        <v>9.218407960199002</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.760338814150471</v>
+        <v>4.608955223880602</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02044686195612276</v>
+        <v>0.02043229602790267</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.324583870965411</v>
+        <v>0.3243526440232999</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909753504945897</v>
+        <v>0.02909758296696929</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04266353304091999</v>
+        <v>0.04228669269848182</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869492979645464</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.03</v>
+        <v>39.05</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-25 20:43:43.770596+05:30</t>
+          <t>2026-09-28 15:23:01.009966+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.520677628300943, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.218407960199002, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001079447322945}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-28 18:09 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="19" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>STRONG BUY</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1864,7 +1864,7 @@
         <v>11.7</v>
       </c>
       <c r="R2" t="n">
-        <v>49.02</v>
+        <v>49.03</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1884,22 +1884,22 @@
         <v>1984.8</v>
       </c>
       <c r="X2" t="n">
-        <v>2010</v>
+        <v>2010.7</v>
       </c>
       <c r="Y2" t="n">
-        <v>2010</v>
+        <v>2010.7</v>
       </c>
       <c r="Z2" t="n">
-        <v>926358</v>
+        <v>950438</v>
       </c>
       <c r="AA2" t="n">
-        <v>1714906</v>
+        <v>1716110</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.54</v>
+        <v>0.55</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.15</v>
+        <v>0.18</v>
       </c>
       <c r="AD2" t="n">
         <v>-0.35</v>
@@ -1926,34 +1926,34 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>3.31</v>
+        <v>3.34</v>
       </c>
       <c r="AM2" t="n">
-        <v>8.220000000000001</v>
+        <v>8.26</v>
       </c>
       <c r="AN2" t="n">
-        <v>49.1</v>
+        <v>49.16</v>
       </c>
       <c r="AO2" t="n">
-        <v>63.8</v>
+        <v>63.88</v>
       </c>
       <c r="AP2" t="n">
-        <v>2.08</v>
+        <v>2.12</v>
       </c>
       <c r="AQ2" t="n">
-        <v>34.6</v>
+        <v>34.65</v>
       </c>
       <c r="AR2" t="n">
-        <v>2010</v>
+        <v>2010.7</v>
       </c>
       <c r="AS2" t="n">
-        <v>2195.29</v>
+        <v>2195.99</v>
       </c>
       <c r="AT2" t="n">
-        <v>1917.36</v>
+        <v>1918.06</v>
       </c>
       <c r="AU2" t="n">
-        <v>2010</v>
+        <v>2010.699951171875</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
@@ -2026,10 +2026,10 @@
         <v>0.245</v>
       </c>
       <c r="BT2" t="n">
-        <v>1485.18</v>
+        <v>1485.44</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.83</v>
+        <v>-13.82</v>
       </c>
       <c r="BV2" t="n">
         <v>2.05</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>89.45</v>
+        <v>88.98999999999999</v>
       </c>
       <c r="CO2" t="n">
-        <v>35.06</v>
+        <v>34.9</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2124,7 +2124,7 @@
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.218400000000001</v>
+        <v>9.215199999999999</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2151,13 +2151,13 @@
         <v>4.0087</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.609</v>
+        <v>4.6074</v>
       </c>
       <c r="DJ2" t="n">
-        <v>32.57</v>
+        <v>32.65</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.609</v>
+        <v>4.6074</v>
       </c>
       <c r="DL2" t="n">
         <v>2.0001</v>
@@ -2178,7 +2178,7 @@
         <v>92.64</v>
       </c>
       <c r="DR2" t="n">
-        <v>74.08</v>
+        <v>72.63</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.9043</v>
+        <v>0.9217</v>
       </c>
       <c r="DX2" t="n">
-        <v>90.5</v>
+        <v>90.3</v>
       </c>
       <c r="DY2" t="n">
-        <v>27</v>
+        <v>27.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>88.426</v>
+        <v>88.093</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>92.77</v>
+        <v>91.73999999999999</v>
       </c>
       <c r="ED2" t="n">
-        <v>99.98</v>
+        <v>100</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.9043</v>
+        <v>0.9217</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.54</v>
+        <v>0.55</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.2434</v>
+        <v>0.248</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.008</v>
+        <v>4.0066</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0285</v>
+        <v>0.029</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7144</v>
+        <v>0.7141999999999999</v>
       </c>
       <c r="EK2" t="n">
-        <v>85.68000000000001</v>
+        <v>84.06</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2249,34 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>5.95</v>
+        <v>5.71</v>
       </c>
       <c r="EP2" t="n">
-        <v>0.6961000000000001</v>
+        <v>0.6681</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.06320000000000001</v>
+        <v>0.0644</v>
       </c>
       <c r="ER2" t="n">
-        <v>17.0741</v>
+        <v>16.7636</v>
       </c>
       <c r="ES2" t="n">
-        <v>9.8697</v>
+        <v>9.8939</v>
       </c>
       <c r="ET2" t="n">
-        <v>34.985</v>
+        <v>34.849</v>
       </c>
       <c r="EU2" t="n">
-        <v>1.1232</v>
+        <v>1.166</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.4935</v>
+        <v>1.4839</v>
       </c>
       <c r="EW2" t="n">
-        <v>5.3223</v>
+        <v>5.0813</v>
       </c>
       <c r="EX2" t="n">
-        <v>43.12</v>
+        <v>43.24</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2293,28 +2293,28 @@
         <v>63.92</v>
       </c>
       <c r="FC2" t="n">
-        <v>23.42</v>
+        <v>23.53</v>
       </c>
       <c r="FD2" t="n">
         <v>73.19</v>
       </c>
       <c r="FE2" t="n">
-        <v>87.565</v>
+        <v>86.52500000000001</v>
       </c>
       <c r="FF2" t="n">
-        <v>39.09</v>
+        <v>39.07</v>
       </c>
       <c r="FG2" t="n">
-        <v>27.1061</v>
+        <v>26.9667</v>
       </c>
       <c r="FH2" t="n">
-        <v>67.419</v>
+        <v>67.30500000000001</v>
       </c>
       <c r="FI2" t="n">
-        <v>53.325</v>
+        <v>52.64</v>
       </c>
       <c r="FJ2" t="n">
-        <v>67.15000000000001</v>
+        <v>67.61</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>76.47</v>
+        <v>76.8</v>
       </c>
       <c r="FO2" t="n">
-        <v>64.73999999999999</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="FP2" t="n">
-        <v>63.59</v>
+        <v>62.6</v>
       </c>
       <c r="FQ2" t="n">
-        <v>75.56</v>
+        <v>74.56</v>
       </c>
       <c r="FR2" t="n">
-        <v>86.31999999999999</v>
+        <v>86.3</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>72.58750000000001</v>
+        <v>72.464</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260928_152300</t>
+          <t>20260928_233859</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46293.64098367205</v>
+        <v>46293.98541051801</v>
       </c>
     </row>
   </sheetData>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46293.64097222222</v>
+        <v>46293.98540509259</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46293</v>
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>2010</v>
+        <v>2010.7</v>
       </c>
       <c r="L2" t="n">
         <v>2000</v>
@@ -2693,34 +2693,34 @@
         <v>1984.8</v>
       </c>
       <c r="O2" t="n">
-        <v>2010</v>
+        <v>2010.7</v>
       </c>
       <c r="P2" t="n">
-        <v>926358</v>
+        <v>950438</v>
       </c>
       <c r="Q2" t="n">
-        <v>2010</v>
+        <v>2010.7</v>
       </c>
       <c r="R2" t="n">
-        <v>2195.29</v>
+        <v>2195.99</v>
       </c>
       <c r="S2" t="n">
-        <v>1917.36</v>
+        <v>1918.06</v>
       </c>
       <c r="T2" t="n">
-        <v>9.218407960199002</v>
+        <v>9.215198687024406</v>
       </c>
       <c r="U2" t="n">
-        <v>185.29</v>
+        <v>185.2899999999997</v>
       </c>
       <c r="V2" t="n">
-        <v>4.608955223880602</v>
+        <v>4.607350673894668</v>
       </c>
       <c r="W2" t="n">
         <v>92.6400000000001</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000107944732294</v>
+        <v>2.000107944732292</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.218407960199002</v>
+        <v>9.215198687024406</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.608955223880602</v>
+        <v>4.607350673894668</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02043229602790267</v>
+        <v>0.02043227326117071</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3243526440232999</v>
+        <v>0.3243522826126344</v>
       </c>
     </row>
     <row r="7">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228669269848182</v>
+        <v>0.04228669813764343</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869492979645463</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-28 15:23:01.009966+05:30</t>
+          <t>2026-09-28 23:38:59.514424+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.218407960199002, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001079447322945}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.215198687024406, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001079447322923}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-29 09:54 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="19" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1816,16 +1816,14 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46293</v>
-      </c>
-      <c r="E2" s="1" t="n">
-        <v>46293</v>
-      </c>
+        <v>46294</v>
+      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H2" t="n">
         <v>8.699999999999999</v>
@@ -1849,72 +1847,68 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="P2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.7</v>
+        <v>11.61</v>
       </c>
       <c r="R2" t="n">
-        <v>49.03</v>
+        <v>49.27</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
       </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>UPTREND</t>
-        </is>
-      </c>
+      <c r="T2" t="inlineStr"/>
       <c r="U2" t="n">
-        <v>2000</v>
+        <v>2020.7</v>
       </c>
       <c r="V2" t="n">
-        <v>2012.3</v>
+        <v>2024.9</v>
       </c>
       <c r="W2" t="n">
-        <v>1984.8</v>
+        <v>1985.7</v>
       </c>
       <c r="X2" t="n">
-        <v>2010.7</v>
+        <v>1994.5</v>
       </c>
       <c r="Y2" t="n">
-        <v>2010.7</v>
+        <v>1994.5</v>
       </c>
       <c r="Z2" t="n">
-        <v>950438</v>
+        <v>2212362</v>
       </c>
       <c r="AA2" t="n">
-        <v>1716110</v>
+        <v>1650210</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.55</v>
+        <v>1.34</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.18</v>
+        <v>-0.8100000000000001</v>
       </c>
       <c r="AD2" t="n">
-        <v>-0.35</v>
+        <v>0.5</v>
       </c>
       <c r="AE2" t="n">
-        <v>27.5</v>
+        <v>39.2</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.37</v>
+        <v>1.97</v>
       </c>
       <c r="AG2" t="n">
-        <v>46.32</v>
+        <v>45.81</v>
       </c>
       <c r="AH2" t="n">
-        <v>46.32</v>
+        <v>45.81</v>
       </c>
       <c r="AI2" t="n">
         <v>2.3</v>
@@ -1926,50 +1920,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>3.34</v>
+        <v>2.16</v>
       </c>
       <c r="AM2" t="n">
-        <v>8.26</v>
+        <v>6.92</v>
       </c>
       <c r="AN2" t="n">
-        <v>49.16</v>
+        <v>47.42</v>
       </c>
       <c r="AO2" t="n">
-        <v>63.88</v>
+        <v>60.54</v>
       </c>
       <c r="AP2" t="n">
-        <v>2.12</v>
+        <v>3.51</v>
       </c>
       <c r="AQ2" t="n">
-        <v>34.65</v>
+        <v>30.53</v>
       </c>
       <c r="AR2" t="n">
-        <v>2010.7</v>
+        <v>1994.5</v>
       </c>
       <c r="AS2" t="n">
-        <v>2195.99</v>
+        <v>2177.75</v>
       </c>
       <c r="AT2" t="n">
-        <v>1918.06</v>
+        <v>1902.87</v>
       </c>
       <c r="AU2" t="n">
-        <v>2010.699951171875</v>
+        <v>1994.5</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.220000000000001</v>
+        <v>9.19</v>
       </c>
       <c r="AY2" t="n">
-        <v>185.29</v>
+        <v>183.25</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.61</v>
+        <v>4.59</v>
       </c>
       <c r="BA2" t="n">
-        <v>92.64</v>
+        <v>91.63</v>
       </c>
       <c r="BB2" t="n">
         <v>2.05</v>
@@ -1978,43 +1972,43 @@
         <v>214</v>
       </c>
       <c r="BD2" t="n">
-        <v>32</v>
+        <v>31.9</v>
       </c>
       <c r="BE2" t="n">
         <v>327</v>
       </c>
       <c r="BF2" t="n">
-        <v>48.9</v>
+        <v>48.8</v>
       </c>
       <c r="BG2" t="n">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.7</v>
+        <v>18.5</v>
       </c>
       <c r="BI2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BM2" t="n">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="BN2" t="n">
         <v>49.9</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.22</v>
+        <v>2.21</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.699999999999999</v>
+        <v>8.69</v>
       </c>
       <c r="BQ2" t="n">
         <v>-4.24</v>
@@ -2023,22 +2017,22 @@
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.245</v>
+        <v>0.243</v>
       </c>
       <c r="BT2" t="n">
-        <v>1485.44</v>
+        <v>1478.06</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.82</v>
+        <v>-14.04</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.05</v>
+        <v>2.04</v>
       </c>
       <c r="BW2" t="n">
         <v>2.05</v>
       </c>
       <c r="BX2" t="n">
-        <v>2.0001</v>
+        <v>1.9999</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2047,7 +2041,7 @@
         <v>8</v>
       </c>
       <c r="CA2" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="CB2" t="n">
         <v>0</v>
@@ -2058,10 +2052,10 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>44.4</v>
+        <v>44.2</v>
       </c>
       <c r="CE2" t="n">
-        <v>52.5</v>
+        <v>52</v>
       </c>
       <c r="CF2" t="n">
         <v>68.3</v>
@@ -2088,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>88.98999999999999</v>
+        <v>95.63</v>
       </c>
       <c r="CO2" t="n">
-        <v>34.9</v>
+        <v>42.96</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2124,7 +2118,7 @@
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.215199999999999</v>
+        <v>9.187799999999999</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,52 +2127,52 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6147</v>
+        <v>0.6127</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3073</v>
+        <v>0.306</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0922</v>
+        <v>0.0919</v>
       </c>
       <c r="DF2" t="n">
-        <v>2</v>
+        <v>2.0022</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.0787</v>
+        <v>1.067</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0087</v>
+        <v>3.9957</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.6074</v>
+        <v>4.5941</v>
       </c>
       <c r="DJ2" t="n">
-        <v>32.65</v>
+        <v>33.86</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.6074</v>
+        <v>4.5941</v>
       </c>
       <c r="DL2" t="n">
-        <v>2.0001</v>
+        <v>1.9999</v>
       </c>
       <c r="DM2" t="n">
-        <v>2.0043</v>
+        <v>1.9957</v>
       </c>
       <c r="DN2" t="n">
-        <v>4.0087</v>
+        <v>3.9957</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0003</v>
+        <v>2.0023</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8696</v>
+        <v>0.8705000000000001</v>
       </c>
       <c r="DQ2" t="n">
-        <v>92.64</v>
+        <v>91.63</v>
       </c>
       <c r="DR2" t="n">
-        <v>72.63</v>
+        <v>82.08</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2193,16 +2187,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.9217</v>
+        <v>1.5261</v>
       </c>
       <c r="DX2" t="n">
-        <v>90.3</v>
+        <v>98.65000000000001</v>
       </c>
       <c r="DY2" t="n">
-        <v>27.5</v>
+        <v>67</v>
       </c>
       <c r="DZ2" t="n">
-        <v>88.093</v>
+        <v>87.554</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,35 +2205,35 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>91.73999999999999</v>
+        <v>78.73999999999999</v>
       </c>
       <c r="ED2" t="n">
         <v>100</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.9217</v>
+        <v>1.5261</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.55</v>
+        <v>1.34</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.248</v>
+        <v>0.4075</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0066</v>
+        <v>3.9947</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.029</v>
+        <v>0.0473</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7141999999999999</v>
+        <v>0.7146</v>
       </c>
       <c r="EK2" t="n">
-        <v>84.06</v>
+        <v>78</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
-          <t>Excellent</t>
+          <t>Strong</t>
         </is>
       </c>
       <c r="EM2" t="n">
@@ -2249,34 +2243,34 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>5.71</v>
+        <v>39.32</v>
       </c>
       <c r="EP2" t="n">
-        <v>0.6681</v>
+        <v>4.5651</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0644</v>
+        <v>0.1556</v>
       </c>
       <c r="ER2" t="n">
-        <v>16.7636</v>
+        <v>6.8582</v>
       </c>
       <c r="ES2" t="n">
-        <v>9.8939</v>
+        <v>10.2606</v>
       </c>
       <c r="ET2" t="n">
-        <v>34.849</v>
+        <v>48.027</v>
       </c>
       <c r="EU2" t="n">
-        <v>1.166</v>
+        <v>4.7034</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.4839</v>
+        <v>0.9829</v>
       </c>
       <c r="EW2" t="n">
-        <v>5.0813</v>
+        <v>37.6017</v>
       </c>
       <c r="EX2" t="n">
-        <v>43.24</v>
+        <v>49.95</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2284,37 +2278,37 @@
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="FA2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.92</v>
+        <v>63.49</v>
       </c>
       <c r="FC2" t="n">
-        <v>23.53</v>
+        <v>24.06</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.19</v>
+        <v>73.3</v>
       </c>
       <c r="FE2" t="n">
-        <v>86.52500000000001</v>
+        <v>86.815</v>
       </c>
       <c r="FF2" t="n">
-        <v>39.07</v>
+        <v>46.455</v>
       </c>
       <c r="FG2" t="n">
-        <v>26.9667</v>
+        <v>28.9788</v>
       </c>
       <c r="FH2" t="n">
-        <v>67.30500000000001</v>
+        <v>70.42400000000001</v>
       </c>
       <c r="FI2" t="n">
-        <v>52.64</v>
+        <v>57.97</v>
       </c>
       <c r="FJ2" t="n">
-        <v>67.61</v>
+        <v>70.72</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2322,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>76.8</v>
+        <v>81.89</v>
       </c>
       <c r="FO2" t="n">
-        <v>66.40000000000001</v>
+        <v>67.53</v>
       </c>
       <c r="FP2" t="n">
-        <v>62.6</v>
+        <v>76.73999999999999</v>
       </c>
       <c r="FQ2" t="n">
-        <v>74.56</v>
+        <v>79.33</v>
       </c>
       <c r="FR2" t="n">
-        <v>86.3</v>
+        <v>89.31999999999999</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,7 +2351,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>72.464</v>
+        <v>76.19499999999999</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260928_233859</t>
+          <t>20260929_152447</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46293.98541051801</v>
+        <v>46294.64221582825</v>
       </c>
     </row>
   </sheetData>
@@ -2444,8 +2438,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -2465,7 +2459,7 @@
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="19" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
@@ -2647,14 +2641,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46293.98540509259</v>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>46293</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>46308</v>
-      </c>
+        <v>46294.64221064815</v>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>LAURUSLABS</t>
@@ -2673,54 +2663,50 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.7</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>UPTREND</t>
-        </is>
-      </c>
+        <v>11.61</v>
+      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>2010.7</v>
+        <v>1994.5</v>
       </c>
       <c r="L2" t="n">
-        <v>2000</v>
+        <v>2020.7</v>
       </c>
       <c r="M2" t="n">
-        <v>2012.3</v>
+        <v>2024.9</v>
       </c>
       <c r="N2" t="n">
-        <v>1984.8</v>
+        <v>1985.7</v>
       </c>
       <c r="O2" t="n">
-        <v>2010.7</v>
+        <v>1994.5</v>
       </c>
       <c r="P2" t="n">
-        <v>950438</v>
+        <v>2212362</v>
       </c>
       <c r="Q2" t="n">
-        <v>2010.7</v>
+        <v>1994.5</v>
       </c>
       <c r="R2" t="n">
-        <v>2195.99</v>
+        <v>2177.75</v>
       </c>
       <c r="S2" t="n">
-        <v>1918.06</v>
+        <v>1902.87</v>
       </c>
       <c r="T2" t="n">
-        <v>9.215198687024406</v>
+        <v>9.187766357483078</v>
       </c>
       <c r="U2" t="n">
-        <v>185.2899999999997</v>
+        <v>183.25</v>
       </c>
       <c r="V2" t="n">
-        <v>4.607350673894668</v>
+        <v>4.594133868137383</v>
       </c>
       <c r="W2" t="n">
-        <v>92.6400000000001</v>
+        <v>91.63000000000011</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000107944732292</v>
+        <v>1.999890865437081</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.215198687024406</v>
+        <v>9.187766357483078</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.607350673894668</v>
+        <v>4.594133868137383</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02043227326117071</v>
+        <v>0.02042166637530506</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3243522826126344</v>
+        <v>0.3241839035195223</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909758296696929</v>
+        <v>0.02909145652070655</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228669813764343</v>
+        <v>0.04228669796214085</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645463</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.05</v>
+        <v>39.07</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-28 23:38:59.514424+05:30</t>
+          <t>2026-09-29 15:24:47.485952+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.215198687024406, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001079447322923}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.187766357483078, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998908654370815}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-29 16:29 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -1847,7 +1847,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>STRONG BUY</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1859,10 +1859,10 @@
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.61</v>
+        <v>11.56</v>
       </c>
       <c r="R2" t="n">
-        <v>49.27</v>
+        <v>49.2</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,43 +1875,43 @@
         <v>2024.9</v>
       </c>
       <c r="W2" t="n">
-        <v>1985.7</v>
+        <v>1979</v>
       </c>
       <c r="X2" t="n">
-        <v>1994.5</v>
+        <v>1979</v>
       </c>
       <c r="Y2" t="n">
-        <v>1994.5</v>
+        <v>1979</v>
       </c>
       <c r="Z2" t="n">
-        <v>2212362</v>
+        <v>2425137</v>
       </c>
       <c r="AA2" t="n">
-        <v>1650210</v>
+        <v>1660849</v>
       </c>
       <c r="AB2" t="n">
-        <v>1.34</v>
+        <v>1.46</v>
       </c>
       <c r="AC2" t="n">
-        <v>-0.8100000000000001</v>
+        <v>-1.58</v>
       </c>
       <c r="AD2" t="n">
         <v>0.5</v>
       </c>
       <c r="AE2" t="n">
-        <v>39.2</v>
+        <v>45.9</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.97</v>
+        <v>2.32</v>
       </c>
       <c r="AG2" t="n">
-        <v>45.81</v>
+        <v>46.29</v>
       </c>
       <c r="AH2" t="n">
-        <v>45.81</v>
+        <v>46.29</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.3</v>
+        <v>2.34</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,53 +1920,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>2.16</v>
+        <v>1.41</v>
       </c>
       <c r="AM2" t="n">
-        <v>6.92</v>
+        <v>6.11</v>
       </c>
       <c r="AN2" t="n">
-        <v>47.42</v>
+        <v>46.28</v>
       </c>
       <c r="AO2" t="n">
-        <v>60.54</v>
+        <v>57.65</v>
       </c>
       <c r="AP2" t="n">
-        <v>3.51</v>
+        <v>2.7</v>
       </c>
       <c r="AQ2" t="n">
-        <v>30.53</v>
+        <v>29.52</v>
       </c>
       <c r="AR2" t="n">
-        <v>1994.5</v>
+        <v>1979</v>
       </c>
       <c r="AS2" t="n">
-        <v>2177.75</v>
+        <v>2164.17</v>
       </c>
       <c r="AT2" t="n">
-        <v>1902.87</v>
+        <v>1886.42</v>
       </c>
       <c r="AU2" t="n">
-        <v>1994.5</v>
+        <v>1979</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.19</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="AY2" t="n">
-        <v>183.25</v>
+        <v>185.17</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.59</v>
+        <v>4.68</v>
       </c>
       <c r="BA2" t="n">
-        <v>91.63</v>
+        <v>92.58</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.05</v>
+        <v>2.04</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
@@ -2005,34 +2005,34 @@
         <v>49.9</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.21</v>
+        <v>2.2</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.69</v>
+        <v>8.68</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.24</v>
+        <v>-4.25</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.243</v>
+        <v>0.242</v>
       </c>
       <c r="BT2" t="n">
-        <v>1478.06</v>
+        <v>1471.65</v>
       </c>
       <c r="BU2" t="n">
-        <v>-14.04</v>
+        <v>-14.19</v>
       </c>
       <c r="BV2" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="BW2" t="n">
         <v>2.04</v>
       </c>
-      <c r="BW2" t="n">
-        <v>2.05</v>
-      </c>
       <c r="BX2" t="n">
-        <v>1.9999</v>
+        <v>2.0001</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2052,13 +2052,13 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>44.2</v>
+        <v>44</v>
       </c>
       <c r="CE2" t="n">
-        <v>52</v>
+        <v>51.5</v>
       </c>
       <c r="CF2" t="n">
-        <v>68.3</v>
+        <v>68</v>
       </c>
       <c r="CG2" t="n">
         <v>71.3</v>
@@ -2082,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>95.63</v>
+        <v>94.56999999999999</v>
       </c>
       <c r="CO2" t="n">
-        <v>42.96</v>
+        <v>43.29</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2118,7 +2118,7 @@
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.187799999999999</v>
+        <v>9.3567</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,52 +2127,52 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6127</v>
+        <v>0.624</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.306</v>
+        <v>0.312</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0919</v>
+        <v>0.0936</v>
       </c>
       <c r="DF2" t="n">
-        <v>2.0022</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.067</v>
+        <v>1.082</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9957</v>
+        <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.5941</v>
+        <v>4.6781</v>
       </c>
       <c r="DJ2" t="n">
-        <v>33.86</v>
+        <v>35.7</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.5941</v>
+        <v>4.6781</v>
       </c>
       <c r="DL2" t="n">
-        <v>1.9999</v>
+        <v>2.0001</v>
       </c>
       <c r="DM2" t="n">
-        <v>1.9957</v>
+        <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9957</v>
+        <v>4</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0023</v>
+        <v>2</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8705000000000001</v>
+        <v>0.8547</v>
       </c>
       <c r="DQ2" t="n">
-        <v>91.63</v>
+        <v>92.58</v>
       </c>
       <c r="DR2" t="n">
-        <v>82.08</v>
+        <v>74.22</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2187,16 +2187,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.5261</v>
+        <v>1.1538</v>
       </c>
       <c r="DX2" t="n">
-        <v>98.65000000000001</v>
+        <v>94.125</v>
       </c>
       <c r="DY2" t="n">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="DZ2" t="n">
-        <v>87.554</v>
+        <v>87.23399999999999</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2205,31 +2205,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>78.73999999999999</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="ED2" t="n">
         <v>100</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.5261</v>
+        <v>1.1538</v>
       </c>
       <c r="EF2" t="n">
-        <v>1.34</v>
+        <v>1.46</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.4075</v>
+        <v>0.3121</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9947</v>
+        <v>3.9986</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0473</v>
+        <v>0.0361</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7146</v>
+        <v>0.704</v>
       </c>
       <c r="EK2" t="n">
-        <v>78</v>
+        <v>78.04000000000001</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2243,34 +2243,34 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>39.32</v>
+        <v>28.14</v>
       </c>
       <c r="EP2" t="n">
-        <v>4.5651</v>
+        <v>3.253</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.1556</v>
+        <v>0.1688</v>
       </c>
       <c r="ER2" t="n">
-        <v>6.8582</v>
+        <v>6.411</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.2606</v>
+        <v>10.6886</v>
       </c>
       <c r="ET2" t="n">
-        <v>48.027</v>
+        <v>44.736</v>
       </c>
       <c r="EU2" t="n">
-        <v>4.7034</v>
+        <v>3.942</v>
       </c>
       <c r="EV2" t="n">
-        <v>0.9829</v>
+        <v>0.9512</v>
       </c>
       <c r="EW2" t="n">
-        <v>37.6017</v>
+        <v>26.612</v>
       </c>
       <c r="EX2" t="n">
-        <v>49.95</v>
+        <v>50.63</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2284,31 +2284,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.49</v>
+        <v>63.26</v>
       </c>
       <c r="FC2" t="n">
-        <v>24.06</v>
+        <v>25.88</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.3</v>
+        <v>72.77</v>
       </c>
       <c r="FE2" t="n">
-        <v>86.815</v>
+        <v>86.30500000000001</v>
       </c>
       <c r="FF2" t="n">
-        <v>46.455</v>
+        <v>46.96</v>
       </c>
       <c r="FG2" t="n">
-        <v>28.9788</v>
+        <v>28.3144</v>
       </c>
       <c r="FH2" t="n">
-        <v>70.42400000000001</v>
+        <v>70.127</v>
       </c>
       <c r="FI2" t="n">
-        <v>57.97</v>
+        <v>54.96</v>
       </c>
       <c r="FJ2" t="n">
-        <v>70.72</v>
+        <v>70.31999999999999</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,19 +2322,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>81.89</v>
+        <v>79.59</v>
       </c>
       <c r="FO2" t="n">
-        <v>67.53</v>
+        <v>68.98</v>
       </c>
       <c r="FP2" t="n">
-        <v>76.73999999999999</v>
+        <v>72.31</v>
       </c>
       <c r="FQ2" t="n">
-        <v>79.33</v>
+        <v>75.38</v>
       </c>
       <c r="FR2" t="n">
-        <v>89.31999999999999</v>
+        <v>87.05</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>76.19499999999999</v>
+        <v>74.077</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260929_152447</t>
+          <t>20260929_215943</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46294.64221582825</v>
+        <v>46294.91648072562</v>
       </c>
     </row>
   </sheetData>
@@ -2458,7 +2458,7 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46294.64221064815</v>
+        <v>46294.91646990741</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2663,11 +2663,11 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.61</v>
+        <v>11.56</v>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>1994.5</v>
+        <v>1979</v>
       </c>
       <c r="L2" t="n">
         <v>2020.7</v>
@@ -2676,37 +2676,37 @@
         <v>2024.9</v>
       </c>
       <c r="N2" t="n">
-        <v>1985.7</v>
+        <v>1979</v>
       </c>
       <c r="O2" t="n">
-        <v>1994.5</v>
+        <v>1979</v>
       </c>
       <c r="P2" t="n">
-        <v>2212362</v>
+        <v>2425137</v>
       </c>
       <c r="Q2" t="n">
-        <v>1994.5</v>
+        <v>1979</v>
       </c>
       <c r="R2" t="n">
-        <v>2177.75</v>
+        <v>2164.17</v>
       </c>
       <c r="S2" t="n">
-        <v>1902.87</v>
+        <v>1886.42</v>
       </c>
       <c r="T2" t="n">
-        <v>9.187766357483078</v>
+        <v>9.356745831227895</v>
       </c>
       <c r="U2" t="n">
-        <v>183.25</v>
+        <v>185.1700000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>4.594133868137383</v>
+        <v>4.678120262758966</v>
       </c>
       <c r="W2" t="n">
-        <v>91.63000000000011</v>
+        <v>92.57999999999993</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999890865437081</v>
+        <v>2.00010801469</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.187766357483078</v>
+        <v>9.356745831227895</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.594133868137383</v>
+        <v>4.678120262758966</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02042166637530506</v>
+        <v>0.02042947499362337</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3241839035195223</v>
+        <v>0.3243078614924418</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909145652070655</v>
+        <v>0.02909156378633574</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228669796214085</v>
+        <v>0.0422866889062618</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869492979645464</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.07</v>
+        <v>39.06</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:24:47.485952+05:30</t>
+          <t>2026-09-29 21:59:43.968216+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.187766357483078, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998908654370815}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.356745831227895, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001080146900003}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-30 09:47 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -1816,14 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46294</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
+        <v>46295</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>46295</v>
+      </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H2" t="n">
         <v>8.699999999999999</v>
@@ -1852,66 +1854,70 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="P2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.56</v>
+        <v>11.44</v>
       </c>
       <c r="R2" t="n">
-        <v>49.2</v>
+        <v>48.86</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
       </c>
-      <c r="T2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>UPTREND</t>
+        </is>
+      </c>
       <c r="U2" t="n">
-        <v>2020.7</v>
+        <v>1993</v>
       </c>
       <c r="V2" t="n">
-        <v>2024.9</v>
+        <v>2001.6</v>
       </c>
       <c r="W2" t="n">
-        <v>1979</v>
+        <v>1955.1</v>
       </c>
       <c r="X2" t="n">
-        <v>1979</v>
+        <v>1988</v>
       </c>
       <c r="Y2" t="n">
-        <v>1979</v>
+        <v>1988</v>
       </c>
       <c r="Z2" t="n">
-        <v>2425137</v>
+        <v>1329932</v>
       </c>
       <c r="AA2" t="n">
-        <v>1660849</v>
+        <v>1614386</v>
       </c>
       <c r="AB2" t="n">
-        <v>1.46</v>
+        <v>0.82</v>
       </c>
       <c r="AC2" t="n">
-        <v>-1.58</v>
+        <v>0.45</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.5</v>
+        <v>0.71</v>
       </c>
       <c r="AE2" t="n">
-        <v>45.9</v>
+        <v>46.5</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.32</v>
+        <v>2.34</v>
       </c>
       <c r="AG2" t="n">
-        <v>46.29</v>
+        <v>46.31</v>
       </c>
       <c r="AH2" t="n">
-        <v>46.29</v>
+        <v>46.31</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.34</v>
+        <v>2.33</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>1.41</v>
+        <v>1.54</v>
       </c>
       <c r="AM2" t="n">
-        <v>6.11</v>
+        <v>6.13</v>
       </c>
       <c r="AN2" t="n">
-        <v>46.28</v>
+        <v>46.41</v>
       </c>
       <c r="AO2" t="n">
-        <v>57.65</v>
+        <v>58.88</v>
       </c>
       <c r="AP2" t="n">
-        <v>2.7</v>
+        <v>4.33</v>
       </c>
       <c r="AQ2" t="n">
-        <v>29.52</v>
+        <v>28.9</v>
       </c>
       <c r="AR2" t="n">
-        <v>1979</v>
+        <v>1988</v>
       </c>
       <c r="AS2" t="n">
-        <v>2164.17</v>
+        <v>2173.23</v>
       </c>
       <c r="AT2" t="n">
-        <v>1886.42</v>
+        <v>1895.39</v>
       </c>
       <c r="AU2" t="n">
-        <v>1979</v>
+        <v>1988</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.359999999999999</v>
+        <v>9.32</v>
       </c>
       <c r="AY2" t="n">
-        <v>185.17</v>
+        <v>185.23</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.68</v>
+        <v>4.66</v>
       </c>
       <c r="BA2" t="n">
-        <v>92.58</v>
+        <v>92.61</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.04</v>
+        <v>2.06</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
@@ -1975,61 +1981,61 @@
         <v>31.9</v>
       </c>
       <c r="BE2" t="n">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="BF2" t="n">
-        <v>48.8</v>
+        <v>49.6</v>
       </c>
       <c r="BG2" t="n">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.5</v>
+        <v>18.2</v>
       </c>
       <c r="BI2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="BM2" t="n">
         <v>670</v>
       </c>
       <c r="BN2" t="n">
-        <v>49.9</v>
+        <v>49.6</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.2</v>
+        <v>2.19</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.68</v>
+        <v>8.73</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.25</v>
+        <v>-4.24</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.242</v>
+        <v>0.241</v>
       </c>
       <c r="BT2" t="n">
-        <v>1471.65</v>
+        <v>1466.03</v>
       </c>
       <c r="BU2" t="n">
-        <v>-14.19</v>
+        <v>-14.01</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.03</v>
+        <v>2.02</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.04</v>
+        <v>2.06</v>
       </c>
       <c r="BX2" t="n">
         <v>2.0001</v>
@@ -2041,7 +2047,7 @@
         <v>8</v>
       </c>
       <c r="CA2" t="n">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="CB2" t="n">
         <v>0</v>
@@ -2052,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>44</v>
+        <v>43.8</v>
       </c>
       <c r="CE2" t="n">
-        <v>51.5</v>
+        <v>51</v>
       </c>
       <c r="CF2" t="n">
-        <v>68</v>
+        <v>68.7</v>
       </c>
       <c r="CG2" t="n">
-        <v>71.3</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2082,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>94.56999999999999</v>
+        <v>95.53</v>
       </c>
       <c r="CO2" t="n">
-        <v>43.29</v>
+        <v>37.92</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2115,10 +2121,10 @@
         <v>54.54545454545454</v>
       </c>
       <c r="CY2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.3567</v>
+        <v>9.317399999999999</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,31 +2133,31 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.624</v>
+        <v>0.6213</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.312</v>
+        <v>0.3107</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0936</v>
+        <v>0.09320000000000001</v>
       </c>
       <c r="DF2" t="n">
         <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.082</v>
+        <v>1.0662</v>
       </c>
       <c r="DH2" t="n">
         <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.6781</v>
+        <v>4.6585</v>
       </c>
       <c r="DJ2" t="n">
-        <v>35.7</v>
+        <v>35.26</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.6781</v>
+        <v>4.6585</v>
       </c>
       <c r="DL2" t="n">
         <v>2.0001</v>
@@ -2163,22 +2169,22 @@
         <v>4</v>
       </c>
       <c r="DO2" t="n">
-        <v>2</v>
+        <v>1.9997</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8547</v>
+        <v>0.8584000000000001</v>
       </c>
       <c r="DQ2" t="n">
-        <v>92.58</v>
+        <v>92.61</v>
       </c>
       <c r="DR2" t="n">
-        <v>74.22</v>
+        <v>47.32</v>
       </c>
       <c r="DS2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="DT2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.1538</v>
+        <v>1.8584</v>
       </c>
       <c r="DX2" t="n">
-        <v>94.125</v>
+        <v>97.2</v>
       </c>
       <c r="DY2" t="n">
-        <v>73</v>
+        <v>41</v>
       </c>
       <c r="DZ2" t="n">
-        <v>87.23399999999999</v>
+        <v>87.581</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2205,35 +2211,35 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>81.40000000000001</v>
+        <v>88.26000000000001</v>
       </c>
       <c r="ED2" t="n">
         <v>100</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.1538</v>
+        <v>1.8584</v>
       </c>
       <c r="EF2" t="n">
-        <v>1.46</v>
+        <v>0.82</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.3121</v>
+        <v>0.4954</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9986</v>
+        <v>3.9989</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0361</v>
+        <v>0.0567</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.704</v>
+        <v>0.7065</v>
       </c>
       <c r="EK2" t="n">
-        <v>78.04000000000001</v>
+        <v>82.73999999999999</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Excellent</t>
         </is>
       </c>
       <c r="EM2" t="n">
@@ -2243,72 +2249,72 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>28.14</v>
+        <v>11.03</v>
       </c>
       <c r="EP2" t="n">
-        <v>3.253</v>
+        <v>1.2618</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.1688</v>
+        <v>0.09379999999999999</v>
       </c>
       <c r="ER2" t="n">
-        <v>6.411</v>
+        <v>11.3659</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.6886</v>
+        <v>10.5886</v>
       </c>
       <c r="ET2" t="n">
-        <v>44.736</v>
+        <v>37.284</v>
       </c>
       <c r="EU2" t="n">
-        <v>3.942</v>
+        <v>3.5506</v>
       </c>
       <c r="EV2" t="n">
-        <v>0.9512</v>
+        <v>1.2802</v>
       </c>
       <c r="EW2" t="n">
-        <v>26.612</v>
+        <v>10.537</v>
       </c>
       <c r="EX2" t="n">
-        <v>50.63</v>
+        <v>27.81</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="FA2" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.26</v>
+        <v>62.69</v>
       </c>
       <c r="FC2" t="n">
-        <v>25.88</v>
+        <v>25.29</v>
       </c>
       <c r="FD2" t="n">
-        <v>72.77</v>
+        <v>73.83</v>
       </c>
       <c r="FE2" t="n">
-        <v>86.30500000000001</v>
+        <v>89.13500000000001</v>
       </c>
       <c r="FF2" t="n">
-        <v>46.96</v>
+        <v>32.865</v>
       </c>
       <c r="FG2" t="n">
-        <v>28.3144</v>
+        <v>28.6877</v>
       </c>
       <c r="FH2" t="n">
-        <v>70.127</v>
+        <v>65.566</v>
       </c>
       <c r="FI2" t="n">
-        <v>54.96</v>
+        <v>41.29</v>
       </c>
       <c r="FJ2" t="n">
-        <v>70.31999999999999</v>
+        <v>67.63</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>79.59</v>
+        <v>69.15000000000001</v>
       </c>
       <c r="FO2" t="n">
-        <v>68.98</v>
+        <v>69.2</v>
       </c>
       <c r="FP2" t="n">
-        <v>72.31</v>
+        <v>45.22</v>
       </c>
       <c r="FQ2" t="n">
-        <v>75.38</v>
+        <v>64.28</v>
       </c>
       <c r="FR2" t="n">
-        <v>87.05</v>
+        <v>76.2</v>
       </c>
       <c r="FS2" t="n">
-        <v>100</v>
+        <v>90.9091</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2347,11 +2353,11 @@
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>74.077</v>
+        <v>64.01300000000001</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260929_215943</t>
+          <t>20260930_151739</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46294.91648072562</v>
+        <v>46295.63726752185</v>
       </c>
     </row>
   </sheetData>
@@ -2438,8 +2444,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -2458,9 +2464,9 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
-    <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="19" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2641,10 +2647,14 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46294.91646990741</v>
-      </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
+        <v>46295.63725694444</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>46310</v>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>LAURUSLABS</t>
@@ -2663,50 +2673,54 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.56</v>
-      </c>
-      <c r="J2" t="inlineStr"/>
+        <v>11.44</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>UPTREND</t>
+        </is>
+      </c>
       <c r="K2" t="n">
-        <v>1979</v>
+        <v>1988</v>
       </c>
       <c r="L2" t="n">
-        <v>2020.7</v>
+        <v>1993</v>
       </c>
       <c r="M2" t="n">
-        <v>2024.9</v>
+        <v>2001.6</v>
       </c>
       <c r="N2" t="n">
-        <v>1979</v>
+        <v>1955.1</v>
       </c>
       <c r="O2" t="n">
-        <v>1979</v>
+        <v>1988</v>
       </c>
       <c r="P2" t="n">
-        <v>2425137</v>
+        <v>1329932</v>
       </c>
       <c r="Q2" t="n">
-        <v>1979</v>
+        <v>1988</v>
       </c>
       <c r="R2" t="n">
-        <v>2164.17</v>
+        <v>2173.23</v>
       </c>
       <c r="S2" t="n">
-        <v>1886.42</v>
+        <v>1895.39</v>
       </c>
       <c r="T2" t="n">
-        <v>9.356745831227895</v>
+        <v>9.317404426559357</v>
       </c>
       <c r="U2" t="n">
-        <v>185.1700000000001</v>
+        <v>185.23</v>
       </c>
       <c r="V2" t="n">
-        <v>4.678120262758966</v>
+        <v>4.658450704225347</v>
       </c>
       <c r="W2" t="n">
-        <v>92.57999999999993</v>
+        <v>92.6099999999999</v>
       </c>
       <c r="X2" t="n">
-        <v>2.00010801469</v>
+        <v>2.000107979699819</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2727,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.356745831227895</v>
+        <v>9.317404426559357</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.678120262758966</v>
+        <v>4.658450704225347</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02042947499362337</v>
+        <v>0.02041505258251645</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3243078614924418</v>
+        <v>0.3240789128138727</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909156378633574</v>
+        <v>0.02908554460570219</v>
       </c>
     </row>
     <row r="12">
@@ -2905,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.06</v>
+        <v>39.07</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-29 21:59:43.968216+05:30</t>
+          <t>2026-09-30 15:17:39.952447+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.356745831227895, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001080146900003}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.317404426559357, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000107979699819}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-09-30 16:23 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -1864,7 +1864,7 @@
         <v>11.44</v>
       </c>
       <c r="R2" t="n">
-        <v>48.86</v>
+        <v>48.88</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1884,22 +1884,22 @@
         <v>1955.1</v>
       </c>
       <c r="X2" t="n">
-        <v>1988</v>
+        <v>1980</v>
       </c>
       <c r="Y2" t="n">
-        <v>1988</v>
+        <v>1980</v>
       </c>
       <c r="Z2" t="n">
-        <v>1329932</v>
+        <v>1397688</v>
       </c>
       <c r="AA2" t="n">
-        <v>1614386</v>
+        <v>1617773</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.82</v>
+        <v>0.86</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.45</v>
+        <v>0.05</v>
       </c>
       <c r="AD2" t="n">
         <v>0.71</v>
@@ -1908,7 +1908,7 @@
         <v>46.5</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.34</v>
+        <v>2.35</v>
       </c>
       <c r="AG2" t="n">
         <v>46.31</v>
@@ -1917,7 +1917,7 @@
         <v>46.31</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.33</v>
+        <v>2.34</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,47 +1926,47 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>1.54</v>
+        <v>1.16</v>
       </c>
       <c r="AM2" t="n">
-        <v>6.13</v>
+        <v>5.71</v>
       </c>
       <c r="AN2" t="n">
-        <v>46.41</v>
+        <v>45.83</v>
       </c>
       <c r="AO2" t="n">
-        <v>58.88</v>
+        <v>57.79</v>
       </c>
       <c r="AP2" t="n">
-        <v>4.33</v>
+        <v>3.91</v>
       </c>
       <c r="AQ2" t="n">
-        <v>28.9</v>
+        <v>28.38</v>
       </c>
       <c r="AR2" t="n">
-        <v>1988</v>
+        <v>1980</v>
       </c>
       <c r="AS2" t="n">
-        <v>2173.23</v>
+        <v>2165.23</v>
       </c>
       <c r="AT2" t="n">
-        <v>1895.39</v>
+        <v>1887.39</v>
       </c>
       <c r="AU2" t="n">
-        <v>1988</v>
+        <v>1980</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.32</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="AY2" t="n">
         <v>185.23</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.66</v>
+        <v>4.68</v>
       </c>
       <c r="BA2" t="n">
         <v>92.61</v>
@@ -2026,7 +2026,7 @@
         <v>0.241</v>
       </c>
       <c r="BT2" t="n">
-        <v>1466.03</v>
+        <v>1465.25</v>
       </c>
       <c r="BU2" t="n">
         <v>-14.01</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>95.53</v>
+        <v>94.45999999999999</v>
       </c>
       <c r="CO2" t="n">
-        <v>37.92</v>
+        <v>37.23</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2124,7 +2124,7 @@
         <v>3</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.317399999999999</v>
+        <v>9.3551</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,31 +2133,31 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6213</v>
+        <v>0.624</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3107</v>
+        <v>0.312</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.09320000000000001</v>
+        <v>0.0936</v>
       </c>
       <c r="DF2" t="n">
         <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.0662</v>
+        <v>1.0708</v>
       </c>
       <c r="DH2" t="n">
         <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.6585</v>
+        <v>4.6773</v>
       </c>
       <c r="DJ2" t="n">
-        <v>35.26</v>
+        <v>35.03</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.6585</v>
+        <v>4.6773</v>
       </c>
       <c r="DL2" t="n">
         <v>2.0001</v>
@@ -2169,22 +2169,22 @@
         <v>4</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9997</v>
+        <v>2</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8584000000000001</v>
+        <v>0.8547</v>
       </c>
       <c r="DQ2" t="n">
         <v>92.61</v>
       </c>
       <c r="DR2" t="n">
-        <v>47.32</v>
+        <v>50.64</v>
       </c>
       <c r="DS2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.8584</v>
+        <v>1.6709</v>
       </c>
       <c r="DX2" t="n">
-        <v>97.2</v>
+        <v>94.47499999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="DZ2" t="n">
-        <v>87.581</v>
+        <v>86.886</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>88.26000000000001</v>
+        <v>85.81</v>
       </c>
       <c r="ED2" t="n">
         <v>100</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.8584</v>
+        <v>1.6709</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.82</v>
+        <v>0.86</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.4954</v>
+        <v>0.4473</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9989</v>
+        <v>3.9979</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0567</v>
+        <v>0.0512</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7065</v>
+        <v>0.7039</v>
       </c>
       <c r="EK2" t="n">
-        <v>82.73999999999999</v>
+        <v>80.48</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2249,34 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>11.03</v>
+        <v>11.43</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.2618</v>
+        <v>1.3076</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.09379999999999999</v>
+        <v>0.0984</v>
       </c>
       <c r="ER2" t="n">
-        <v>11.3659</v>
+        <v>10.8837</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.5886</v>
+        <v>10.488</v>
       </c>
       <c r="ET2" t="n">
-        <v>37.284</v>
+        <v>37.128</v>
       </c>
       <c r="EU2" t="n">
-        <v>3.5506</v>
+        <v>3.3626</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.2802</v>
+        <v>1.2581</v>
       </c>
       <c r="EW2" t="n">
-        <v>10.537</v>
+        <v>10.7968</v>
       </c>
       <c r="EX2" t="n">
-        <v>27.81</v>
+        <v>27.88</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2293,28 +2293,28 @@
         <v>62.69</v>
       </c>
       <c r="FC2" t="n">
-        <v>25.29</v>
+        <v>24.8</v>
       </c>
       <c r="FD2" t="n">
         <v>73.83</v>
       </c>
       <c r="FE2" t="n">
-        <v>89.13500000000001</v>
+        <v>87.47</v>
       </c>
       <c r="FF2" t="n">
-        <v>32.865</v>
+        <v>32.555</v>
       </c>
       <c r="FG2" t="n">
-        <v>28.6877</v>
+        <v>28.2814</v>
       </c>
       <c r="FH2" t="n">
-        <v>65.566</v>
+        <v>65.259</v>
       </c>
       <c r="FI2" t="n">
-        <v>41.29</v>
+        <v>42.835</v>
       </c>
       <c r="FJ2" t="n">
-        <v>67.63</v>
+        <v>67.65000000000001</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>69.15000000000001</v>
+        <v>69.64</v>
       </c>
       <c r="FO2" t="n">
-        <v>69.2</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="FP2" t="n">
-        <v>45.22</v>
+        <v>46.28</v>
       </c>
       <c r="FQ2" t="n">
-        <v>64.28</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="FR2" t="n">
-        <v>76.2</v>
+        <v>74.31999999999999</v>
       </c>
       <c r="FS2" t="n">
         <v>90.9091</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>64.01300000000001</v>
+        <v>63.5405</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260930_151739</t>
+          <t>20260930_215357</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46295.63726752185</v>
+        <v>46295.91247494507</v>
       </c>
     </row>
   </sheetData>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46295.63725694444</v>
+        <v>46295.91246527778</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46295</v>
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1988</v>
+        <v>1980</v>
       </c>
       <c r="L2" t="n">
         <v>1993</v>
@@ -2693,28 +2693,28 @@
         <v>1955.1</v>
       </c>
       <c r="O2" t="n">
-        <v>1988</v>
+        <v>1980</v>
       </c>
       <c r="P2" t="n">
-        <v>1329932</v>
+        <v>1397688</v>
       </c>
       <c r="Q2" t="n">
-        <v>1988</v>
+        <v>1980</v>
       </c>
       <c r="R2" t="n">
-        <v>2173.23</v>
+        <v>2165.23</v>
       </c>
       <c r="S2" t="n">
-        <v>1895.39</v>
+        <v>1887.39</v>
       </c>
       <c r="T2" t="n">
-        <v>9.317404426559357</v>
+        <v>9.355050505050507</v>
       </c>
       <c r="U2" t="n">
         <v>185.23</v>
       </c>
       <c r="V2" t="n">
-        <v>4.658450704225347</v>
+        <v>4.677272727272722</v>
       </c>
       <c r="W2" t="n">
         <v>92.6099999999999</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.317404426559357</v>
+        <v>9.355050505050507</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.658450704225347</v>
+        <v>4.677272727272722</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02041505258251645</v>
+        <v>0.02041506973087686</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3240789128138727</v>
+        <v>0.324079185035655</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02908554460570219</v>
+        <v>0.02908554432243104</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.0422866889062618</v>
+        <v>0.04228670527526088</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869493934347617</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-30 15:17:39.952447+05:30</t>
+          <t>2026-09-30 21:53:57.874306+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.317404426559357, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000107979699819}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.355050505050507, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000107979699819}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-01 10:13 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H2" t="n">
         <v>8.699999999999999</v>
@@ -1864,7 +1864,7 @@
         <v>11.44</v>
       </c>
       <c r="R2" t="n">
-        <v>48.88</v>
+        <v>48.83</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1993</v>
+        <v>1973.6</v>
       </c>
       <c r="V2" t="n">
-        <v>2001.6</v>
+        <v>2006.9</v>
       </c>
       <c r="W2" t="n">
-        <v>1955.1</v>
+        <v>1952.1</v>
       </c>
       <c r="X2" t="n">
-        <v>1980</v>
+        <v>1984</v>
       </c>
       <c r="Y2" t="n">
-        <v>1980</v>
+        <v>1984</v>
       </c>
       <c r="Z2" t="n">
-        <v>1397688</v>
+        <v>1459404</v>
       </c>
       <c r="AA2" t="n">
-        <v>1617773</v>
+        <v>1615437</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.71</v>
+        <v>-0.32</v>
       </c>
       <c r="AE2" t="n">
-        <v>46.5</v>
+        <v>54.8</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.35</v>
+        <v>2.76</v>
       </c>
       <c r="AG2" t="n">
-        <v>46.31</v>
+        <v>46.91</v>
       </c>
       <c r="AH2" t="n">
-        <v>46.31</v>
+        <v>46.91</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.34</v>
+        <v>2.36</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>1.16</v>
+        <v>1.06</v>
       </c>
       <c r="AM2" t="n">
-        <v>5.71</v>
+        <v>5.45</v>
       </c>
       <c r="AN2" t="n">
-        <v>45.83</v>
+        <v>45.59</v>
       </c>
       <c r="AO2" t="n">
-        <v>57.79</v>
+        <v>58.38</v>
       </c>
       <c r="AP2" t="n">
-        <v>3.91</v>
+        <v>1.84</v>
       </c>
       <c r="AQ2" t="n">
-        <v>28.38</v>
+        <v>29.74</v>
       </c>
       <c r="AR2" t="n">
-        <v>1980</v>
+        <v>1984</v>
       </c>
       <c r="AS2" t="n">
-        <v>2165.23</v>
+        <v>2171.65</v>
       </c>
       <c r="AT2" t="n">
-        <v>1887.39</v>
+        <v>1890.17</v>
       </c>
       <c r="AU2" t="n">
-        <v>1980</v>
+        <v>1984</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.359999999999999</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="AY2" t="n">
-        <v>185.23</v>
+        <v>187.65</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.68</v>
+        <v>4.73</v>
       </c>
       <c r="BA2" t="n">
-        <v>92.61</v>
+        <v>93.83</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.06</v>
+        <v>2.05</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
@@ -1984,13 +1984,13 @@
         <v>332</v>
       </c>
       <c r="BF2" t="n">
-        <v>49.6</v>
+        <v>49.5</v>
       </c>
       <c r="BG2" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.2</v>
+        <v>18.3</v>
       </c>
       <c r="BI2" t="n">
         <v>2</v>
@@ -2005,16 +2005,16 @@
         <v>2</v>
       </c>
       <c r="BM2" t="n">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="BN2" t="n">
         <v>49.6</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.19</v>
+        <v>2.18</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.73</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="BQ2" t="n">
         <v>-4.24</v>
@@ -2026,19 +2026,19 @@
         <v>0.241</v>
       </c>
       <c r="BT2" t="n">
-        <v>1465.25</v>
+        <v>1465.91</v>
       </c>
       <c r="BU2" t="n">
-        <v>-14.01</v>
+        <v>-13.98</v>
       </c>
       <c r="BV2" t="n">
         <v>2.02</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.06</v>
+        <v>2.05</v>
       </c>
       <c r="BX2" t="n">
-        <v>2.0001</v>
+        <v>1.9999</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2047,7 +2047,7 @@
         <v>8</v>
       </c>
       <c r="CA2" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="CB2" t="n">
         <v>0</v>
@@ -2058,13 +2058,13 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>43.8</v>
+        <v>43.6</v>
       </c>
       <c r="CE2" t="n">
         <v>51</v>
       </c>
       <c r="CF2" t="n">
-        <v>68.7</v>
+        <v>68.3</v>
       </c>
       <c r="CG2" t="n">
         <v>70.90000000000001</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>94.45999999999999</v>
+        <v>87.31999999999999</v>
       </c>
       <c r="CO2" t="n">
-        <v>37.23</v>
+        <v>36.27</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2124,7 +2124,7 @@
         <v>3</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.3551</v>
+        <v>9.4582</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.624</v>
+        <v>0.6307</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.312</v>
+        <v>0.3153</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0936</v>
+        <v>0.0946</v>
       </c>
       <c r="DF2" t="n">
         <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.0708</v>
+        <v>1.0822</v>
       </c>
       <c r="DH2" t="n">
-        <v>4</v>
+        <v>4.0085</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.6773</v>
+        <v>4.7293</v>
       </c>
       <c r="DJ2" t="n">
-        <v>35.03</v>
+        <v>35.45</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.6773</v>
+        <v>4.7293</v>
       </c>
       <c r="DL2" t="n">
-        <v>2.0001</v>
+        <v>1.9999</v>
       </c>
       <c r="DM2" t="n">
-        <v>2</v>
+        <v>2.0042</v>
       </c>
       <c r="DN2" t="n">
-        <v>4</v>
+        <v>4.0085</v>
       </c>
       <c r="DO2" t="n">
-        <v>2</v>
+        <v>2.0003</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8547</v>
+        <v>0.8475</v>
       </c>
       <c r="DQ2" t="n">
-        <v>92.61</v>
+        <v>93.83</v>
       </c>
       <c r="DR2" t="n">
-        <v>50.64</v>
+        <v>69.22</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,49 +2193,49 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.6709</v>
+        <v>0.7796999999999999</v>
       </c>
       <c r="DX2" t="n">
-        <v>94.47499999999999</v>
+        <v>95.95</v>
       </c>
       <c r="DY2" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="DZ2" t="n">
-        <v>86.886</v>
+        <v>89.01900000000001</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
       </c>
       <c r="EB2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>85.81</v>
+        <v>92.65000000000001</v>
       </c>
       <c r="ED2" t="n">
         <v>100</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.6709</v>
+        <v>0.7796999999999999</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.4473</v>
+        <v>0.2105</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9979</v>
+        <v>4.0077</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0512</v>
+        <v>0.0241</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7039</v>
+        <v>0.6994</v>
       </c>
       <c r="EK2" t="n">
-        <v>80.48</v>
+        <v>84.38</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2249,34 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>11.43</v>
+        <v>12.24</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.3076</v>
+        <v>1.4003</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0984</v>
+        <v>0.103</v>
       </c>
       <c r="ER2" t="n">
-        <v>10.8837</v>
+        <v>10.5111</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.488</v>
+        <v>10.5506</v>
       </c>
       <c r="ET2" t="n">
-        <v>37.128</v>
+        <v>36.987</v>
       </c>
       <c r="EU2" t="n">
-        <v>3.3626</v>
+        <v>1.656</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.2581</v>
+        <v>1.2421</v>
       </c>
       <c r="EW2" t="n">
-        <v>10.7968</v>
+        <v>10.688</v>
       </c>
       <c r="EX2" t="n">
-        <v>27.88</v>
+        <v>29.8</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2293,28 +2293,28 @@
         <v>62.69</v>
       </c>
       <c r="FC2" t="n">
-        <v>24.8</v>
+        <v>25.62</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.83</v>
+        <v>73.3</v>
       </c>
       <c r="FE2" t="n">
-        <v>87.47</v>
+        <v>85.84999999999999</v>
       </c>
       <c r="FF2" t="n">
-        <v>32.555</v>
+        <v>33.035</v>
       </c>
       <c r="FG2" t="n">
-        <v>28.2814</v>
+        <v>25.9881</v>
       </c>
       <c r="FH2" t="n">
-        <v>65.259</v>
+        <v>63.501</v>
       </c>
       <c r="FI2" t="n">
-        <v>42.835</v>
+        <v>52.335</v>
       </c>
       <c r="FJ2" t="n">
-        <v>67.65000000000001</v>
+        <v>68.18000000000001</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>69.64</v>
+        <v>77.23</v>
       </c>
       <c r="FO2" t="n">
-        <v>68.90000000000001</v>
+        <v>68.33</v>
       </c>
       <c r="FP2" t="n">
-        <v>46.28</v>
+        <v>59.61</v>
       </c>
       <c r="FQ2" t="n">
-        <v>65.09999999999999</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="FR2" t="n">
-        <v>74.31999999999999</v>
+        <v>81.18000000000001</v>
       </c>
       <c r="FS2" t="n">
         <v>90.9091</v>
@@ -2353,11 +2353,11 @@
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>63.5405</v>
+        <v>69.9265</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20260930_215357</t>
+          <t>20261001_154354</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46295.91247494507</v>
+        <v>46296.65548923887</v>
       </c>
     </row>
   </sheetData>
@@ -2465,7 +2465,7 @@
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="19" customWidth="1" min="23" max="23"/>
     <col width="19" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46295.91246527778</v>
+        <v>46296.65548611111</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1980</v>
+        <v>1984</v>
       </c>
       <c r="L2" t="n">
-        <v>1993</v>
+        <v>1973.6</v>
       </c>
       <c r="M2" t="n">
-        <v>2001.6</v>
+        <v>2006.9</v>
       </c>
       <c r="N2" t="n">
-        <v>1955.1</v>
+        <v>1952.1</v>
       </c>
       <c r="O2" t="n">
-        <v>1980</v>
+        <v>1984</v>
       </c>
       <c r="P2" t="n">
-        <v>1397688</v>
+        <v>1459404</v>
       </c>
       <c r="Q2" t="n">
-        <v>1980</v>
+        <v>1984</v>
       </c>
       <c r="R2" t="n">
-        <v>2165.23</v>
+        <v>2171.65</v>
       </c>
       <c r="S2" t="n">
-        <v>1887.39</v>
+        <v>1890.17</v>
       </c>
       <c r="T2" t="n">
-        <v>9.355050505050507</v>
+        <v>9.458165322580649</v>
       </c>
       <c r="U2" t="n">
-        <v>185.23</v>
+        <v>187.6500000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>4.677272727272722</v>
+        <v>4.729334677419351</v>
       </c>
       <c r="W2" t="n">
-        <v>92.6099999999999</v>
+        <v>93.82999999999993</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000107979699819</v>
+        <v>1.999893424277952</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.355050505050507</v>
+        <v>9.458165322580649</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.677272727272722</v>
+        <v>4.729334677419351</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02041506973087686</v>
+        <v>0.02040055973410541</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.324079185035655</v>
+        <v>0.3238488459777654</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02908554432243104</v>
+        <v>0.02907953966364668</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228670527526088</v>
+        <v>0.04228671263421219</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347617</v>
+        <v>0.1869493934347614</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.07</v>
+        <v>39.09</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-30 21:53:57.874306+05:30</t>
+          <t>2026-10-01 15:43:54.309479+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.355050505050507, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000107979699819}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.45816532258065, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.999893424277952}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-01 17:00 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -2026,7 +2026,7 @@
         <v>0.241</v>
       </c>
       <c r="BT2" t="n">
-        <v>1465.91</v>
+        <v>1465.92</v>
       </c>
       <c r="BU2" t="n">
         <v>-13.98</v>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261001_154354</t>
+          <t>20261001_223052</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46296.65548923887</v>
+        <v>46296.93810992716</v>
       </c>
     </row>
   </sheetData>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46296.65548611111</v>
+        <v>46296.93810185185</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46296</v>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02040055973410541</v>
+        <v>0.02040055780919982</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3238488459777654</v>
+        <v>0.3238488154208364</v>
       </c>
     </row>
     <row r="7">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228671263421219</v>
+        <v>0.04228670884492124</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347614</v>
+        <v>0.1869493934347613</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-01 15:43:54.309479+05:30</t>
+          <t>2026-10-01 22:30:52.734703+05:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-02 09:51 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -1890,10 +1890,10 @@
         <v>1984</v>
       </c>
       <c r="Z2" t="n">
-        <v>1459404</v>
+        <v>1459687</v>
       </c>
       <c r="AA2" t="n">
-        <v>1615437</v>
+        <v>1615452</v>
       </c>
       <c r="AB2" t="n">
         <v>0.9</v>
@@ -2026,7 +2026,7 @@
         <v>0.241</v>
       </c>
       <c r="BT2" t="n">
-        <v>1465.92</v>
+        <v>1465.91</v>
       </c>
       <c r="BU2" t="n">
         <v>-13.98</v>
@@ -2091,7 +2091,7 @@
         <v>87.31999999999999</v>
       </c>
       <c r="CO2" t="n">
-        <v>36.27</v>
+        <v>36.24</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2264,7 +2264,7 @@
         <v>10.5506</v>
       </c>
       <c r="ET2" t="n">
-        <v>36.987</v>
+        <v>36.975</v>
       </c>
       <c r="EU2" t="n">
         <v>1.656</v>
@@ -2276,7 +2276,7 @@
         <v>10.688</v>
       </c>
       <c r="EX2" t="n">
-        <v>29.8</v>
+        <v>29.79</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2302,13 +2302,13 @@
         <v>85.84999999999999</v>
       </c>
       <c r="FF2" t="n">
-        <v>33.035</v>
+        <v>33.015</v>
       </c>
       <c r="FG2" t="n">
         <v>25.9881</v>
       </c>
       <c r="FH2" t="n">
-        <v>63.501</v>
+        <v>63.499</v>
       </c>
       <c r="FI2" t="n">
         <v>52.335</v>
@@ -2334,13 +2334,13 @@
         <v>68.33</v>
       </c>
       <c r="FP2" t="n">
-        <v>59.61</v>
+        <v>59.6</v>
       </c>
       <c r="FQ2" t="n">
-        <v>76.40000000000001</v>
+        <v>76.41</v>
       </c>
       <c r="FR2" t="n">
-        <v>81.18000000000001</v>
+        <v>81.19</v>
       </c>
       <c r="FS2" t="n">
         <v>90.9091</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>69.9265</v>
+        <v>69.9315</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261001_223052</t>
+          <t>20261002_152125</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46296.93810992716</v>
+        <v>46297.63987567084</v>
       </c>
     </row>
   </sheetData>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46296.93810185185</v>
+        <v>46297.63987268518</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46296</v>
@@ -2696,7 +2696,7 @@
         <v>1984</v>
       </c>
       <c r="P2" t="n">
-        <v>1459404</v>
+        <v>1459687</v>
       </c>
       <c r="Q2" t="n">
         <v>1984</v>
@@ -2726,13 +2726,13 @@
         <v>15</v>
       </c>
       <c r="Z2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AB2" t="n">
-        <v>0</v>
+        <v>6.666666666666667</v>
       </c>
       <c r="AC2" t="n">
         <v>0</v>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02040055780919982</v>
+        <v>0.02040055602716745</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3238488154208364</v>
+        <v>0.3238487871319495</v>
       </c>
     </row>
     <row r="7">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228670884492124</v>
+        <v>0.04228670193426839</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347613</v>
+        <v>0.1869492979645464</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-01 22:30:52.734703+05:30</t>
+          <t>2026-10-02 15:21:25.301588+05:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-02 16:15 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -2026,7 +2026,7 @@
         <v>0.241</v>
       </c>
       <c r="BT2" t="n">
-        <v>1465.91</v>
+        <v>1465.9</v>
       </c>
       <c r="BU2" t="n">
         <v>-13.98</v>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261002_152125</t>
+          <t>20261002_214530</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46297.63987567084</v>
+        <v>46297.90660359216</v>
       </c>
     </row>
   </sheetData>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46297.63987268518</v>
+        <v>46297.90659722222</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46296</v>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02040055602716745</v>
+        <v>0.02040055533151923</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3238487871319495</v>
+        <v>0.3238487760888763</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02907953966364668</v>
+        <v>0.02907952500016192</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228670193426839</v>
+        <v>0.0422867071950403</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-02 15:21:25.301588+05:30</t>
+          <t>2026-10-02 21:45:30.576251+05:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-05 10:33 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="17" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,19 +1816,17 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46296</v>
-      </c>
-      <c r="E2" s="1" t="n">
-        <v>46296</v>
-      </c>
+        <v>46300</v>
+      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="H2" t="n">
-        <v>8.699999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -1854,61 +1852,57 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="P2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.44</v>
+        <v>11.35</v>
       </c>
       <c r="R2" t="n">
-        <v>48.83</v>
+        <v>48.84</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
       </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>UPTREND</t>
-        </is>
-      </c>
+      <c r="T2" t="inlineStr"/>
       <c r="U2" t="n">
-        <v>1973.6</v>
+        <v>1994</v>
       </c>
       <c r="V2" t="n">
-        <v>2006.9</v>
+        <v>2002</v>
       </c>
       <c r="W2" t="n">
-        <v>1952.1</v>
+        <v>1955.1</v>
       </c>
       <c r="X2" t="n">
-        <v>1984</v>
+        <v>1971.4</v>
       </c>
       <c r="Y2" t="n">
-        <v>1984</v>
+        <v>1971.4</v>
       </c>
       <c r="Z2" t="n">
-        <v>1459687</v>
+        <v>1371692</v>
       </c>
       <c r="AA2" t="n">
-        <v>1615452</v>
+        <v>1630239</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.9</v>
+        <v>0.84</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.2</v>
+        <v>-0.64</v>
       </c>
       <c r="AD2" t="n">
-        <v>-0.32</v>
+        <v>0.5</v>
       </c>
       <c r="AE2" t="n">
-        <v>54.8</v>
+        <v>46.9</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.76</v>
+        <v>2.38</v>
       </c>
       <c r="AG2" t="n">
         <v>46.91</v>
@@ -1917,7 +1911,7 @@
         <v>46.91</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.36</v>
+        <v>2.38</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,119 +1920,119 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>1.06</v>
+        <v>0.09</v>
       </c>
       <c r="AM2" t="n">
-        <v>5.45</v>
+        <v>4.37</v>
       </c>
       <c r="AN2" t="n">
-        <v>45.59</v>
+        <v>44.16</v>
       </c>
       <c r="AO2" t="n">
-        <v>58.38</v>
+        <v>55.73</v>
       </c>
       <c r="AP2" t="n">
-        <v>1.84</v>
+        <v>0.89</v>
       </c>
       <c r="AQ2" t="n">
-        <v>29.74</v>
+        <v>33.44</v>
       </c>
       <c r="AR2" t="n">
-        <v>1984</v>
+        <v>1971.4</v>
       </c>
       <c r="AS2" t="n">
-        <v>2171.65</v>
+        <v>2159.05</v>
       </c>
       <c r="AT2" t="n">
-        <v>1890.17</v>
+        <v>1877.58</v>
       </c>
       <c r="AU2" t="n">
-        <v>1984</v>
+        <v>1971.400024414062</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.460000000000001</v>
+        <v>9.52</v>
       </c>
       <c r="AY2" t="n">
         <v>187.65</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.73</v>
+        <v>4.76</v>
       </c>
       <c r="BA2" t="n">
-        <v>93.83</v>
+        <v>93.81999999999999</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.05</v>
+        <v>2.07</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
       </c>
       <c r="BD2" t="n">
-        <v>31.9</v>
+        <v>31.8</v>
       </c>
       <c r="BE2" t="n">
         <v>332</v>
       </c>
       <c r="BF2" t="n">
-        <v>49.5</v>
+        <v>49.4</v>
       </c>
       <c r="BG2" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.3</v>
+        <v>18.2</v>
       </c>
       <c r="BI2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="BM2" t="n">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="BN2" t="n">
-        <v>49.6</v>
+        <v>49.4</v>
       </c>
       <c r="BO2" t="n">
         <v>2.18</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.699999999999999</v>
+        <v>8.73</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.24</v>
+        <v>-4.22</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.241</v>
+        <v>0.24</v>
       </c>
       <c r="BT2" t="n">
-        <v>1465.9</v>
+        <v>1462.76</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.98</v>
+        <v>-14.16</v>
       </c>
       <c r="BV2" t="n">
         <v>2.02</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.05</v>
+        <v>2.07</v>
       </c>
       <c r="BX2" t="n">
-        <v>1.9999</v>
+        <v>2.0001</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2047,14 +2041,14 @@
         <v>8</v>
       </c>
       <c r="CA2" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="CB2" t="n">
         <v>0</v>
       </c>
       <c r="CC2" t="inlineStr">
         <is>
-          <t>limited history: 8.7y (&lt;10y) - lower confidence</t>
+          <t>limited history: 8.8y (&lt;10y) - lower confidence</t>
         </is>
       </c>
       <c r="CD2" t="n">
@@ -2064,10 +2058,10 @@
         <v>51</v>
       </c>
       <c r="CF2" t="n">
-        <v>68.3</v>
+        <v>69</v>
       </c>
       <c r="CG2" t="n">
-        <v>70.90000000000001</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>87.31999999999999</v>
+        <v>89.86</v>
       </c>
       <c r="CO2" t="n">
-        <v>36.24</v>
+        <v>37.11</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2121,10 +2115,10 @@
         <v>54.54545454545454</v>
       </c>
       <c r="CY2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.4582</v>
+        <v>9.518599999999999</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2127,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6307</v>
+        <v>0.6347</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3153</v>
+        <v>0.3173</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0946</v>
+        <v>0.09520000000000001</v>
       </c>
       <c r="DF2" t="n">
         <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.0822</v>
+        <v>1.0805</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0085</v>
+        <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.7293</v>
+        <v>4.7591</v>
       </c>
       <c r="DJ2" t="n">
-        <v>35.45</v>
+        <v>30.66</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.7293</v>
+        <v>4.7591</v>
       </c>
       <c r="DL2" t="n">
-        <v>1.9999</v>
+        <v>2.0001</v>
       </c>
       <c r="DM2" t="n">
-        <v>2.0042</v>
+        <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>4.0085</v>
+        <v>4</v>
       </c>
       <c r="DO2" t="n">
         <v>2.0003</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8475</v>
+        <v>0.8403</v>
       </c>
       <c r="DQ2" t="n">
-        <v>93.83</v>
+        <v>93.81999999999999</v>
       </c>
       <c r="DR2" t="n">
-        <v>69.22</v>
+        <v>55.85</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2187,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.7796999999999999</v>
+        <v>0.3739</v>
       </c>
       <c r="DX2" t="n">
-        <v>95.95</v>
+        <v>89.32499999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="DZ2" t="n">
-        <v>89.01900000000001</v>
+        <v>87.72799999999999</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,35 +2205,35 @@
         <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>92.65000000000001</v>
+        <v>85.78</v>
       </c>
       <c r="ED2" t="n">
-        <v>100</v>
+        <v>97.23999999999999</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.7796999999999999</v>
+        <v>0.3739</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.9</v>
+        <v>0.84</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.2105</v>
+        <v>0.101</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0077</v>
+        <v>3.9994</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0241</v>
+        <v>0.0115</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6994</v>
+        <v>0.6943</v>
       </c>
       <c r="EK2" t="n">
-        <v>84.38</v>
+        <v>79.88</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
-          <t>Excellent</t>
+          <t>Strong</t>
         </is>
       </c>
       <c r="EM2" t="n">
@@ -2249,72 +2243,72 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>12.24</v>
+        <v>25.46</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.4003</v>
+        <v>2.8897</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.103</v>
+        <v>0.0953</v>
       </c>
       <c r="ER2" t="n">
-        <v>10.5111</v>
+        <v>11.3333</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.5506</v>
+        <v>9.071</v>
       </c>
       <c r="ET2" t="n">
-        <v>36.975</v>
+        <v>41.16</v>
       </c>
       <c r="EU2" t="n">
-        <v>1.656</v>
+        <v>0.7476</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.2421</v>
+        <v>1.2935</v>
       </c>
       <c r="EW2" t="n">
-        <v>10.688</v>
+        <v>22.8784</v>
       </c>
       <c r="EX2" t="n">
-        <v>29.79</v>
+        <v>56.46</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="FA2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="FB2" t="n">
-        <v>62.69</v>
+        <v>62.26</v>
       </c>
       <c r="FC2" t="n">
-        <v>25.62</v>
+        <v>19.66</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.3</v>
+        <v>74.36</v>
       </c>
       <c r="FE2" t="n">
-        <v>85.84999999999999</v>
+        <v>84.87</v>
       </c>
       <c r="FF2" t="n">
-        <v>33.015</v>
+        <v>46.785</v>
       </c>
       <c r="FG2" t="n">
-        <v>25.9881</v>
+        <v>26.5858</v>
       </c>
       <c r="FH2" t="n">
-        <v>63.499</v>
+        <v>69.38</v>
       </c>
       <c r="FI2" t="n">
-        <v>52.335</v>
+        <v>43.255</v>
       </c>
       <c r="FJ2" t="n">
-        <v>68.18000000000001</v>
+        <v>68.26000000000001</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2322,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>77.23</v>
+        <v>78.27</v>
       </c>
       <c r="FO2" t="n">
-        <v>68.33</v>
+        <v>64.53</v>
       </c>
       <c r="FP2" t="n">
-        <v>59.6</v>
+        <v>76.81</v>
       </c>
       <c r="FQ2" t="n">
-        <v>76.41</v>
+        <v>73.01000000000001</v>
       </c>
       <c r="FR2" t="n">
-        <v>81.19</v>
+        <v>89.48999999999999</v>
       </c>
       <c r="FS2" t="n">
-        <v>90.9091</v>
+        <v>100</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2357,7 +2351,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>69.9315</v>
+        <v>71.37350000000001</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261002_214530</t>
+          <t>20261005_160320</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46297.90660359216</v>
+        <v>46300.66898909498</v>
       </c>
     </row>
   </sheetData>
@@ -2444,8 +2438,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -2647,14 +2641,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46297.90659722222</v>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>46296</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>46311</v>
-      </c>
+        <v>46300.66898148148</v>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>LAURUSLABS</t>
@@ -2673,66 +2663,62 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.44</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>UPTREND</t>
-        </is>
-      </c>
+        <v>11.35</v>
+      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>1984</v>
+        <v>1971.4</v>
       </c>
       <c r="L2" t="n">
-        <v>1973.6</v>
+        <v>1994</v>
       </c>
       <c r="M2" t="n">
-        <v>2006.9</v>
+        <v>2002</v>
       </c>
       <c r="N2" t="n">
-        <v>1952.1</v>
+        <v>1955.1</v>
       </c>
       <c r="O2" t="n">
-        <v>1984</v>
+        <v>1971.4</v>
       </c>
       <c r="P2" t="n">
-        <v>1459687</v>
+        <v>1371692</v>
       </c>
       <c r="Q2" t="n">
-        <v>1984</v>
+        <v>1971.4</v>
       </c>
       <c r="R2" t="n">
-        <v>2171.65</v>
+        <v>2159.05</v>
       </c>
       <c r="S2" t="n">
-        <v>1890.17</v>
+        <v>1877.58</v>
       </c>
       <c r="T2" t="n">
-        <v>9.458165322580649</v>
+        <v>9.518616211829162</v>
       </c>
       <c r="U2" t="n">
         <v>187.6500000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>4.729334677419351</v>
+        <v>4.759054479050429</v>
       </c>
       <c r="W2" t="n">
-        <v>93.82999999999993</v>
+        <v>93.82000000000016</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999893424277952</v>
+        <v>2.000106587081643</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
       </c>
       <c r="Z2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="AB2" t="n">
-        <v>6.666666666666667</v>
+        <v>0</v>
       </c>
       <c r="AC2" t="n">
         <v>0</v>
@@ -2741,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.458165322580649</v>
+        <v>9.518616211829162</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.729334677419351</v>
+        <v>4.759054479050429</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02040055533151923</v>
+        <v>0.02038884116137439</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3238487760888763</v>
+        <v>0.3236628194027639</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02907952500016192</v>
+        <v>0.0290735062444351</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.0422867071950403</v>
+        <v>0.04228669903469408</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869492979645462</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.09</v>
+        <v>39.11</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-02 21:45:30.576251+05:30</t>
+          <t>2026-10-05 16:03:20.680814+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.45816532258065, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.999893424277952}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.518616211829162, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000106587081643}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-05 19:17 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="20" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="17" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,17 +1816,19 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46300</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
+        <v>46296</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>46296</v>
+      </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46300</v>
+        <v>46296</v>
       </c>
       <c r="H2" t="n">
-        <v>8.800000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -1852,57 +1854,61 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="P2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.35</v>
+        <v>11.44</v>
       </c>
       <c r="R2" t="n">
-        <v>48.84</v>
+        <v>48.83</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
       </c>
-      <c r="T2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>UPTREND</t>
+        </is>
+      </c>
       <c r="U2" t="n">
-        <v>1994</v>
+        <v>1973.6</v>
       </c>
       <c r="V2" t="n">
-        <v>2002</v>
+        <v>2006.9</v>
       </c>
       <c r="W2" t="n">
-        <v>1955.1</v>
+        <v>1952.1</v>
       </c>
       <c r="X2" t="n">
-        <v>1971.4</v>
+        <v>1984</v>
       </c>
       <c r="Y2" t="n">
-        <v>1971.4</v>
+        <v>1984</v>
       </c>
       <c r="Z2" t="n">
-        <v>1371692</v>
+        <v>1459687</v>
       </c>
       <c r="AA2" t="n">
-        <v>1630239</v>
+        <v>1615452</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.84</v>
+        <v>0.9</v>
       </c>
       <c r="AC2" t="n">
-        <v>-0.64</v>
+        <v>0.2</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.5</v>
+        <v>-0.32</v>
       </c>
       <c r="AE2" t="n">
-        <v>46.9</v>
+        <v>54.8</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.38</v>
+        <v>2.76</v>
       </c>
       <c r="AG2" t="n">
         <v>46.91</v>
@@ -1911,7 +1917,7 @@
         <v>46.91</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.38</v>
+        <v>2.36</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,119 +1926,119 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>0.09</v>
+        <v>1.06</v>
       </c>
       <c r="AM2" t="n">
-        <v>4.37</v>
+        <v>5.45</v>
       </c>
       <c r="AN2" t="n">
-        <v>44.16</v>
+        <v>45.59</v>
       </c>
       <c r="AO2" t="n">
-        <v>55.73</v>
+        <v>58.38</v>
       </c>
       <c r="AP2" t="n">
-        <v>0.89</v>
+        <v>1.84</v>
       </c>
       <c r="AQ2" t="n">
-        <v>33.44</v>
+        <v>29.74</v>
       </c>
       <c r="AR2" t="n">
-        <v>1971.4</v>
+        <v>1984</v>
       </c>
       <c r="AS2" t="n">
-        <v>2159.05</v>
+        <v>2171.65</v>
       </c>
       <c r="AT2" t="n">
-        <v>1877.58</v>
+        <v>1890.17</v>
       </c>
       <c r="AU2" t="n">
-        <v>1971.400024414062</v>
+        <v>1984</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.52</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="AY2" t="n">
         <v>187.65</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.76</v>
+        <v>4.73</v>
       </c>
       <c r="BA2" t="n">
-        <v>93.81999999999999</v>
+        <v>93.83</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.07</v>
+        <v>2.05</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
       </c>
       <c r="BD2" t="n">
-        <v>31.8</v>
+        <v>31.9</v>
       </c>
       <c r="BE2" t="n">
         <v>332</v>
       </c>
       <c r="BF2" t="n">
-        <v>49.4</v>
+        <v>49.5</v>
       </c>
       <c r="BG2" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.2</v>
+        <v>18.3</v>
       </c>
       <c r="BI2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="BM2" t="n">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="BN2" t="n">
-        <v>49.4</v>
+        <v>49.6</v>
       </c>
       <c r="BO2" t="n">
         <v>2.18</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.73</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.22</v>
+        <v>-4.24</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.24</v>
+        <v>0.241</v>
       </c>
       <c r="BT2" t="n">
-        <v>1462.76</v>
+        <v>1465.9</v>
       </c>
       <c r="BU2" t="n">
-        <v>-14.16</v>
+        <v>-13.98</v>
       </c>
       <c r="BV2" t="n">
         <v>2.02</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.07</v>
+        <v>2.05</v>
       </c>
       <c r="BX2" t="n">
-        <v>2.0001</v>
+        <v>1.9999</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2041,14 +2047,14 @@
         <v>8</v>
       </c>
       <c r="CA2" t="n">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="CB2" t="n">
         <v>0</v>
       </c>
       <c r="CC2" t="inlineStr">
         <is>
-          <t>limited history: 8.8y (&lt;10y) - lower confidence</t>
+          <t>limited history: 8.7y (&lt;10y) - lower confidence</t>
         </is>
       </c>
       <c r="CD2" t="n">
@@ -2058,10 +2064,10 @@
         <v>51</v>
       </c>
       <c r="CF2" t="n">
-        <v>69</v>
+        <v>68.3</v>
       </c>
       <c r="CG2" t="n">
-        <v>70.59999999999999</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2082,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>89.86</v>
+        <v>87.31999999999999</v>
       </c>
       <c r="CO2" t="n">
-        <v>37.11</v>
+        <v>36.24</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2115,10 +2121,10 @@
         <v>54.54545454545454</v>
       </c>
       <c r="CY2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.518599999999999</v>
+        <v>9.4582</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6347</v>
+        <v>0.6307</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3173</v>
+        <v>0.3153</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.09520000000000001</v>
+        <v>0.0946</v>
       </c>
       <c r="DF2" t="n">
         <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.0805</v>
+        <v>1.0822</v>
       </c>
       <c r="DH2" t="n">
-        <v>4</v>
+        <v>4.0085</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.7591</v>
+        <v>4.7293</v>
       </c>
       <c r="DJ2" t="n">
-        <v>30.66</v>
+        <v>35.45</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.7591</v>
+        <v>4.7293</v>
       </c>
       <c r="DL2" t="n">
-        <v>2.0001</v>
+        <v>1.9999</v>
       </c>
       <c r="DM2" t="n">
-        <v>2</v>
+        <v>2.0042</v>
       </c>
       <c r="DN2" t="n">
-        <v>4</v>
+        <v>4.0085</v>
       </c>
       <c r="DO2" t="n">
         <v>2.0003</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8403</v>
+        <v>0.8475</v>
       </c>
       <c r="DQ2" t="n">
-        <v>93.81999999999999</v>
+        <v>93.83</v>
       </c>
       <c r="DR2" t="n">
-        <v>55.85</v>
+        <v>69.22</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.3739</v>
+        <v>0.7796999999999999</v>
       </c>
       <c r="DX2" t="n">
-        <v>89.32499999999999</v>
+        <v>95.95</v>
       </c>
       <c r="DY2" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="DZ2" t="n">
-        <v>87.72799999999999</v>
+        <v>89.01900000000001</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2205,35 +2211,35 @@
         <v>9</v>
       </c>
       <c r="EC2" t="n">
-        <v>85.78</v>
+        <v>92.65000000000001</v>
       </c>
       <c r="ED2" t="n">
-        <v>97.23999999999999</v>
+        <v>100</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.3739</v>
+        <v>0.7796999999999999</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.84</v>
+        <v>0.9</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.101</v>
+        <v>0.2105</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9994</v>
+        <v>4.0077</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0115</v>
+        <v>0.0241</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6943</v>
+        <v>0.6994</v>
       </c>
       <c r="EK2" t="n">
-        <v>79.88</v>
+        <v>84.38</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Excellent</t>
         </is>
       </c>
       <c r="EM2" t="n">
@@ -2243,72 +2249,72 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>25.46</v>
+        <v>12.24</v>
       </c>
       <c r="EP2" t="n">
-        <v>2.8897</v>
+        <v>1.4003</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0953</v>
+        <v>0.103</v>
       </c>
       <c r="ER2" t="n">
-        <v>11.3333</v>
+        <v>10.5111</v>
       </c>
       <c r="ES2" t="n">
-        <v>9.071</v>
+        <v>10.5506</v>
       </c>
       <c r="ET2" t="n">
-        <v>41.16</v>
+        <v>36.975</v>
       </c>
       <c r="EU2" t="n">
-        <v>0.7476</v>
+        <v>1.656</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.2935</v>
+        <v>1.2421</v>
       </c>
       <c r="EW2" t="n">
-        <v>22.8784</v>
+        <v>10.688</v>
       </c>
       <c r="EX2" t="n">
-        <v>56.46</v>
+        <v>29.79</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="FA2" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="FB2" t="n">
-        <v>62.26</v>
+        <v>62.69</v>
       </c>
       <c r="FC2" t="n">
-        <v>19.66</v>
+        <v>25.62</v>
       </c>
       <c r="FD2" t="n">
-        <v>74.36</v>
+        <v>73.3</v>
       </c>
       <c r="FE2" t="n">
-        <v>84.87</v>
+        <v>85.84999999999999</v>
       </c>
       <c r="FF2" t="n">
-        <v>46.785</v>
+        <v>33.015</v>
       </c>
       <c r="FG2" t="n">
-        <v>26.5858</v>
+        <v>25.9881</v>
       </c>
       <c r="FH2" t="n">
-        <v>69.38</v>
+        <v>63.499</v>
       </c>
       <c r="FI2" t="n">
-        <v>43.255</v>
+        <v>52.335</v>
       </c>
       <c r="FJ2" t="n">
-        <v>68.26000000000001</v>
+        <v>68.18000000000001</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>78.27</v>
+        <v>77.23</v>
       </c>
       <c r="FO2" t="n">
-        <v>64.53</v>
+        <v>68.33</v>
       </c>
       <c r="FP2" t="n">
-        <v>76.81</v>
+        <v>59.6</v>
       </c>
       <c r="FQ2" t="n">
-        <v>73.01000000000001</v>
+        <v>76.41</v>
       </c>
       <c r="FR2" t="n">
-        <v>89.48999999999999</v>
+        <v>81.18000000000001</v>
       </c>
       <c r="FS2" t="n">
-        <v>100</v>
+        <v>90.9091</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2351,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>71.37350000000001</v>
+        <v>69.9265</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261005_160320</t>
+          <t>20261006_004724</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46300.66898909498</v>
+        <v>46301.03291937124</v>
       </c>
     </row>
   </sheetData>
@@ -2438,8 +2444,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -2641,10 +2647,14 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46300.66898148148</v>
-      </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
+        <v>46301.03291666666</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>46311</v>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>LAURUSLABS</t>
@@ -2663,62 +2673,66 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.35</v>
-      </c>
-      <c r="J2" t="inlineStr"/>
+        <v>11.44</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>UPTREND</t>
+        </is>
+      </c>
       <c r="K2" t="n">
-        <v>1971.4</v>
+        <v>1984</v>
       </c>
       <c r="L2" t="n">
-        <v>1994</v>
+        <v>1973.6</v>
       </c>
       <c r="M2" t="n">
-        <v>2002</v>
+        <v>2006.9</v>
       </c>
       <c r="N2" t="n">
-        <v>1955.1</v>
+        <v>1952.1</v>
       </c>
       <c r="O2" t="n">
-        <v>1971.4</v>
+        <v>1984</v>
       </c>
       <c r="P2" t="n">
-        <v>1371692</v>
+        <v>1459687</v>
       </c>
       <c r="Q2" t="n">
-        <v>1971.4</v>
+        <v>1984</v>
       </c>
       <c r="R2" t="n">
-        <v>2159.05</v>
+        <v>2171.65</v>
       </c>
       <c r="S2" t="n">
-        <v>1877.58</v>
+        <v>1890.17</v>
       </c>
       <c r="T2" t="n">
-        <v>9.518616211829162</v>
+        <v>9.458165322580649</v>
       </c>
       <c r="U2" t="n">
         <v>187.6500000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>4.759054479050429</v>
+        <v>4.729334677419351</v>
       </c>
       <c r="W2" t="n">
-        <v>93.82000000000016</v>
+        <v>93.82999999999993</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000106587081643</v>
+        <v>1.999893424277952</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
       </c>
       <c r="Z2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AA2" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="AB2" t="n">
-        <v>0</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="AC2" t="n">
         <v>0</v>
@@ -2727,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.518616211829162</v>
+        <v>9.458165322580649</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.759054479050429</v>
+        <v>4.729334677419351</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02038884116137439</v>
+        <v>0.02040055546603376</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3236628194027639</v>
+        <v>0.3238487782242284</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.0290735062444351</v>
+        <v>0.02907952542506864</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228669903469408</v>
+        <v>0.0422866948954063</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645462</v>
+        <v>0.1869492979645464</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.11</v>
+        <v>39.09</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-05 16:03:20.680814+05:30</t>
+          <t>2026-10-06 00:47:24.274513+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.518616211829162, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000106587081643}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.45816532258065, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.999893424277952}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-06 10:25 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -1816,19 +1816,19 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46296</v>
+        <v>46301</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46296</v>
+        <v>46301</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46296</v>
+        <v>46301</v>
       </c>
       <c r="H2" t="n">
-        <v>8.699999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1861,181 +1861,181 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.44</v>
+        <v>11.65</v>
       </c>
       <c r="R2" t="n">
+        <v>49.22</v>
+      </c>
+      <c r="S2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>UPTREND</t>
+        </is>
+      </c>
+      <c r="U2" t="n">
+        <v>1968.9</v>
+      </c>
+      <c r="V2" t="n">
+        <v>2054.9</v>
+      </c>
+      <c r="W2" t="n">
+        <v>1958</v>
+      </c>
+      <c r="X2" t="n">
+        <v>2050</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>2050</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>2196922</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>1577002</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>-0.13</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>96.90000000000001</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>4.73</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>47.59</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>47.59</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="AJ2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>3.52</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>7.89</v>
+      </c>
+      <c r="AN2" t="n">
         <v>48.83</v>
       </c>
-      <c r="S2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>UPTREND</t>
-        </is>
-      </c>
-      <c r="U2" t="n">
-        <v>1973.6</v>
-      </c>
-      <c r="V2" t="n">
-        <v>2006.9</v>
-      </c>
-      <c r="W2" t="n">
-        <v>1952.1</v>
-      </c>
-      <c r="X2" t="n">
-        <v>1984</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>1984</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>1459687</v>
-      </c>
-      <c r="AA2" t="n">
-        <v>1615452</v>
-      </c>
-      <c r="AB2" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="AC2" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="AD2" t="n">
-        <v>-0.32</v>
-      </c>
-      <c r="AE2" t="n">
-        <v>54.8</v>
-      </c>
-      <c r="AF2" t="n">
-        <v>2.76</v>
-      </c>
-      <c r="AG2" t="n">
-        <v>46.91</v>
-      </c>
-      <c r="AH2" t="n">
-        <v>46.91</v>
-      </c>
-      <c r="AI2" t="n">
-        <v>2.36</v>
-      </c>
-      <c r="AJ2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AK2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AL2" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="AM2" t="n">
-        <v>5.45</v>
-      </c>
-      <c r="AN2" t="n">
-        <v>45.59</v>
-      </c>
       <c r="AO2" t="n">
-        <v>58.38</v>
+        <v>66.51000000000001</v>
       </c>
       <c r="AP2" t="n">
-        <v>1.84</v>
+        <v>2.17</v>
       </c>
       <c r="AQ2" t="n">
-        <v>29.74</v>
+        <v>36</v>
       </c>
       <c r="AR2" t="n">
-        <v>1984</v>
+        <v>2050</v>
       </c>
       <c r="AS2" t="n">
-        <v>2171.65</v>
+        <v>2240.37</v>
       </c>
       <c r="AT2" t="n">
-        <v>1890.17</v>
+        <v>1954.81</v>
       </c>
       <c r="AU2" t="n">
-        <v>1984</v>
+        <v>2050</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.460000000000001</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="AY2" t="n">
-        <v>187.65</v>
+        <v>190.37</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.73</v>
+        <v>4.64</v>
       </c>
       <c r="BA2" t="n">
-        <v>93.83</v>
+        <v>95.19</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.05</v>
+        <v>2.03</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
       </c>
       <c r="BD2" t="n">
-        <v>31.9</v>
+        <v>31.8</v>
       </c>
       <c r="BE2" t="n">
         <v>332</v>
       </c>
       <c r="BF2" t="n">
-        <v>49.5</v>
+        <v>49.3</v>
       </c>
       <c r="BG2" t="n">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.3</v>
+        <v>18.9</v>
       </c>
       <c r="BI2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BM2" t="n">
-        <v>671</v>
+        <v>673</v>
       </c>
       <c r="BN2" t="n">
-        <v>49.6</v>
+        <v>50.1</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.18</v>
+        <v>2.2</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.699999999999999</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.24</v>
+        <v>-4.25</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.241</v>
+        <v>0.243</v>
       </c>
       <c r="BT2" t="n">
-        <v>1465.9</v>
+        <v>1479.26</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.98</v>
+        <v>-13.68</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.02</v>
+        <v>2.04</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.05</v>
+        <v>2.03</v>
       </c>
       <c r="BX2" t="n">
         <v>1.9999</v>
@@ -2054,20 +2054,20 @@
       </c>
       <c r="CC2" t="inlineStr">
         <is>
-          <t>limited history: 8.7y (&lt;10y) - lower confidence</t>
+          <t>limited history: 8.8y (&lt;10y) - lower confidence</t>
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>43.6</v>
+        <v>44</v>
       </c>
       <c r="CE2" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="CF2" t="n">
-        <v>68.3</v>
+        <v>67.7</v>
       </c>
       <c r="CG2" t="n">
-        <v>70.90000000000001</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>87.31999999999999</v>
+        <v>83.37</v>
       </c>
       <c r="CO2" t="n">
-        <v>36.24</v>
+        <v>41.63</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2106,7 +2106,7 @@
         <v>100</v>
       </c>
       <c r="CT2" t="n">
-        <v>95.45454545454545</v>
+        <v>100</v>
       </c>
       <c r="CU2" t="n">
         <v>95.45454545454545</v>
@@ -2121,10 +2121,10 @@
         <v>54.54545454545454</v>
       </c>
       <c r="CY2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.4582</v>
+        <v>9.286300000000001</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,52 +2133,52 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6307</v>
+        <v>0.6193</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3153</v>
+        <v>0.3093</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0946</v>
+        <v>0.0929</v>
       </c>
       <c r="DF2" t="n">
-        <v>2</v>
+        <v>2.0022</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.0822</v>
+        <v>1.0823</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0085</v>
+        <v>4.0043</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.7293</v>
+        <v>4.6434</v>
       </c>
       <c r="DJ2" t="n">
-        <v>35.45</v>
+        <v>39.07</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.7293</v>
+        <v>4.6434</v>
       </c>
       <c r="DL2" t="n">
         <v>1.9999</v>
       </c>
       <c r="DM2" t="n">
-        <v>2.0042</v>
+        <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>4.0085</v>
+        <v>4.0043</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0003</v>
+        <v>2.0023</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8475</v>
+        <v>0.863</v>
       </c>
       <c r="DQ2" t="n">
-        <v>93.83</v>
+        <v>95.19</v>
       </c>
       <c r="DR2" t="n">
-        <v>69.22</v>
+        <v>70.73</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2193,53 +2193,53 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.7796999999999999</v>
+        <v>0.9353</v>
       </c>
       <c r="DX2" t="n">
-        <v>95.95</v>
+        <v>83.72499999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>45</v>
+        <v>69.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>89.01900000000001</v>
+        <v>86.208</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
       </c>
       <c r="EB2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>92.65000000000001</v>
+        <v>75.41</v>
       </c>
       <c r="ED2" t="n">
-        <v>100</v>
+        <v>93.68000000000001</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.7796999999999999</v>
+        <v>0.9353</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.9</v>
+        <v>1.39</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.2105</v>
+        <v>0.2528</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0077</v>
+        <v>4.0027</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0241</v>
+        <v>0.0295</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6994</v>
+        <v>0.7097</v>
       </c>
       <c r="EK2" t="n">
-        <v>84.38</v>
+        <v>75.03</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
-          <t>Excellent</t>
+          <t>Strong</t>
         </is>
       </c>
       <c r="EM2" t="n">
@@ -2249,72 +2249,72 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>12.24</v>
+        <v>35.85</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.4003</v>
+        <v>4.1765</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.103</v>
+        <v>0.1619</v>
       </c>
       <c r="ER2" t="n">
-        <v>10.5111</v>
+        <v>6.6835</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.5506</v>
+        <v>11.7681</v>
       </c>
       <c r="ET2" t="n">
-        <v>36.975</v>
+        <v>46.511</v>
       </c>
       <c r="EU2" t="n">
-        <v>1.656</v>
+        <v>3.0163</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.2421</v>
+        <v>0.9707</v>
       </c>
       <c r="EW2" t="n">
-        <v>10.688</v>
+        <v>29.8881</v>
       </c>
       <c r="EX2" t="n">
-        <v>29.79</v>
+        <v>63</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Strong</t>
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="FA2" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>62.69</v>
+        <v>63.68</v>
       </c>
       <c r="FC2" t="n">
-        <v>25.62</v>
+        <v>26.86</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.3</v>
+        <v>72.23999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>85.84999999999999</v>
+        <v>79.2</v>
       </c>
       <c r="FF2" t="n">
-        <v>33.015</v>
+        <v>52.315</v>
       </c>
       <c r="FG2" t="n">
-        <v>25.9881</v>
+        <v>25.1114</v>
       </c>
       <c r="FH2" t="n">
-        <v>63.499</v>
+        <v>69.45099999999999</v>
       </c>
       <c r="FI2" t="n">
-        <v>52.335</v>
+        <v>54.9</v>
       </c>
       <c r="FJ2" t="n">
-        <v>68.18000000000001</v>
+        <v>70.14</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>77.23</v>
+        <v>81.12</v>
       </c>
       <c r="FO2" t="n">
-        <v>68.33</v>
+        <v>65.97</v>
       </c>
       <c r="FP2" t="n">
-        <v>59.6</v>
+        <v>86.15000000000001</v>
       </c>
       <c r="FQ2" t="n">
-        <v>76.41</v>
+        <v>76.86</v>
       </c>
       <c r="FR2" t="n">
-        <v>81.18000000000001</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="FS2" t="n">
-        <v>90.9091</v>
+        <v>100</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>69.9265</v>
+        <v>75.44799999999999</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261006_004724</t>
+          <t>20261006_155509</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46301.03291937124</v>
+        <v>46301.66330461224</v>
       </c>
     </row>
   </sheetData>
@@ -2466,7 +2466,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="19" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46301.03291666666</v>
+        <v>46301.66329861111</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46296</v>
+        <v>46301</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46311</v>
+        <v>46316</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.44</v>
+        <v>11.65</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,58 +2681,58 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>1984</v>
+        <v>2050</v>
       </c>
       <c r="L2" t="n">
-        <v>1973.6</v>
+        <v>1968.9</v>
       </c>
       <c r="M2" t="n">
-        <v>2006.9</v>
+        <v>2054.9</v>
       </c>
       <c r="N2" t="n">
-        <v>1952.1</v>
+        <v>1958</v>
       </c>
       <c r="O2" t="n">
-        <v>1984</v>
+        <v>2050</v>
       </c>
       <c r="P2" t="n">
-        <v>1459687</v>
+        <v>2196922</v>
       </c>
       <c r="Q2" t="n">
-        <v>1984</v>
+        <v>2050</v>
       </c>
       <c r="R2" t="n">
-        <v>2171.65</v>
+        <v>2240.37</v>
       </c>
       <c r="S2" t="n">
-        <v>1890.17</v>
+        <v>1954.81</v>
       </c>
       <c r="T2" t="n">
-        <v>9.458165322580649</v>
+        <v>9.286341463414628</v>
       </c>
       <c r="U2" t="n">
-        <v>187.6500000000001</v>
+        <v>190.3699999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.729334677419351</v>
+        <v>4.643414634146344</v>
       </c>
       <c r="W2" t="n">
-        <v>93.82999999999993</v>
+        <v>95.19000000000005</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999893424277952</v>
+        <v>1.999894946948207</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
       </c>
       <c r="Z2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AA2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="AB2" t="n">
-        <v>33.33333333333333</v>
+        <v>0</v>
       </c>
       <c r="AC2" t="n">
         <v>0</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.458165322580649</v>
+        <v>9.286341463414628</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.729334677419351</v>
+        <v>4.643414634146344</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02040055546603376</v>
+        <v>0.02042267491940029</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3238487782242284</v>
+        <v>0.3241999136606955</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02907952542506864</v>
+        <v>0.02906751079476494</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.0422866948954063</v>
+        <v>0.04228670014074916</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869492979645463</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.09</v>
+        <v>39.06</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-06 00:47:24.274513+05:30</t>
+          <t>2026-10-06 15:55:09.589655+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.45816532258065, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.999893424277952}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.286341463414628, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998949469482066}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-06 16:45 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>STRONG BUY</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -2088,19 +2088,19 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>83.37</v>
+        <v>83.29000000000001</v>
       </c>
       <c r="CO2" t="n">
-        <v>41.63</v>
+        <v>41.6</v>
       </c>
       <c r="CP2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CQ2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CR2" t="n">
-        <v>86.36363636363636</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="CS2" t="n">
         <v>100</v>
@@ -2109,16 +2109,16 @@
         <v>100</v>
       </c>
       <c r="CU2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CV2" t="n">
-        <v>86.36363636363636</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="CW2" t="n">
-        <v>68.18181818181817</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="CX2" t="n">
-        <v>54.54545454545454</v>
+        <v>57.14285714285714</v>
       </c>
       <c r="CY2" t="n">
         <v>1</v>
@@ -2154,7 +2154,7 @@
         <v>4.6434</v>
       </c>
       <c r="DJ2" t="n">
-        <v>39.07</v>
+        <v>39.09</v>
       </c>
       <c r="DK2" t="n">
         <v>4.6434</v>
@@ -2178,7 +2178,7 @@
         <v>95.19</v>
       </c>
       <c r="DR2" t="n">
-        <v>70.73</v>
+        <v>74.98</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2202,7 +2202,7 @@
         <v>69.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>86.208</v>
+        <v>86.333</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,10 +2211,10 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>75.41</v>
+        <v>75.31</v>
       </c>
       <c r="ED2" t="n">
-        <v>93.68000000000001</v>
+        <v>93.67</v>
       </c>
       <c r="EE2" t="n">
         <v>0.9353</v>
@@ -2235,7 +2235,7 @@
         <v>0.7097</v>
       </c>
       <c r="EK2" t="n">
-        <v>75.03</v>
+        <v>74.95</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,10 +2249,10 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>35.85</v>
+        <v>37.4</v>
       </c>
       <c r="EP2" t="n">
-        <v>4.1765</v>
+        <v>4.3571</v>
       </c>
       <c r="EQ2" t="n">
         <v>0.1619</v>
@@ -2261,10 +2261,10 @@
         <v>6.6835</v>
       </c>
       <c r="ES2" t="n">
-        <v>11.7681</v>
+        <v>11.7741</v>
       </c>
       <c r="ET2" t="n">
-        <v>46.511</v>
+        <v>46.877</v>
       </c>
       <c r="EU2" t="n">
         <v>3.0163</v>
@@ -2273,10 +2273,10 @@
         <v>0.9707</v>
       </c>
       <c r="EW2" t="n">
-        <v>29.8881</v>
+        <v>31.1505</v>
       </c>
       <c r="EX2" t="n">
-        <v>63</v>
+        <v>63.09</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2290,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.68</v>
+        <v>63.39</v>
       </c>
       <c r="FC2" t="n">
-        <v>26.86</v>
+        <v>26.83</v>
       </c>
       <c r="FD2" t="n">
-        <v>72.23999999999999</v>
+        <v>72.14</v>
       </c>
       <c r="FE2" t="n">
-        <v>79.2</v>
+        <v>79.12</v>
       </c>
       <c r="FF2" t="n">
-        <v>52.315</v>
+        <v>52.345</v>
       </c>
       <c r="FG2" t="n">
-        <v>25.1114</v>
+        <v>25.0873</v>
       </c>
       <c r="FH2" t="n">
-        <v>69.45099999999999</v>
+        <v>69.3</v>
       </c>
       <c r="FI2" t="n">
-        <v>54.9</v>
+        <v>57.035</v>
       </c>
       <c r="FJ2" t="n">
-        <v>70.14</v>
+        <v>69.95</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>81.12</v>
+        <v>81.04000000000001</v>
       </c>
       <c r="FO2" t="n">
-        <v>65.97</v>
+        <v>65.88</v>
       </c>
       <c r="FP2" t="n">
-        <v>86.15000000000001</v>
+        <v>86.02</v>
       </c>
       <c r="FQ2" t="n">
-        <v>76.86</v>
+        <v>76.83</v>
       </c>
       <c r="FR2" t="n">
-        <v>89.90000000000001</v>
+        <v>89.65000000000001</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>75.44799999999999</v>
+        <v>75.9255</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261006_155509</t>
+          <t>20261006_221541</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46301.66330461224</v>
+        <v>46301.92756253383</v>
       </c>
     </row>
   </sheetData>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46301.66329861111</v>
+        <v>46301.92755787037</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46301</v>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02042267491940029</v>
+        <v>0.02042267391435136</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3241999136606955</v>
+        <v>0.3241998977060384</v>
       </c>
     </row>
     <row r="7">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228670014074916</v>
+        <v>0.04228668955374454</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645463</v>
+        <v>0.1869492979645462</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-06 15:55:09.589655+05:30</t>
+          <t>2026-10-06 22:15:41.423194+05:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-07 10:20 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="19" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="17" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="H2" t="n">
         <v>8.800000000000001</v>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.65</v>
+        <v>11.58</v>
       </c>
       <c r="R2" t="n">
-        <v>49.22</v>
+        <v>49.06</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1968.9</v>
+        <v>2052</v>
       </c>
       <c r="V2" t="n">
-        <v>2054.9</v>
+        <v>2065.2</v>
       </c>
       <c r="W2" t="n">
-        <v>1958</v>
+        <v>2035.6</v>
       </c>
       <c r="X2" t="n">
-        <v>2050</v>
+        <v>2052.8</v>
       </c>
       <c r="Y2" t="n">
-        <v>2050</v>
+        <v>2052.8</v>
       </c>
       <c r="Z2" t="n">
-        <v>2196922</v>
+        <v>1499554</v>
       </c>
       <c r="AA2" t="n">
-        <v>1577002</v>
+        <v>1560888</v>
       </c>
       <c r="AB2" t="n">
-        <v>1.39</v>
+        <v>0.96</v>
       </c>
       <c r="AC2" t="n">
-        <v>3.99</v>
+        <v>0.14</v>
       </c>
       <c r="AD2" t="n">
-        <v>-0.13</v>
+        <v>0.1</v>
       </c>
       <c r="AE2" t="n">
-        <v>96.90000000000001</v>
+        <v>29.6</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.73</v>
+        <v>1.44</v>
       </c>
       <c r="AG2" t="n">
-        <v>47.59</v>
+        <v>46.31</v>
       </c>
       <c r="AH2" t="n">
-        <v>47.59</v>
+        <v>46.31</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.32</v>
+        <v>2.26</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>3.52</v>
+        <v>3.36</v>
       </c>
       <c r="AM2" t="n">
-        <v>7.89</v>
+        <v>7.73</v>
       </c>
       <c r="AN2" t="n">
-        <v>48.83</v>
+        <v>48.5</v>
       </c>
       <c r="AO2" t="n">
-        <v>66.51000000000001</v>
+        <v>66.81999999999999</v>
       </c>
       <c r="AP2" t="n">
-        <v>2.17</v>
+        <v>0.92</v>
       </c>
       <c r="AQ2" t="n">
-        <v>36</v>
+        <v>33.49</v>
       </c>
       <c r="AR2" t="n">
-        <v>2050</v>
+        <v>2052.8</v>
       </c>
       <c r="AS2" t="n">
-        <v>2240.37</v>
+        <v>2238.03</v>
       </c>
       <c r="AT2" t="n">
-        <v>1954.81</v>
+        <v>1960.18</v>
       </c>
       <c r="AU2" t="n">
-        <v>2050</v>
+        <v>2052.800048828125</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.289999999999999</v>
+        <v>9.02</v>
       </c>
       <c r="AY2" t="n">
-        <v>190.37</v>
+        <v>185.23</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.64</v>
+        <v>4.51</v>
       </c>
       <c r="BA2" t="n">
-        <v>95.19</v>
+        <v>92.62</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.03</v>
+        <v>2.04</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
@@ -1987,10 +1987,10 @@
         <v>49.3</v>
       </c>
       <c r="BG2" t="n">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.9</v>
+        <v>19</v>
       </c>
       <c r="BI2" t="n">
         <v>0</v>
@@ -2005,10 +2005,10 @@
         <v>0</v>
       </c>
       <c r="BM2" t="n">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="BN2" t="n">
-        <v>50.1</v>
+        <v>50</v>
       </c>
       <c r="BO2" t="n">
         <v>2.2</v>
@@ -2017,25 +2017,25 @@
         <v>8.630000000000001</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.25</v>
+        <v>-4.24</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.243</v>
+        <v>0.242</v>
       </c>
       <c r="BT2" t="n">
-        <v>1479.26</v>
+        <v>1479.65</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.68</v>
+        <v>-13.69</v>
       </c>
       <c r="BV2" t="n">
         <v>2.04</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.03</v>
+        <v>2.04</v>
       </c>
       <c r="BX2" t="n">
         <v>1.9999</v>
@@ -2047,7 +2047,7 @@
         <v>8</v>
       </c>
       <c r="CA2" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="CB2" t="n">
         <v>0</v>
@@ -2064,10 +2064,10 @@
         <v>52</v>
       </c>
       <c r="CF2" t="n">
-        <v>67.7</v>
+        <v>68</v>
       </c>
       <c r="CG2" t="n">
-        <v>71.59999999999999</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,19 +2088,19 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>83.29000000000001</v>
+        <v>83.38</v>
       </c>
       <c r="CO2" t="n">
-        <v>41.6</v>
+        <v>38.72</v>
       </c>
       <c r="CP2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CQ2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CR2" t="n">
-        <v>85.71428571428571</v>
+        <v>86.36363636363636</v>
       </c>
       <c r="CS2" t="n">
         <v>100</v>
@@ -2109,22 +2109,22 @@
         <v>100</v>
       </c>
       <c r="CU2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CV2" t="n">
-        <v>85.71428571428571</v>
+        <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>66.66666666666666</v>
+        <v>68.18181818181817</v>
       </c>
       <c r="CX2" t="n">
-        <v>57.14285714285714</v>
+        <v>54.54545454545454</v>
       </c>
       <c r="CY2" t="n">
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.286300000000001</v>
+        <v>9.023300000000001</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6193</v>
+        <v>0.6012999999999999</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3093</v>
+        <v>0.3007</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0929</v>
+        <v>0.0902</v>
       </c>
       <c r="DF2" t="n">
-        <v>2.0022</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.0823</v>
+        <v>1.0445</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0043</v>
+        <v>3.9912</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.6434</v>
+        <v>4.5119</v>
       </c>
       <c r="DJ2" t="n">
-        <v>39.09</v>
+        <v>29.55</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.6434</v>
+        <v>4.5119</v>
       </c>
       <c r="DL2" t="n">
         <v>1.9999</v>
       </c>
       <c r="DM2" t="n">
-        <v>2</v>
+        <v>1.9956</v>
       </c>
       <c r="DN2" t="n">
-        <v>4.0043</v>
+        <v>3.9912</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0023</v>
+        <v>1.9997</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.863</v>
+        <v>0.885</v>
       </c>
       <c r="DQ2" t="n">
-        <v>95.19</v>
+        <v>92.62</v>
       </c>
       <c r="DR2" t="n">
-        <v>74.98</v>
+        <v>50.42</v>
       </c>
       <c r="DS2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="DT2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.9353</v>
+        <v>0.4071</v>
       </c>
       <c r="DX2" t="n">
-        <v>83.72499999999999</v>
+        <v>82.95000000000002</v>
       </c>
       <c r="DY2" t="n">
-        <v>69.5</v>
+        <v>48</v>
       </c>
       <c r="DZ2" t="n">
-        <v>86.333</v>
+        <v>84.904</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>75.31</v>
+        <v>72.17</v>
       </c>
       <c r="ED2" t="n">
-        <v>93.67</v>
+        <v>90.27</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.9353</v>
+        <v>0.4071</v>
       </c>
       <c r="EF2" t="n">
-        <v>1.39</v>
+        <v>0.96</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.2528</v>
+        <v>0.1065</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0027</v>
+        <v>3.9926</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0295</v>
+        <v>0.0123</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7097</v>
+        <v>0.7246</v>
       </c>
       <c r="EK2" t="n">
-        <v>74.95</v>
+        <v>68.61</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,38 +2249,38 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>37.4</v>
+        <v>32.53</v>
       </c>
       <c r="EP2" t="n">
-        <v>4.3571</v>
+        <v>3.767</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.1619</v>
+        <v>0.1112</v>
       </c>
       <c r="ER2" t="n">
-        <v>6.6835</v>
+        <v>9.395799999999999</v>
       </c>
       <c r="ES2" t="n">
-        <v>11.7741</v>
+        <v>9.064399999999999</v>
       </c>
       <c r="ET2" t="n">
-        <v>46.877</v>
+        <v>44.252</v>
       </c>
       <c r="EU2" t="n">
-        <v>3.0163</v>
+        <v>0.8832</v>
       </c>
       <c r="EV2" t="n">
-        <v>0.9707</v>
+        <v>1.1531</v>
       </c>
       <c r="EW2" t="n">
-        <v>31.1505</v>
+        <v>27.1235</v>
       </c>
       <c r="EX2" t="n">
-        <v>63.09</v>
+        <v>58.72</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="EZ2" t="n">
@@ -2290,31 +2290,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.39</v>
+        <v>63.35</v>
       </c>
       <c r="FC2" t="n">
-        <v>26.83</v>
+        <v>20.46</v>
       </c>
       <c r="FD2" t="n">
-        <v>72.14</v>
+        <v>72.77</v>
       </c>
       <c r="FE2" t="n">
-        <v>79.12</v>
+        <v>75.995</v>
       </c>
       <c r="FF2" t="n">
-        <v>52.345</v>
+        <v>48.72</v>
       </c>
       <c r="FG2" t="n">
-        <v>25.0873</v>
+        <v>25.5767</v>
       </c>
       <c r="FH2" t="n">
-        <v>69.3</v>
+        <v>68.43300000000001</v>
       </c>
       <c r="FI2" t="n">
-        <v>57.035</v>
+        <v>39.985</v>
       </c>
       <c r="FJ2" t="n">
-        <v>69.95</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>81.04000000000001</v>
+        <v>73.06</v>
       </c>
       <c r="FO2" t="n">
-        <v>65.88</v>
+        <v>58.41</v>
       </c>
       <c r="FP2" t="n">
-        <v>86.02</v>
+        <v>74.27</v>
       </c>
       <c r="FQ2" t="n">
-        <v>76.83</v>
+        <v>69.83</v>
       </c>
       <c r="FR2" t="n">
-        <v>89.65000000000001</v>
+        <v>84.86</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>75.9255</v>
+        <v>67.6455</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261006_221541</t>
+          <t>20261007_155053</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46301.92756253383</v>
+        <v>46302.66034685935</v>
       </c>
     </row>
   </sheetData>
@@ -2464,7 +2464,7 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46301.92755787037</v>
+        <v>46302.66033564815</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.65</v>
+        <v>11.58</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>2050</v>
+        <v>2052.8</v>
       </c>
       <c r="L2" t="n">
-        <v>1968.9</v>
+        <v>2052</v>
       </c>
       <c r="M2" t="n">
-        <v>2054.9</v>
+        <v>2065.2</v>
       </c>
       <c r="N2" t="n">
-        <v>1958</v>
+        <v>2035.6</v>
       </c>
       <c r="O2" t="n">
-        <v>2050</v>
+        <v>2052.8</v>
       </c>
       <c r="P2" t="n">
-        <v>2196922</v>
+        <v>1499554</v>
       </c>
       <c r="Q2" t="n">
-        <v>2050</v>
+        <v>2052.8</v>
       </c>
       <c r="R2" t="n">
-        <v>2240.37</v>
+        <v>2238.03</v>
       </c>
       <c r="S2" t="n">
-        <v>1954.81</v>
+        <v>1960.18</v>
       </c>
       <c r="T2" t="n">
-        <v>9.286341463414628</v>
+        <v>9.023285268901013</v>
       </c>
       <c r="U2" t="n">
-        <v>190.3699999999999</v>
+        <v>185.23</v>
       </c>
       <c r="V2" t="n">
-        <v>4.643414634146344</v>
+        <v>4.51188620420889</v>
       </c>
       <c r="W2" t="n">
-        <v>95.19000000000005</v>
+        <v>92.62000000000012</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999894946948207</v>
+        <v>1.999892031958538</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.286341463414628</v>
+        <v>9.023285268901013</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.643414634146344</v>
+        <v>4.51188620420889</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02042267391435136</v>
+        <v>0.02040826084955815</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3241998977060384</v>
+        <v>0.3239710973955998</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02906751079476494</v>
+        <v>0.02906149636032406</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228668955374454</v>
+        <v>0.04228670115330902</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645462</v>
+        <v>0.1869492979645464</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.06</v>
+        <v>39.08</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-06 22:15:41.423194+05:30</t>
+          <t>2026-10-07 15:50:53.990994+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.286341463414628, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998949469482066}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.023285268901013, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998920319585378}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-07 17:24 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -2026,7 +2026,7 @@
         <v>0.242</v>
       </c>
       <c r="BT2" t="n">
-        <v>1479.65</v>
+        <v>1479.64</v>
       </c>
       <c r="BU2" t="n">
         <v>-13.69</v>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261007_155053</t>
+          <t>20261007_225449</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46302.66034685935</v>
+        <v>46302.95474260203</v>
       </c>
     </row>
   </sheetData>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46302.66033564815</v>
+        <v>46302.95473379629</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46302</v>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02040826084955815</v>
+        <v>0.02040825742936484</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3239710973955998</v>
+        <v>0.3239710431017142</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02906149636032406</v>
+        <v>0.02906138809988556</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228670115330902</v>
+        <v>0.04228669646808489</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869493934347617</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-07 15:50:53.990994+05:30</t>
+          <t>2026-10-07 22:54:49.782942+05:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-08 10:41 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="19" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="17" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="H2" t="n">
         <v>8.800000000000001</v>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.58</v>
+        <v>11.33</v>
       </c>
       <c r="R2" t="n">
-        <v>49.06</v>
+        <v>48.81</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>2052</v>
+        <v>2055</v>
       </c>
       <c r="V2" t="n">
-        <v>2065.2</v>
+        <v>2055</v>
       </c>
       <c r="W2" t="n">
-        <v>2035.6</v>
+        <v>1997.9</v>
       </c>
       <c r="X2" t="n">
-        <v>2052.8</v>
+        <v>1997.9</v>
       </c>
       <c r="Y2" t="n">
-        <v>2052.8</v>
+        <v>1997.9</v>
       </c>
       <c r="Z2" t="n">
-        <v>1499554</v>
+        <v>1393893</v>
       </c>
       <c r="AA2" t="n">
-        <v>1560888</v>
+        <v>1577224</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.96</v>
+        <v>0.88</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.14</v>
+        <v>-2.67</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="AE2" t="n">
-        <v>29.6</v>
+        <v>57.1</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.44</v>
+        <v>2.86</v>
       </c>
       <c r="AG2" t="n">
-        <v>46.31</v>
+        <v>47.08</v>
       </c>
       <c r="AH2" t="n">
-        <v>46.31</v>
+        <v>47.08</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.26</v>
+        <v>2.36</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,119 +1926,119 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>3.36</v>
+        <v>0.46</v>
       </c>
       <c r="AM2" t="n">
-        <v>7.73</v>
+        <v>4.61</v>
       </c>
       <c r="AN2" t="n">
-        <v>48.5</v>
+        <v>44.05</v>
       </c>
       <c r="AO2" t="n">
-        <v>66.81999999999999</v>
+        <v>55.78</v>
       </c>
       <c r="AP2" t="n">
-        <v>0.92</v>
+        <v>-1.4</v>
       </c>
       <c r="AQ2" t="n">
-        <v>33.49</v>
+        <v>28.19</v>
       </c>
       <c r="AR2" t="n">
-        <v>2052.8</v>
+        <v>1997.9</v>
       </c>
       <c r="AS2" t="n">
-        <v>2238.03</v>
+        <v>2186.22</v>
       </c>
       <c r="AT2" t="n">
-        <v>1960.18</v>
+        <v>1903.74</v>
       </c>
       <c r="AU2" t="n">
-        <v>2052.800048828125</v>
+        <v>1997.900024414062</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.02</v>
+        <v>9.43</v>
       </c>
       <c r="AY2" t="n">
-        <v>185.23</v>
+        <v>188.32</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.51</v>
+        <v>4.71</v>
       </c>
       <c r="BA2" t="n">
-        <v>92.62</v>
+        <v>94.16</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.04</v>
+        <v>2.06</v>
       </c>
       <c r="BC2" t="n">
         <v>214</v>
       </c>
       <c r="BD2" t="n">
-        <v>31.8</v>
+        <v>31.7</v>
       </c>
       <c r="BE2" t="n">
         <v>332</v>
       </c>
       <c r="BF2" t="n">
-        <v>49.3</v>
+        <v>49.2</v>
       </c>
       <c r="BG2" t="n">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="BH2" t="n">
-        <v>19</v>
+        <v>18.5</v>
       </c>
       <c r="BI2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="BM2" t="n">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="BN2" t="n">
-        <v>50</v>
+        <v>49.5</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.2</v>
+        <v>2.17</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.630000000000001</v>
+        <v>8.68</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.24</v>
+        <v>-4.21</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.242</v>
+        <v>0.239</v>
       </c>
       <c r="BT2" t="n">
-        <v>1479.64</v>
+        <v>1462.43</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.69</v>
+        <v>-14.2</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.04</v>
+        <v>2.02</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.04</v>
+        <v>2.06</v>
       </c>
       <c r="BX2" t="n">
-        <v>1.9999</v>
+        <v>2</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>44</v>
+        <v>43.4</v>
       </c>
       <c r="CE2" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="CF2" t="n">
-        <v>68</v>
+        <v>68.7</v>
       </c>
       <c r="CG2" t="n">
-        <v>71.40000000000001</v>
+        <v>70.7</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>83.38</v>
+        <v>82.53</v>
       </c>
       <c r="CO2" t="n">
-        <v>38.72</v>
+        <v>24.55</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2121,10 +2121,10 @@
         <v>54.54545454545454</v>
       </c>
       <c r="CY2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.023300000000001</v>
+        <v>9.4259</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6012999999999999</v>
+        <v>0.6287</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3007</v>
+        <v>0.314</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0902</v>
+        <v>0.09429999999999999</v>
       </c>
       <c r="DF2" t="n">
+        <v>2.0021</v>
+      </c>
+      <c r="DG2" t="n">
+        <v>1.0684</v>
+      </c>
+      <c r="DH2" t="n">
+        <v>3.9958</v>
+      </c>
+      <c r="DI2" t="n">
+        <v>4.7129</v>
+      </c>
+      <c r="DJ2" t="n">
+        <v>26.56</v>
+      </c>
+      <c r="DK2" t="n">
+        <v>4.7129</v>
+      </c>
+      <c r="DL2" t="n">
         <v>2</v>
       </c>
-      <c r="DG2" t="n">
-        <v>1.0445</v>
-      </c>
-      <c r="DH2" t="n">
-        <v>3.9912</v>
-      </c>
-      <c r="DI2" t="n">
-        <v>4.5119</v>
-      </c>
-      <c r="DJ2" t="n">
-        <v>29.55</v>
-      </c>
-      <c r="DK2" t="n">
-        <v>4.5119</v>
-      </c>
-      <c r="DL2" t="n">
-        <v>1.9999</v>
-      </c>
       <c r="DM2" t="n">
-        <v>1.9956</v>
+        <v>1.9958</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9912</v>
+        <v>3.9958</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9997</v>
+        <v>2.0022</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.885</v>
+        <v>0.8484</v>
       </c>
       <c r="DQ2" t="n">
-        <v>92.62</v>
+        <v>94.16</v>
       </c>
       <c r="DR2" t="n">
-        <v>50.42</v>
+        <v>79.28</v>
       </c>
       <c r="DS2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.4071</v>
+        <v>-0.5931999999999999</v>
       </c>
       <c r="DX2" t="n">
-        <v>82.95000000000002</v>
+        <v>89.45</v>
       </c>
       <c r="DY2" t="n">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="DZ2" t="n">
-        <v>84.904</v>
+        <v>81.794</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>72.17</v>
+        <v>70.19</v>
       </c>
       <c r="ED2" t="n">
-        <v>90.27</v>
+        <v>100</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.4071</v>
+        <v>-0.5931999999999999</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.96</v>
+        <v>0.88</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.1065</v>
+        <v>-0.1586</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9926</v>
+        <v>3.994</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0123</v>
+        <v>-0.018</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.7246</v>
+        <v>0.6995</v>
       </c>
       <c r="EK2" t="n">
-        <v>68.61</v>
+        <v>68.81999999999999</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,72 +2249,72 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>32.53</v>
+        <v>7.37</v>
       </c>
       <c r="EP2" t="n">
-        <v>3.767</v>
+        <v>0.835</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.1112</v>
+        <v>0.0997</v>
       </c>
       <c r="ER2" t="n">
-        <v>9.395799999999999</v>
+        <v>10.7159</v>
       </c>
       <c r="ES2" t="n">
-        <v>9.064399999999999</v>
+        <v>7.9048</v>
       </c>
       <c r="ET2" t="n">
-        <v>44.252</v>
+        <v>30.679</v>
       </c>
       <c r="EU2" t="n">
-        <v>0.8832</v>
+        <v>-1.232</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.1531</v>
+        <v>1.2553</v>
       </c>
       <c r="EW2" t="n">
-        <v>27.1235</v>
+        <v>6.0825</v>
       </c>
       <c r="EX2" t="n">
-        <v>58.72</v>
+        <v>31.45</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="EZ2" t="n">
+        <v>3</v>
+      </c>
+      <c r="FA2" t="n">
         <v>5</v>
       </c>
-      <c r="FA2" t="n">
-        <v>10</v>
-      </c>
       <c r="FB2" t="n">
-        <v>63.35</v>
+        <v>62.16</v>
       </c>
       <c r="FC2" t="n">
-        <v>20.46</v>
+        <v>18.16</v>
       </c>
       <c r="FD2" t="n">
-        <v>72.77</v>
+        <v>73.83</v>
       </c>
       <c r="FE2" t="n">
-        <v>75.995</v>
+        <v>75.675</v>
       </c>
       <c r="FF2" t="n">
-        <v>48.72</v>
+        <v>28</v>
       </c>
       <c r="FG2" t="n">
-        <v>25.5767</v>
+        <v>24.5625</v>
       </c>
       <c r="FH2" t="n">
-        <v>68.43300000000001</v>
+        <v>62.129</v>
       </c>
       <c r="FI2" t="n">
-        <v>39.985</v>
+        <v>52.92</v>
       </c>
       <c r="FJ2" t="n">
-        <v>66.09999999999999</v>
+        <v>65.23999999999999</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>73.06</v>
+        <v>75.04000000000001</v>
       </c>
       <c r="FO2" t="n">
-        <v>58.41</v>
+        <v>60.18</v>
       </c>
       <c r="FP2" t="n">
-        <v>74.27</v>
+        <v>60.4</v>
       </c>
       <c r="FQ2" t="n">
-        <v>69.83</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="FR2" t="n">
-        <v>84.86</v>
+        <v>83.27</v>
       </c>
       <c r="FS2" t="n">
-        <v>100</v>
+        <v>95.4545</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>67.6455</v>
+        <v>70.559</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261007_225449</t>
+          <t>20261008_161129</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46302.95474260203</v>
+        <v>46303.67464687106</v>
       </c>
     </row>
   </sheetData>
@@ -2464,7 +2464,7 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46302.95473379629</v>
+        <v>46303.6746412037</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.58</v>
+        <v>11.33</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>2052.8</v>
+        <v>1997.9</v>
       </c>
       <c r="L2" t="n">
-        <v>2052</v>
+        <v>2055</v>
       </c>
       <c r="M2" t="n">
-        <v>2065.2</v>
+        <v>2055</v>
       </c>
       <c r="N2" t="n">
-        <v>2035.6</v>
+        <v>1997.9</v>
       </c>
       <c r="O2" t="n">
-        <v>2052.8</v>
+        <v>1997.9</v>
       </c>
       <c r="P2" t="n">
-        <v>1499554</v>
+        <v>1393893</v>
       </c>
       <c r="Q2" t="n">
-        <v>2052.8</v>
+        <v>1997.9</v>
       </c>
       <c r="R2" t="n">
-        <v>2238.03</v>
+        <v>2186.22</v>
       </c>
       <c r="S2" t="n">
-        <v>1960.18</v>
+        <v>1903.74</v>
       </c>
       <c r="T2" t="n">
-        <v>9.023285268901013</v>
+        <v>9.425897192051639</v>
       </c>
       <c r="U2" t="n">
-        <v>185.23</v>
+        <v>188.3199999999997</v>
       </c>
       <c r="V2" t="n">
-        <v>4.51188620420889</v>
+        <v>4.712948596025831</v>
       </c>
       <c r="W2" t="n">
-        <v>92.62000000000012</v>
+        <v>94.16000000000008</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999892031958538</v>
+        <v>1.999999999999995</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.023285268901013</v>
+        <v>9.425897192051639</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.51188620420889</v>
+        <v>4.712948596025831</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2767,7 +2767,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02040825742936484</v>
+        <v>0.02040946862370053</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3239710431017142</v>
+        <v>0.3239902702157238</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02906138809988556</v>
+        <v>0.0290494295219009</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228669646808489</v>
+        <v>0.04228670255513612</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347617</v>
+        <v>0.1869492979645462</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-07 22:54:49.782942+05:30</t>
+          <t>2026-10-08 16:11:29.529707+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.023285268901013, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998920319585378}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.42589719205164, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9999999999999951}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-08 17:23 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -2026,7 +2026,7 @@
         <v>0.239</v>
       </c>
       <c r="BT2" t="n">
-        <v>1462.43</v>
+        <v>1462.42</v>
       </c>
       <c r="BU2" t="n">
         <v>-14.2</v>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261008_161129</t>
+          <t>20261008_225328</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46303.67464687106</v>
+        <v>46303.95380754121</v>
       </c>
     </row>
   </sheetData>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46303.6746412037</v>
+        <v>46303.95379629629</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46303</v>
@@ -2767,7 +2767,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02040946862370053</v>
+        <v>0.02040946744253115</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3239902702157238</v>
+        <v>0.3239902514652412</v>
       </c>
     </row>
     <row r="7">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228670255513612</v>
+        <v>0.04228669269848182</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645462</v>
+        <v>0.1869492979645464</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-08 16:11:29.529707+05:30</t>
+          <t>2026-10-08 22:53:29.009944+05:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-09 10:40 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="H2" t="n">
         <v>8.800000000000001</v>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.33</v>
+        <v>11.56</v>
       </c>
       <c r="R2" t="n">
-        <v>48.81</v>
+        <v>48.72</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>2055</v>
+        <v>1997.9</v>
       </c>
       <c r="V2" t="n">
-        <v>2055</v>
+        <v>2048</v>
       </c>
       <c r="W2" t="n">
-        <v>1997.9</v>
+        <v>1988.9</v>
       </c>
       <c r="X2" t="n">
-        <v>1997.9</v>
+        <v>2036.6</v>
       </c>
       <c r="Y2" t="n">
-        <v>1997.9</v>
+        <v>2036.6</v>
       </c>
       <c r="Z2" t="n">
-        <v>1393893</v>
+        <v>1358109</v>
       </c>
       <c r="AA2" t="n">
-        <v>1577224</v>
+        <v>1698526</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.88</v>
+        <v>0.8</v>
       </c>
       <c r="AC2" t="n">
-        <v>-2.67</v>
+        <v>1.94</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.11</v>
+        <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>57.1</v>
+        <v>59.1</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.86</v>
+        <v>2.9</v>
       </c>
       <c r="AG2" t="n">
-        <v>47.08</v>
+        <v>51.16</v>
       </c>
       <c r="AH2" t="n">
-        <v>47.08</v>
+        <v>51.16</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.36</v>
+        <v>2.51</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,116 +1926,116 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>0.46</v>
+        <v>2.34</v>
       </c>
       <c r="AM2" t="n">
-        <v>4.61</v>
+        <v>6.79</v>
       </c>
       <c r="AN2" t="n">
-        <v>44.05</v>
+        <v>47.72</v>
       </c>
       <c r="AO2" t="n">
-        <v>55.78</v>
+        <v>60.75</v>
       </c>
       <c r="AP2" t="n">
-        <v>-1.4</v>
+        <v>0.51</v>
       </c>
       <c r="AQ2" t="n">
-        <v>28.19</v>
+        <v>32.44</v>
       </c>
       <c r="AR2" t="n">
-        <v>1997.9</v>
+        <v>2036.6</v>
       </c>
       <c r="AS2" t="n">
-        <v>2186.22</v>
+        <v>2241.24</v>
       </c>
       <c r="AT2" t="n">
-        <v>1903.74</v>
+        <v>1934.28</v>
       </c>
       <c r="AU2" t="n">
-        <v>1997.900024414062</v>
+        <v>2036.599975585938</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.43</v>
+        <v>10.05</v>
       </c>
       <c r="AY2" t="n">
-        <v>188.32</v>
+        <v>204.64</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.71</v>
+        <v>5.02</v>
       </c>
       <c r="BA2" t="n">
-        <v>94.16</v>
+        <v>102.32</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.06</v>
+        <v>2.02</v>
       </c>
       <c r="BC2" t="n">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="BD2" t="n">
         <v>31.7</v>
       </c>
       <c r="BE2" t="n">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="BF2" t="n">
-        <v>49.2</v>
+        <v>49</v>
       </c>
       <c r="BG2" t="n">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.5</v>
+        <v>19.1</v>
       </c>
       <c r="BI2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.6</v>
+        <v>0.1</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="BM2" t="n">
-        <v>675</v>
+        <v>671</v>
       </c>
       <c r="BN2" t="n">
-        <v>49.5</v>
+        <v>50.1</v>
       </c>
       <c r="BO2" t="n">
         <v>2.17</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.68</v>
+        <v>8.59</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.21</v>
+        <v>-4.26</v>
       </c>
       <c r="BR2" t="n">
-        <v>9.1</v>
+        <v>9</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.239</v>
+        <v>0.241</v>
       </c>
       <c r="BT2" t="n">
-        <v>1462.42</v>
+        <v>1458.95</v>
       </c>
       <c r="BU2" t="n">
-        <v>-14.2</v>
+        <v>-13.38</v>
       </c>
       <c r="BV2" t="n">
         <v>2.02</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.06</v>
+        <v>2.02</v>
       </c>
       <c r="BX2" t="n">
         <v>2</v>
@@ -2047,7 +2047,7 @@
         <v>8</v>
       </c>
       <c r="CA2" t="n">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="CB2" t="n">
         <v>0</v>
@@ -2064,10 +2064,10 @@
         <v>51</v>
       </c>
       <c r="CF2" t="n">
-        <v>68.7</v>
+        <v>67.3</v>
       </c>
       <c r="CG2" t="n">
-        <v>70.7</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>82.53</v>
+        <v>87.18000000000001</v>
       </c>
       <c r="CO2" t="n">
-        <v>24.55</v>
+        <v>27.21</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2118,13 +2118,13 @@
         <v>68.18181818181817</v>
       </c>
       <c r="CX2" t="n">
-        <v>54.54545454545454</v>
+        <v>63.63636363636363</v>
       </c>
       <c r="CY2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.4259</v>
+        <v>10.0481</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,52 +2133,52 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6287</v>
+        <v>0.67</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.314</v>
+        <v>0.3347</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.09429999999999999</v>
+        <v>0.1005</v>
       </c>
       <c r="DF2" t="n">
-        <v>2.0021</v>
+        <v>2.002</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.0684</v>
+        <v>1.1618</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9958</v>
+        <v>4.004</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.7129</v>
+        <v>5.0241</v>
       </c>
       <c r="DJ2" t="n">
-        <v>26.56</v>
+        <v>28.49</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.7129</v>
+        <v>5.0241</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>1.9958</v>
+        <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9958</v>
+        <v>4.004</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0022</v>
+        <v>2.0018</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8484</v>
+        <v>0.7976</v>
       </c>
       <c r="DQ2" t="n">
-        <v>94.16</v>
+        <v>102.32</v>
       </c>
       <c r="DR2" t="n">
-        <v>79.28</v>
+        <v>58.02</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>-0.5931999999999999</v>
+        <v>0.2032</v>
       </c>
       <c r="DX2" t="n">
-        <v>89.45</v>
+        <v>98.125</v>
       </c>
       <c r="DY2" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="DZ2" t="n">
-        <v>81.794</v>
+        <v>84.018</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,35 +2211,35 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>70.19</v>
+        <v>74.59</v>
       </c>
       <c r="ED2" t="n">
         <v>100</v>
       </c>
       <c r="EE2" t="n">
-        <v>-0.5931999999999999</v>
+        <v>0.2032</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.88</v>
+        <v>0.8</v>
       </c>
       <c r="EG2" t="n">
-        <v>-0.1586</v>
+        <v>0.059</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.994</v>
+        <v>4.0032</v>
       </c>
       <c r="EI2" t="n">
-        <v>-0.018</v>
+        <v>0.0068</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6995</v>
+        <v>0.665</v>
       </c>
       <c r="EK2" t="n">
-        <v>68.81999999999999</v>
+        <v>81.05</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Excellent</t>
         </is>
       </c>
       <c r="EM2" t="n">
@@ -2249,72 +2249,72 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>7.37</v>
+        <v>16.41</v>
       </c>
       <c r="EP2" t="n">
-        <v>0.835</v>
+        <v>1.897</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0997</v>
+        <v>0.0925</v>
       </c>
       <c r="ER2" t="n">
-        <v>10.7159</v>
+        <v>12.5625</v>
       </c>
       <c r="ES2" t="n">
-        <v>7.9048</v>
+        <v>8.1168</v>
       </c>
       <c r="ET2" t="n">
-        <v>30.679</v>
+        <v>34.677</v>
       </c>
       <c r="EU2" t="n">
-        <v>-1.232</v>
+        <v>0.408</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.2553</v>
+        <v>1.3944</v>
       </c>
       <c r="EW2" t="n">
-        <v>6.0825</v>
+        <v>14.3062</v>
       </c>
       <c r="EX2" t="n">
-        <v>31.45</v>
+        <v>44.36</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="FA2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>62.16</v>
+        <v>62.9</v>
       </c>
       <c r="FC2" t="n">
-        <v>18.16</v>
+        <v>19.71</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.83</v>
+        <v>72.18000000000001</v>
       </c>
       <c r="FE2" t="n">
-        <v>75.675</v>
+        <v>84.11499999999999</v>
       </c>
       <c r="FF2" t="n">
-        <v>28</v>
+        <v>35.785</v>
       </c>
       <c r="FG2" t="n">
-        <v>24.5625</v>
+        <v>24.8376</v>
       </c>
       <c r="FH2" t="n">
-        <v>62.129</v>
+        <v>66.476</v>
       </c>
       <c r="FI2" t="n">
-        <v>52.92</v>
+        <v>43.255</v>
       </c>
       <c r="FJ2" t="n">
-        <v>65.23999999999999</v>
+        <v>66.81</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>75.04000000000001</v>
+        <v>76.41</v>
       </c>
       <c r="FO2" t="n">
-        <v>60.18</v>
+        <v>63.84</v>
       </c>
       <c r="FP2" t="n">
-        <v>60.4</v>
+        <v>67.23</v>
       </c>
       <c r="FQ2" t="n">
-        <v>76.90000000000001</v>
+        <v>72.78</v>
       </c>
       <c r="FR2" t="n">
-        <v>83.27</v>
+        <v>87.89</v>
       </c>
       <c r="FS2" t="n">
-        <v>95.4545</v>
+        <v>100</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>70.559</v>
+        <v>70.2835</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261008_225328</t>
+          <t>20261009_161005</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46303.95380754121</v>
+        <v>46304.67368008956</v>
       </c>
     </row>
   </sheetData>
@@ -2465,8 +2465,8 @@
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46303.95379629629</v>
+        <v>46304.67366898148</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.33</v>
+        <v>11.56</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
+        <v>2036.6</v>
+      </c>
+      <c r="L2" t="n">
         <v>1997.9</v>
       </c>
-      <c r="L2" t="n">
-        <v>2055</v>
-      </c>
       <c r="M2" t="n">
-        <v>2055</v>
+        <v>2048</v>
       </c>
       <c r="N2" t="n">
-        <v>1997.9</v>
+        <v>1988.9</v>
       </c>
       <c r="O2" t="n">
-        <v>1997.9</v>
+        <v>2036.6</v>
       </c>
       <c r="P2" t="n">
-        <v>1393893</v>
+        <v>1358109</v>
       </c>
       <c r="Q2" t="n">
-        <v>1997.9</v>
+        <v>2036.6</v>
       </c>
       <c r="R2" t="n">
-        <v>2186.22</v>
+        <v>2241.24</v>
       </c>
       <c r="S2" t="n">
-        <v>1903.74</v>
+        <v>1934.28</v>
       </c>
       <c r="T2" t="n">
-        <v>9.425897192051639</v>
+        <v>10.04811941471079</v>
       </c>
       <c r="U2" t="n">
-        <v>188.3199999999997</v>
+        <v>204.6399999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.712948596025831</v>
+        <v>5.024059707355393</v>
       </c>
       <c r="W2" t="n">
-        <v>94.16000000000008</v>
+        <v>102.3199999999999</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999999999999995</v>
+        <v>2</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.425897192051639</v>
+        <v>10.04811941471079</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.712948596025831</v>
+        <v>5.024059707355393</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02040946744253115</v>
+        <v>0.02046166485663698</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3239902514652412</v>
+        <v>0.3248188597260694</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.0290494295219009</v>
+        <v>0.02906748706380155</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228669269848182</v>
+        <v>0.04228670854841523</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869492979645462</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.08</v>
+        <v>39.01</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-08 22:53:29.009944+05:30</t>
+          <t>2026-10-09 16:10:05.996236+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.42589719205164, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9999999999999951}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.048119414710786, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-09 16:58 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -2026,7 +2026,7 @@
         <v>0.241</v>
       </c>
       <c r="BT2" t="n">
-        <v>1458.95</v>
+        <v>1458.96</v>
       </c>
       <c r="BU2" t="n">
         <v>-13.38</v>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261009_161005</t>
+          <t>20261009_222837</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46304.67368008956</v>
+        <v>46304.93654488589</v>
       </c>
     </row>
   </sheetData>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46304.67366898148</v>
+        <v>46304.93653935185</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46304</v>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02046166485663698</v>
+        <v>0.02046166109638705</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3248188597260694</v>
+        <v>0.3248188000339522</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02906748706380155</v>
+        <v>0.02906751079476494</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228670854841523</v>
+        <v>0.04228669594893958</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645462</v>
+        <v>0.1869492979645464</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-09 16:10:05.996236+05:30</t>
+          <t>2026-10-09 22:28:37.517889+05:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-12 10:57 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="20" customWidth="1" min="47" max="47"/>
+    <col width="19" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="17" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46304</v>
+        <v>46307</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46304</v>
+        <v>46307</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46304</v>
+        <v>46307</v>
       </c>
       <c r="H2" t="n">
         <v>8.800000000000001</v>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>STRONG BUY</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.56</v>
+        <v>11.65</v>
       </c>
       <c r="R2" t="n">
-        <v>48.72</v>
+        <v>48.85</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1997.9</v>
+        <v>2044.1</v>
       </c>
       <c r="V2" t="n">
-        <v>2048</v>
+        <v>2069.2</v>
       </c>
       <c r="W2" t="n">
-        <v>1988.9</v>
+        <v>2036.1</v>
       </c>
       <c r="X2" t="n">
-        <v>2036.6</v>
+        <v>2069.2</v>
       </c>
       <c r="Y2" t="n">
-        <v>2036.6</v>
+        <v>2069.2</v>
       </c>
       <c r="Z2" t="n">
-        <v>1358109</v>
+        <v>1416822</v>
       </c>
       <c r="AA2" t="n">
-        <v>1698526</v>
+        <v>1715994</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
       <c r="AC2" t="n">
-        <v>1.94</v>
+        <v>1.6</v>
       </c>
       <c r="AD2" t="n">
-        <v>0</v>
+        <v>0.37</v>
       </c>
       <c r="AE2" t="n">
-        <v>59.1</v>
+        <v>33.1</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.9</v>
+        <v>1.6</v>
       </c>
       <c r="AG2" t="n">
-        <v>51.16</v>
+        <v>49.87</v>
       </c>
       <c r="AH2" t="n">
-        <v>51.16</v>
+        <v>49.87</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.51</v>
+        <v>2.41</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>2.34</v>
+        <v>3.65</v>
       </c>
       <c r="AM2" t="n">
-        <v>6.79</v>
+        <v>8.17</v>
       </c>
       <c r="AN2" t="n">
-        <v>47.72</v>
+        <v>49.51</v>
       </c>
       <c r="AO2" t="n">
-        <v>60.75</v>
+        <v>64.17</v>
       </c>
       <c r="AP2" t="n">
-        <v>0.51</v>
+        <v>3.1</v>
       </c>
       <c r="AQ2" t="n">
-        <v>32.44</v>
+        <v>32.76</v>
       </c>
       <c r="AR2" t="n">
-        <v>2036.6</v>
+        <v>2069.2</v>
       </c>
       <c r="AS2" t="n">
-        <v>2241.24</v>
+        <v>2268.68</v>
       </c>
       <c r="AT2" t="n">
-        <v>1934.28</v>
+        <v>1969.46</v>
       </c>
       <c r="AU2" t="n">
-        <v>2036.599975585938</v>
+        <v>2069.199951171875</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>10.05</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="AY2" t="n">
-        <v>204.64</v>
+        <v>199.48</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.02</v>
+        <v>4.82</v>
       </c>
       <c r="BA2" t="n">
-        <v>102.32</v>
+        <v>99.73999999999999</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.02</v>
+        <v>2.01</v>
       </c>
       <c r="BC2" t="n">
         <v>213</v>
@@ -1987,55 +1987,55 @@
         <v>49</v>
       </c>
       <c r="BG2" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="BH2" t="n">
-        <v>19.1</v>
+        <v>19.3</v>
       </c>
       <c r="BI2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BM2" t="n">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="BN2" t="n">
-        <v>50.1</v>
+        <v>50.3</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.17</v>
+        <v>2.19</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.59</v>
+        <v>8.57</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.26</v>
+        <v>-4.27</v>
       </c>
       <c r="BR2" t="n">
         <v>9</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.241</v>
+        <v>0.242</v>
       </c>
       <c r="BT2" t="n">
-        <v>1458.96</v>
+        <v>1470.41</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.38</v>
+        <v>-13.15</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.02</v>
+        <v>2.03</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.02</v>
+        <v>2.01</v>
       </c>
       <c r="BX2" t="n">
         <v>2</v>
@@ -2047,7 +2047,7 @@
         <v>8</v>
       </c>
       <c r="CA2" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="CB2" t="n">
         <v>0</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>43.4</v>
+        <v>43.8</v>
       </c>
       <c r="CE2" t="n">
-        <v>51</v>
+        <v>51.5</v>
       </c>
       <c r="CF2" t="n">
-        <v>67.3</v>
+        <v>67</v>
       </c>
       <c r="CG2" t="n">
-        <v>71.59999999999999</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>87.18000000000001</v>
+        <v>96.23</v>
       </c>
       <c r="CO2" t="n">
-        <v>27.21</v>
+        <v>28.82</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2115,7 +2115,7 @@
         <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>68.18181818181817</v>
+        <v>72.72727272727273</v>
       </c>
       <c r="CX2" t="n">
         <v>63.63636363636363</v>
@@ -2124,7 +2124,7 @@
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>10.0481</v>
+        <v>9.6404</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,31 +2133,31 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.67</v>
+        <v>0.6427</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3347</v>
+        <v>0.3213</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1005</v>
+        <v>0.0964</v>
       </c>
       <c r="DF2" t="n">
-        <v>2.002</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1618</v>
+        <v>1.1231</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.004</v>
+        <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.0241</v>
+        <v>4.8202</v>
       </c>
       <c r="DJ2" t="n">
-        <v>28.49</v>
+        <v>25.24</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.0241</v>
+        <v>4.8202</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
@@ -2166,19 +2166,19 @@
         <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>4.004</v>
+        <v>4</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0018</v>
+        <v>2.0003</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.7976</v>
+        <v>0.8299</v>
       </c>
       <c r="DQ2" t="n">
-        <v>102.32</v>
+        <v>99.73999999999999</v>
       </c>
       <c r="DR2" t="n">
-        <v>58.02</v>
+        <v>54.84</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.2032</v>
+        <v>1.2863</v>
       </c>
       <c r="DX2" t="n">
-        <v>98.125</v>
+        <v>89.57499999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>40</v>
+        <v>41.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>84.018</v>
+        <v>89.149</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>74.59</v>
+        <v>89.56999999999999</v>
       </c>
       <c r="ED2" t="n">
-        <v>100</v>
+        <v>98.56999999999999</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.2032</v>
+        <v>1.2863</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.059</v>
+        <v>0.3612</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0032</v>
+        <v>4.0002</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0068</v>
+        <v>0.0421</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.665</v>
+        <v>0.6873</v>
       </c>
       <c r="EK2" t="n">
-        <v>81.05</v>
+        <v>89.83</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2249,34 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>16.41</v>
+        <v>22.78</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.897</v>
+        <v>2.6539</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0925</v>
+        <v>0.09669999999999999</v>
       </c>
       <c r="ER2" t="n">
-        <v>12.5625</v>
+        <v>11.6145</v>
       </c>
       <c r="ES2" t="n">
-        <v>8.1168</v>
+        <v>7.4018</v>
       </c>
       <c r="ET2" t="n">
-        <v>34.677</v>
+        <v>37.361</v>
       </c>
       <c r="EU2" t="n">
-        <v>0.408</v>
+        <v>2.573</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.3944</v>
+        <v>1.3169</v>
       </c>
       <c r="EW2" t="n">
-        <v>14.3062</v>
+        <v>21.9212</v>
       </c>
       <c r="EX2" t="n">
-        <v>44.36</v>
+        <v>44.23</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2290,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>62.9</v>
+        <v>63.33</v>
       </c>
       <c r="FC2" t="n">
-        <v>19.71</v>
+        <v>15.13</v>
       </c>
       <c r="FD2" t="n">
-        <v>72.18000000000001</v>
+        <v>71.65000000000001</v>
       </c>
       <c r="FE2" t="n">
-        <v>84.11499999999999</v>
+        <v>93.03</v>
       </c>
       <c r="FF2" t="n">
-        <v>35.785</v>
+        <v>36.525</v>
       </c>
       <c r="FG2" t="n">
-        <v>24.8376</v>
+        <v>28.2199</v>
       </c>
       <c r="FH2" t="n">
-        <v>66.476</v>
+        <v>69.38</v>
       </c>
       <c r="FI2" t="n">
-        <v>43.255</v>
+        <v>40.04</v>
       </c>
       <c r="FJ2" t="n">
-        <v>66.81</v>
+        <v>66.7</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>76.41</v>
+        <v>75.45999999999999</v>
       </c>
       <c r="FO2" t="n">
-        <v>63.84</v>
+        <v>65.22</v>
       </c>
       <c r="FP2" t="n">
-        <v>67.23</v>
+        <v>61.83</v>
       </c>
       <c r="FQ2" t="n">
-        <v>72.78</v>
+        <v>70.39</v>
       </c>
       <c r="FR2" t="n">
-        <v>87.89</v>
+        <v>83.56999999999999</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>70.2835</v>
+        <v>67.137</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261009_222837</t>
+          <t>20261012_162756</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46304.93654488589</v>
+        <v>46307.68606791035</v>
       </c>
     </row>
   </sheetData>
@@ -2465,8 +2465,8 @@
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="20" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="19" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46304.93653935185</v>
+        <v>46307.68606481481</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46304</v>
+        <v>46307</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.56</v>
+        <v>11.65</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>2036.6</v>
+        <v>2069.2</v>
       </c>
       <c r="L2" t="n">
-        <v>1997.9</v>
+        <v>2044.1</v>
       </c>
       <c r="M2" t="n">
-        <v>2048</v>
+        <v>2069.2</v>
       </c>
       <c r="N2" t="n">
-        <v>1988.9</v>
+        <v>2036.1</v>
       </c>
       <c r="O2" t="n">
-        <v>2036.6</v>
+        <v>2069.2</v>
       </c>
       <c r="P2" t="n">
-        <v>1358109</v>
+        <v>1416822</v>
       </c>
       <c r="Q2" t="n">
-        <v>2036.6</v>
+        <v>2069.2</v>
       </c>
       <c r="R2" t="n">
-        <v>2241.24</v>
+        <v>2268.68</v>
       </c>
       <c r="S2" t="n">
-        <v>1934.28</v>
+        <v>1969.46</v>
       </c>
       <c r="T2" t="n">
-        <v>10.04811941471079</v>
+        <v>9.640440750048329</v>
       </c>
       <c r="U2" t="n">
-        <v>204.6399999999999</v>
+        <v>199.48</v>
       </c>
       <c r="V2" t="n">
-        <v>5.024059707355393</v>
+        <v>4.820220375024153</v>
       </c>
       <c r="W2" t="n">
-        <v>102.3199999999999</v>
+        <v>99.73999999999978</v>
       </c>
       <c r="X2" t="n">
-        <v>2</v>
+        <v>2.000000000000004</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>10.04811941471079</v>
+        <v>9.640440750048329</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.024059707355393</v>
+        <v>4.820220375024153</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02046166109638705</v>
+        <v>0.0204533657525738</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3248188000339522</v>
+        <v>0.3246871155333343</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02906751079476494</v>
+        <v>0.02906146703335455</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228669594893958</v>
+        <v>0.04228670307940854</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.01</v>
+        <v>39.03</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-09 22:28:37.517889+05:30</t>
+          <t>2026-10-12 16:27:56.286821+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.048119414710786, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.64044075004833, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0000000000000044}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-12 19:47 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="19" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="17" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46307</v>
+        <v>46304</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46307</v>
+        <v>46304</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46307</v>
+        <v>46304</v>
       </c>
       <c r="H2" t="n">
         <v>8.800000000000001</v>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.65</v>
+        <v>11.56</v>
       </c>
       <c r="R2" t="n">
-        <v>48.85</v>
+        <v>48.72</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>2044.1</v>
+        <v>1997.9</v>
       </c>
       <c r="V2" t="n">
-        <v>2069.2</v>
+        <v>2048</v>
       </c>
       <c r="W2" t="n">
-        <v>2036.1</v>
+        <v>1988.9</v>
       </c>
       <c r="X2" t="n">
-        <v>2069.2</v>
+        <v>2036.6</v>
       </c>
       <c r="Y2" t="n">
-        <v>2069.2</v>
+        <v>2036.6</v>
       </c>
       <c r="Z2" t="n">
-        <v>1416822</v>
+        <v>1358268</v>
       </c>
       <c r="AA2" t="n">
-        <v>1715994</v>
+        <v>1698534</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.83</v>
+        <v>0.8</v>
       </c>
       <c r="AC2" t="n">
-        <v>1.6</v>
+        <v>1.94</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.37</v>
+        <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>33.1</v>
+        <v>59.1</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.6</v>
+        <v>2.9</v>
       </c>
       <c r="AG2" t="n">
-        <v>49.87</v>
+        <v>51.16</v>
       </c>
       <c r="AH2" t="n">
-        <v>49.87</v>
+        <v>51.16</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.41</v>
+        <v>2.51</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>3.65</v>
+        <v>2.34</v>
       </c>
       <c r="AM2" t="n">
-        <v>8.17</v>
+        <v>6.79</v>
       </c>
       <c r="AN2" t="n">
-        <v>49.51</v>
+        <v>47.72</v>
       </c>
       <c r="AO2" t="n">
-        <v>64.17</v>
+        <v>60.75</v>
       </c>
       <c r="AP2" t="n">
-        <v>3.1</v>
+        <v>0.51</v>
       </c>
       <c r="AQ2" t="n">
-        <v>32.76</v>
+        <v>32.44</v>
       </c>
       <c r="AR2" t="n">
-        <v>2069.2</v>
+        <v>2036.6</v>
       </c>
       <c r="AS2" t="n">
-        <v>2268.68</v>
+        <v>2241.24</v>
       </c>
       <c r="AT2" t="n">
-        <v>1969.46</v>
+        <v>1934.28</v>
       </c>
       <c r="AU2" t="n">
-        <v>2069.199951171875</v>
+        <v>2036.599975585938</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.640000000000001</v>
+        <v>10.05</v>
       </c>
       <c r="AY2" t="n">
-        <v>199.48</v>
+        <v>204.64</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.82</v>
+        <v>5.02</v>
       </c>
       <c r="BA2" t="n">
-        <v>99.73999999999999</v>
+        <v>102.32</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.01</v>
+        <v>2.02</v>
       </c>
       <c r="BC2" t="n">
         <v>213</v>
@@ -1987,55 +1987,55 @@
         <v>49</v>
       </c>
       <c r="BG2" t="n">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="BH2" t="n">
-        <v>19.3</v>
+        <v>19.1</v>
       </c>
       <c r="BI2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BM2" t="n">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="BN2" t="n">
-        <v>50.3</v>
+        <v>50.1</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.19</v>
+        <v>2.17</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.57</v>
+        <v>8.59</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.27</v>
+        <v>-4.26</v>
       </c>
       <c r="BR2" t="n">
         <v>9</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.242</v>
+        <v>0.241</v>
       </c>
       <c r="BT2" t="n">
-        <v>1470.41</v>
+        <v>1458.94</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.15</v>
+        <v>-13.38</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.03</v>
+        <v>2.02</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.01</v>
+        <v>2.02</v>
       </c>
       <c r="BX2" t="n">
         <v>2</v>
@@ -2047,7 +2047,7 @@
         <v>8</v>
       </c>
       <c r="CA2" t="n">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="CB2" t="n">
         <v>0</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>43.8</v>
+        <v>43.4</v>
       </c>
       <c r="CE2" t="n">
-        <v>51.5</v>
+        <v>51</v>
       </c>
       <c r="CF2" t="n">
-        <v>67</v>
+        <v>67.3</v>
       </c>
       <c r="CG2" t="n">
-        <v>71.90000000000001</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>96.23</v>
+        <v>87.18000000000001</v>
       </c>
       <c r="CO2" t="n">
-        <v>28.82</v>
+        <v>27.21</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2115,7 +2115,7 @@
         <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>72.72727272727273</v>
+        <v>68.18181818181817</v>
       </c>
       <c r="CX2" t="n">
         <v>63.63636363636363</v>
@@ -2124,7 +2124,7 @@
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.6404</v>
+        <v>10.0481</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,31 +2133,31 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6427</v>
+        <v>0.67</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3213</v>
+        <v>0.3347</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0964</v>
+        <v>0.1005</v>
       </c>
       <c r="DF2" t="n">
-        <v>2</v>
+        <v>2.002</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1231</v>
+        <v>1.1618</v>
       </c>
       <c r="DH2" t="n">
-        <v>4</v>
+        <v>4.004</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.8202</v>
+        <v>5.0241</v>
       </c>
       <c r="DJ2" t="n">
-        <v>25.24</v>
+        <v>28.49</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.8202</v>
+        <v>5.0241</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
@@ -2166,19 +2166,19 @@
         <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>4</v>
+        <v>4.004</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0003</v>
+        <v>2.0018</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8299</v>
+        <v>0.7976</v>
       </c>
       <c r="DQ2" t="n">
-        <v>99.73999999999999</v>
+        <v>102.32</v>
       </c>
       <c r="DR2" t="n">
-        <v>54.84</v>
+        <v>58.02</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.2863</v>
+        <v>0.2032</v>
       </c>
       <c r="DX2" t="n">
-        <v>89.57499999999999</v>
+        <v>98.125</v>
       </c>
       <c r="DY2" t="n">
-        <v>41.5</v>
+        <v>40</v>
       </c>
       <c r="DZ2" t="n">
-        <v>89.149</v>
+        <v>84.018</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>89.56999999999999</v>
+        <v>74.59</v>
       </c>
       <c r="ED2" t="n">
-        <v>98.56999999999999</v>
+        <v>100</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.2863</v>
+        <v>0.2032</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.83</v>
+        <v>0.8</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.3612</v>
+        <v>0.059</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0002</v>
+        <v>4.0032</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0421</v>
+        <v>0.0068</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6873</v>
+        <v>0.665</v>
       </c>
       <c r="EK2" t="n">
-        <v>89.83</v>
+        <v>81.05</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2249,34 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>22.78</v>
+        <v>16.41</v>
       </c>
       <c r="EP2" t="n">
-        <v>2.6539</v>
+        <v>1.897</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.09669999999999999</v>
+        <v>0.0925</v>
       </c>
       <c r="ER2" t="n">
-        <v>11.6145</v>
+        <v>12.5625</v>
       </c>
       <c r="ES2" t="n">
-        <v>7.4018</v>
+        <v>8.1168</v>
       </c>
       <c r="ET2" t="n">
-        <v>37.361</v>
+        <v>34.677</v>
       </c>
       <c r="EU2" t="n">
-        <v>2.573</v>
+        <v>0.408</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.3169</v>
+        <v>1.3944</v>
       </c>
       <c r="EW2" t="n">
-        <v>21.9212</v>
+        <v>14.3062</v>
       </c>
       <c r="EX2" t="n">
-        <v>44.23</v>
+        <v>44.36</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2290,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.33</v>
+        <v>62.9</v>
       </c>
       <c r="FC2" t="n">
-        <v>15.13</v>
+        <v>19.71</v>
       </c>
       <c r="FD2" t="n">
-        <v>71.65000000000001</v>
+        <v>72.18000000000001</v>
       </c>
       <c r="FE2" t="n">
-        <v>93.03</v>
+        <v>84.11499999999999</v>
       </c>
       <c r="FF2" t="n">
-        <v>36.525</v>
+        <v>35.785</v>
       </c>
       <c r="FG2" t="n">
-        <v>28.2199</v>
+        <v>24.8376</v>
       </c>
       <c r="FH2" t="n">
-        <v>69.38</v>
+        <v>66.476</v>
       </c>
       <c r="FI2" t="n">
-        <v>40.04</v>
+        <v>43.255</v>
       </c>
       <c r="FJ2" t="n">
-        <v>66.7</v>
+        <v>66.81</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>75.45999999999999</v>
+        <v>76.41</v>
       </c>
       <c r="FO2" t="n">
-        <v>65.22</v>
+        <v>63.84</v>
       </c>
       <c r="FP2" t="n">
-        <v>61.83</v>
+        <v>67.23</v>
       </c>
       <c r="FQ2" t="n">
-        <v>70.39</v>
+        <v>72.78</v>
       </c>
       <c r="FR2" t="n">
-        <v>83.56999999999999</v>
+        <v>87.89</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>67.137</v>
+        <v>70.2835</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261012_162756</t>
+          <t>20261013_011725</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46307.68606791035</v>
+        <v>46308.05376659927</v>
       </c>
     </row>
   </sheetData>
@@ -2465,8 +2465,8 @@
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46307.68606481481</v>
+        <v>46308.05376157408</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46307</v>
+        <v>46304</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46322</v>
+        <v>46319</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.65</v>
+        <v>11.56</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,58 +2681,58 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>2069.2</v>
+        <v>2036.6</v>
       </c>
       <c r="L2" t="n">
-        <v>2044.1</v>
+        <v>1997.9</v>
       </c>
       <c r="M2" t="n">
-        <v>2069.2</v>
+        <v>2048</v>
       </c>
       <c r="N2" t="n">
-        <v>2036.1</v>
+        <v>1988.9</v>
       </c>
       <c r="O2" t="n">
-        <v>2069.2</v>
+        <v>2036.6</v>
       </c>
       <c r="P2" t="n">
-        <v>1416822</v>
+        <v>1358268</v>
       </c>
       <c r="Q2" t="n">
-        <v>2069.2</v>
+        <v>2036.6</v>
       </c>
       <c r="R2" t="n">
-        <v>2268.68</v>
+        <v>2241.24</v>
       </c>
       <c r="S2" t="n">
-        <v>1969.46</v>
+        <v>1934.28</v>
       </c>
       <c r="T2" t="n">
-        <v>9.640440750048329</v>
+        <v>10.04811941471079</v>
       </c>
       <c r="U2" t="n">
-        <v>199.48</v>
+        <v>204.6399999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.820220375024153</v>
+        <v>5.024059707355393</v>
       </c>
       <c r="W2" t="n">
-        <v>99.73999999999978</v>
+        <v>102.3199999999999</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000000000000004</v>
+        <v>2</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
       </c>
       <c r="Z2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AA2" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="AB2" t="n">
-        <v>0</v>
+        <v>26.66666666666667</v>
       </c>
       <c r="AC2" t="n">
         <v>0</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.640440750048329</v>
+        <v>10.04811941471079</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.820220375024153</v>
+        <v>5.024059707355393</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0204533657525738</v>
+        <v>0.0204616615097953</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3246871155333343</v>
+        <v>0.3248188065966047</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02906146703335455</v>
+        <v>0.02906748635562367</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228670307940854</v>
+        <v>0.04228670527526088</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869493934347617</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.03</v>
+        <v>39.01</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-12 16:27:56.286821+05:30</t>
+          <t>2026-10-13 01:17:25.472792+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.64044075004833, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0000000000000044}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.048119414710786, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-13 10:42 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="20" customWidth="1" min="47" max="47"/>
+    <col width="18" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="H2" t="n">
         <v>8.800000000000001</v>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>STRONG BUY</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1861,7 +1861,7 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.56</v>
+        <v>11.65</v>
       </c>
       <c r="R2" t="n">
         <v>48.72</v>
@@ -1875,46 +1875,46 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>1997.9</v>
+        <v>2047.1</v>
       </c>
       <c r="V2" t="n">
-        <v>2048</v>
+        <v>2065</v>
       </c>
       <c r="W2" t="n">
-        <v>1988.9</v>
+        <v>2007.8</v>
       </c>
       <c r="X2" t="n">
-        <v>2036.6</v>
+        <v>2059.4</v>
       </c>
       <c r="Y2" t="n">
-        <v>2036.6</v>
+        <v>2059.4</v>
       </c>
       <c r="Z2" t="n">
-        <v>1358268</v>
+        <v>1140915</v>
       </c>
       <c r="AA2" t="n">
-        <v>1698534</v>
+        <v>1702199</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.8</v>
+        <v>0.67</v>
       </c>
       <c r="AC2" t="n">
-        <v>1.94</v>
+        <v>1.12</v>
       </c>
       <c r="AD2" t="n">
-        <v>0</v>
+        <v>0.52</v>
       </c>
       <c r="AE2" t="n">
-        <v>59.1</v>
+        <v>57.2</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.9</v>
+        <v>2.78</v>
       </c>
       <c r="AG2" t="n">
-        <v>51.16</v>
+        <v>51.59</v>
       </c>
       <c r="AH2" t="n">
-        <v>51.16</v>
+        <v>51.59</v>
       </c>
       <c r="AI2" t="n">
         <v>2.51</v>
@@ -1926,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>2.34</v>
+        <v>3.19</v>
       </c>
       <c r="AM2" t="n">
-        <v>6.79</v>
+        <v>7.67</v>
       </c>
       <c r="AN2" t="n">
-        <v>47.72</v>
+        <v>48.81</v>
       </c>
       <c r="AO2" t="n">
-        <v>60.75</v>
+        <v>63.21</v>
       </c>
       <c r="AP2" t="n">
-        <v>0.51</v>
+        <v>2.61</v>
       </c>
       <c r="AQ2" t="n">
-        <v>32.44</v>
+        <v>32.13</v>
       </c>
       <c r="AR2" t="n">
-        <v>2036.6</v>
+        <v>2059.4</v>
       </c>
       <c r="AS2" t="n">
-        <v>2241.24</v>
+        <v>2265.76</v>
       </c>
       <c r="AT2" t="n">
-        <v>1934.28</v>
+        <v>1956.22</v>
       </c>
       <c r="AU2" t="n">
-        <v>2036.599975585938</v>
+        <v>2059.39990234375</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>10.05</v>
+        <v>10.02</v>
       </c>
       <c r="AY2" t="n">
-        <v>204.64</v>
+        <v>206.36</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.02</v>
+        <v>5.01</v>
       </c>
       <c r="BA2" t="n">
-        <v>102.32</v>
+        <v>103.18</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.02</v>
+        <v>2</v>
       </c>
       <c r="BC2" t="n">
         <v>213</v>
@@ -1987,55 +1987,55 @@
         <v>49</v>
       </c>
       <c r="BG2" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="BH2" t="n">
-        <v>19.1</v>
+        <v>19.3</v>
       </c>
       <c r="BI2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BM2" t="n">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="BN2" t="n">
-        <v>50.1</v>
+        <v>50.3</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.17</v>
+        <v>2.18</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.59</v>
+        <v>8.56</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.26</v>
+        <v>-4.27</v>
       </c>
       <c r="BR2" t="n">
         <v>9</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.241</v>
+        <v>0.242</v>
       </c>
       <c r="BT2" t="n">
-        <v>1458.94</v>
+        <v>1466.77</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.38</v>
+        <v>-13.24</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.02</v>
+        <v>2.03</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.02</v>
+        <v>2</v>
       </c>
       <c r="BX2" t="n">
         <v>2</v>
@@ -2047,7 +2047,7 @@
         <v>8</v>
       </c>
       <c r="CA2" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="CB2" t="n">
         <v>0</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>43.4</v>
+        <v>43.6</v>
       </c>
       <c r="CE2" t="n">
-        <v>51</v>
+        <v>51.5</v>
       </c>
       <c r="CF2" t="n">
-        <v>67.3</v>
+        <v>66.7</v>
       </c>
       <c r="CG2" t="n">
-        <v>71.59999999999999</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>87.18000000000001</v>
+        <v>81.11</v>
       </c>
       <c r="CO2" t="n">
-        <v>27.21</v>
+        <v>34.13</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2115,16 +2115,16 @@
         <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>68.18181818181817</v>
+        <v>72.72727272727273</v>
       </c>
       <c r="CX2" t="n">
         <v>63.63636363636363</v>
       </c>
       <c r="CY2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>10.0481</v>
+        <v>10.0204</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,52 +2133,52 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.67</v>
+        <v>0.668</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3347</v>
+        <v>0.334</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1005</v>
+        <v>0.1002</v>
       </c>
       <c r="DF2" t="n">
-        <v>2.002</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1618</v>
+        <v>1.1673</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.004</v>
+        <v>3.992</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.0241</v>
+        <v>5.0102</v>
       </c>
       <c r="DJ2" t="n">
-        <v>28.49</v>
+        <v>31.06</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.0241</v>
+        <v>5.0102</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
       </c>
       <c r="DM2" t="n">
+        <v>1.996</v>
+      </c>
+      <c r="DN2" t="n">
+        <v>3.992</v>
+      </c>
+      <c r="DO2" t="n">
         <v>2</v>
       </c>
-      <c r="DN2" t="n">
-        <v>4.004</v>
-      </c>
-      <c r="DO2" t="n">
-        <v>2.0018</v>
-      </c>
       <c r="DP2" t="n">
-        <v>0.7976</v>
+        <v>0.7968</v>
       </c>
       <c r="DQ2" t="n">
-        <v>102.32</v>
+        <v>103.18</v>
       </c>
       <c r="DR2" t="n">
-        <v>58.02</v>
+        <v>51.61</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.2032</v>
+        <v>1.0398</v>
       </c>
       <c r="DX2" t="n">
-        <v>98.125</v>
+        <v>91.97499999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>40</v>
+        <v>33.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>84.018</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,35 +2211,35 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>74.59</v>
+        <v>81.31999999999999</v>
       </c>
       <c r="ED2" t="n">
-        <v>100</v>
+        <v>98.58</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.2032</v>
+        <v>1.0398</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.8</v>
+        <v>0.67</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.059</v>
+        <v>0.3041</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0032</v>
+        <v>3.9922</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0068</v>
+        <v>0.0354</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.665</v>
+        <v>0.6643</v>
       </c>
       <c r="EK2" t="n">
-        <v>81.05</v>
+        <v>79.52</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
-          <t>Excellent</t>
+          <t>Strong</t>
         </is>
       </c>
       <c r="EM2" t="n">
@@ -2249,34 +2249,34 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>16.41</v>
+        <v>5.04</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.897</v>
+        <v>0.5872000000000001</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0925</v>
+        <v>0.0781</v>
       </c>
       <c r="ER2" t="n">
-        <v>12.5625</v>
+        <v>14.9552</v>
       </c>
       <c r="ES2" t="n">
-        <v>8.1168</v>
+        <v>8.849</v>
       </c>
       <c r="ET2" t="n">
-        <v>34.677</v>
+        <v>34.163</v>
       </c>
       <c r="EU2" t="n">
-        <v>0.408</v>
+        <v>1.7487</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.3944</v>
+        <v>1.503</v>
       </c>
       <c r="EW2" t="n">
-        <v>14.3062</v>
+        <v>4.0879</v>
       </c>
       <c r="EX2" t="n">
-        <v>44.36</v>
+        <v>42.2</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2284,37 +2284,37 @@
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="FA2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="FB2" t="n">
-        <v>62.9</v>
+        <v>63.33</v>
       </c>
       <c r="FC2" t="n">
-        <v>19.71</v>
+        <v>20.65</v>
       </c>
       <c r="FD2" t="n">
-        <v>72.18000000000001</v>
+        <v>71.13</v>
       </c>
       <c r="FE2" t="n">
-        <v>84.11499999999999</v>
+        <v>80.315</v>
       </c>
       <c r="FF2" t="n">
-        <v>35.785</v>
+        <v>38.165</v>
       </c>
       <c r="FG2" t="n">
-        <v>24.8376</v>
+        <v>23.1083</v>
       </c>
       <c r="FH2" t="n">
-        <v>66.476</v>
+        <v>64.438</v>
       </c>
       <c r="FI2" t="n">
-        <v>43.255</v>
+        <v>41.335</v>
       </c>
       <c r="FJ2" t="n">
-        <v>66.81</v>
+        <v>66.7</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>76.41</v>
+        <v>73.03</v>
       </c>
       <c r="FO2" t="n">
-        <v>63.84</v>
+        <v>64.91</v>
       </c>
       <c r="FP2" t="n">
-        <v>67.23</v>
+        <v>58.88</v>
       </c>
       <c r="FQ2" t="n">
-        <v>72.78</v>
+        <v>68.8</v>
       </c>
       <c r="FR2" t="n">
-        <v>87.89</v>
+        <v>81.68000000000001</v>
       </c>
       <c r="FS2" t="n">
-        <v>100</v>
+        <v>95.4545</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>70.2835</v>
+        <v>66.5805</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261013_011725</t>
+          <t>20261013_161201</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46308.05376659927</v>
+        <v>46308.67502042748</v>
       </c>
     </row>
   </sheetData>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46308.05376157408</v>
+        <v>46308.67501157407</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46319</v>
+        <v>46323</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.56</v>
+        <v>11.65</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,43 +2681,43 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>2036.6</v>
+        <v>2059.4</v>
       </c>
       <c r="L2" t="n">
-        <v>1997.9</v>
+        <v>2047.1</v>
       </c>
       <c r="M2" t="n">
-        <v>2048</v>
+        <v>2065</v>
       </c>
       <c r="N2" t="n">
-        <v>1988.9</v>
+        <v>2007.8</v>
       </c>
       <c r="O2" t="n">
-        <v>2036.6</v>
+        <v>2059.4</v>
       </c>
       <c r="P2" t="n">
-        <v>1358268</v>
+        <v>1140915</v>
       </c>
       <c r="Q2" t="n">
-        <v>2036.6</v>
+        <v>2059.4</v>
       </c>
       <c r="R2" t="n">
-        <v>2241.24</v>
+        <v>2265.76</v>
       </c>
       <c r="S2" t="n">
-        <v>1934.28</v>
+        <v>1956.22</v>
       </c>
       <c r="T2" t="n">
-        <v>10.04811941471079</v>
+        <v>10.02039428959892</v>
       </c>
       <c r="U2" t="n">
-        <v>204.6399999999999</v>
+        <v>206.3600000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>5.024059707355393</v>
+        <v>5.010197144799458</v>
       </c>
       <c r="W2" t="n">
-        <v>102.3199999999999</v>
+        <v>103.1800000000001</v>
       </c>
       <c r="X2" t="n">
         <v>2</v>
@@ -2726,13 +2726,13 @@
         <v>15</v>
       </c>
       <c r="Z2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AA2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="AB2" t="n">
-        <v>26.66666666666667</v>
+        <v>0</v>
       </c>
       <c r="AC2" t="n">
         <v>0</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>10.04811941471079</v>
+        <v>10.02039428959892</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.024059707355393</v>
+        <v>5.010197144799458</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0204616615097953</v>
+        <v>0.02044971194770667</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3248188065966047</v>
+        <v>0.3246291131792289</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02906748635562367</v>
+        <v>0.02906146703335455</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228670527526088</v>
+        <v>0.04228670340767787</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347617</v>
+        <v>0.1869493934347615</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.01</v>
+        <v>39.03</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-13 01:17:25.472792+05:30</t>
+          <t>2026-10-13 16:12:01.784351+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.048119414710786, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.020394289598917, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-13 17:34 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -2026,7 +2026,7 @@
         <v>0.242</v>
       </c>
       <c r="BT2" t="n">
-        <v>1466.77</v>
+        <v>1466.78</v>
       </c>
       <c r="BU2" t="n">
         <v>-13.24</v>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261013_161201</t>
+          <t>20261013_230436</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46308.67502042748</v>
+        <v>46308.96153171048</v>
       </c>
     </row>
   </sheetData>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46308.67501157407</v>
+        <v>46308.96152777778</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46308</v>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02044971194770667</v>
+        <v>0.02044971010222153</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3246291131792289</v>
+        <v>0.3246290838830605</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02906146703335455</v>
+        <v>0.02906149636032406</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228670340767787</v>
+        <v>0.04228669780900114</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347615</v>
+        <v>0.1869492979645464</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-13 16:12:01.784351+05:30</t>
+          <t>2026-10-13 23:04:36.379636+05:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-14 08:47 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="18" customWidth="1" min="47" max="47"/>
+    <col width="19" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="H2" t="n">
         <v>8.800000000000001</v>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.65</v>
+        <v>11.32</v>
       </c>
       <c r="R2" t="n">
-        <v>48.72</v>
+        <v>48.6</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>2047.1</v>
+        <v>2049</v>
       </c>
       <c r="V2" t="n">
-        <v>2065</v>
+        <v>2057.3</v>
       </c>
       <c r="W2" t="n">
-        <v>2007.8</v>
+        <v>2021.2</v>
       </c>
       <c r="X2" t="n">
-        <v>2059.4</v>
+        <v>2027.2</v>
       </c>
       <c r="Y2" t="n">
-        <v>2059.4</v>
+        <v>2027.2</v>
       </c>
       <c r="Z2" t="n">
-        <v>1140915</v>
+        <v>1017383</v>
       </c>
       <c r="AA2" t="n">
-        <v>1702199</v>
+        <v>1633163</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.67</v>
+        <v>0.62</v>
       </c>
       <c r="AC2" t="n">
-        <v>1.12</v>
+        <v>-1.56</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.52</v>
+        <v>-0.5</v>
       </c>
       <c r="AE2" t="n">
-        <v>57.2</v>
+        <v>36.1</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.78</v>
+        <v>1.78</v>
       </c>
       <c r="AG2" t="n">
-        <v>51.59</v>
+        <v>49.8</v>
       </c>
       <c r="AH2" t="n">
-        <v>51.59</v>
+        <v>49.8</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.51</v>
+        <v>2.46</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,116 +1926,116 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>3.19</v>
+        <v>1.06</v>
       </c>
       <c r="AM2" t="n">
-        <v>7.67</v>
+        <v>5.47</v>
       </c>
       <c r="AN2" t="n">
-        <v>48.81</v>
+        <v>45.44</v>
       </c>
       <c r="AO2" t="n">
-        <v>63.21</v>
+        <v>56.89</v>
       </c>
       <c r="AP2" t="n">
-        <v>2.61</v>
+        <v>2.44</v>
       </c>
       <c r="AQ2" t="n">
-        <v>32.13</v>
+        <v>30.43</v>
       </c>
       <c r="AR2" t="n">
-        <v>2059.4</v>
+        <v>2027.2</v>
       </c>
       <c r="AS2" t="n">
-        <v>2265.76</v>
+        <v>2226.4</v>
       </c>
       <c r="AT2" t="n">
-        <v>1956.22</v>
+        <v>1927.6</v>
       </c>
       <c r="AU2" t="n">
-        <v>2059.39990234375</v>
+        <v>2027.199951171875</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>10.02</v>
+        <v>9.83</v>
       </c>
       <c r="AY2" t="n">
-        <v>206.36</v>
+        <v>199.2</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.01</v>
+        <v>4.91</v>
       </c>
       <c r="BA2" t="n">
-        <v>103.18</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="BB2" t="n">
-        <v>2</v>
+        <v>2.04</v>
       </c>
       <c r="BC2" t="n">
         <v>213</v>
       </c>
       <c r="BD2" t="n">
-        <v>31.7</v>
+        <v>31.6</v>
       </c>
       <c r="BE2" t="n">
         <v>329</v>
       </c>
       <c r="BF2" t="n">
-        <v>49</v>
+        <v>48.8</v>
       </c>
       <c r="BG2" t="n">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="BH2" t="n">
-        <v>19.3</v>
+        <v>19</v>
       </c>
       <c r="BI2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="BM2" t="n">
-        <v>672</v>
+        <v>674</v>
       </c>
       <c r="BN2" t="n">
-        <v>50.3</v>
+        <v>49.7</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.18</v>
+        <v>2.15</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.56</v>
+        <v>8.609999999999999</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.27</v>
+        <v>-4.22</v>
       </c>
       <c r="BR2" t="n">
         <v>9</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.242</v>
+        <v>0.238</v>
       </c>
       <c r="BT2" t="n">
-        <v>1466.78</v>
+        <v>1452.38</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.24</v>
+        <v>-13.53</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.03</v>
+        <v>2.02</v>
       </c>
       <c r="BW2" t="n">
-        <v>2</v>
+        <v>2.04</v>
       </c>
       <c r="BX2" t="n">
         <v>2</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>43.6</v>
+        <v>43</v>
       </c>
       <c r="CE2" t="n">
-        <v>51.5</v>
+        <v>51</v>
       </c>
       <c r="CF2" t="n">
-        <v>66.7</v>
+        <v>68</v>
       </c>
       <c r="CG2" t="n">
-        <v>71.90000000000001</v>
+        <v>71</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>81.11</v>
+        <v>73.20999999999999</v>
       </c>
       <c r="CO2" t="n">
-        <v>34.13</v>
+        <v>34.49</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2115,16 +2115,16 @@
         <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>72.72727272727273</v>
+        <v>68.18181818181817</v>
       </c>
       <c r="CX2" t="n">
         <v>63.63636363636363</v>
       </c>
       <c r="CY2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="CZ2" t="n">
-        <v>10.0204</v>
+        <v>9.8264</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,52 +2133,52 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.668</v>
+        <v>0.6553</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.334</v>
+        <v>0.3273</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1002</v>
+        <v>0.0983</v>
       </c>
       <c r="DF2" t="n">
-        <v>2</v>
+        <v>2.002</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1673</v>
+        <v>1.1128</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.992</v>
+        <v>3.9959</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.0102</v>
+        <v>4.9132</v>
       </c>
       <c r="DJ2" t="n">
-        <v>31.06</v>
+        <v>29.58</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.0102</v>
+        <v>4.9132</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>1.996</v>
+        <v>1.9959</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.992</v>
+        <v>3.9959</v>
       </c>
       <c r="DO2" t="n">
-        <v>2</v>
+        <v>2.0021</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.7968</v>
+        <v>0.8138</v>
       </c>
       <c r="DQ2" t="n">
-        <v>103.18</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="DR2" t="n">
-        <v>51.61</v>
+        <v>61.5</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.0398</v>
+        <v>0.9919</v>
       </c>
       <c r="DX2" t="n">
-        <v>91.97499999999999</v>
+        <v>92.22499999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>33.5</v>
+        <v>31</v>
       </c>
       <c r="DZ2" t="n">
-        <v>84.90000000000001</v>
+        <v>76.712</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>81.31999999999999</v>
+        <v>60.94</v>
       </c>
       <c r="ED2" t="n">
-        <v>98.58</v>
+        <v>96.22</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.0398</v>
+        <v>0.9919</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.67</v>
+        <v>0.62</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.3041</v>
+        <v>0.2762</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9922</v>
+        <v>3.9945</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0354</v>
+        <v>0.0313</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6643</v>
+        <v>0.6758999999999999</v>
       </c>
       <c r="EK2" t="n">
-        <v>79.52</v>
+        <v>67.79000000000001</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2246,41 +2246,41 @@
         <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>5.04</v>
+        <v>12.28</v>
       </c>
       <c r="EP2" t="n">
-        <v>0.5872000000000001</v>
+        <v>1.3901</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0781</v>
+        <v>0.0702</v>
       </c>
       <c r="ER2" t="n">
-        <v>14.9552</v>
+        <v>15.8548</v>
       </c>
       <c r="ES2" t="n">
-        <v>8.849</v>
+        <v>8.549099999999999</v>
       </c>
       <c r="ET2" t="n">
-        <v>34.163</v>
+        <v>36.011</v>
       </c>
       <c r="EU2" t="n">
-        <v>1.7487</v>
+        <v>1.5128</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.503</v>
+        <v>1.5185</v>
       </c>
       <c r="EW2" t="n">
-        <v>4.0879</v>
+        <v>8.9902</v>
       </c>
       <c r="EX2" t="n">
-        <v>42.2</v>
+        <v>37.34</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="EZ2" t="n">
@@ -2290,31 +2290,31 @@
         <v>8</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.33</v>
+        <v>61.77</v>
       </c>
       <c r="FC2" t="n">
-        <v>20.65</v>
+        <v>19.7</v>
       </c>
       <c r="FD2" t="n">
-        <v>71.13</v>
+        <v>73.23999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>80.315</v>
+        <v>70.5</v>
       </c>
       <c r="FF2" t="n">
-        <v>38.165</v>
+        <v>35.915</v>
       </c>
       <c r="FG2" t="n">
-        <v>23.1083</v>
+        <v>21.159</v>
       </c>
       <c r="FH2" t="n">
-        <v>64.438</v>
+        <v>60.316</v>
       </c>
       <c r="FI2" t="n">
-        <v>41.335</v>
+        <v>45.54</v>
       </c>
       <c r="FJ2" t="n">
-        <v>66.7</v>
+        <v>63.08</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>73.03</v>
+        <v>69.84999999999999</v>
       </c>
       <c r="FO2" t="n">
-        <v>64.91</v>
+        <v>53.94</v>
       </c>
       <c r="FP2" t="n">
-        <v>58.88</v>
+        <v>64.45</v>
       </c>
       <c r="FQ2" t="n">
-        <v>68.8</v>
+        <v>72.27</v>
       </c>
       <c r="FR2" t="n">
-        <v>81.68000000000001</v>
+        <v>82.38</v>
       </c>
       <c r="FS2" t="n">
-        <v>95.4545</v>
+        <v>90.9091</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>66.5805</v>
+        <v>67.468</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261013_230436</t>
+          <t>20261014_141757</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46308.96153171048</v>
+        <v>46309.595806736</v>
       </c>
     </row>
   </sheetData>
@@ -2464,9 +2464,9 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="20" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46308.96152777778</v>
+        <v>46309.59579861111</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.65</v>
+        <v>11.32</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>2059.4</v>
+        <v>2027.2</v>
       </c>
       <c r="L2" t="n">
-        <v>2047.1</v>
+        <v>2049</v>
       </c>
       <c r="M2" t="n">
-        <v>2065</v>
+        <v>2057.3</v>
       </c>
       <c r="N2" t="n">
-        <v>2007.8</v>
+        <v>2021.2</v>
       </c>
       <c r="O2" t="n">
-        <v>2059.4</v>
+        <v>2027.2</v>
       </c>
       <c r="P2" t="n">
-        <v>1140915</v>
+        <v>1017383</v>
       </c>
       <c r="Q2" t="n">
-        <v>2059.4</v>
+        <v>2027.2</v>
       </c>
       <c r="R2" t="n">
-        <v>2265.76</v>
+        <v>2226.4</v>
       </c>
       <c r="S2" t="n">
-        <v>1956.22</v>
+        <v>1927.6</v>
       </c>
       <c r="T2" t="n">
-        <v>10.02039428959892</v>
+        <v>9.826361483820049</v>
       </c>
       <c r="U2" t="n">
-        <v>206.3600000000001</v>
+        <v>199.2</v>
       </c>
       <c r="V2" t="n">
-        <v>5.010197144799458</v>
+        <v>4.91318074191003</v>
       </c>
       <c r="W2" t="n">
-        <v>103.1800000000001</v>
+        <v>99.60000000000014</v>
       </c>
       <c r="X2" t="n">
-        <v>2</v>
+        <v>1.999999999999998</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>10.02039428959892</v>
+        <v>9.826361483820049</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.010197144799458</v>
+        <v>4.91318074191003</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02044971010222153</v>
+        <v>0.02043784535893707</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3246290838830605</v>
+        <v>0.3244407369224587</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02906149636032406</v>
+        <v>0.02904936073155717</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228669780900114</v>
+        <v>0.0422867080737743</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.03</v>
+        <v>39.04</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-13 23:04:36.379636+05:30</t>
+          <t>2026-10-14 14:17:57.725245+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.020394289598917, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.82636148382005, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9999999999999978}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-14 15:04 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="19" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.32</v>
+        <v>11.42</v>
       </c>
       <c r="R2" t="n">
-        <v>48.6</v>
+        <v>48.7</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1881,43 +1881,43 @@
         <v>2057.3</v>
       </c>
       <c r="W2" t="n">
-        <v>2021.2</v>
+        <v>2019.2</v>
       </c>
       <c r="X2" t="n">
-        <v>2027.2</v>
+        <v>2036.9</v>
       </c>
       <c r="Y2" t="n">
-        <v>2027.2</v>
+        <v>2036.9</v>
       </c>
       <c r="Z2" t="n">
-        <v>1017383</v>
+        <v>1300927</v>
       </c>
       <c r="AA2" t="n">
-        <v>1633163</v>
+        <v>1647340</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.62</v>
+        <v>0.79</v>
       </c>
       <c r="AC2" t="n">
-        <v>-1.56</v>
+        <v>-1.09</v>
       </c>
       <c r="AD2" t="n">
         <v>-0.5</v>
       </c>
       <c r="AE2" t="n">
-        <v>36.1</v>
+        <v>38.1</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.78</v>
+        <v>1.87</v>
       </c>
       <c r="AG2" t="n">
-        <v>49.8</v>
+        <v>49.94</v>
       </c>
       <c r="AH2" t="n">
-        <v>49.8</v>
+        <v>49.94</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.46</v>
+        <v>2.45</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>1.06</v>
+        <v>1.52</v>
       </c>
       <c r="AM2" t="n">
-        <v>5.47</v>
+        <v>5.96</v>
       </c>
       <c r="AN2" t="n">
-        <v>45.44</v>
+        <v>46.13</v>
       </c>
       <c r="AO2" t="n">
-        <v>56.89</v>
+        <v>58.45</v>
       </c>
       <c r="AP2" t="n">
-        <v>2.44</v>
+        <v>2.93</v>
       </c>
       <c r="AQ2" t="n">
-        <v>30.43</v>
+        <v>31.05</v>
       </c>
       <c r="AR2" t="n">
-        <v>2027.2</v>
+        <v>2036.9</v>
       </c>
       <c r="AS2" t="n">
-        <v>2226.4</v>
+        <v>2236.67</v>
       </c>
       <c r="AT2" t="n">
-        <v>1927.6</v>
+        <v>1937.01</v>
       </c>
       <c r="AU2" t="n">
-        <v>2027.199951171875</v>
+        <v>2036.900024414062</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.83</v>
+        <v>9.81</v>
       </c>
       <c r="AY2" t="n">
-        <v>199.2</v>
+        <v>199.77</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.91</v>
+        <v>4.9</v>
       </c>
       <c r="BA2" t="n">
-        <v>99.59999999999999</v>
+        <v>99.89</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.04</v>
+        <v>2.03</v>
       </c>
       <c r="BC2" t="n">
         <v>213</v>
@@ -2008,37 +2008,37 @@
         <v>674</v>
       </c>
       <c r="BN2" t="n">
-        <v>49.7</v>
+        <v>49.9</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.15</v>
+        <v>2.16</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.609999999999999</v>
+        <v>8.59</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.22</v>
+        <v>-4.23</v>
       </c>
       <c r="BR2" t="n">
         <v>9</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.238</v>
+        <v>0.239</v>
       </c>
       <c r="BT2" t="n">
-        <v>1452.38</v>
+        <v>1457.02</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.53</v>
+        <v>-13.44</v>
       </c>
       <c r="BV2" t="n">
         <v>2.02</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.04</v>
+        <v>2.03</v>
       </c>
       <c r="BX2" t="n">
-        <v>2</v>
+        <v>1.9999</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>43</v>
+        <v>43.2</v>
       </c>
       <c r="CE2" t="n">
         <v>51</v>
       </c>
       <c r="CF2" t="n">
-        <v>68</v>
+        <v>67.7</v>
       </c>
       <c r="CG2" t="n">
-        <v>71</v>
+        <v>71.3</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>73.20999999999999</v>
+        <v>72.31</v>
       </c>
       <c r="CO2" t="n">
-        <v>34.49</v>
+        <v>31.53</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2124,7 +2124,7 @@
         <v>3</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.8264</v>
+        <v>9.807600000000001</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,52 +2133,52 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6553</v>
+        <v>0.654</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3273</v>
+        <v>0.3267</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0983</v>
+        <v>0.09810000000000001</v>
       </c>
       <c r="DF2" t="n">
         <v>2.002</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1128</v>
+        <v>1.1203</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9959</v>
+        <v>4.0041</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.9132</v>
+        <v>4.904</v>
       </c>
       <c r="DJ2" t="n">
-        <v>29.58</v>
+        <v>29.72</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.9132</v>
+        <v>4.904</v>
       </c>
       <c r="DL2" t="n">
+        <v>1.9999</v>
+      </c>
+      <c r="DM2" t="n">
         <v>2</v>
       </c>
-      <c r="DM2" t="n">
-        <v>1.9959</v>
-      </c>
       <c r="DN2" t="n">
-        <v>3.9959</v>
+        <v>4.0041</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0021</v>
+        <v>2.0018</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8138</v>
+        <v>0.8172</v>
       </c>
       <c r="DQ2" t="n">
-        <v>99.59999999999999</v>
+        <v>99.89</v>
       </c>
       <c r="DR2" t="n">
-        <v>61.5</v>
+        <v>59.74</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.9919</v>
+        <v>1.1959</v>
       </c>
       <c r="DX2" t="n">
-        <v>92.22499999999999</v>
+        <v>96.125</v>
       </c>
       <c r="DY2" t="n">
-        <v>31</v>
+        <v>39.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>76.712</v>
+        <v>74.73399999999999</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>60.94</v>
+        <v>56.76</v>
       </c>
       <c r="ED2" t="n">
-        <v>96.22</v>
+        <v>100</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.9919</v>
+        <v>1.1959</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.62</v>
+        <v>0.79</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.2762</v>
+        <v>0.3346</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9945</v>
+        <v>4.0031</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0313</v>
+        <v>0.0382</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6758999999999999</v>
+        <v>0.6785</v>
       </c>
       <c r="EK2" t="n">
-        <v>67.79000000000001</v>
+        <v>70.06</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2249,34 @@
         <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>12.28</v>
+        <v>11.12</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.3901</v>
+        <v>1.2699</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0702</v>
+        <v>0.0902</v>
       </c>
       <c r="ER2" t="n">
-        <v>15.8548</v>
+        <v>12.4177</v>
       </c>
       <c r="ES2" t="n">
-        <v>8.549099999999999</v>
+        <v>8.6145</v>
       </c>
       <c r="ET2" t="n">
-        <v>36.011</v>
+        <v>34.62</v>
       </c>
       <c r="EU2" t="n">
-        <v>1.5128</v>
+        <v>2.3147</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.5185</v>
+        <v>1.3687</v>
       </c>
       <c r="EW2" t="n">
-        <v>8.9902</v>
+        <v>8.040900000000001</v>
       </c>
       <c r="EX2" t="n">
-        <v>37.34</v>
+        <v>36.08</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2290,31 @@
         <v>8</v>
       </c>
       <c r="FB2" t="n">
-        <v>61.77</v>
+        <v>62.24</v>
       </c>
       <c r="FC2" t="n">
-        <v>19.7</v>
+        <v>19.8</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.23999999999999</v>
+        <v>72.70999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>70.5</v>
+        <v>71.185</v>
       </c>
       <c r="FF2" t="n">
-        <v>35.915</v>
+        <v>33.805</v>
       </c>
       <c r="FG2" t="n">
-        <v>21.159</v>
+        <v>20.9594</v>
       </c>
       <c r="FH2" t="n">
-        <v>60.316</v>
+        <v>60.029</v>
       </c>
       <c r="FI2" t="n">
-        <v>45.54</v>
+        <v>44.73</v>
       </c>
       <c r="FJ2" t="n">
-        <v>63.08</v>
+        <v>62.42</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>69.84999999999999</v>
+        <v>69.43000000000001</v>
       </c>
       <c r="FO2" t="n">
-        <v>53.94</v>
+        <v>54.23</v>
       </c>
       <c r="FP2" t="n">
-        <v>64.45</v>
+        <v>63</v>
       </c>
       <c r="FQ2" t="n">
-        <v>72.27</v>
+        <v>71.55</v>
       </c>
       <c r="FR2" t="n">
-        <v>82.38</v>
+        <v>79.31</v>
       </c>
       <c r="FS2" t="n">
         <v>90.9091</v>
@@ -2353,11 +2353,11 @@
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>67.468</v>
+        <v>65.55800000000001</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261014_141757</t>
+          <t>20261014_203451</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46309.595806736</v>
+        <v>46309.85753952918</v>
       </c>
     </row>
   </sheetData>
@@ -2464,8 +2464,8 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
-    <col width="19" customWidth="1" min="23" max="23"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46309.59579861111</v>
+        <v>46309.85753472222</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46309</v>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.32</v>
+        <v>11.42</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>2027.2</v>
+        <v>2036.9</v>
       </c>
       <c r="L2" t="n">
         <v>2049</v>
@@ -2690,37 +2690,37 @@
         <v>2057.3</v>
       </c>
       <c r="N2" t="n">
-        <v>2021.2</v>
+        <v>2019.2</v>
       </c>
       <c r="O2" t="n">
-        <v>2027.2</v>
+        <v>2036.9</v>
       </c>
       <c r="P2" t="n">
-        <v>1017383</v>
+        <v>1300927</v>
       </c>
       <c r="Q2" t="n">
-        <v>2027.2</v>
+        <v>2036.9</v>
       </c>
       <c r="R2" t="n">
-        <v>2226.4</v>
+        <v>2236.67</v>
       </c>
       <c r="S2" t="n">
-        <v>1927.6</v>
+        <v>1937.01</v>
       </c>
       <c r="T2" t="n">
-        <v>9.826361483820049</v>
+        <v>9.807550689773674</v>
       </c>
       <c r="U2" t="n">
-        <v>199.2</v>
+        <v>199.77</v>
       </c>
       <c r="V2" t="n">
-        <v>4.91318074191003</v>
+        <v>4.904020815945804</v>
       </c>
       <c r="W2" t="n">
-        <v>99.60000000000014</v>
+        <v>99.8900000000001</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999999999999998</v>
+        <v>1.999899889878864</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.826361483820049</v>
+        <v>9.807550689773674</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.91318074191003</v>
+        <v>4.904020815945804</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02043784535893707</v>
+        <v>0.02043267390781192</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3244407369224587</v>
+        <v>0.3243586426808918</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02904936073155717</v>
+        <v>0.0290494283888163</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.0422867080737743</v>
+        <v>0.04228671062017354</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869493934347614</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.04</v>
+        <v>39.05</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-14 14:17:57.725245+05:30</t>
+          <t>2026-10-14 20:34:51.456887+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.82636148382005, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9999999999999978}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.807550689773674, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998998898788645}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-15 08:23 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="20" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="17" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="H2" t="n">
         <v>8.800000000000001</v>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.42</v>
+        <v>11.3</v>
       </c>
       <c r="R2" t="n">
-        <v>48.7</v>
+        <v>48.53</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>2049</v>
+        <v>2025</v>
       </c>
       <c r="V2" t="n">
-        <v>2057.3</v>
+        <v>2046.3</v>
       </c>
       <c r="W2" t="n">
-        <v>2019.2</v>
+        <v>2008</v>
       </c>
       <c r="X2" t="n">
-        <v>2036.9</v>
+        <v>2028</v>
       </c>
       <c r="Y2" t="n">
-        <v>2036.9</v>
+        <v>2028</v>
       </c>
       <c r="Z2" t="n">
-        <v>1300927</v>
+        <v>606348</v>
       </c>
       <c r="AA2" t="n">
-        <v>1647340</v>
+        <v>1534093</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.79</v>
+        <v>0.4</v>
       </c>
       <c r="AC2" t="n">
-        <v>-1.09</v>
+        <v>-0.44</v>
       </c>
       <c r="AD2" t="n">
-        <v>-0.5</v>
+        <v>-0.58</v>
       </c>
       <c r="AE2" t="n">
-        <v>38.1</v>
+        <v>38.3</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.87</v>
+        <v>1.89</v>
       </c>
       <c r="AG2" t="n">
-        <v>49.94</v>
+        <v>49.11</v>
       </c>
       <c r="AH2" t="n">
-        <v>49.94</v>
+        <v>49.11</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.45</v>
+        <v>2.42</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>1.52</v>
+        <v>0.77</v>
       </c>
       <c r="AM2" t="n">
-        <v>5.96</v>
+        <v>5.31</v>
       </c>
       <c r="AN2" t="n">
-        <v>46.13</v>
+        <v>44.99</v>
       </c>
       <c r="AO2" t="n">
-        <v>58.45</v>
+        <v>56.91</v>
       </c>
       <c r="AP2" t="n">
-        <v>2.93</v>
+        <v>2.42</v>
       </c>
       <c r="AQ2" t="n">
-        <v>31.05</v>
+        <v>30.2</v>
       </c>
       <c r="AR2" t="n">
-        <v>2036.9</v>
+        <v>2028</v>
       </c>
       <c r="AS2" t="n">
-        <v>2236.67</v>
+        <v>2224.45</v>
       </c>
       <c r="AT2" t="n">
-        <v>1937.01</v>
+        <v>1929.78</v>
       </c>
       <c r="AU2" t="n">
-        <v>2036.900024414062</v>
+        <v>2028</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.81</v>
+        <v>9.69</v>
       </c>
       <c r="AY2" t="n">
-        <v>199.77</v>
+        <v>196.45</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.9</v>
+        <v>4.84</v>
       </c>
       <c r="BA2" t="n">
-        <v>99.89</v>
+        <v>98.22</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.03</v>
+        <v>2.05</v>
       </c>
       <c r="BC2" t="n">
         <v>213</v>
@@ -1984,13 +1984,13 @@
         <v>329</v>
       </c>
       <c r="BF2" t="n">
-        <v>48.8</v>
+        <v>48.7</v>
       </c>
       <c r="BG2" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="BH2" t="n">
-        <v>19</v>
+        <v>19.1</v>
       </c>
       <c r="BI2" t="n">
         <v>4</v>
@@ -2005,40 +2005,40 @@
         <v>4</v>
       </c>
       <c r="BM2" t="n">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="BN2" t="n">
-        <v>49.9</v>
+        <v>49.6</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.16</v>
+        <v>2.15</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.59</v>
+        <v>8.609999999999999</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.23</v>
+        <v>-4.21</v>
       </c>
       <c r="BR2" t="n">
         <v>9</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.239</v>
+        <v>0.238</v>
       </c>
       <c r="BT2" t="n">
-        <v>1457.02</v>
+        <v>1452.74</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.44</v>
+        <v>-13.4</v>
       </c>
       <c r="BV2" t="n">
         <v>2.02</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.03</v>
+        <v>2.05</v>
       </c>
       <c r="BX2" t="n">
-        <v>1.9999</v>
+        <v>2.0001</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>43.2</v>
+        <v>43</v>
       </c>
       <c r="CE2" t="n">
         <v>51</v>
       </c>
       <c r="CF2" t="n">
-        <v>67.7</v>
+        <v>68.3</v>
       </c>
       <c r="CG2" t="n">
-        <v>71.3</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>72.31</v>
+        <v>78.11</v>
       </c>
       <c r="CO2" t="n">
-        <v>31.53</v>
+        <v>23.53</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2115,16 +2115,16 @@
         <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>68.18181818181817</v>
+        <v>72.72727272727273</v>
       </c>
       <c r="CX2" t="n">
         <v>63.63636363636363</v>
       </c>
       <c r="CY2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.807600000000001</v>
+        <v>9.6869</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,34 +2133,34 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.654</v>
+        <v>0.646</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3267</v>
+        <v>0.3227</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.09810000000000001</v>
+        <v>0.0969</v>
       </c>
       <c r="DF2" t="n">
-        <v>2.002</v>
+        <v>2.0021</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1203</v>
+        <v>1.095</v>
       </c>
       <c r="DH2" t="n">
         <v>4.0041</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.904</v>
+        <v>4.8432</v>
       </c>
       <c r="DJ2" t="n">
-        <v>29.72</v>
+        <v>29.81</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.904</v>
+        <v>4.8432</v>
       </c>
       <c r="DL2" t="n">
-        <v>1.9999</v>
+        <v>2.0001</v>
       </c>
       <c r="DM2" t="n">
         <v>2</v>
@@ -2169,22 +2169,22 @@
         <v>4.0041</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0018</v>
+        <v>2.0019</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8172</v>
+        <v>0.8273</v>
       </c>
       <c r="DQ2" t="n">
-        <v>99.89</v>
+        <v>98.22</v>
       </c>
       <c r="DR2" t="n">
-        <v>59.74</v>
+        <v>61.8</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.1959</v>
+        <v>1</v>
       </c>
       <c r="DX2" t="n">
-        <v>96.125</v>
+        <v>92.27499999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>39.5</v>
+        <v>20</v>
       </c>
       <c r="DZ2" t="n">
-        <v>74.73399999999999</v>
+        <v>82.26600000000001</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>56.76</v>
+        <v>72.56999999999999</v>
       </c>
       <c r="ED2" t="n">
-        <v>100</v>
+        <v>99.58</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.1959</v>
+        <v>1</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.79</v>
+        <v>0.4</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.3346</v>
+        <v>0.2735</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0031</v>
+        <v>4.0029</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0382</v>
+        <v>0.0309</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6785</v>
+        <v>0.6854</v>
       </c>
       <c r="EK2" t="n">
-        <v>70.06</v>
+        <v>72.58</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2246,37 +2246,37 @@
         <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>11.12</v>
+        <v>5.79</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.2699</v>
+        <v>0.6543</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0902</v>
+        <v>0.0452</v>
       </c>
       <c r="ER2" t="n">
-        <v>12.4177</v>
+        <v>24.225</v>
       </c>
       <c r="ES2" t="n">
-        <v>8.6145</v>
+        <v>8.7164</v>
       </c>
       <c r="ET2" t="n">
-        <v>34.62</v>
+        <v>29.65</v>
       </c>
       <c r="EU2" t="n">
-        <v>2.3147</v>
+        <v>0.968</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.3687</v>
+        <v>1.7286</v>
       </c>
       <c r="EW2" t="n">
-        <v>8.040900000000001</v>
+        <v>4.5226</v>
       </c>
       <c r="EX2" t="n">
-        <v>36.08</v>
+        <v>37.1</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2290,31 @@
         <v>8</v>
       </c>
       <c r="FB2" t="n">
-        <v>62.24</v>
+        <v>61.67</v>
       </c>
       <c r="FC2" t="n">
-        <v>19.8</v>
+        <v>20.23</v>
       </c>
       <c r="FD2" t="n">
-        <v>72.70999999999999</v>
+        <v>73.76000000000001</v>
       </c>
       <c r="FE2" t="n">
-        <v>71.185</v>
+        <v>75.345</v>
       </c>
       <c r="FF2" t="n">
-        <v>33.805</v>
+        <v>30.315</v>
       </c>
       <c r="FG2" t="n">
-        <v>20.9594</v>
+        <v>22.8392</v>
       </c>
       <c r="FH2" t="n">
-        <v>60.029</v>
+        <v>61.688</v>
       </c>
       <c r="FI2" t="n">
-        <v>44.73</v>
+        <v>45.805</v>
       </c>
       <c r="FJ2" t="n">
-        <v>62.42</v>
+        <v>62.82</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,28 +2328,28 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>69.43000000000001</v>
+        <v>71.69</v>
       </c>
       <c r="FO2" t="n">
-        <v>54.23</v>
+        <v>57.23</v>
       </c>
       <c r="FP2" t="n">
-        <v>63</v>
+        <v>60.97</v>
       </c>
       <c r="FQ2" t="n">
-        <v>71.55</v>
+        <v>73.17</v>
       </c>
       <c r="FR2" t="n">
-        <v>79.31</v>
+        <v>78.83</v>
       </c>
       <c r="FS2" t="n">
-        <v>90.9091</v>
+        <v>86.36360000000001</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
       </c>
       <c r="FU2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="FV2" t="inlineStr">
         <is>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>65.55800000000001</v>
+        <v>65.7205</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2365,13 +2365,13 @@
         </is>
       </c>
       <c r="FY2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="FZ2" t="b">
         <v>1</v>
       </c>
       <c r="GA2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="GB2" t="b">
         <v>0</v>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261014_203451</t>
+          <t>20261015_135306</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46309.85753952918</v>
+        <v>46310.57854972719</v>
       </c>
     </row>
   </sheetData>
@@ -2465,7 +2465,7 @@
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="19" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46309.85753472222</v>
+        <v>46310.57854166667</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.42</v>
+        <v>11.3</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>2036.9</v>
+        <v>2028</v>
       </c>
       <c r="L2" t="n">
-        <v>2049</v>
+        <v>2025</v>
       </c>
       <c r="M2" t="n">
-        <v>2057.3</v>
+        <v>2046.3</v>
       </c>
       <c r="N2" t="n">
-        <v>2019.2</v>
+        <v>2008</v>
       </c>
       <c r="O2" t="n">
-        <v>2036.9</v>
+        <v>2028</v>
       </c>
       <c r="P2" t="n">
-        <v>1300927</v>
+        <v>606348</v>
       </c>
       <c r="Q2" t="n">
-        <v>2036.9</v>
+        <v>2028</v>
       </c>
       <c r="R2" t="n">
-        <v>2236.67</v>
+        <v>2224.45</v>
       </c>
       <c r="S2" t="n">
-        <v>1937.01</v>
+        <v>1929.78</v>
       </c>
       <c r="T2" t="n">
-        <v>9.807550689773674</v>
+        <v>9.686883629191312</v>
       </c>
       <c r="U2" t="n">
-        <v>199.77</v>
+        <v>196.4499999999998</v>
       </c>
       <c r="V2" t="n">
-        <v>4.904020815945804</v>
+        <v>4.843195266272191</v>
       </c>
       <c r="W2" t="n">
-        <v>99.8900000000001</v>
+        <v>98.22000000000003</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999899889878864</v>
+        <v>2.000101812258194</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.807550689773674</v>
+        <v>9.686883629191312</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.904020815945804</v>
+        <v>4.843195266272191</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02043267390781192</v>
+        <v>0.02042802464580288</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3243586426808918</v>
+        <v>0.3242848379345565</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.0290494283888163</v>
+        <v>0.02904946749144232</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228671062017354</v>
+        <v>0.04228670049474639</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347614</v>
+        <v>0.1869492979645464</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.05</v>
+        <v>39.06</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-14 20:34:51.456887+05:30</t>
+          <t>2026-10-15 13:53:06.734396+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.807550689773674, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9998998898788645}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.686883629191312, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001018122581935}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-15 14:58 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="17" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.3</v>
+        <v>11.19</v>
       </c>
       <c r="R2" t="n">
-        <v>48.53</v>
+        <v>48.5</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1884,22 +1884,22 @@
         <v>2008</v>
       </c>
       <c r="X2" t="n">
-        <v>2028</v>
+        <v>2018.5</v>
       </c>
       <c r="Y2" t="n">
-        <v>2028</v>
+        <v>2018.5</v>
       </c>
       <c r="Z2" t="n">
-        <v>606348</v>
+        <v>858424</v>
       </c>
       <c r="AA2" t="n">
-        <v>1534093</v>
+        <v>1546697</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.4</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="AC2" t="n">
-        <v>-0.44</v>
+        <v>-0.9</v>
       </c>
       <c r="AD2" t="n">
         <v>-0.58</v>
@@ -1908,7 +1908,7 @@
         <v>38.3</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.89</v>
+        <v>1.9</v>
       </c>
       <c r="AG2" t="n">
         <v>49.11</v>
@@ -1917,7 +1917,7 @@
         <v>49.11</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.42</v>
+        <v>2.43</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>0.77</v>
+        <v>0.32</v>
       </c>
       <c r="AM2" t="n">
-        <v>5.31</v>
+        <v>4.82</v>
       </c>
       <c r="AN2" t="n">
-        <v>44.99</v>
+        <v>44.32</v>
       </c>
       <c r="AO2" t="n">
-        <v>56.91</v>
+        <v>55.35</v>
       </c>
       <c r="AP2" t="n">
-        <v>2.42</v>
+        <v>1.94</v>
       </c>
       <c r="AQ2" t="n">
-        <v>30.2</v>
+        <v>29.59</v>
       </c>
       <c r="AR2" t="n">
-        <v>2028</v>
+        <v>2018.5</v>
       </c>
       <c r="AS2" t="n">
-        <v>2224.45</v>
+        <v>2214.95</v>
       </c>
       <c r="AT2" t="n">
-        <v>1929.78</v>
+        <v>1920.28</v>
       </c>
       <c r="AU2" t="n">
-        <v>2028</v>
+        <v>2018.5</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.69</v>
+        <v>9.73</v>
       </c>
       <c r="AY2" t="n">
         <v>196.45</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.84</v>
+        <v>4.87</v>
       </c>
       <c r="BA2" t="n">
         <v>98.22</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.05</v>
+        <v>2.06</v>
       </c>
       <c r="BC2" t="n">
         <v>213</v>
@@ -1987,55 +1987,55 @@
         <v>48.7</v>
       </c>
       <c r="BG2" t="n">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="BH2" t="n">
-        <v>19.1</v>
+        <v>18.7</v>
       </c>
       <c r="BI2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="BM2" t="n">
         <v>675</v>
       </c>
       <c r="BN2" t="n">
-        <v>49.6</v>
+        <v>49.3</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.15</v>
+        <v>2.14</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.609999999999999</v>
+        <v>8.65</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.21</v>
+        <v>-4.19</v>
       </c>
       <c r="BR2" t="n">
         <v>9</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.238</v>
+        <v>0.237</v>
       </c>
       <c r="BT2" t="n">
-        <v>1452.74</v>
+        <v>1447.53</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.4</v>
+        <v>-13.49</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.02</v>
+        <v>2.01</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.05</v>
+        <v>2.06</v>
       </c>
       <c r="BX2" t="n">
         <v>2.0001</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>43</v>
+        <v>42.8</v>
       </c>
       <c r="CE2" t="n">
-        <v>51</v>
+        <v>50.5</v>
       </c>
       <c r="CF2" t="n">
-        <v>68.3</v>
+        <v>68.7</v>
       </c>
       <c r="CG2" t="n">
-        <v>70.90000000000001</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>78.11</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="CO2" t="n">
-        <v>23.53</v>
+        <v>23.74</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2115,16 +2115,16 @@
         <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>72.72727272727273</v>
+        <v>68.18181818181817</v>
       </c>
       <c r="CX2" t="n">
         <v>63.63636363636363</v>
       </c>
       <c r="CY2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.6869</v>
+        <v>9.7325</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.646</v>
+        <v>0.6487000000000001</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3227</v>
+        <v>0.3247</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0969</v>
+        <v>0.0973</v>
       </c>
       <c r="DF2" t="n">
-        <v>2.0021</v>
+        <v>1.9979</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.095</v>
+        <v>1.0888</v>
       </c>
       <c r="DH2" t="n">
         <v>4.0041</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.8432</v>
+        <v>4.866</v>
       </c>
       <c r="DJ2" t="n">
-        <v>29.81</v>
+        <v>29.7</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.8432</v>
+        <v>4.866</v>
       </c>
       <c r="DL2" t="n">
         <v>2.0001</v>
       </c>
       <c r="DM2" t="n">
-        <v>2</v>
+        <v>2.0041</v>
       </c>
       <c r="DN2" t="n">
         <v>4.0041</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0019</v>
+        <v>1.9978</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8273</v>
+        <v>0.8222</v>
       </c>
       <c r="DQ2" t="n">
         <v>98.22</v>
       </c>
       <c r="DR2" t="n">
-        <v>61.8</v>
+        <v>43.19</v>
       </c>
       <c r="DS2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="DT2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1</v>
+        <v>0.7984</v>
       </c>
       <c r="DX2" t="n">
-        <v>92.27499999999999</v>
+        <v>88.375</v>
       </c>
       <c r="DY2" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="DZ2" t="n">
-        <v>82.26600000000001</v>
+        <v>81.78100000000001</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>72.56999999999999</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="ED2" t="n">
-        <v>99.58</v>
+        <v>93.72</v>
       </c>
       <c r="EE2" t="n">
-        <v>1</v>
+        <v>0.7984</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.4</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.2735</v>
+        <v>0.2171</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0029</v>
+        <v>4.0051</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0309</v>
+        <v>0.0243</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6854</v>
+        <v>0.6823</v>
       </c>
       <c r="EK2" t="n">
-        <v>72.58</v>
+        <v>73.61</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2249,34 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>5.79</v>
+        <v>6.57</v>
       </c>
       <c r="EP2" t="n">
-        <v>0.6543</v>
+        <v>0.7352</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0452</v>
+        <v>0.06270000000000001</v>
       </c>
       <c r="ER2" t="n">
-        <v>24.225</v>
+        <v>17.375</v>
       </c>
       <c r="ES2" t="n">
-        <v>8.7164</v>
+        <v>8.658899999999999</v>
       </c>
       <c r="ET2" t="n">
-        <v>29.65</v>
+        <v>29.812</v>
       </c>
       <c r="EU2" t="n">
-        <v>0.968</v>
+        <v>1.0864</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.7286</v>
+        <v>1.5577</v>
       </c>
       <c r="EW2" t="n">
-        <v>4.5226</v>
+        <v>5.1108</v>
       </c>
       <c r="EX2" t="n">
-        <v>37.1</v>
+        <v>39.53</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2290,31 @@
         <v>8</v>
       </c>
       <c r="FB2" t="n">
-        <v>61.67</v>
+        <v>61.15</v>
       </c>
       <c r="FC2" t="n">
-        <v>20.23</v>
+        <v>20.57</v>
       </c>
       <c r="FD2" t="n">
-        <v>73.76000000000001</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="FE2" t="n">
-        <v>75.345</v>
+        <v>75.7</v>
       </c>
       <c r="FF2" t="n">
-        <v>30.315</v>
+        <v>31.635</v>
       </c>
       <c r="FG2" t="n">
-        <v>22.8392</v>
+        <v>22.6793</v>
       </c>
       <c r="FH2" t="n">
-        <v>61.688</v>
+        <v>61.818</v>
       </c>
       <c r="FI2" t="n">
-        <v>45.805</v>
+        <v>36.445</v>
       </c>
       <c r="FJ2" t="n">
-        <v>62.82</v>
+        <v>62.01</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,28 +2328,28 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>71.69</v>
+        <v>65.13</v>
       </c>
       <c r="FO2" t="n">
-        <v>57.23</v>
+        <v>57.67</v>
       </c>
       <c r="FP2" t="n">
-        <v>60.97</v>
+        <v>51.35</v>
       </c>
       <c r="FQ2" t="n">
-        <v>73.17</v>
+        <v>62.62</v>
       </c>
       <c r="FR2" t="n">
-        <v>78.83</v>
+        <v>68.52</v>
       </c>
       <c r="FS2" t="n">
-        <v>86.36360000000001</v>
+        <v>77.2727</v>
       </c>
       <c r="FT2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="FU2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="FV2" t="inlineStr">
         <is>
@@ -2357,18 +2357,18 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>65.7205</v>
+        <v>57.5955</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="FY2" t="b">
         <v>0</v>
       </c>
       <c r="FZ2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="GA2" t="b">
         <v>0</v>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261015_135306</t>
+          <t>20261015_202804</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46310.57854972719</v>
+        <v>46310.85282827693</v>
       </c>
     </row>
   </sheetData>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46310.57854166667</v>
+        <v>46310.85282407407</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46310</v>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.3</v>
+        <v>11.19</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>2028</v>
+        <v>2018.5</v>
       </c>
       <c r="L2" t="n">
         <v>2025</v>
@@ -2693,28 +2693,28 @@
         <v>2008</v>
       </c>
       <c r="O2" t="n">
-        <v>2028</v>
+        <v>2018.5</v>
       </c>
       <c r="P2" t="n">
-        <v>606348</v>
+        <v>858424</v>
       </c>
       <c r="Q2" t="n">
-        <v>2028</v>
+        <v>2018.5</v>
       </c>
       <c r="R2" t="n">
-        <v>2224.45</v>
+        <v>2214.95</v>
       </c>
       <c r="S2" t="n">
-        <v>1929.78</v>
+        <v>1920.28</v>
       </c>
       <c r="T2" t="n">
-        <v>9.686883629191312</v>
+        <v>9.732474609858798</v>
       </c>
       <c r="U2" t="n">
         <v>196.4499999999998</v>
       </c>
       <c r="V2" t="n">
-        <v>4.843195266272191</v>
+        <v>4.865989596234829</v>
       </c>
       <c r="W2" t="n">
         <v>98.22000000000003</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.686883629191312</v>
+        <v>9.732474609858798</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.843195266272191</v>
+        <v>4.865989596234829</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02042802464580288</v>
+        <v>0.02042292925838663</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3242848379345565</v>
+        <v>0.3242039511669349</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02904946749144232</v>
+        <v>0.02904345305700145</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228670049474639</v>
+        <v>0.04228669940338745</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869492979645463</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-15 13:53:06.734396+05:30</t>
+          <t>2026-10-15 20:28:04.402682+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.686883629191312, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001018122581935}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.732474609858798, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001018122581935}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-16 08:15 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="18" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="H2" t="n">
         <v>8.800000000000001</v>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.19</v>
+        <v>11.72</v>
       </c>
       <c r="R2" t="n">
-        <v>48.5</v>
+        <v>48.87</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,46 +1875,46 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>2025</v>
+        <v>2030.4</v>
       </c>
       <c r="V2" t="n">
-        <v>2046.3</v>
+        <v>2086</v>
       </c>
       <c r="W2" t="n">
-        <v>2008</v>
+        <v>2028.7</v>
       </c>
       <c r="X2" t="n">
-        <v>2018.5</v>
+        <v>2073.9</v>
       </c>
       <c r="Y2" t="n">
-        <v>2018.5</v>
+        <v>2073.9</v>
       </c>
       <c r="Z2" t="n">
-        <v>858424</v>
+        <v>1191605</v>
       </c>
       <c r="AA2" t="n">
-        <v>1546697</v>
+        <v>1524036</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.78</v>
       </c>
       <c r="AC2" t="n">
-        <v>-0.9</v>
+        <v>2.74</v>
       </c>
       <c r="AD2" t="n">
-        <v>-0.58</v>
+        <v>0.59</v>
       </c>
       <c r="AE2" t="n">
-        <v>38.3</v>
+        <v>57.3</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.9</v>
+        <v>2.76</v>
       </c>
       <c r="AG2" t="n">
-        <v>49.11</v>
+        <v>50.42</v>
       </c>
       <c r="AH2" t="n">
-        <v>49.11</v>
+        <v>50.42</v>
       </c>
       <c r="AI2" t="n">
         <v>2.43</v>
@@ -1926,34 +1926,34 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>0.32</v>
+        <v>2.76</v>
       </c>
       <c r="AM2" t="n">
-        <v>4.82</v>
+        <v>7.43</v>
       </c>
       <c r="AN2" t="n">
-        <v>44.32</v>
+        <v>47.75</v>
       </c>
       <c r="AO2" t="n">
-        <v>55.35</v>
+        <v>61.9</v>
       </c>
       <c r="AP2" t="n">
-        <v>1.94</v>
+        <v>4.53</v>
       </c>
       <c r="AQ2" t="n">
-        <v>29.59</v>
+        <v>35.57</v>
       </c>
       <c r="AR2" t="n">
-        <v>2018.5</v>
+        <v>2073.9</v>
       </c>
       <c r="AS2" t="n">
-        <v>2214.95</v>
+        <v>2275.6</v>
       </c>
       <c r="AT2" t="n">
-        <v>1920.28</v>
+        <v>1973.05</v>
       </c>
       <c r="AU2" t="n">
-        <v>2018.5</v>
+        <v>2073.89990234375</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
@@ -1963,22 +1963,22 @@
         <v>9.73</v>
       </c>
       <c r="AY2" t="n">
-        <v>196.45</v>
+        <v>201.7</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.87</v>
+        <v>4.86</v>
       </c>
       <c r="BA2" t="n">
-        <v>98.22</v>
+        <v>100.85</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.06</v>
+        <v>1.99</v>
       </c>
       <c r="BC2" t="n">
         <v>213</v>
       </c>
       <c r="BD2" t="n">
-        <v>31.6</v>
+        <v>31.5</v>
       </c>
       <c r="BE2" t="n">
         <v>329</v>
@@ -1987,58 +1987,58 @@
         <v>48.7</v>
       </c>
       <c r="BG2" t="n">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.7</v>
+        <v>19.8</v>
       </c>
       <c r="BI2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="BJ2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="BM2" t="n">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="BN2" t="n">
-        <v>49.3</v>
+        <v>50.6</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.14</v>
+        <v>2.19</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.65</v>
+        <v>8.49</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.19</v>
+        <v>-4.27</v>
       </c>
       <c r="BR2" t="n">
         <v>9</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.237</v>
+        <v>0.242</v>
       </c>
       <c r="BT2" t="n">
-        <v>1447.53</v>
+        <v>1477.14</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.49</v>
+        <v>-13.04</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.01</v>
+        <v>2.04</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.06</v>
+        <v>1.99</v>
       </c>
       <c r="BX2" t="n">
-        <v>2.0001</v>
+        <v>2</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>42.8</v>
+        <v>43.8</v>
       </c>
       <c r="CE2" t="n">
-        <v>50.5</v>
+        <v>52</v>
       </c>
       <c r="CF2" t="n">
-        <v>68.7</v>
+        <v>66.3</v>
       </c>
       <c r="CG2" t="n">
-        <v>70.40000000000001</v>
+        <v>72.3</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>77.79000000000001</v>
+        <v>89.98999999999999</v>
       </c>
       <c r="CO2" t="n">
-        <v>23.74</v>
+        <v>45.91</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2115,16 +2115,16 @@
         <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>68.18181818181817</v>
+        <v>77.27272727272727</v>
       </c>
       <c r="CX2" t="n">
         <v>63.63636363636363</v>
       </c>
       <c r="CY2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.7325</v>
+        <v>9.7256</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2136,55 +2136,55 @@
         <v>0.6487000000000001</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3247</v>
+        <v>0.324</v>
       </c>
       <c r="DE2" t="n">
         <v>0.0973</v>
       </c>
       <c r="DF2" t="n">
-        <v>1.9979</v>
+        <v>2.0021</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.0888</v>
+        <v>1.1404</v>
       </c>
       <c r="DH2" t="n">
         <v>4.0041</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.866</v>
+        <v>4.8628</v>
       </c>
       <c r="DJ2" t="n">
-        <v>29.7</v>
+        <v>33.28</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.866</v>
+        <v>4.8628</v>
       </c>
       <c r="DL2" t="n">
-        <v>2.0001</v>
+        <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>2.0041</v>
+        <v>2</v>
       </c>
       <c r="DN2" t="n">
         <v>4.0041</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9978</v>
+        <v>2.0022</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8222</v>
+        <v>0.8239</v>
       </c>
       <c r="DQ2" t="n">
-        <v>98.22</v>
+        <v>100.85</v>
       </c>
       <c r="DR2" t="n">
-        <v>43.19</v>
+        <v>60.48</v>
       </c>
       <c r="DS2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.7984</v>
+        <v>1.8642</v>
       </c>
       <c r="DX2" t="n">
-        <v>88.375</v>
+        <v>95.25</v>
       </c>
       <c r="DY2" t="n">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="DZ2" t="n">
-        <v>81.78100000000001</v>
+        <v>90.333</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>74.59999999999999</v>
+        <v>77.02</v>
       </c>
       <c r="ED2" t="n">
-        <v>93.72</v>
+        <v>93.93000000000001</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.7984</v>
+        <v>1.8642</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.78</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.2171</v>
+        <v>0.5309</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0051</v>
+        <v>4.0023</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0243</v>
+        <v>0.0622</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6823</v>
+        <v>0.6830000000000001</v>
       </c>
       <c r="EK2" t="n">
-        <v>73.61</v>
+        <v>76.14</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,72 +2249,72 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>6.57</v>
+        <v>72.27</v>
       </c>
       <c r="EP2" t="n">
-        <v>0.7352</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.06270000000000001</v>
+        <v>0.0914</v>
       </c>
       <c r="ER2" t="n">
-        <v>17.375</v>
+        <v>12.4744</v>
       </c>
       <c r="ES2" t="n">
-        <v>8.658899999999999</v>
+        <v>9.7026</v>
       </c>
       <c r="ET2" t="n">
-        <v>29.812</v>
+        <v>59.143</v>
       </c>
       <c r="EU2" t="n">
-        <v>1.0864</v>
+        <v>3.5334</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.5577</v>
+        <v>1.3652</v>
       </c>
       <c r="EW2" t="n">
-        <v>5.1108</v>
+        <v>65.03579999999999</v>
       </c>
       <c r="EX2" t="n">
-        <v>39.53</v>
+        <v>56.5</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="EZ2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="FA2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>61.15</v>
+        <v>63.66</v>
       </c>
       <c r="FC2" t="n">
-        <v>20.57</v>
+        <v>23.86</v>
       </c>
       <c r="FD2" t="n">
-        <v>74.29000000000001</v>
+        <v>70.47</v>
       </c>
       <c r="FE2" t="n">
-        <v>75.7</v>
+        <v>83.065</v>
       </c>
       <c r="FF2" t="n">
-        <v>31.635</v>
+        <v>51.205</v>
       </c>
       <c r="FG2" t="n">
-        <v>22.6793</v>
+        <v>26.2362</v>
       </c>
       <c r="FH2" t="n">
-        <v>61.818</v>
+        <v>70.127</v>
       </c>
       <c r="FI2" t="n">
-        <v>36.445</v>
+        <v>46.88</v>
       </c>
       <c r="FJ2" t="n">
-        <v>62.01</v>
+        <v>67.65000000000001</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,50 +2328,50 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>65.13</v>
+        <v>78.70999999999999</v>
       </c>
       <c r="FO2" t="n">
-        <v>57.67</v>
+        <v>61.83</v>
       </c>
       <c r="FP2" t="n">
-        <v>51.35</v>
+        <v>82.14</v>
       </c>
       <c r="FQ2" t="n">
-        <v>62.62</v>
+        <v>76.73999999999999</v>
       </c>
       <c r="FR2" t="n">
-        <v>68.52</v>
+        <v>88.31</v>
       </c>
       <c r="FS2" t="n">
-        <v>77.2727</v>
+        <v>100</v>
       </c>
       <c r="FT2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="FU2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>57.5955</v>
+        <v>71.749</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Strong</t>
         </is>
       </c>
       <c r="FY2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="FZ2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="GA2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="GB2" t="b">
         <v>0</v>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261015_202804</t>
+          <t>20261016_134533</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46310.85282827693</v>
+        <v>46311.5732998367</v>
       </c>
     </row>
   </sheetData>
@@ -2465,7 +2465,7 @@
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="19" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46310.85282407407</v>
+        <v>46311.57329861111</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.19</v>
+        <v>11.72</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>2018.5</v>
+        <v>2073.9</v>
       </c>
       <c r="L2" t="n">
-        <v>2025</v>
+        <v>2030.4</v>
       </c>
       <c r="M2" t="n">
-        <v>2046.3</v>
+        <v>2086</v>
       </c>
       <c r="N2" t="n">
-        <v>2008</v>
+        <v>2028.7</v>
       </c>
       <c r="O2" t="n">
-        <v>2018.5</v>
+        <v>2073.9</v>
       </c>
       <c r="P2" t="n">
-        <v>858424</v>
+        <v>1191605</v>
       </c>
       <c r="Q2" t="n">
-        <v>2018.5</v>
+        <v>2073.9</v>
       </c>
       <c r="R2" t="n">
-        <v>2214.95</v>
+        <v>2275.6</v>
       </c>
       <c r="S2" t="n">
-        <v>1920.28</v>
+        <v>1973.05</v>
       </c>
       <c r="T2" t="n">
-        <v>9.732474609858798</v>
+        <v>9.725637687448758</v>
       </c>
       <c r="U2" t="n">
-        <v>196.4499999999998</v>
+        <v>201.6999999999998</v>
       </c>
       <c r="V2" t="n">
-        <v>4.865989596234829</v>
+        <v>4.862818843724391</v>
       </c>
       <c r="W2" t="n">
-        <v>98.22000000000003</v>
+        <v>100.8500000000001</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000101812258194</v>
+        <v>1.999999999999996</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.732474609858798</v>
+        <v>9.725637687448758</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.865989596234829</v>
+        <v>4.862818843724391</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02042292925838663</v>
+        <v>0.02043952678175495</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3242039511669349</v>
+        <v>0.3244674286822077</v>
       </c>
     </row>
     <row r="7">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228669940338745</v>
+        <v>0.04228670539922998</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645463</v>
+        <v>0.1869492979645465</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.06</v>
+        <v>39.04</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-15 20:28:04.402682+05:30</t>
+          <t>2026-10-16 13:45:33.130220+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.732474609858798, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0001018122581935}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.725637687448758, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9999999999999956}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-16 14:48 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.72</v>
+        <v>11.63</v>
       </c>
       <c r="R2" t="n">
-        <v>48.87</v>
+        <v>48.82</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1884,22 +1884,22 @@
         <v>2028.7</v>
       </c>
       <c r="X2" t="n">
-        <v>2073.9</v>
+        <v>2060.1</v>
       </c>
       <c r="Y2" t="n">
-        <v>2073.9</v>
+        <v>2060.1</v>
       </c>
       <c r="Z2" t="n">
-        <v>1191605</v>
+        <v>1606316</v>
       </c>
       <c r="AA2" t="n">
-        <v>1524036</v>
+        <v>1544771</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.78</v>
+        <v>1.04</v>
       </c>
       <c r="AC2" t="n">
-        <v>2.74</v>
+        <v>2.06</v>
       </c>
       <c r="AD2" t="n">
         <v>0.59</v>
@@ -1908,7 +1908,7 @@
         <v>57.3</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.76</v>
+        <v>2.78</v>
       </c>
       <c r="AG2" t="n">
         <v>50.42</v>
@@ -1917,7 +1917,7 @@
         <v>50.42</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.43</v>
+        <v>2.45</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>2.76</v>
+        <v>2.11</v>
       </c>
       <c r="AM2" t="n">
-        <v>7.43</v>
+        <v>6.73</v>
       </c>
       <c r="AN2" t="n">
-        <v>47.75</v>
+        <v>46.78</v>
       </c>
       <c r="AO2" t="n">
-        <v>61.9</v>
+        <v>60.45</v>
       </c>
       <c r="AP2" t="n">
-        <v>4.53</v>
+        <v>3.84</v>
       </c>
       <c r="AQ2" t="n">
-        <v>35.57</v>
+        <v>34.66</v>
       </c>
       <c r="AR2" t="n">
-        <v>2073.9</v>
+        <v>2060.1</v>
       </c>
       <c r="AS2" t="n">
-        <v>2275.6</v>
+        <v>2261.8</v>
       </c>
       <c r="AT2" t="n">
-        <v>1973.05</v>
+        <v>1959.25</v>
       </c>
       <c r="AU2" t="n">
-        <v>2073.89990234375</v>
+        <v>2060.10009765625</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.73</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="AY2" t="n">
         <v>201.7</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.86</v>
+        <v>4.9</v>
       </c>
       <c r="BA2" t="n">
         <v>100.85</v>
       </c>
       <c r="BB2" t="n">
-        <v>1.99</v>
+        <v>1.98</v>
       </c>
       <c r="BC2" t="n">
         <v>213</v>
@@ -2011,10 +2011,10 @@
         <v>50.6</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.19</v>
+        <v>2.17</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.49</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="BQ2" t="n">
         <v>-4.27</v>
@@ -2023,19 +2023,19 @@
         <v>9</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.242</v>
+        <v>0.24</v>
       </c>
       <c r="BT2" t="n">
-        <v>1477.14</v>
+        <v>1470.02</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.04</v>
+        <v>-13.15</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.04</v>
+        <v>2.03</v>
       </c>
       <c r="BW2" t="n">
-        <v>1.99</v>
+        <v>1.98</v>
       </c>
       <c r="BX2" t="n">
         <v>2</v>
@@ -2058,13 +2058,13 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>43.8</v>
+        <v>43.4</v>
       </c>
       <c r="CE2" t="n">
-        <v>52</v>
+        <v>51.5</v>
       </c>
       <c r="CF2" t="n">
-        <v>66.3</v>
+        <v>66</v>
       </c>
       <c r="CG2" t="n">
         <v>72.3</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>89.98999999999999</v>
+        <v>87.59</v>
       </c>
       <c r="CO2" t="n">
-        <v>45.91</v>
+        <v>42.01</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2121,10 +2121,10 @@
         <v>63.63636363636363</v>
       </c>
       <c r="CY2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.7256</v>
+        <v>9.790800000000001</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,31 +2133,31 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6487000000000001</v>
+        <v>0.6526999999999999</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.324</v>
+        <v>0.3267</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0973</v>
+        <v>0.0979</v>
       </c>
       <c r="DF2" t="n">
-        <v>2.0021</v>
+        <v>1.998</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1404</v>
+        <v>1.1386</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0041</v>
+        <v>3.9959</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.8628</v>
+        <v>4.8954</v>
       </c>
       <c r="DJ2" t="n">
-        <v>33.28</v>
+        <v>35.28</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.8628</v>
+        <v>4.8954</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
@@ -2166,25 +2166,25 @@
         <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>4.0041</v>
+        <v>3.9959</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0022</v>
+        <v>1.9979</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8239</v>
+        <v>0.8155</v>
       </c>
       <c r="DQ2" t="n">
         <v>100.85</v>
       </c>
       <c r="DR2" t="n">
-        <v>60.48</v>
+        <v>44.1</v>
       </c>
       <c r="DS2" t="n">
+        <v>3</v>
+      </c>
+      <c r="DT2" t="n">
         <v>5</v>
-      </c>
-      <c r="DT2" t="n">
-        <v>10</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.8642</v>
+        <v>1.5673</v>
       </c>
       <c r="DX2" t="n">
-        <v>95.25</v>
+        <v>98.875</v>
       </c>
       <c r="DY2" t="n">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="DZ2" t="n">
-        <v>90.333</v>
+        <v>88.31699999999999</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>77.02</v>
+        <v>71.28</v>
       </c>
       <c r="ED2" t="n">
-        <v>93.93000000000001</v>
+        <v>100</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.8642</v>
+        <v>1.5673</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.78</v>
+        <v>1.04</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.5309</v>
+        <v>0.4466</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0023</v>
+        <v>3.9962</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0622</v>
+        <v>0.0519</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6830000000000001</v>
+        <v>0.6773</v>
       </c>
       <c r="EK2" t="n">
-        <v>76.14</v>
+        <v>70.38</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2249,34 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>72.27</v>
+        <v>69.65000000000001</v>
       </c>
       <c r="EP2" t="n">
-        <v>8.470000000000001</v>
+        <v>8.100300000000001</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0914</v>
+        <v>0.121</v>
       </c>
       <c r="ER2" t="n">
-        <v>12.4744</v>
+        <v>9.413500000000001</v>
       </c>
       <c r="ES2" t="n">
-        <v>9.7026</v>
+        <v>10.2261</v>
       </c>
       <c r="ET2" t="n">
-        <v>59.143</v>
+        <v>56.668</v>
       </c>
       <c r="EU2" t="n">
-        <v>3.5334</v>
+        <v>3.9936</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.3652</v>
+        <v>1.201</v>
       </c>
       <c r="EW2" t="n">
-        <v>65.03579999999999</v>
+        <v>61.0064</v>
       </c>
       <c r="EX2" t="n">
-        <v>56.5</v>
+        <v>57.64</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2290,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.66</v>
+        <v>63.23</v>
       </c>
       <c r="FC2" t="n">
-        <v>23.86</v>
+        <v>25.34</v>
       </c>
       <c r="FD2" t="n">
-        <v>70.47</v>
+        <v>69.94</v>
       </c>
       <c r="FE2" t="n">
-        <v>83.065</v>
+        <v>78.985</v>
       </c>
       <c r="FF2" t="n">
-        <v>51.205</v>
+        <v>49.825</v>
       </c>
       <c r="FG2" t="n">
-        <v>26.2362</v>
+        <v>25.3884</v>
       </c>
       <c r="FH2" t="n">
-        <v>70.127</v>
+        <v>69.42</v>
       </c>
       <c r="FI2" t="n">
-        <v>46.88</v>
+        <v>39.69</v>
       </c>
       <c r="FJ2" t="n">
-        <v>67.65000000000001</v>
+        <v>66.2</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>78.70999999999999</v>
+        <v>69.68000000000001</v>
       </c>
       <c r="FO2" t="n">
-        <v>61.83</v>
+        <v>61.2</v>
       </c>
       <c r="FP2" t="n">
-        <v>82.14</v>
+        <v>69.58</v>
       </c>
       <c r="FQ2" t="n">
-        <v>76.73999999999999</v>
+        <v>63.86</v>
       </c>
       <c r="FR2" t="n">
-        <v>88.31</v>
+        <v>81.27</v>
       </c>
       <c r="FS2" t="n">
-        <v>100</v>
+        <v>90.9091</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>71.749</v>
+        <v>65.782</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261016_134533</t>
+          <t>20261016_201834</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46311.5732998367</v>
+        <v>46311.84622931224</v>
       </c>
     </row>
   </sheetData>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46311.57329861111</v>
+        <v>46311.84622685185</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46311</v>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.72</v>
+        <v>11.63</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>2073.9</v>
+        <v>2060.1</v>
       </c>
       <c r="L2" t="n">
         <v>2030.4</v>
@@ -2693,34 +2693,34 @@
         <v>2028.7</v>
       </c>
       <c r="O2" t="n">
-        <v>2073.9</v>
+        <v>2060.1</v>
       </c>
       <c r="P2" t="n">
-        <v>1191605</v>
+        <v>1606316</v>
       </c>
       <c r="Q2" t="n">
-        <v>2073.9</v>
+        <v>2060.1</v>
       </c>
       <c r="R2" t="n">
-        <v>2275.6</v>
+        <v>2261.8</v>
       </c>
       <c r="S2" t="n">
-        <v>1973.05</v>
+        <v>1959.25</v>
       </c>
       <c r="T2" t="n">
-        <v>9.725637687448758</v>
+        <v>9.790786855007052</v>
       </c>
       <c r="U2" t="n">
-        <v>201.6999999999998</v>
+        <v>201.7000000000003</v>
       </c>
       <c r="V2" t="n">
-        <v>4.862818843724391</v>
+        <v>4.895393427503516</v>
       </c>
       <c r="W2" t="n">
-        <v>100.8500000000001</v>
+        <v>100.8499999999999</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999999999999996</v>
+        <v>2.000000000000004</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.725637687448758</v>
+        <v>9.790786855007052</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.862818843724391</v>
+        <v>4.895393427503516</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02043952678175495</v>
+        <v>0.02041972787390557</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3244674286822077</v>
+        <v>0.3241531307638069</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02904345305700145</v>
+        <v>0.02903743862256058</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228670539922998</v>
+        <v>0.04228669642138508</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645465</v>
+        <v>0.1869492979645464</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.04</v>
+        <v>39.07</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-16 13:45:33.130220+05:30</t>
+          <t>2026-10-16 20:18:34.247300+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.725637687448758, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9999999999999956}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.790786855007052, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0000000000000044}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-19 08:59 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="17" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46311</v>
+        <v>46314</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46311</v>
+        <v>46314</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46311</v>
+        <v>46314</v>
       </c>
       <c r="H2" t="n">
         <v>8.800000000000001</v>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.63</v>
+        <v>11.65</v>
       </c>
       <c r="R2" t="n">
-        <v>48.82</v>
+        <v>48.7</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,101 +1875,101 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>2030.4</v>
+        <v>2060.1</v>
       </c>
       <c r="V2" t="n">
-        <v>2086</v>
+        <v>2089</v>
       </c>
       <c r="W2" t="n">
-        <v>2028.7</v>
+        <v>2052.2</v>
       </c>
       <c r="X2" t="n">
-        <v>2060.1</v>
+        <v>2064.9</v>
       </c>
       <c r="Y2" t="n">
-        <v>2060.1</v>
+        <v>2064.9</v>
       </c>
       <c r="Z2" t="n">
-        <v>1606316</v>
+        <v>942561</v>
       </c>
       <c r="AA2" t="n">
-        <v>1544771</v>
+        <v>1459117</v>
       </c>
       <c r="AB2" t="n">
-        <v>1.04</v>
+        <v>0.65</v>
       </c>
       <c r="AC2" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>36.8</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>49.45</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>49.45</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="AJ2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL2" t="n">
         <v>2.06</v>
       </c>
-      <c r="AD2" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="AE2" t="n">
-        <v>57.3</v>
-      </c>
-      <c r="AF2" t="n">
-        <v>2.78</v>
-      </c>
-      <c r="AG2" t="n">
-        <v>50.42</v>
-      </c>
-      <c r="AH2" t="n">
-        <v>50.42</v>
-      </c>
-      <c r="AI2" t="n">
-        <v>2.45</v>
-      </c>
-      <c r="AJ2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AK2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AL2" t="n">
-        <v>2.11</v>
-      </c>
       <c r="AM2" t="n">
-        <v>6.73</v>
+        <v>6.72</v>
       </c>
       <c r="AN2" t="n">
-        <v>46.78</v>
+        <v>46.61</v>
       </c>
       <c r="AO2" t="n">
-        <v>60.45</v>
+        <v>61.01</v>
       </c>
       <c r="AP2" t="n">
-        <v>3.84</v>
+        <v>4.74</v>
       </c>
       <c r="AQ2" t="n">
-        <v>34.66</v>
+        <v>32.46</v>
       </c>
       <c r="AR2" t="n">
-        <v>2060.1</v>
+        <v>2064.9</v>
       </c>
       <c r="AS2" t="n">
-        <v>2261.8</v>
+        <v>2262.71</v>
       </c>
       <c r="AT2" t="n">
-        <v>1959.25</v>
+        <v>1966</v>
       </c>
       <c r="AU2" t="n">
-        <v>2060.10009765625</v>
+        <v>2064.89990234375</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.789999999999999</v>
+        <v>9.58</v>
       </c>
       <c r="AY2" t="n">
-        <v>201.7</v>
+        <v>197.81</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.9</v>
+        <v>4.79</v>
       </c>
       <c r="BA2" t="n">
-        <v>100.85</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="BB2" t="n">
         <v>1.98</v>
@@ -1984,13 +1984,13 @@
         <v>329</v>
       </c>
       <c r="BF2" t="n">
-        <v>48.7</v>
+        <v>48.6</v>
       </c>
       <c r="BG2" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="BH2" t="n">
-        <v>19.8</v>
+        <v>19.9</v>
       </c>
       <c r="BI2" t="n">
         <v>0</v>
@@ -2005,16 +2005,16 @@
         <v>0</v>
       </c>
       <c r="BM2" t="n">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="BN2" t="n">
-        <v>50.6</v>
+        <v>50.7</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.17</v>
+        <v>2.18</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.470000000000001</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="BQ2" t="n">
         <v>-4.27</v>
@@ -2026,10 +2026,10 @@
         <v>0.24</v>
       </c>
       <c r="BT2" t="n">
-        <v>1470.02</v>
+        <v>1472.52</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.15</v>
+        <v>-13.23</v>
       </c>
       <c r="BV2" t="n">
         <v>2.03</v>
@@ -2038,7 +2038,7 @@
         <v>1.98</v>
       </c>
       <c r="BX2" t="n">
-        <v>2</v>
+        <v>2.0001</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2058,7 +2058,7 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>43.4</v>
+        <v>43.6</v>
       </c>
       <c r="CE2" t="n">
         <v>51.5</v>
@@ -2067,7 +2067,7 @@
         <v>66</v>
       </c>
       <c r="CG2" t="n">
-        <v>72.3</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>87.59</v>
+        <v>88.91</v>
       </c>
       <c r="CO2" t="n">
-        <v>42.01</v>
+        <v>39.37</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2118,13 +2118,13 @@
         <v>77.27272727272727</v>
       </c>
       <c r="CX2" t="n">
-        <v>63.63636363636363</v>
+        <v>59.09090909090909</v>
       </c>
       <c r="CY2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.790800000000001</v>
+        <v>9.579599999999999</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6526999999999999</v>
+        <v>0.6387</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3267</v>
+        <v>0.3193</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0979</v>
+        <v>0.0958</v>
       </c>
       <c r="DF2" t="n">
-        <v>1.998</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1386</v>
+        <v>1.1161</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9959</v>
+        <v>4.0084</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.8954</v>
+        <v>4.7896</v>
       </c>
       <c r="DJ2" t="n">
-        <v>35.28</v>
+        <v>28.67</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.8954</v>
+        <v>4.7896</v>
       </c>
       <c r="DL2" t="n">
-        <v>2</v>
+        <v>2.0001</v>
       </c>
       <c r="DM2" t="n">
-        <v>2</v>
+        <v>2.0042</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9959</v>
+        <v>4.0084</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9979</v>
+        <v>2.0003</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.8155</v>
+        <v>0.8368</v>
       </c>
       <c r="DQ2" t="n">
-        <v>100.85</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="DR2" t="n">
-        <v>44.1</v>
+        <v>67.41</v>
       </c>
       <c r="DS2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.5673</v>
+        <v>1.9833</v>
       </c>
       <c r="DX2" t="n">
-        <v>98.875</v>
+        <v>97.47500000000001</v>
       </c>
       <c r="DY2" t="n">
-        <v>52</v>
+        <v>32.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>88.31699999999999</v>
+        <v>90.20999999999999</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,35 +2211,35 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>71.28</v>
+        <v>93.72</v>
       </c>
       <c r="ED2" t="n">
         <v>100</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.5673</v>
+        <v>1.9833</v>
       </c>
       <c r="EF2" t="n">
-        <v>1.04</v>
+        <v>0.65</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.4466</v>
+        <v>0.5522</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9962</v>
+        <v>4.0082</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0519</v>
+        <v>0.0643</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6773</v>
+        <v>0.6923</v>
       </c>
       <c r="EK2" t="n">
-        <v>70.38</v>
+        <v>87.20999999999999</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Excellent</t>
         </is>
       </c>
       <c r="EM2" t="n">
@@ -2249,38 +2249,38 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>69.65000000000001</v>
+        <v>20.94</v>
       </c>
       <c r="EP2" t="n">
-        <v>8.100300000000001</v>
+        <v>2.4395</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.121</v>
+        <v>0.0757</v>
       </c>
       <c r="ER2" t="n">
-        <v>9.413500000000001</v>
+        <v>14.7385</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.2261</v>
+        <v>8.4572</v>
       </c>
       <c r="ET2" t="n">
-        <v>56.668</v>
+        <v>41.029</v>
       </c>
       <c r="EU2" t="n">
-        <v>3.9936</v>
+        <v>3.081</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.201</v>
+        <v>1.4485</v>
       </c>
       <c r="EW2" t="n">
-        <v>61.0064</v>
+        <v>18.6178</v>
       </c>
       <c r="EX2" t="n">
-        <v>57.64</v>
+        <v>63.15</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Strong</t>
         </is>
       </c>
       <c r="EZ2" t="n">
@@ -2290,31 +2290,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.23</v>
+        <v>63.33</v>
       </c>
       <c r="FC2" t="n">
-        <v>25.34</v>
+        <v>17.24</v>
       </c>
       <c r="FD2" t="n">
-        <v>69.94</v>
+        <v>70.06999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>78.985</v>
+        <v>88.06</v>
       </c>
       <c r="FF2" t="n">
-        <v>49.825</v>
+        <v>51.26</v>
       </c>
       <c r="FG2" t="n">
-        <v>25.3884</v>
+        <v>26.2271</v>
       </c>
       <c r="FH2" t="n">
-        <v>69.42</v>
+        <v>70.968</v>
       </c>
       <c r="FI2" t="n">
-        <v>39.69</v>
+        <v>48.04</v>
       </c>
       <c r="FJ2" t="n">
-        <v>66.2</v>
+        <v>68.76000000000001</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>69.68000000000001</v>
+        <v>81.48</v>
       </c>
       <c r="FO2" t="n">
-        <v>61.2</v>
+        <v>67.22</v>
       </c>
       <c r="FP2" t="n">
-        <v>69.58</v>
+        <v>83.86</v>
       </c>
       <c r="FQ2" t="n">
-        <v>63.86</v>
+        <v>72.66</v>
       </c>
       <c r="FR2" t="n">
-        <v>81.27</v>
+        <v>92.66</v>
       </c>
       <c r="FS2" t="n">
-        <v>90.9091</v>
+        <v>100</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>65.782</v>
+        <v>74.494</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261016_201834</t>
+          <t>20261019_142928</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46311.84622931224</v>
+        <v>46314.60380311091</v>
       </c>
     </row>
   </sheetData>
@@ -2465,8 +2465,8 @@
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="20" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="19" customWidth="1" min="23" max="23"/>
+    <col width="19" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46311.84622685185</v>
+        <v>46314.60379629629</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46311</v>
+        <v>46314</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46326</v>
+        <v>46329</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.63</v>
+        <v>11.65</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
+        <v>2064.9</v>
+      </c>
+      <c r="L2" t="n">
         <v>2060.1</v>
       </c>
-      <c r="L2" t="n">
-        <v>2030.4</v>
-      </c>
       <c r="M2" t="n">
-        <v>2086</v>
+        <v>2089</v>
       </c>
       <c r="N2" t="n">
-        <v>2028.7</v>
+        <v>2052.2</v>
       </c>
       <c r="O2" t="n">
-        <v>2060.1</v>
+        <v>2064.9</v>
       </c>
       <c r="P2" t="n">
-        <v>1606316</v>
+        <v>942561</v>
       </c>
       <c r="Q2" t="n">
-        <v>2060.1</v>
+        <v>2064.9</v>
       </c>
       <c r="R2" t="n">
-        <v>2261.8</v>
+        <v>2262.71</v>
       </c>
       <c r="S2" t="n">
-        <v>1959.25</v>
+        <v>1966</v>
       </c>
       <c r="T2" t="n">
-        <v>9.790786855007052</v>
+        <v>9.579640660564673</v>
       </c>
       <c r="U2" t="n">
-        <v>201.7000000000003</v>
+        <v>197.8099999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.895393427503516</v>
+        <v>4.789578187805709</v>
       </c>
       <c r="W2" t="n">
-        <v>100.8499999999999</v>
+        <v>98.90000000000009</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000000000000004</v>
+        <v>2.000101112234578</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.790786855007052</v>
+        <v>9.579640660564673</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.895393427503516</v>
+        <v>4.789578187805709</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02041972787390557</v>
+        <v>0.02040536832899545</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3241531307638069</v>
+        <v>0.3239251800551735</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02903743862256058</v>
+        <v>0.02903131967906458</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228669642138508</v>
+        <v>0.04228670559729215</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.07</v>
+        <v>39.09</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-16 20:18:34.247300+05:30</t>
+          <t>2026-10-19 14:29:28.628052+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.790786855007052, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0000000000000044}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.579640660564673, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000101112234578}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-19 16:58 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="18" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="17" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.65</v>
+        <v>11.7</v>
       </c>
       <c r="R2" t="n">
-        <v>48.7</v>
+        <v>48.75</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1884,22 +1884,22 @@
         <v>2052.2</v>
       </c>
       <c r="X2" t="n">
-        <v>2064.9</v>
+        <v>2069</v>
       </c>
       <c r="Y2" t="n">
-        <v>2064.9</v>
+        <v>2069</v>
       </c>
       <c r="Z2" t="n">
-        <v>942561</v>
+        <v>1132511</v>
       </c>
       <c r="AA2" t="n">
-        <v>1459117</v>
+        <v>1468615</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.65</v>
+        <v>0.77</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.23</v>
+        <v>0.43</v>
       </c>
       <c r="AD2" t="n">
         <v>0</v>
@@ -1926,47 +1926,47 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>2.06</v>
+        <v>2.26</v>
       </c>
       <c r="AM2" t="n">
-        <v>6.72</v>
+        <v>6.93</v>
       </c>
       <c r="AN2" t="n">
-        <v>46.61</v>
+        <v>46.9</v>
       </c>
       <c r="AO2" t="n">
-        <v>61.01</v>
+        <v>61.47</v>
       </c>
       <c r="AP2" t="n">
-        <v>4.74</v>
+        <v>4.95</v>
       </c>
       <c r="AQ2" t="n">
-        <v>32.46</v>
+        <v>32.72</v>
       </c>
       <c r="AR2" t="n">
-        <v>2064.9</v>
+        <v>2069</v>
       </c>
       <c r="AS2" t="n">
-        <v>2262.71</v>
+        <v>2266.81</v>
       </c>
       <c r="AT2" t="n">
-        <v>1966</v>
+        <v>1970.1</v>
       </c>
       <c r="AU2" t="n">
-        <v>2064.89990234375</v>
+        <v>2069</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.58</v>
+        <v>9.56</v>
       </c>
       <c r="AY2" t="n">
         <v>197.81</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.79</v>
+        <v>4.78</v>
       </c>
       <c r="BA2" t="n">
         <v>98.90000000000001</v>
@@ -2014,7 +2014,7 @@
         <v>2.18</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.449999999999999</v>
+        <v>8.460000000000001</v>
       </c>
       <c r="BQ2" t="n">
         <v>-4.27</v>
@@ -2023,13 +2023,13 @@
         <v>9</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.24</v>
+        <v>0.241</v>
       </c>
       <c r="BT2" t="n">
-        <v>1472.52</v>
+        <v>1474.78</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.23</v>
+        <v>-13.19</v>
       </c>
       <c r="BV2" t="n">
         <v>2.03</v>
@@ -2088,10 +2088,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>88.91</v>
+        <v>88.48999999999999</v>
       </c>
       <c r="CO2" t="n">
-        <v>39.37</v>
+        <v>37.63</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2115,7 +2115,7 @@
         <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>77.27272727272727</v>
+        <v>72.72727272727273</v>
       </c>
       <c r="CX2" t="n">
         <v>59.09090909090909</v>
@@ -2124,7 +2124,7 @@
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.579599999999999</v>
+        <v>9.560700000000001</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,43 +2133,43 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6387</v>
+        <v>0.6373</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3193</v>
+        <v>0.3187</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0958</v>
+        <v>0.0956</v>
       </c>
       <c r="DF2" t="n">
         <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1161</v>
+        <v>1.1185</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0084</v>
+        <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.7896</v>
+        <v>4.7801</v>
       </c>
       <c r="DJ2" t="n">
-        <v>28.67</v>
+        <v>27.95</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.7896</v>
+        <v>4.7801</v>
       </c>
       <c r="DL2" t="n">
         <v>2.0001</v>
       </c>
       <c r="DM2" t="n">
-        <v>2.0042</v>
+        <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>4.0084</v>
+        <v>4</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0003</v>
+        <v>1.9997</v>
       </c>
       <c r="DP2" t="n">
         <v>0.8368</v>
@@ -2178,7 +2178,7 @@
         <v>98.90000000000001</v>
       </c>
       <c r="DR2" t="n">
-        <v>67.41</v>
+        <v>61.29</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.9833</v>
+        <v>2.0711</v>
       </c>
       <c r="DX2" t="n">
-        <v>97.47500000000001</v>
+        <v>96.325</v>
       </c>
       <c r="DY2" t="n">
-        <v>32.5</v>
+        <v>38.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>90.20999999999999</v>
+        <v>90.279</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>93.72</v>
+        <v>94.75</v>
       </c>
       <c r="ED2" t="n">
-        <v>100</v>
+        <v>99.92</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.9833</v>
+        <v>2.0711</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.65</v>
+        <v>0.77</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.5522</v>
+        <v>0.5790999999999999</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0082</v>
+        <v>4.0003</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0643</v>
+        <v>0.0678</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6923</v>
+        <v>0.6921</v>
       </c>
       <c r="EK2" t="n">
-        <v>87.20999999999999</v>
+        <v>82.81</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2249,34 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>20.94</v>
+        <v>18.54</v>
       </c>
       <c r="EP2" t="n">
-        <v>2.4395</v>
+        <v>2.1692</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0757</v>
+        <v>0.0901</v>
       </c>
       <c r="ER2" t="n">
-        <v>14.7385</v>
+        <v>12.4156</v>
       </c>
       <c r="ES2" t="n">
-        <v>8.4572</v>
+        <v>8.2448</v>
       </c>
       <c r="ET2" t="n">
-        <v>41.029</v>
+        <v>39.682</v>
       </c>
       <c r="EU2" t="n">
-        <v>3.081</v>
+        <v>3.8115</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.4485</v>
+        <v>1.3503</v>
       </c>
       <c r="EW2" t="n">
-        <v>18.6178</v>
+        <v>16.406</v>
       </c>
       <c r="EX2" t="n">
-        <v>63.15</v>
+        <v>62.34</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2290,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.33</v>
+        <v>63.56</v>
       </c>
       <c r="FC2" t="n">
-        <v>17.24</v>
+        <v>16.52</v>
       </c>
       <c r="FD2" t="n">
         <v>70.06999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>88.06</v>
+        <v>85.65000000000001</v>
       </c>
       <c r="FF2" t="n">
-        <v>51.26</v>
+        <v>49.985</v>
       </c>
       <c r="FG2" t="n">
-        <v>26.2271</v>
+        <v>26.1032</v>
       </c>
       <c r="FH2" t="n">
-        <v>70.968</v>
+        <v>70.795</v>
       </c>
       <c r="FI2" t="n">
-        <v>48.04</v>
+        <v>44.62</v>
       </c>
       <c r="FJ2" t="n">
-        <v>68.76000000000001</v>
+        <v>66.98</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>81.48</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="FO2" t="n">
-        <v>67.22</v>
+        <v>63.59</v>
       </c>
       <c r="FP2" t="n">
-        <v>83.86</v>
+        <v>80.58</v>
       </c>
       <c r="FQ2" t="n">
-        <v>72.66</v>
+        <v>71.04000000000001</v>
       </c>
       <c r="FR2" t="n">
-        <v>92.66</v>
+        <v>87.89</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>74.494</v>
+        <v>70.727</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261019_142928</t>
+          <t>20261019_222819</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46314.60380311091</v>
+        <v>46314.93633222378</v>
       </c>
     </row>
   </sheetData>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46314.60379629629</v>
+        <v>46314.93633101852</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46314</v>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.65</v>
+        <v>11.7</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>2064.9</v>
+        <v>2069</v>
       </c>
       <c r="L2" t="n">
         <v>2060.1</v>
@@ -2693,28 +2693,28 @@
         <v>2052.2</v>
       </c>
       <c r="O2" t="n">
-        <v>2064.9</v>
+        <v>2069</v>
       </c>
       <c r="P2" t="n">
-        <v>942561</v>
+        <v>1132511</v>
       </c>
       <c r="Q2" t="n">
-        <v>2064.9</v>
+        <v>2069</v>
       </c>
       <c r="R2" t="n">
-        <v>2262.71</v>
+        <v>2266.81</v>
       </c>
       <c r="S2" t="n">
-        <v>1966</v>
+        <v>1970.1</v>
       </c>
       <c r="T2" t="n">
-        <v>9.579640660564673</v>
+        <v>9.560657322377958</v>
       </c>
       <c r="U2" t="n">
         <v>197.8099999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.789578187805709</v>
+        <v>4.780086998550029</v>
       </c>
       <c r="W2" t="n">
         <v>98.90000000000009</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.579640660564673</v>
+        <v>9.560657322377958</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.789578187805709</v>
+        <v>4.780086998550029</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02040536832899545</v>
+        <v>0.02040546308265652</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3239251800551735</v>
+        <v>0.3239266842229115</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02903131967906458</v>
+        <v>0.02903137198000025</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228670559729215</v>
+        <v>0.04228669670202969</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869492979645463</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-19 14:29:28.628052+05:30</t>
+          <t>2026-10-19 22:28:19.142152+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.579640660564673, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000101112234578}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.560657322377958, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000101112234578}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-20 08:38 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -1890,10 +1890,10 @@
         <v>2069</v>
       </c>
       <c r="Z2" t="n">
-        <v>1132511</v>
+        <v>1133053</v>
       </c>
       <c r="AA2" t="n">
-        <v>1468615</v>
+        <v>1468642</v>
       </c>
       <c r="AB2" t="n">
         <v>0.77</v>
@@ -2091,7 +2091,7 @@
         <v>88.48999999999999</v>
       </c>
       <c r="CO2" t="n">
-        <v>37.63</v>
+        <v>37.62</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2115,7 +2115,7 @@
         <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>72.72727272727273</v>
+        <v>77.27272727272727</v>
       </c>
       <c r="CX2" t="n">
         <v>59.09090909090909</v>
@@ -2264,7 +2264,7 @@
         <v>8.2448</v>
       </c>
       <c r="ET2" t="n">
-        <v>39.682</v>
+        <v>39.678</v>
       </c>
       <c r="EU2" t="n">
         <v>3.8115</v>
@@ -2302,7 +2302,7 @@
         <v>85.65000000000001</v>
       </c>
       <c r="FF2" t="n">
-        <v>49.985</v>
+        <v>49.98</v>
       </c>
       <c r="FG2" t="n">
         <v>26.1032</v>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261019_222819</t>
+          <t>20261020_140818</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46314.93633222378</v>
+        <v>46315.58910402795</v>
       </c>
     </row>
   </sheetData>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46314.93633101852</v>
+        <v>46315.58909722222</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46314</v>
@@ -2696,7 +2696,7 @@
         <v>2069</v>
       </c>
       <c r="P2" t="n">
-        <v>1132511</v>
+        <v>1133053</v>
       </c>
       <c r="Q2" t="n">
         <v>2069</v>
@@ -2726,13 +2726,13 @@
         <v>15</v>
       </c>
       <c r="Z2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AB2" t="n">
-        <v>0</v>
+        <v>6.666666666666667</v>
       </c>
       <c r="AC2" t="n">
         <v>0</v>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02040546308265652</v>
+        <v>0.02040546536817222</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3239266842229115</v>
+        <v>0.3239267205043485</v>
       </c>
     </row>
     <row r="7">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228669670202969</v>
+        <v>0.04228670026262123</v>
       </c>
     </row>
     <row r="13">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-19 22:28:19.142152+05:30</t>
+          <t>2026-10-20 14:08:18.627117+05:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-20 15:01 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -2026,7 +2026,7 @@
         <v>0.241</v>
       </c>
       <c r="BT2" t="n">
-        <v>1474.78</v>
+        <v>1474.8</v>
       </c>
       <c r="BU2" t="n">
         <v>-13.19</v>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261020_140818</t>
+          <t>20261020_203131</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46315.58910402795</v>
+        <v>46315.85522760463</v>
       </c>
     </row>
   </sheetData>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46315.58909722222</v>
+        <v>46315.8552199074</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46314</v>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02040546536817222</v>
+        <v>0.02040546296035075</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3239267205043485</v>
+        <v>0.3239266822813676</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02903137198000025</v>
+        <v>0.02903142418811971</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228670026262123</v>
+        <v>0.04228670352865471</v>
       </c>
     </row>
     <row r="13">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-20 14:08:18.627117+05:30</t>
+          <t>2026-10-20 20:31:31.706918+05:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-21 08:39 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46314</v>
+        <v>46316</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46314</v>
+        <v>46316</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46314</v>
+        <v>46316</v>
       </c>
       <c r="H2" t="n">
         <v>8.800000000000001</v>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.7</v>
+        <v>10.96</v>
       </c>
       <c r="R2" t="n">
-        <v>48.75</v>
+        <v>48.29</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>2060.1</v>
+        <v>2052.9</v>
       </c>
       <c r="V2" t="n">
-        <v>2089</v>
+        <v>2079.8</v>
       </c>
       <c r="W2" t="n">
-        <v>2052.2</v>
+        <v>2003.2</v>
       </c>
       <c r="X2" t="n">
-        <v>2069</v>
+        <v>2004.4</v>
       </c>
       <c r="Y2" t="n">
-        <v>2069</v>
+        <v>2004.4</v>
       </c>
       <c r="Z2" t="n">
-        <v>1133053</v>
+        <v>872558</v>
       </c>
       <c r="AA2" t="n">
-        <v>1468642</v>
+        <v>1403757</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.77</v>
+        <v>0.62</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.43</v>
+        <v>-3.12</v>
       </c>
       <c r="AD2" t="n">
-        <v>0</v>
+        <v>-0.78</v>
       </c>
       <c r="AE2" t="n">
-        <v>36.8</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.78</v>
+        <v>3.82</v>
       </c>
       <c r="AG2" t="n">
-        <v>49.45</v>
+        <v>51.39</v>
       </c>
       <c r="AH2" t="n">
-        <v>49.45</v>
+        <v>51.39</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.39</v>
+        <v>2.56</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,119 +1926,119 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>2.26</v>
+        <v>-0.9</v>
       </c>
       <c r="AM2" t="n">
-        <v>6.93</v>
+        <v>3.42</v>
       </c>
       <c r="AN2" t="n">
-        <v>46.9</v>
+        <v>41.84</v>
       </c>
       <c r="AO2" t="n">
-        <v>61.47</v>
+        <v>51.2</v>
       </c>
       <c r="AP2" t="n">
-        <v>4.95</v>
+        <v>-2.22</v>
       </c>
       <c r="AQ2" t="n">
-        <v>32.72</v>
+        <v>25.81</v>
       </c>
       <c r="AR2" t="n">
-        <v>2069</v>
+        <v>2004.4</v>
       </c>
       <c r="AS2" t="n">
-        <v>2266.81</v>
+        <v>2209.96</v>
       </c>
       <c r="AT2" t="n">
-        <v>1970.1</v>
+        <v>1901.62</v>
       </c>
       <c r="AU2" t="n">
-        <v>2069</v>
+        <v>2004.400024414062</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>9.56</v>
+        <v>10.26</v>
       </c>
       <c r="AY2" t="n">
-        <v>197.81</v>
+        <v>205.56</v>
       </c>
       <c r="AZ2" t="n">
-        <v>4.78</v>
+        <v>5.13</v>
       </c>
       <c r="BA2" t="n">
-        <v>98.90000000000001</v>
+        <v>102.78</v>
       </c>
       <c r="BB2" t="n">
-        <v>1.98</v>
+        <v>2.06</v>
       </c>
       <c r="BC2" t="n">
         <v>213</v>
       </c>
       <c r="BD2" t="n">
-        <v>31.5</v>
+        <v>31.4</v>
       </c>
       <c r="BE2" t="n">
         <v>329</v>
       </c>
       <c r="BF2" t="n">
-        <v>48.6</v>
+        <v>48.5</v>
       </c>
       <c r="BG2" t="n">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="BH2" t="n">
-        <v>19.9</v>
+        <v>18.4</v>
       </c>
       <c r="BI2" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="BM2" t="n">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="BN2" t="n">
-        <v>50.7</v>
+        <v>49.1</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.18</v>
+        <v>2.11</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.460000000000001</v>
+        <v>8.65</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.27</v>
+        <v>-4.19</v>
       </c>
       <c r="BR2" t="n">
-        <v>9</v>
+        <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.241</v>
+        <v>0.233</v>
       </c>
       <c r="BT2" t="n">
-        <v>1474.8</v>
+        <v>1432.79</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.19</v>
+        <v>-13.73</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.03</v>
+        <v>1.99</v>
       </c>
       <c r="BW2" t="n">
-        <v>1.98</v>
+        <v>2.06</v>
       </c>
       <c r="BX2" t="n">
-        <v>2.0001</v>
+        <v>2</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>43.6</v>
+        <v>42.2</v>
       </c>
       <c r="CE2" t="n">
-        <v>51.5</v>
+        <v>49.5</v>
       </c>
       <c r="CF2" t="n">
-        <v>66</v>
+        <v>68.7</v>
       </c>
       <c r="CG2" t="n">
-        <v>72.40000000000001</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,43 +2088,43 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>88.48999999999999</v>
+        <v>96.55</v>
       </c>
       <c r="CO2" t="n">
-        <v>37.62</v>
+        <v>35.8</v>
       </c>
       <c r="CP2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CQ2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CR2" t="n">
-        <v>86.36363636363636</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="CS2" t="n">
         <v>100</v>
       </c>
       <c r="CT2" t="n">
-        <v>100</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CU2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CV2" t="n">
-        <v>86.36363636363636</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="CW2" t="n">
-        <v>77.27272727272727</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="CX2" t="n">
-        <v>59.09090909090909</v>
+        <v>57.14285714285714</v>
       </c>
       <c r="CY2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CZ2" t="n">
-        <v>9.560700000000001</v>
+        <v>10.2554</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,52 +2133,52 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6373</v>
+        <v>0.6840000000000001</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3187</v>
+        <v>0.342</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.0956</v>
+        <v>0.1026</v>
       </c>
       <c r="DF2" t="n">
         <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1185</v>
+        <v>1.1245</v>
       </c>
       <c r="DH2" t="n">
-        <v>4</v>
+        <v>4.0078</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.7801</v>
+        <v>5.1277</v>
       </c>
       <c r="DJ2" t="n">
-        <v>27.95</v>
+        <v>31.54</v>
       </c>
       <c r="DK2" t="n">
-        <v>4.7801</v>
+        <v>5.1277</v>
       </c>
       <c r="DL2" t="n">
-        <v>2.0001</v>
+        <v>2</v>
       </c>
       <c r="DM2" t="n">
+        <v>2.0039</v>
+      </c>
+      <c r="DN2" t="n">
+        <v>4.0078</v>
+      </c>
+      <c r="DO2" t="n">
         <v>2</v>
       </c>
-      <c r="DN2" t="n">
-        <v>4</v>
-      </c>
-      <c r="DO2" t="n">
-        <v>1.9997</v>
-      </c>
       <c r="DP2" t="n">
-        <v>0.8368</v>
+        <v>0.7812</v>
       </c>
       <c r="DQ2" t="n">
-        <v>98.90000000000001</v>
+        <v>102.78</v>
       </c>
       <c r="DR2" t="n">
-        <v>61.29</v>
+        <v>66.31999999999999</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>2.0711</v>
+        <v>-0.8672</v>
       </c>
       <c r="DX2" t="n">
-        <v>96.325</v>
+        <v>78</v>
       </c>
       <c r="DY2" t="n">
-        <v>38.5</v>
+        <v>31</v>
       </c>
       <c r="DZ2" t="n">
-        <v>90.279</v>
+        <v>86.53100000000001</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>94.75</v>
+        <v>85.84</v>
       </c>
       <c r="ED2" t="n">
-        <v>99.92</v>
+        <v>98.81999999999999</v>
       </c>
       <c r="EE2" t="n">
-        <v>2.0711</v>
+        <v>-0.8672</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.77</v>
+        <v>0.62</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.5790999999999999</v>
+        <v>-0.2433</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0003</v>
+        <v>4.006</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0678</v>
+        <v>-0.0267</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6921</v>
+        <v>0.6535</v>
       </c>
       <c r="EK2" t="n">
-        <v>82.81</v>
+        <v>87.33</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,38 +2249,38 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>18.54</v>
+        <v>10.15</v>
       </c>
       <c r="EP2" t="n">
-        <v>2.1692</v>
+        <v>1.1124</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0901</v>
+        <v>0.068</v>
       </c>
       <c r="ER2" t="n">
-        <v>12.4156</v>
+        <v>16.5484</v>
       </c>
       <c r="ES2" t="n">
-        <v>8.2448</v>
+        <v>8.8596</v>
       </c>
       <c r="ET2" t="n">
-        <v>39.678</v>
+        <v>35.29</v>
       </c>
       <c r="EU2" t="n">
-        <v>3.8115</v>
+        <v>-1.3764</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.3503</v>
+        <v>1.5802</v>
       </c>
       <c r="EW2" t="n">
-        <v>16.406</v>
+        <v>9.799799999999999</v>
       </c>
       <c r="EX2" t="n">
-        <v>62.34</v>
+        <v>47.77</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="EZ2" t="n">
@@ -2290,31 +2290,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>63.56</v>
+        <v>59.75</v>
       </c>
       <c r="FC2" t="n">
-        <v>16.52</v>
+        <v>20.85</v>
       </c>
       <c r="FD2" t="n">
-        <v>70.06999999999999</v>
+        <v>74.18000000000001</v>
       </c>
       <c r="FE2" t="n">
-        <v>85.65000000000001</v>
+        <v>91.94</v>
       </c>
       <c r="FF2" t="n">
-        <v>49.98</v>
+        <v>41.785</v>
       </c>
       <c r="FG2" t="n">
-        <v>26.1032</v>
+        <v>27.1208</v>
       </c>
       <c r="FH2" t="n">
-        <v>70.795</v>
+        <v>68.39400000000001</v>
       </c>
       <c r="FI2" t="n">
-        <v>44.62</v>
+        <v>48.93</v>
       </c>
       <c r="FJ2" t="n">
-        <v>66.98</v>
+        <v>68.84</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>78.09999999999999</v>
+        <v>78.62</v>
       </c>
       <c r="FO2" t="n">
-        <v>63.59</v>
+        <v>67.29000000000001</v>
       </c>
       <c r="FP2" t="n">
-        <v>80.58</v>
+        <v>71.26000000000001</v>
       </c>
       <c r="FQ2" t="n">
-        <v>71.04000000000001</v>
+        <v>73.84999999999999</v>
       </c>
       <c r="FR2" t="n">
-        <v>87.89</v>
+        <v>85.77</v>
       </c>
       <c r="FS2" t="n">
-        <v>100</v>
+        <v>90.47620000000001</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>70.727</v>
+        <v>71.33199999999999</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261020_203131</t>
+          <t>20261021_140925</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46315.85522760463</v>
+        <v>46316.58987897106</v>
       </c>
     </row>
   </sheetData>
@@ -2466,7 +2466,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="19" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46315.8552199074</v>
+        <v>46316.58987268519</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46314</v>
+        <v>46316</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46329</v>
+        <v>46331</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11.7</v>
+        <v>10.96</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,58 +2681,58 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>2069</v>
+        <v>2004.4</v>
       </c>
       <c r="L2" t="n">
-        <v>2060.1</v>
+        <v>2052.9</v>
       </c>
       <c r="M2" t="n">
-        <v>2089</v>
+        <v>2079.8</v>
       </c>
       <c r="N2" t="n">
-        <v>2052.2</v>
+        <v>2003.2</v>
       </c>
       <c r="O2" t="n">
-        <v>2069</v>
+        <v>2004.4</v>
       </c>
       <c r="P2" t="n">
-        <v>1133053</v>
+        <v>872558</v>
       </c>
       <c r="Q2" t="n">
-        <v>2069</v>
+        <v>2004.4</v>
       </c>
       <c r="R2" t="n">
-        <v>2266.81</v>
+        <v>2209.96</v>
       </c>
       <c r="S2" t="n">
-        <v>1970.1</v>
+        <v>1901.62</v>
       </c>
       <c r="T2" t="n">
-        <v>9.560657322377958</v>
+        <v>10.25543803632009</v>
       </c>
       <c r="U2" t="n">
-        <v>197.8099999999999</v>
+        <v>205.5599999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>4.780086998550029</v>
+        <v>5.127719018160057</v>
       </c>
       <c r="W2" t="n">
-        <v>98.90000000000009</v>
+        <v>102.7800000000002</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000101112234578</v>
+        <v>1.999999999999996</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
       </c>
       <c r="Z2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="AB2" t="n">
-        <v>6.666666666666667</v>
+        <v>0</v>
       </c>
       <c r="AC2" t="n">
         <v>0</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>9.560657322377958</v>
+        <v>10.25543803632009</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.780086998550029</v>
+        <v>5.127719018160057</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02040546296035075</v>
+        <v>0.02043047426352121</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3239266822813676</v>
+        <v>0.3243237244102957</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02903142418811971</v>
+        <v>0.02909805661883564</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228670352865471</v>
+        <v>0.04234573888804577</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645463</v>
+        <v>0.1869493934347613</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.09</v>
+        <v>39.05</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-20 20:31:31.706918+05:30</t>
+          <t>2026-10-21 14:09:25.580622+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 9.560657322377958, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000101112234578}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.255438036320093, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9999999999999956}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-21 15:12 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="20" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>10.96</v>
+        <v>11</v>
       </c>
       <c r="R2" t="n">
-        <v>48.29</v>
+        <v>48.53</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1881,43 +1881,43 @@
         <v>2079.8</v>
       </c>
       <c r="W2" t="n">
-        <v>2003.2</v>
+        <v>1993.4</v>
       </c>
       <c r="X2" t="n">
-        <v>2004.4</v>
+        <v>2012.5</v>
       </c>
       <c r="Y2" t="n">
-        <v>2004.4</v>
+        <v>2012.5</v>
       </c>
       <c r="Z2" t="n">
-        <v>872558</v>
+        <v>1273804</v>
       </c>
       <c r="AA2" t="n">
-        <v>1403757</v>
+        <v>1423819</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.62</v>
+        <v>0.89</v>
       </c>
       <c r="AC2" t="n">
-        <v>-3.12</v>
+        <v>-2.73</v>
       </c>
       <c r="AD2" t="n">
         <v>-0.78</v>
       </c>
       <c r="AE2" t="n">
-        <v>76.59999999999999</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="AF2" t="n">
-        <v>3.82</v>
+        <v>4.29</v>
       </c>
       <c r="AG2" t="n">
-        <v>51.39</v>
+        <v>52.09</v>
       </c>
       <c r="AH2" t="n">
-        <v>51.39</v>
+        <v>52.09</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.56</v>
+        <v>2.59</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,53 +1926,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>-0.9</v>
+        <v>-0.52</v>
       </c>
       <c r="AM2" t="n">
-        <v>3.42</v>
+        <v>3.83</v>
       </c>
       <c r="AN2" t="n">
-        <v>41.84</v>
+        <v>42.41</v>
       </c>
       <c r="AO2" t="n">
-        <v>51.2</v>
+        <v>52.29</v>
       </c>
       <c r="AP2" t="n">
-        <v>-2.22</v>
+        <v>-1.83</v>
       </c>
       <c r="AQ2" t="n">
-        <v>25.81</v>
+        <v>26.32</v>
       </c>
       <c r="AR2" t="n">
-        <v>2004.4</v>
+        <v>2012.5</v>
       </c>
       <c r="AS2" t="n">
-        <v>2209.96</v>
+        <v>2220.86</v>
       </c>
       <c r="AT2" t="n">
-        <v>1901.62</v>
+        <v>1908.32</v>
       </c>
       <c r="AU2" t="n">
-        <v>2004.400024414062</v>
+        <v>2012.5</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>10.26</v>
+        <v>10.35</v>
       </c>
       <c r="AY2" t="n">
-        <v>205.56</v>
+        <v>208.36</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.13</v>
+        <v>5.18</v>
       </c>
       <c r="BA2" t="n">
-        <v>102.78</v>
+        <v>104.18</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.06</v>
+        <v>2.07</v>
       </c>
       <c r="BC2" t="n">
         <v>213</v>
@@ -2011,31 +2011,31 @@
         <v>49.1</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.11</v>
+        <v>2.12</v>
       </c>
       <c r="BP2" t="n">
         <v>8.65</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.19</v>
+        <v>-4.18</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.233</v>
+        <v>0.234</v>
       </c>
       <c r="BT2" t="n">
-        <v>1432.79</v>
+        <v>1437.67</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.73</v>
+        <v>-13.74</v>
       </c>
       <c r="BV2" t="n">
-        <v>1.99</v>
+        <v>2</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.06</v>
+        <v>2.07</v>
       </c>
       <c r="BX2" t="n">
         <v>2</v>
@@ -2058,13 +2058,13 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>42.2</v>
+        <v>42.4</v>
       </c>
       <c r="CE2" t="n">
-        <v>49.5</v>
+        <v>50</v>
       </c>
       <c r="CF2" t="n">
-        <v>68.7</v>
+        <v>69</v>
       </c>
       <c r="CG2" t="n">
         <v>70.09999999999999</v>
@@ -2088,43 +2088,43 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>96.55</v>
+        <v>93.14</v>
       </c>
       <c r="CO2" t="n">
-        <v>35.8</v>
+        <v>36.45</v>
       </c>
       <c r="CP2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CQ2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CR2" t="n">
-        <v>85.71428571428571</v>
+        <v>86.36363636363636</v>
       </c>
       <c r="CS2" t="n">
         <v>100</v>
       </c>
       <c r="CT2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CU2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CV2" t="n">
-        <v>85.71428571428571</v>
+        <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>66.66666666666666</v>
+        <v>68.18181818181817</v>
       </c>
       <c r="CX2" t="n">
-        <v>57.14285714285714</v>
+        <v>54.54545454545454</v>
       </c>
       <c r="CY2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>10.2554</v>
+        <v>10.3533</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6840000000000001</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.342</v>
+        <v>0.3453</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1026</v>
+        <v>0.1035</v>
       </c>
       <c r="DF2" t="n">
-        <v>2</v>
+        <v>1.9981</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1245</v>
+        <v>1.1385</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0078</v>
+        <v>3.9961</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.1277</v>
+        <v>5.1766</v>
       </c>
       <c r="DJ2" t="n">
-        <v>31.54</v>
+        <v>33.68</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.1277</v>
+        <v>5.1766</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>2.0039</v>
+        <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>4.0078</v>
+        <v>3.9961</v>
       </c>
       <c r="DO2" t="n">
-        <v>2</v>
+        <v>1.9983</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.7812</v>
+        <v>0.7715</v>
       </c>
       <c r="DQ2" t="n">
-        <v>102.78</v>
+        <v>104.18</v>
       </c>
       <c r="DR2" t="n">
-        <v>66.31999999999999</v>
+        <v>52.98</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>-0.8672</v>
+        <v>-0.7066</v>
       </c>
       <c r="DX2" t="n">
-        <v>78</v>
+        <v>80.72499999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>31</v>
+        <v>44.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>86.53100000000001</v>
+        <v>87.11499999999999</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2211,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>85.84</v>
+        <v>86.27</v>
       </c>
       <c r="ED2" t="n">
-        <v>98.81999999999999</v>
+        <v>100</v>
       </c>
       <c r="EE2" t="n">
-        <v>-0.8672</v>
+        <v>-0.7066</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.62</v>
+        <v>0.89</v>
       </c>
       <c r="EG2" t="n">
-        <v>-0.2433</v>
+        <v>-0.2013</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.006</v>
+        <v>3.9974</v>
       </c>
       <c r="EI2" t="n">
-        <v>-0.0267</v>
+        <v>-0.0221</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6535</v>
+        <v>0.6468</v>
       </c>
       <c r="EK2" t="n">
-        <v>87.33</v>
+        <v>85.55</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2249,34 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>10.15</v>
+        <v>12.34</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.1124</v>
+        <v>1.3574</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.068</v>
+        <v>0.0979</v>
       </c>
       <c r="ER2" t="n">
-        <v>16.5484</v>
+        <v>11.6292</v>
       </c>
       <c r="ES2" t="n">
-        <v>8.8596</v>
+        <v>9.381600000000001</v>
       </c>
       <c r="ET2" t="n">
-        <v>35.29</v>
+        <v>36.354</v>
       </c>
       <c r="EU2" t="n">
-        <v>-1.3764</v>
+        <v>-1.6287</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.5802</v>
+        <v>1.3704</v>
       </c>
       <c r="EW2" t="n">
-        <v>9.799799999999999</v>
+        <v>11.4935</v>
       </c>
       <c r="EX2" t="n">
-        <v>47.77</v>
+        <v>52.7</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2290,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>59.75</v>
+        <v>60.24</v>
       </c>
       <c r="FC2" t="n">
-        <v>20.85</v>
+        <v>22.8</v>
       </c>
       <c r="FD2" t="n">
-        <v>74.18000000000001</v>
+        <v>74.81999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>91.94</v>
+        <v>89.345</v>
       </c>
       <c r="FF2" t="n">
-        <v>41.785</v>
+        <v>44.575</v>
       </c>
       <c r="FG2" t="n">
-        <v>27.1208</v>
+        <v>25.9443</v>
       </c>
       <c r="FH2" t="n">
-        <v>68.39400000000001</v>
+        <v>68.602</v>
       </c>
       <c r="FI2" t="n">
-        <v>48.93</v>
+        <v>43.33</v>
       </c>
       <c r="FJ2" t="n">
-        <v>68.84</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2328,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>78.62</v>
+        <v>73.2</v>
       </c>
       <c r="FO2" t="n">
-        <v>67.29000000000001</v>
+        <v>65.44</v>
       </c>
       <c r="FP2" t="n">
-        <v>71.26000000000001</v>
+        <v>67.93000000000001</v>
       </c>
       <c r="FQ2" t="n">
-        <v>73.84999999999999</v>
+        <v>66.52</v>
       </c>
       <c r="FR2" t="n">
-        <v>85.77</v>
+        <v>82.05</v>
       </c>
       <c r="FS2" t="n">
-        <v>90.47620000000001</v>
+        <v>95.4545</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>71.33199999999999</v>
+        <v>67.404</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261021_140925</t>
+          <t>20261021_204203</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46316.58987897106</v>
+        <v>46316.86254281009</v>
       </c>
     </row>
   </sheetData>
@@ -2465,8 +2465,8 @@
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46316.58987268519</v>
+        <v>46316.86253472222</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46316</v>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>10.96</v>
+        <v>11</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>2004.4</v>
+        <v>2012.5</v>
       </c>
       <c r="L2" t="n">
         <v>2052.9</v>
@@ -2690,37 +2690,37 @@
         <v>2079.8</v>
       </c>
       <c r="N2" t="n">
-        <v>2003.2</v>
+        <v>1993.4</v>
       </c>
       <c r="O2" t="n">
-        <v>2004.4</v>
+        <v>2012.5</v>
       </c>
       <c r="P2" t="n">
-        <v>872558</v>
+        <v>1273804</v>
       </c>
       <c r="Q2" t="n">
-        <v>2004.4</v>
+        <v>2012.5</v>
       </c>
       <c r="R2" t="n">
-        <v>2209.96</v>
+        <v>2220.86</v>
       </c>
       <c r="S2" t="n">
-        <v>1901.62</v>
+        <v>1908.32</v>
       </c>
       <c r="T2" t="n">
-        <v>10.25543803632009</v>
+        <v>10.35329192546584</v>
       </c>
       <c r="U2" t="n">
-        <v>205.5599999999999</v>
+        <v>208.3600000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>5.127719018160057</v>
+        <v>5.176645962732922</v>
       </c>
       <c r="W2" t="n">
-        <v>102.7800000000002</v>
+        <v>104.1800000000001</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999999999999996</v>
+        <v>2</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>10.25543803632009</v>
+        <v>10.35329192546584</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.127719018160057</v>
+        <v>5.176645962732922</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02043047426352121</v>
+        <v>0.02042190229720003</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3243237244102957</v>
+        <v>0.3241876486634998</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02909805661883564</v>
+        <v>0.02902530599490038</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04234573888804577</v>
+        <v>0.04228670266997363</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347613</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.05</v>
+        <v>39.06</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-21 14:09:25.580622+05:30</t>
+          <t>2026-10-21 20:42:03.737033+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.255438036320093, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9999999999999956}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.353291925465845, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-22 08:41 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="17" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,16 +1816,14 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46316</v>
-      </c>
-      <c r="E2" s="1" t="n">
-        <v>46316</v>
-      </c>
+        <v>46317</v>
+      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="H2" t="n">
         <v>8.800000000000001</v>
@@ -1854,70 +1852,66 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="P2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>11</v>
+        <v>10.82</v>
       </c>
       <c r="R2" t="n">
-        <v>48.53</v>
+        <v>48.25</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
       </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>UPTREND</t>
-        </is>
-      </c>
+      <c r="T2" t="inlineStr"/>
       <c r="U2" t="n">
-        <v>2052.9</v>
+        <v>1993.5</v>
       </c>
       <c r="V2" t="n">
-        <v>2079.8</v>
+        <v>2019.8</v>
       </c>
       <c r="W2" t="n">
-        <v>1993.4</v>
+        <v>1956.6</v>
       </c>
       <c r="X2" t="n">
-        <v>2012.5</v>
+        <v>2007.6</v>
       </c>
       <c r="Y2" t="n">
-        <v>2012.5</v>
+        <v>2007.6</v>
       </c>
       <c r="Z2" t="n">
-        <v>1273804</v>
+        <v>1224584</v>
       </c>
       <c r="AA2" t="n">
-        <v>1423819</v>
+        <v>1410798</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.89</v>
+        <v>0.87</v>
       </c>
       <c r="AC2" t="n">
-        <v>-2.73</v>
+        <v>-0.24</v>
       </c>
       <c r="AD2" t="n">
-        <v>-0.78</v>
+        <v>-0.9399999999999999</v>
       </c>
       <c r="AE2" t="n">
-        <v>86.40000000000001</v>
+        <v>63.2</v>
       </c>
       <c r="AF2" t="n">
-        <v>4.29</v>
+        <v>3.15</v>
       </c>
       <c r="AG2" t="n">
-        <v>52.09</v>
+        <v>52.88</v>
       </c>
       <c r="AH2" t="n">
-        <v>52.09</v>
+        <v>52.88</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.59</v>
+        <v>2.63</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,53 +1920,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>-0.52</v>
+        <v>-0.77</v>
       </c>
       <c r="AM2" t="n">
-        <v>3.83</v>
+        <v>3.41</v>
       </c>
       <c r="AN2" t="n">
-        <v>42.41</v>
+        <v>41.61</v>
       </c>
       <c r="AO2" t="n">
-        <v>52.29</v>
+        <v>51.58</v>
       </c>
       <c r="AP2" t="n">
-        <v>-1.83</v>
+        <v>-2.2</v>
       </c>
       <c r="AQ2" t="n">
-        <v>26.32</v>
+        <v>27.24</v>
       </c>
       <c r="AR2" t="n">
-        <v>2012.5</v>
+        <v>2007.6</v>
       </c>
       <c r="AS2" t="n">
-        <v>2220.86</v>
+        <v>2219.14</v>
       </c>
       <c r="AT2" t="n">
-        <v>1908.32</v>
+        <v>1901.83</v>
       </c>
       <c r="AU2" t="n">
-        <v>2012.5</v>
+        <v>2007.599975585938</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>10.35</v>
+        <v>10.54</v>
       </c>
       <c r="AY2" t="n">
-        <v>208.36</v>
+        <v>211.54</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.18</v>
+        <v>5.27</v>
       </c>
       <c r="BA2" t="n">
-        <v>104.18</v>
+        <v>105.77</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.07</v>
+        <v>2.06</v>
       </c>
       <c r="BC2" t="n">
         <v>213</v>
@@ -1981,61 +1975,61 @@
         <v>31.4</v>
       </c>
       <c r="BE2" t="n">
-        <v>329</v>
+        <v>342</v>
       </c>
       <c r="BF2" t="n">
-        <v>48.5</v>
+        <v>50.4</v>
       </c>
       <c r="BG2" t="n">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.4</v>
+        <v>18.3</v>
       </c>
       <c r="BI2" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="BJ2" t="n">
-        <v>1.6</v>
+        <v>0</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="BM2" t="n">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="BN2" t="n">
-        <v>49.1</v>
+        <v>48.9</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.12</v>
+        <v>2.09</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.65</v>
+        <v>8.67</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.18</v>
+        <v>-4.2</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.234</v>
+        <v>0.231</v>
       </c>
       <c r="BT2" t="n">
-        <v>1437.67</v>
+        <v>1421.99</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.74</v>
+        <v>-13.85</v>
       </c>
       <c r="BV2" t="n">
-        <v>2</v>
+        <v>1.98</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.07</v>
+        <v>2.06</v>
       </c>
       <c r="BX2" t="n">
         <v>2</v>
@@ -2047,7 +2041,7 @@
         <v>8</v>
       </c>
       <c r="CA2" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="CB2" t="n">
         <v>0</v>
@@ -2058,16 +2052,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>42.4</v>
+        <v>41.8</v>
       </c>
       <c r="CE2" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="CF2" t="n">
-        <v>69</v>
+        <v>68.7</v>
       </c>
       <c r="CG2" t="n">
-        <v>70.09999999999999</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2088,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>93.14</v>
+        <v>85.45999999999999</v>
       </c>
       <c r="CO2" t="n">
-        <v>36.45</v>
+        <v>36.79</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2121,10 +2115,10 @@
         <v>54.54545454545454</v>
       </c>
       <c r="CY2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>10.3533</v>
+        <v>10.537</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2127,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.7027</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3453</v>
+        <v>0.3513</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1035</v>
+        <v>0.1054</v>
       </c>
       <c r="DF2" t="n">
-        <v>1.9981</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1385</v>
+        <v>1.1404</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9961</v>
+        <v>4.0076</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.1766</v>
+        <v>5.2685</v>
       </c>
       <c r="DJ2" t="n">
-        <v>33.68</v>
+        <v>33.97</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.1766</v>
+        <v>5.2685</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>2</v>
+        <v>2.0038</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9961</v>
+        <v>4.0076</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9983</v>
+        <v>2.0003</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.7715</v>
+        <v>0.7605</v>
       </c>
       <c r="DQ2" t="n">
-        <v>104.18</v>
+        <v>105.77</v>
       </c>
       <c r="DR2" t="n">
-        <v>52.98</v>
+        <v>72.06</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2187,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>-0.7066</v>
+        <v>-0.8365</v>
       </c>
       <c r="DX2" t="n">
-        <v>80.72499999999999</v>
+        <v>78.94999999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>44.5</v>
+        <v>43.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>87.11499999999999</v>
+        <v>85.61799999999999</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2211,31 +2205,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>86.27</v>
+        <v>80.08</v>
       </c>
       <c r="ED2" t="n">
-        <v>100</v>
+        <v>97.03</v>
       </c>
       <c r="EE2" t="n">
-        <v>-0.7066</v>
+        <v>-0.8365</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.89</v>
+        <v>0.87</v>
       </c>
       <c r="EG2" t="n">
-        <v>-0.2013</v>
+        <v>-0.238</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9974</v>
+        <v>4.0065</v>
       </c>
       <c r="EI2" t="n">
-        <v>-0.0221</v>
+        <v>-0.0258</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6468</v>
+        <v>0.639</v>
       </c>
       <c r="EK2" t="n">
-        <v>85.55</v>
+        <v>80.23999999999999</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2243,34 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>12.34</v>
+        <v>21.88</v>
       </c>
       <c r="EP2" t="n">
-        <v>1.3574</v>
+        <v>2.3674</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0979</v>
+        <v>0.0941</v>
       </c>
       <c r="ER2" t="n">
-        <v>11.6292</v>
+        <v>12.1149</v>
       </c>
       <c r="ES2" t="n">
-        <v>9.381600000000001</v>
+        <v>9.3581</v>
       </c>
       <c r="ET2" t="n">
-        <v>36.354</v>
+        <v>39.094</v>
       </c>
       <c r="EU2" t="n">
-        <v>-1.6287</v>
+        <v>-1.914</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.3704</v>
+        <v>1.4064</v>
       </c>
       <c r="EW2" t="n">
-        <v>11.4935</v>
+        <v>18.6986</v>
       </c>
       <c r="EX2" t="n">
-        <v>52.7</v>
+        <v>56.27</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2284,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>60.24</v>
+        <v>59.38</v>
       </c>
       <c r="FC2" t="n">
-        <v>22.8</v>
+        <v>22.5</v>
       </c>
       <c r="FD2" t="n">
-        <v>74.81999999999999</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="FE2" t="n">
-        <v>89.345</v>
+        <v>82.84999999999999</v>
       </c>
       <c r="FF2" t="n">
-        <v>44.575</v>
+        <v>46.53</v>
       </c>
       <c r="FG2" t="n">
-        <v>25.9443</v>
+        <v>23.5427</v>
       </c>
       <c r="FH2" t="n">
-        <v>68.602</v>
+        <v>66.58199999999999</v>
       </c>
       <c r="FI2" t="n">
-        <v>43.33</v>
+        <v>53.015</v>
       </c>
       <c r="FJ2" t="n">
-        <v>66.90000000000001</v>
+        <v>66.91</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,22 +2322,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>73.2</v>
+        <v>79.72</v>
       </c>
       <c r="FO2" t="n">
-        <v>65.44</v>
+        <v>63.56</v>
       </c>
       <c r="FP2" t="n">
-        <v>67.93000000000001</v>
+        <v>82.26000000000001</v>
       </c>
       <c r="FQ2" t="n">
-        <v>66.52</v>
+        <v>76.42</v>
       </c>
       <c r="FR2" t="n">
-        <v>82.05</v>
+        <v>88.98999999999999</v>
       </c>
       <c r="FS2" t="n">
-        <v>95.4545</v>
+        <v>100</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2357,7 +2351,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>67.404</v>
+        <v>73.78149999999999</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261021_204203</t>
+          <t>20261022_141137</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46316.86254281009</v>
+        <v>46317.59140913087</v>
       </c>
     </row>
   </sheetData>
@@ -2444,8 +2438,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -2647,14 +2641,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46316.86253472222</v>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>46316</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>46331</v>
-      </c>
+        <v>46317.59140046296</v>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>LAURUSLABS</t>
@@ -2673,51 +2663,47 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>11</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>UPTREND</t>
-        </is>
-      </c>
+        <v>10.82</v>
+      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>2012.5</v>
+        <v>2007.6</v>
       </c>
       <c r="L2" t="n">
-        <v>2052.9</v>
+        <v>1993.5</v>
       </c>
       <c r="M2" t="n">
-        <v>2079.8</v>
+        <v>2019.8</v>
       </c>
       <c r="N2" t="n">
-        <v>1993.4</v>
+        <v>1956.6</v>
       </c>
       <c r="O2" t="n">
-        <v>2012.5</v>
+        <v>2007.6</v>
       </c>
       <c r="P2" t="n">
-        <v>1273804</v>
+        <v>1224584</v>
       </c>
       <c r="Q2" t="n">
-        <v>2012.5</v>
+        <v>2007.6</v>
       </c>
       <c r="R2" t="n">
-        <v>2220.86</v>
+        <v>2219.14</v>
       </c>
       <c r="S2" t="n">
-        <v>1908.32</v>
+        <v>1901.83</v>
       </c>
       <c r="T2" t="n">
-        <v>10.35329192546584</v>
+        <v>10.53695955369595</v>
       </c>
       <c r="U2" t="n">
-        <v>208.3600000000001</v>
+        <v>211.54</v>
       </c>
       <c r="V2" t="n">
-        <v>5.176645962732922</v>
+        <v>5.268479776847977</v>
       </c>
       <c r="W2" t="n">
-        <v>104.1800000000001</v>
+        <v>105.77</v>
       </c>
       <c r="X2" t="n">
         <v>2</v>
@@ -2741,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>10.35329192546584</v>
+        <v>10.53695955369595</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.176645962732922</v>
+        <v>5.268479776847977</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02042190229720003</v>
+        <v>0.02039200714825264</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3241876486634998</v>
+        <v>0.3237130778863675</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02902530599490038</v>
+        <v>0.02902540975367884</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228670266997363</v>
+        <v>0.04228670255183435</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869492979645464</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.06</v>
+        <v>39.1</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-21 20:42:03.737033+05:30</t>
+          <t>2026-10-22 14:11:37.788468+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.353291925465845, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.536959553695954, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-22 15:13 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="20" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="17" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1862,7 +1862,7 @@
         <v>10.82</v>
       </c>
       <c r="R2" t="n">
-        <v>48.25</v>
+        <v>48.34</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1878,22 +1878,22 @@
         <v>1956.6</v>
       </c>
       <c r="X2" t="n">
-        <v>2007.6</v>
+        <v>2002.5</v>
       </c>
       <c r="Y2" t="n">
-        <v>2007.6</v>
+        <v>2002.5</v>
       </c>
       <c r="Z2" t="n">
-        <v>1224584</v>
+        <v>1538706</v>
       </c>
       <c r="AA2" t="n">
-        <v>1410798</v>
+        <v>1426504</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.87</v>
+        <v>1.08</v>
       </c>
       <c r="AC2" t="n">
-        <v>-0.24</v>
+        <v>-0.5</v>
       </c>
       <c r="AD2" t="n">
         <v>-0.9399999999999999</v>
@@ -1902,7 +1902,7 @@
         <v>63.2</v>
       </c>
       <c r="AF2" t="n">
-        <v>3.15</v>
+        <v>3.16</v>
       </c>
       <c r="AG2" t="n">
         <v>52.88</v>
@@ -1911,7 +1911,7 @@
         <v>52.88</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.63</v>
+        <v>2.64</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,47 +1920,47 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>-0.77</v>
+        <v>-1.01</v>
       </c>
       <c r="AM2" t="n">
-        <v>3.41</v>
+        <v>3.16</v>
       </c>
       <c r="AN2" t="n">
-        <v>41.61</v>
+        <v>41.25</v>
       </c>
       <c r="AO2" t="n">
-        <v>51.58</v>
+        <v>50.85</v>
       </c>
       <c r="AP2" t="n">
-        <v>-2.2</v>
+        <v>-2.45</v>
       </c>
       <c r="AQ2" t="n">
-        <v>27.24</v>
+        <v>26.92</v>
       </c>
       <c r="AR2" t="n">
-        <v>2007.6</v>
+        <v>2002.5</v>
       </c>
       <c r="AS2" t="n">
-        <v>2219.14</v>
+        <v>2214.04</v>
       </c>
       <c r="AT2" t="n">
-        <v>1901.83</v>
+        <v>1896.73</v>
       </c>
       <c r="AU2" t="n">
-        <v>2007.599975585938</v>
+        <v>2002.5</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>10.54</v>
+        <v>10.56</v>
       </c>
       <c r="AY2" t="n">
         <v>211.54</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.27</v>
+        <v>5.28</v>
       </c>
       <c r="BA2" t="n">
         <v>105.77</v>
@@ -2020,10 +2020,10 @@
         <v>0.231</v>
       </c>
       <c r="BT2" t="n">
-        <v>1421.99</v>
+        <v>1421.77</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.85</v>
+        <v>-13.87</v>
       </c>
       <c r="BV2" t="n">
         <v>1.98</v>
@@ -2082,43 +2082,43 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>85.45999999999999</v>
+        <v>84.67</v>
       </c>
       <c r="CO2" t="n">
-        <v>36.79</v>
+        <v>36.37</v>
       </c>
       <c r="CP2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CQ2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CR2" t="n">
-        <v>86.36363636363636</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="CS2" t="n">
         <v>100</v>
       </c>
       <c r="CT2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CU2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CV2" t="n">
-        <v>86.36363636363636</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="CW2" t="n">
-        <v>68.18181818181817</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="CX2" t="n">
-        <v>54.54545454545454</v>
+        <v>57.14285714285714</v>
       </c>
       <c r="CY2" t="n">
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>10.537</v>
+        <v>10.5638</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,52 +2127,52 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.7027</v>
+        <v>0.704</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3513</v>
+        <v>0.352</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1054</v>
+        <v>0.1056</v>
       </c>
       <c r="DF2" t="n">
         <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1404</v>
+        <v>1.1426</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0076</v>
+        <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.2685</v>
+        <v>5.2819</v>
       </c>
       <c r="DJ2" t="n">
-        <v>33.97</v>
+        <v>34.44</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.2685</v>
+        <v>5.2819</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>2.0038</v>
+        <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>4.0076</v>
+        <v>4</v>
       </c>
       <c r="DO2" t="n">
-        <v>2.0003</v>
+        <v>2</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.7605</v>
+        <v>0.7576000000000001</v>
       </c>
       <c r="DQ2" t="n">
         <v>105.77</v>
       </c>
       <c r="DR2" t="n">
-        <v>72.06</v>
+        <v>72.34</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
@@ -2187,16 +2187,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>-0.8365</v>
+        <v>-0.928</v>
       </c>
       <c r="DX2" t="n">
-        <v>78.94999999999999</v>
+        <v>77.125</v>
       </c>
       <c r="DY2" t="n">
-        <v>43.5</v>
+        <v>54</v>
       </c>
       <c r="DZ2" t="n">
-        <v>85.61799999999999</v>
+        <v>83.771</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2205,35 +2205,35 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>80.08</v>
+        <v>75.54000000000001</v>
       </c>
       <c r="ED2" t="n">
-        <v>97.03</v>
+        <v>93.59</v>
       </c>
       <c r="EE2" t="n">
-        <v>-0.8365</v>
+        <v>-0.928</v>
       </c>
       <c r="EF2" t="n">
-        <v>0.87</v>
+        <v>1.08</v>
       </c>
       <c r="EG2" t="n">
-        <v>-0.238</v>
+        <v>-0.2651</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0065</v>
+        <v>4.0014</v>
       </c>
       <c r="EI2" t="n">
-        <v>-0.0258</v>
+        <v>-0.0287</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.639</v>
+        <v>0.6372</v>
       </c>
       <c r="EK2" t="n">
-        <v>80.23999999999999</v>
+        <v>77.59</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
-          <t>Excellent</t>
+          <t>Strong</t>
         </is>
       </c>
       <c r="EM2" t="n">
@@ -2243,34 +2243,34 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>21.88</v>
+        <v>23.91</v>
       </c>
       <c r="EP2" t="n">
-        <v>2.3674</v>
+        <v>2.5871</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.0941</v>
+        <v>0.1169</v>
       </c>
       <c r="ER2" t="n">
-        <v>12.1149</v>
+        <v>9.777799999999999</v>
       </c>
       <c r="ES2" t="n">
-        <v>9.3581</v>
+        <v>9.461499999999999</v>
       </c>
       <c r="ET2" t="n">
-        <v>39.094</v>
+        <v>39.442</v>
       </c>
       <c r="EU2" t="n">
-        <v>-1.914</v>
+        <v>-2.646</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.4064</v>
+        <v>1.2692</v>
       </c>
       <c r="EW2" t="n">
-        <v>18.6986</v>
+        <v>20.2446</v>
       </c>
       <c r="EX2" t="n">
-        <v>56.27</v>
+        <v>57.13</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2284,31 +2284,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>59.38</v>
+        <v>59.07</v>
       </c>
       <c r="FC2" t="n">
-        <v>22.5</v>
+        <v>22.91</v>
       </c>
       <c r="FD2" t="n">
-        <v>74.29000000000001</v>
+        <v>74.18000000000001</v>
       </c>
       <c r="FE2" t="n">
-        <v>82.84999999999999</v>
+        <v>81.13</v>
       </c>
       <c r="FF2" t="n">
-        <v>46.53</v>
+        <v>46.75</v>
       </c>
       <c r="FG2" t="n">
-        <v>23.5427</v>
+        <v>23.261</v>
       </c>
       <c r="FH2" t="n">
-        <v>66.58199999999999</v>
+        <v>66.36199999999999</v>
       </c>
       <c r="FI2" t="n">
-        <v>53.015</v>
+        <v>53.39</v>
       </c>
       <c r="FJ2" t="n">
-        <v>66.91</v>
+        <v>65.70999999999999</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,19 +2322,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>79.72</v>
+        <v>77.51000000000001</v>
       </c>
       <c r="FO2" t="n">
-        <v>63.56</v>
+        <v>62.04</v>
       </c>
       <c r="FP2" t="n">
-        <v>82.26000000000001</v>
+        <v>81.14</v>
       </c>
       <c r="FQ2" t="n">
-        <v>76.42</v>
+        <v>74.06999999999999</v>
       </c>
       <c r="FR2" t="n">
-        <v>88.98999999999999</v>
+        <v>90.67</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>73.78149999999999</v>
+        <v>74.494</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261022_141137</t>
+          <t>20261022_204320</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46317.59140913087</v>
+        <v>46317.86343316094</v>
       </c>
     </row>
   </sheetData>
@@ -2458,7 +2458,7 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="22" max="22"/>
     <col width="20" customWidth="1" min="23" max="23"/>
     <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46317.59140046296</v>
+        <v>46317.86342592593</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2667,7 +2667,7 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>2007.6</v>
+        <v>2002.5</v>
       </c>
       <c r="L2" t="n">
         <v>1993.5</v>
@@ -2679,28 +2679,28 @@
         <v>1956.6</v>
       </c>
       <c r="O2" t="n">
-        <v>2007.6</v>
+        <v>2002.5</v>
       </c>
       <c r="P2" t="n">
-        <v>1224584</v>
+        <v>1538706</v>
       </c>
       <c r="Q2" t="n">
-        <v>2007.6</v>
+        <v>2002.5</v>
       </c>
       <c r="R2" t="n">
-        <v>2219.14</v>
+        <v>2214.04</v>
       </c>
       <c r="S2" t="n">
-        <v>1901.83</v>
+        <v>1896.73</v>
       </c>
       <c r="T2" t="n">
-        <v>10.53695955369595</v>
+        <v>10.56379525593008</v>
       </c>
       <c r="U2" t="n">
         <v>211.54</v>
       </c>
       <c r="V2" t="n">
-        <v>5.268479776847977</v>
+        <v>5.281897627965042</v>
       </c>
       <c r="W2" t="n">
         <v>105.77</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>10.53695955369595</v>
+        <v>10.56379525593008</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.268479776847977</v>
+        <v>5.281897627965042</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02039200714825264</v>
+        <v>0.0204095306894342</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3237130778863675</v>
+        <v>0.3239912554787012</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02902540975367884</v>
+        <v>0.02901929231073619</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228670255183435</v>
+        <v>0.04228669418851912</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645464</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.1</v>
+        <v>39.08</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-22 14:11:37.788468+05:30</t>
+          <t>2026-10-22 20:43:20.657110+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.536959553695954, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.563795255930085, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-23 08:37 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="17" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,14 +1816,14 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="H2" t="n">
         <v>8.800000000000001</v>
@@ -1859,59 +1859,59 @@
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>10.82</v>
+        <v>10.77</v>
       </c>
       <c r="R2" t="n">
-        <v>48.34</v>
+        <v>48.26</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="n">
-        <v>1993.5</v>
+        <v>1987.5</v>
       </c>
       <c r="V2" t="n">
-        <v>2019.8</v>
+        <v>2009.6</v>
       </c>
       <c r="W2" t="n">
+        <v>1933.5</v>
+      </c>
+      <c r="X2" t="n">
         <v>1956.6</v>
       </c>
-      <c r="X2" t="n">
-        <v>2002.5</v>
-      </c>
       <c r="Y2" t="n">
-        <v>2002.5</v>
+        <v>1956.6</v>
       </c>
       <c r="Z2" t="n">
-        <v>1538706</v>
+        <v>1480043</v>
       </c>
       <c r="AA2" t="n">
-        <v>1426504</v>
+        <v>1432307</v>
       </c>
       <c r="AB2" t="n">
-        <v>1.08</v>
+        <v>1.03</v>
       </c>
       <c r="AC2" t="n">
-        <v>-0.5</v>
+        <v>-2.29</v>
       </c>
       <c r="AD2" t="n">
-        <v>-0.9399999999999999</v>
+        <v>-0.75</v>
       </c>
       <c r="AE2" t="n">
-        <v>63.2</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="AF2" t="n">
-        <v>3.16</v>
+        <v>3.89</v>
       </c>
       <c r="AG2" t="n">
-        <v>52.88</v>
+        <v>54.54</v>
       </c>
       <c r="AH2" t="n">
-        <v>52.88</v>
+        <v>54.54</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.64</v>
+        <v>2.79</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,53 +1920,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>-1.01</v>
+        <v>-3.09</v>
       </c>
       <c r="AM2" t="n">
-        <v>3.16</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="AN2" t="n">
-        <v>41.25</v>
+        <v>37.6</v>
       </c>
       <c r="AO2" t="n">
-        <v>50.85</v>
+        <v>44.73</v>
       </c>
       <c r="AP2" t="n">
-        <v>-2.45</v>
+        <v>-2.07</v>
       </c>
       <c r="AQ2" t="n">
-        <v>26.92</v>
+        <v>24.76</v>
       </c>
       <c r="AR2" t="n">
-        <v>2002.5</v>
+        <v>1956.6</v>
       </c>
       <c r="AS2" t="n">
-        <v>2214.04</v>
+        <v>2174.77</v>
       </c>
       <c r="AT2" t="n">
-        <v>1896.73</v>
+        <v>1847.51</v>
       </c>
       <c r="AU2" t="n">
-        <v>2002.5</v>
+        <v>1956.599975585938</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>10.56</v>
+        <v>11.15</v>
       </c>
       <c r="AY2" t="n">
-        <v>211.54</v>
+        <v>218.17</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.28</v>
+        <v>5.58</v>
       </c>
       <c r="BA2" t="n">
-        <v>105.77</v>
+        <v>109.09</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.06</v>
+        <v>2.07</v>
       </c>
       <c r="BC2" t="n">
         <v>213</v>
@@ -1981,37 +1981,37 @@
         <v>50.4</v>
       </c>
       <c r="BG2" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.3</v>
+        <v>18.1</v>
       </c>
       <c r="BI2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BM2" t="n">
         <v>679</v>
       </c>
       <c r="BN2" t="n">
-        <v>48.9</v>
+        <v>48.7</v>
       </c>
       <c r="BO2" t="n">
         <v>2.09</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.67</v>
+        <v>8.69</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.2</v>
+        <v>-4.19</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
@@ -2020,19 +2020,19 @@
         <v>0.231</v>
       </c>
       <c r="BT2" t="n">
-        <v>1421.77</v>
+        <v>1419.54</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.87</v>
+        <v>-14.1</v>
       </c>
       <c r="BV2" t="n">
-        <v>1.98</v>
+        <v>1.97</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.06</v>
+        <v>2.07</v>
       </c>
       <c r="BX2" t="n">
-        <v>2</v>
+        <v>1.9999</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2055,13 +2055,13 @@
         <v>41.8</v>
       </c>
       <c r="CE2" t="n">
-        <v>49</v>
+        <v>48.5</v>
       </c>
       <c r="CF2" t="n">
-        <v>68.7</v>
+        <v>69</v>
       </c>
       <c r="CG2" t="n">
-        <v>69.90000000000001</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2082,43 +2082,43 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>84.67</v>
+        <v>95.78</v>
       </c>
       <c r="CO2" t="n">
-        <v>36.37</v>
+        <v>39.73</v>
       </c>
       <c r="CP2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CQ2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CR2" t="n">
-        <v>85.71428571428571</v>
+        <v>86.36363636363636</v>
       </c>
       <c r="CS2" t="n">
         <v>100</v>
       </c>
       <c r="CT2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CU2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CV2" t="n">
-        <v>85.71428571428571</v>
+        <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>66.66666666666666</v>
+        <v>68.18181818181817</v>
       </c>
       <c r="CX2" t="n">
-        <v>57.14285714285714</v>
+        <v>54.54545454545454</v>
       </c>
       <c r="CY2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>10.5638</v>
+        <v>11.1505</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,58 +2127,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.704</v>
+        <v>0.7433</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.352</v>
+        <v>0.372</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1056</v>
+        <v>0.1115</v>
       </c>
       <c r="DF2" t="n">
-        <v>2</v>
+        <v>1.9982</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1426</v>
+        <v>1.2009</v>
       </c>
       <c r="DH2" t="n">
-        <v>4</v>
+        <v>3.9964</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.2819</v>
+        <v>5.5755</v>
       </c>
       <c r="DJ2" t="n">
-        <v>34.44</v>
+        <v>39.16</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.2819</v>
+        <v>5.5755</v>
       </c>
       <c r="DL2" t="n">
-        <v>2</v>
+        <v>1.9999</v>
       </c>
       <c r="DM2" t="n">
         <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>4</v>
+        <v>3.9964</v>
       </c>
       <c r="DO2" t="n">
-        <v>2</v>
+        <v>1.9981</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.7576000000000001</v>
+        <v>0.7161999999999999</v>
       </c>
       <c r="DQ2" t="n">
-        <v>105.77</v>
+        <v>109.09</v>
       </c>
       <c r="DR2" t="n">
-        <v>72.34</v>
+        <v>40.42</v>
       </c>
       <c r="DS2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="DT2" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,16 +2187,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>-0.928</v>
+        <v>-0.7419</v>
       </c>
       <c r="DX2" t="n">
-        <v>77.125</v>
+        <v>61.82499999999999</v>
       </c>
       <c r="DY2" t="n">
-        <v>54</v>
+        <v>51.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>83.771</v>
+        <v>87.931</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2205,72 +2205,72 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>75.54000000000001</v>
+        <v>82.51000000000001</v>
       </c>
       <c r="ED2" t="n">
-        <v>93.59</v>
+        <v>91.89</v>
       </c>
       <c r="EE2" t="n">
-        <v>-0.928</v>
+        <v>-0.7419</v>
       </c>
       <c r="EF2" t="n">
-        <v>1.08</v>
+        <v>1.03</v>
       </c>
       <c r="EG2" t="n">
-        <v>-0.2651</v>
+        <v>-0.2229</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.0014</v>
+        <v>3.9966</v>
       </c>
       <c r="EI2" t="n">
-        <v>-0.0287</v>
+        <v>-0.024</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6372</v>
+        <v>0.6074000000000001</v>
       </c>
       <c r="EK2" t="n">
-        <v>77.59</v>
+        <v>82.11</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Excellent</t>
         </is>
       </c>
       <c r="EM2" t="n">
         <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="EO2" t="n">
-        <v>23.91</v>
+        <v>48</v>
       </c>
       <c r="EP2" t="n">
-        <v>2.5871</v>
+        <v>5.1696</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.1169</v>
+        <v>0.1109</v>
       </c>
       <c r="ER2" t="n">
-        <v>9.777799999999999</v>
+        <v>10.8252</v>
       </c>
       <c r="ES2" t="n">
-        <v>9.461499999999999</v>
+        <v>10.3325</v>
       </c>
       <c r="ET2" t="n">
-        <v>39.442</v>
+        <v>48.034</v>
       </c>
       <c r="EU2" t="n">
-        <v>-2.646</v>
+        <v>-2.1321</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.2692</v>
+        <v>1.3744</v>
       </c>
       <c r="EW2" t="n">
-        <v>20.2446</v>
+        <v>45.9744</v>
       </c>
       <c r="EX2" t="n">
-        <v>57.13</v>
+        <v>55.19</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2284,31 +2284,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>59.07</v>
+        <v>59.14</v>
       </c>
       <c r="FC2" t="n">
-        <v>22.91</v>
+        <v>31.69</v>
       </c>
       <c r="FD2" t="n">
-        <v>74.18000000000001</v>
+        <v>74.81999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>81.13</v>
+        <v>88.94499999999999</v>
       </c>
       <c r="FF2" t="n">
-        <v>46.75</v>
+        <v>47.46</v>
       </c>
       <c r="FG2" t="n">
-        <v>23.261</v>
+        <v>25.2718</v>
       </c>
       <c r="FH2" t="n">
-        <v>66.36199999999999</v>
+        <v>69.342</v>
       </c>
       <c r="FI2" t="n">
-        <v>53.39</v>
+        <v>39.79</v>
       </c>
       <c r="FJ2" t="n">
-        <v>65.70999999999999</v>
+        <v>70.27</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,22 +2322,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>77.51000000000001</v>
+        <v>70.89</v>
       </c>
       <c r="FO2" t="n">
-        <v>62.04</v>
+        <v>69.55</v>
       </c>
       <c r="FP2" t="n">
-        <v>81.14</v>
+        <v>63.87</v>
       </c>
       <c r="FQ2" t="n">
-        <v>74.06999999999999</v>
+        <v>60.56</v>
       </c>
       <c r="FR2" t="n">
-        <v>90.67</v>
+        <v>79.92</v>
       </c>
       <c r="FS2" t="n">
-        <v>100</v>
+        <v>95.4545</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2347,11 +2347,11 @@
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>74.494</v>
+        <v>65.95099999999999</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261022_204320</t>
+          <t>20261023_140725</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46317.86343316094</v>
+        <v>46318.5884930489</v>
       </c>
     </row>
   </sheetData>
@@ -2458,9 +2458,9 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
     <col width="20" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46317.86342592593</v>
+        <v>46318.58848379629</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2663,50 +2663,50 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>10.82</v>
+        <v>10.77</v>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>2002.5</v>
+        <v>1956.6</v>
       </c>
       <c r="L2" t="n">
-        <v>1993.5</v>
+        <v>1987.5</v>
       </c>
       <c r="M2" t="n">
-        <v>2019.8</v>
+        <v>2009.6</v>
       </c>
       <c r="N2" t="n">
+        <v>1933.5</v>
+      </c>
+      <c r="O2" t="n">
         <v>1956.6</v>
       </c>
-      <c r="O2" t="n">
-        <v>2002.5</v>
-      </c>
       <c r="P2" t="n">
-        <v>1538706</v>
+        <v>1480043</v>
       </c>
       <c r="Q2" t="n">
-        <v>2002.5</v>
+        <v>1956.6</v>
       </c>
       <c r="R2" t="n">
-        <v>2214.04</v>
+        <v>2174.77</v>
       </c>
       <c r="S2" t="n">
-        <v>1896.73</v>
+        <v>1847.51</v>
       </c>
       <c r="T2" t="n">
-        <v>10.56379525593008</v>
+        <v>11.15046509250742</v>
       </c>
       <c r="U2" t="n">
-        <v>211.54</v>
+        <v>218.1700000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>5.281897627965042</v>
+        <v>5.575488091587443</v>
       </c>
       <c r="W2" t="n">
-        <v>105.77</v>
+        <v>109.0899999999999</v>
       </c>
       <c r="X2" t="n">
-        <v>2</v>
+        <v>1.99990833256944</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>10.56379525593008</v>
+        <v>11.15046509250742</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.281897627965042</v>
+        <v>5.575488091587443</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0204095306894342</v>
+        <v>0.02042987483925653</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3239912554787012</v>
+        <v>0.3243142088450907</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02901929231073619</v>
+        <v>0.02901939531923797</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228669418851912</v>
+        <v>0.04228671602080091</v>
       </c>
     </row>
     <row r="13">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.08</v>
+        <v>39.05</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-22 20:43:20.657110+05:30</t>
+          <t>2026-10-23 14:07:25.833673+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 10.563795255930085, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 11.150465092507416, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9999083325694402}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-23 15:01 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="20" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="17" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1862,7 +1862,7 @@
         <v>10.77</v>
       </c>
       <c r="R2" t="n">
-        <v>48.26</v>
+        <v>48.38</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1878,22 +1878,22 @@
         <v>1933.5</v>
       </c>
       <c r="X2" t="n">
-        <v>1956.6</v>
+        <v>1970</v>
       </c>
       <c r="Y2" t="n">
-        <v>1956.6</v>
+        <v>1970</v>
       </c>
       <c r="Z2" t="n">
-        <v>1480043</v>
+        <v>1893589</v>
       </c>
       <c r="AA2" t="n">
-        <v>1432307</v>
+        <v>1452985</v>
       </c>
       <c r="AB2" t="n">
-        <v>1.03</v>
+        <v>1.3</v>
       </c>
       <c r="AC2" t="n">
-        <v>-2.29</v>
+        <v>-1.62</v>
       </c>
       <c r="AD2" t="n">
         <v>-0.75</v>
@@ -1902,7 +1902,7 @@
         <v>76.09999999999999</v>
       </c>
       <c r="AF2" t="n">
-        <v>3.89</v>
+        <v>3.86</v>
       </c>
       <c r="AG2" t="n">
         <v>54.54</v>
@@ -1911,7 +1911,7 @@
         <v>54.54</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.79</v>
+        <v>2.77</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,47 +1920,47 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>-3.09</v>
+        <v>-2.46</v>
       </c>
       <c r="AM2" t="n">
-        <v>0.6899999999999999</v>
+        <v>1.37</v>
       </c>
       <c r="AN2" t="n">
-        <v>37.6</v>
+        <v>38.54</v>
       </c>
       <c r="AO2" t="n">
-        <v>44.73</v>
+        <v>46.36</v>
       </c>
       <c r="AP2" t="n">
-        <v>-2.07</v>
+        <v>-1.4</v>
       </c>
       <c r="AQ2" t="n">
-        <v>24.76</v>
+        <v>25.61</v>
       </c>
       <c r="AR2" t="n">
-        <v>1956.6</v>
+        <v>1970</v>
       </c>
       <c r="AS2" t="n">
-        <v>2174.77</v>
+        <v>2188.17</v>
       </c>
       <c r="AT2" t="n">
-        <v>1847.51</v>
+        <v>1860.91</v>
       </c>
       <c r="AU2" t="n">
-        <v>1956.599975585938</v>
+        <v>1970</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>11.15</v>
+        <v>11.07</v>
       </c>
       <c r="AY2" t="n">
         <v>218.17</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.58</v>
+        <v>5.54</v>
       </c>
       <c r="BA2" t="n">
         <v>109.09</v>
@@ -2020,10 +2020,10 @@
         <v>0.231</v>
       </c>
       <c r="BT2" t="n">
-        <v>1419.54</v>
+        <v>1420.2</v>
       </c>
       <c r="BU2" t="n">
-        <v>-14.1</v>
+        <v>-14.03</v>
       </c>
       <c r="BV2" t="n">
         <v>1.97</v>
@@ -2082,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>95.78</v>
+        <v>94.93000000000001</v>
       </c>
       <c r="CO2" t="n">
-        <v>39.73</v>
+        <v>39.25</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2118,7 +2118,7 @@
         <v>2</v>
       </c>
       <c r="CZ2" t="n">
-        <v>11.1505</v>
+        <v>11.0746</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,31 +2127,31 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.7433</v>
+        <v>0.738</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.372</v>
+        <v>0.3693</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1115</v>
+        <v>0.1107</v>
       </c>
       <c r="DF2" t="n">
         <v>1.9982</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.2009</v>
+        <v>1.1922</v>
       </c>
       <c r="DH2" t="n">
         <v>3.9964</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.5755</v>
+        <v>5.5376</v>
       </c>
       <c r="DJ2" t="n">
-        <v>39.16</v>
+        <v>37.58</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.5755</v>
+        <v>5.5376</v>
       </c>
       <c r="DL2" t="n">
         <v>1.9999</v>
@@ -2163,22 +2163,22 @@
         <v>3.9964</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9981</v>
+        <v>1.9984</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.7161999999999999</v>
+        <v>0.7214</v>
       </c>
       <c r="DQ2" t="n">
         <v>109.09</v>
       </c>
       <c r="DR2" t="n">
-        <v>40.42</v>
+        <v>44.6</v>
       </c>
       <c r="DS2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="DT2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,16 +2187,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>-0.7419</v>
+        <v>-0.5054</v>
       </c>
       <c r="DX2" t="n">
-        <v>61.82499999999999</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="DY2" t="n">
-        <v>51.5</v>
+        <v>65</v>
       </c>
       <c r="DZ2" t="n">
-        <v>87.931</v>
+        <v>87.43000000000001</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2205,31 +2205,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>82.51000000000001</v>
+        <v>76.95</v>
       </c>
       <c r="ED2" t="n">
-        <v>91.89</v>
+        <v>96.81</v>
       </c>
       <c r="EE2" t="n">
-        <v>-0.7419</v>
+        <v>-0.5054</v>
       </c>
       <c r="EF2" t="n">
-        <v>1.03</v>
+        <v>1.3</v>
       </c>
       <c r="EG2" t="n">
-        <v>-0.2229</v>
+        <v>-0.1508</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9966</v>
+        <v>3.9981</v>
       </c>
       <c r="EI2" t="n">
-        <v>-0.024</v>
+        <v>-0.0162</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6074000000000001</v>
+        <v>0.6113</v>
       </c>
       <c r="EK2" t="n">
-        <v>82.11</v>
+        <v>81.61</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2240,37 +2240,37 @@
         <v>5</v>
       </c>
       <c r="EN2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>48</v>
+        <v>49.83</v>
       </c>
       <c r="EP2" t="n">
-        <v>5.1696</v>
+        <v>5.3667</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.1109</v>
+        <v>0.14</v>
       </c>
       <c r="ER2" t="n">
-        <v>10.8252</v>
+        <v>8.5154</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.3325</v>
+        <v>9.9682</v>
       </c>
       <c r="ET2" t="n">
-        <v>48.034</v>
+        <v>48.391</v>
       </c>
       <c r="EU2" t="n">
-        <v>-2.1321</v>
+        <v>-1.82</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.3744</v>
+        <v>1.2043</v>
       </c>
       <c r="EW2" t="n">
-        <v>45.9744</v>
+        <v>47.3036</v>
       </c>
       <c r="EX2" t="n">
-        <v>55.19</v>
+        <v>57.31</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2287,28 +2287,28 @@
         <v>59.14</v>
       </c>
       <c r="FC2" t="n">
-        <v>31.69</v>
+        <v>29.98</v>
       </c>
       <c r="FD2" t="n">
         <v>74.81999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>88.94499999999999</v>
+        <v>88.27</v>
       </c>
       <c r="FF2" t="n">
-        <v>47.46</v>
+        <v>48.28</v>
       </c>
       <c r="FG2" t="n">
-        <v>25.2718</v>
+        <v>25.1804</v>
       </c>
       <c r="FH2" t="n">
-        <v>69.342</v>
+        <v>69.511</v>
       </c>
       <c r="FI2" t="n">
-        <v>39.79</v>
+        <v>41.09</v>
       </c>
       <c r="FJ2" t="n">
-        <v>70.27</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,19 +2322,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>70.89</v>
+        <v>73.05</v>
       </c>
       <c r="FO2" t="n">
-        <v>69.55</v>
+        <v>70.01000000000001</v>
       </c>
       <c r="FP2" t="n">
-        <v>63.87</v>
+        <v>66.75</v>
       </c>
       <c r="FQ2" t="n">
-        <v>60.56</v>
+        <v>62.37</v>
       </c>
       <c r="FR2" t="n">
-        <v>79.92</v>
+        <v>83.54000000000001</v>
       </c>
       <c r="FS2" t="n">
         <v>95.4545</v>
@@ -2347,11 +2347,11 @@
       </c>
       <c r="FV2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>65.95099999999999</v>
+        <v>68.17700000000001</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261023_140725</t>
+          <t>20261023_203111</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46318.5884930489</v>
+        <v>46318.85498938241</v>
       </c>
     </row>
   </sheetData>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46318.58848379629</v>
+        <v>46318.85498842593</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2667,7 +2667,7 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>1956.6</v>
+        <v>1970</v>
       </c>
       <c r="L2" t="n">
         <v>1987.5</v>
@@ -2679,28 +2679,28 @@
         <v>1933.5</v>
       </c>
       <c r="O2" t="n">
-        <v>1956.6</v>
+        <v>1970</v>
       </c>
       <c r="P2" t="n">
-        <v>1480043</v>
+        <v>1893589</v>
       </c>
       <c r="Q2" t="n">
-        <v>1956.6</v>
+        <v>1970</v>
       </c>
       <c r="R2" t="n">
-        <v>2174.77</v>
+        <v>2188.17</v>
       </c>
       <c r="S2" t="n">
-        <v>1847.51</v>
+        <v>1860.91</v>
       </c>
       <c r="T2" t="n">
-        <v>11.15046509250742</v>
+        <v>11.07461928934011</v>
       </c>
       <c r="U2" t="n">
         <v>218.1700000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>5.575488091587443</v>
+        <v>5.537563451776646</v>
       </c>
       <c r="W2" t="n">
         <v>109.0899999999999</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>11.15046509250742</v>
+        <v>11.07461928934011</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.575488091587443</v>
+        <v>5.537563451776646</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02042987483925653</v>
+        <v>0.02040733964618313</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3243142088450907</v>
+        <v>0.3239564737453765</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02901939531923797</v>
+        <v>0.0290133808847971</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228671602080091</v>
+        <v>0.04228670591851882</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869492979645463</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.05</v>
+        <v>39.08</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-23 14:07:25.833673+05:30</t>
+          <t>2026-10-23 20:31:11.120117+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 11.150465092507416, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9999083325694402}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 11.074619289340106, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9999083325694402}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-26 09:02 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="19" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1816,14 +1816,14 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="H2" t="n">
         <v>8.800000000000001</v>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1859,7 +1859,7 @@
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>10.77</v>
+        <v>10.82</v>
       </c>
       <c r="R2" t="n">
         <v>48.38</v>
@@ -1869,49 +1869,49 @@
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="n">
-        <v>1987.5</v>
+        <v>1960</v>
       </c>
       <c r="V2" t="n">
-        <v>2009.6</v>
+        <v>2058</v>
       </c>
       <c r="W2" t="n">
-        <v>1933.5</v>
+        <v>1951.6</v>
       </c>
       <c r="X2" t="n">
-        <v>1970</v>
+        <v>2051.2</v>
       </c>
       <c r="Y2" t="n">
-        <v>1970</v>
+        <v>2051.2</v>
       </c>
       <c r="Z2" t="n">
-        <v>1893589</v>
+        <v>1614484</v>
       </c>
       <c r="AA2" t="n">
-        <v>1452985</v>
+        <v>1464313</v>
       </c>
       <c r="AB2" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="AC2" t="n">
-        <v>-1.62</v>
+        <v>4.12</v>
       </c>
       <c r="AD2" t="n">
-        <v>-0.75</v>
+        <v>-0.51</v>
       </c>
       <c r="AE2" t="n">
-        <v>76.09999999999999</v>
+        <v>106.4</v>
       </c>
       <c r="AF2" t="n">
-        <v>3.86</v>
+        <v>5.19</v>
       </c>
       <c r="AG2" t="n">
-        <v>54.54</v>
+        <v>58.25</v>
       </c>
       <c r="AH2" t="n">
-        <v>54.54</v>
+        <v>58.25</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.77</v>
+        <v>2.84</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,53 +1920,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>-2.46</v>
+        <v>1.5</v>
       </c>
       <c r="AM2" t="n">
-        <v>1.37</v>
+        <v>5.33</v>
       </c>
       <c r="AN2" t="n">
-        <v>38.54</v>
+        <v>43.77</v>
       </c>
       <c r="AO2" t="n">
-        <v>46.36</v>
+        <v>56.65</v>
       </c>
       <c r="AP2" t="n">
-        <v>-1.4</v>
+        <v>0.72</v>
       </c>
       <c r="AQ2" t="n">
-        <v>25.61</v>
+        <v>28.1</v>
       </c>
       <c r="AR2" t="n">
-        <v>1970</v>
+        <v>2051.2</v>
       </c>
       <c r="AS2" t="n">
-        <v>2188.17</v>
+        <v>2284.19</v>
       </c>
       <c r="AT2" t="n">
-        <v>1860.91</v>
+        <v>1934.71</v>
       </c>
       <c r="AU2" t="n">
-        <v>1970</v>
+        <v>2051.199951171875</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>11.07</v>
+        <v>11.36</v>
       </c>
       <c r="AY2" t="n">
-        <v>218.17</v>
+        <v>232.99</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.54</v>
+        <v>5.68</v>
       </c>
       <c r="BA2" t="n">
-        <v>109.09</v>
+        <v>116.49</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.07</v>
+        <v>2.06</v>
       </c>
       <c r="BC2" t="n">
         <v>213</v>
@@ -1981,37 +1981,37 @@
         <v>50.4</v>
       </c>
       <c r="BG2" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.1</v>
+        <v>18.3</v>
       </c>
       <c r="BI2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="BK2" t="n">
         <v>0</v>
       </c>
       <c r="BL2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BM2" t="n">
         <v>679</v>
       </c>
       <c r="BN2" t="n">
-        <v>48.7</v>
+        <v>48.9</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.09</v>
+        <v>2.1</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.69</v>
+        <v>8.67</v>
       </c>
       <c r="BQ2" t="n">
-        <v>-4.19</v>
+        <v>-4.2</v>
       </c>
       <c r="BR2" t="n">
         <v>9.1</v>
@@ -2020,19 +2020,19 @@
         <v>0.231</v>
       </c>
       <c r="BT2" t="n">
-        <v>1420.2</v>
+        <v>1423.74</v>
       </c>
       <c r="BU2" t="n">
-        <v>-14.03</v>
+        <v>-13.66</v>
       </c>
       <c r="BV2" t="n">
-        <v>1.97</v>
+        <v>1.98</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.07</v>
+        <v>2.06</v>
       </c>
       <c r="BX2" t="n">
-        <v>1.9999</v>
+        <v>2.0001</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2052,16 +2052,16 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>41.8</v>
+        <v>42</v>
       </c>
       <c r="CE2" t="n">
-        <v>48.5</v>
+        <v>49</v>
       </c>
       <c r="CF2" t="n">
-        <v>69</v>
+        <v>68.7</v>
       </c>
       <c r="CG2" t="n">
-        <v>69.59999999999999</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2082,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>94.93000000000001</v>
+        <v>96.92</v>
       </c>
       <c r="CO2" t="n">
-        <v>39.25</v>
+        <v>39.9</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2115,10 +2115,10 @@
         <v>54.54545454545454</v>
       </c>
       <c r="CY2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>11.0746</v>
+        <v>11.3587</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,58 +2127,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.738</v>
+        <v>0.7573</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3693</v>
+        <v>0.3787</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1107</v>
+        <v>0.1136</v>
       </c>
       <c r="DF2" t="n">
-        <v>1.9982</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.1922</v>
+        <v>1.2292</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9964</v>
+        <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.5376</v>
+        <v>5.6791</v>
       </c>
       <c r="DJ2" t="n">
-        <v>37.58</v>
+        <v>42.15</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.5376</v>
+        <v>5.6791</v>
       </c>
       <c r="DL2" t="n">
-        <v>1.9999</v>
+        <v>2.0001</v>
       </c>
       <c r="DM2" t="n">
         <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9964</v>
+        <v>4</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9984</v>
+        <v>1.9997</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.7214</v>
+        <v>0.7042</v>
       </c>
       <c r="DQ2" t="n">
-        <v>109.09</v>
+        <v>116.49</v>
       </c>
       <c r="DR2" t="n">
-        <v>44.6</v>
+        <v>59.36</v>
       </c>
       <c r="DS2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,16 +2187,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>-0.5054</v>
+        <v>0.2535</v>
       </c>
       <c r="DX2" t="n">
-        <v>65.90000000000001</v>
+        <v>91.625</v>
       </c>
       <c r="DY2" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="DZ2" t="n">
-        <v>87.43000000000001</v>
+        <v>90.878</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2205,31 +2205,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>76.95</v>
+        <v>85.88</v>
       </c>
       <c r="ED2" t="n">
-        <v>96.81</v>
+        <v>100</v>
       </c>
       <c r="EE2" t="n">
-        <v>-0.5054</v>
+        <v>0.2535</v>
       </c>
       <c r="EF2" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="EG2" t="n">
-        <v>-0.1508</v>
+        <v>0.0779</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9981</v>
+        <v>3.9995</v>
       </c>
       <c r="EI2" t="n">
-        <v>-0.0162</v>
+        <v>0.008399999999999999</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6113</v>
+        <v>0.5987</v>
       </c>
       <c r="EK2" t="n">
-        <v>81.61</v>
+        <v>85.62</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2243,34 +2243,34 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>49.83</v>
+        <v>51.14</v>
       </c>
       <c r="EP2" t="n">
-        <v>5.3667</v>
+        <v>5.5333</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.14</v>
+        <v>0.119</v>
       </c>
       <c r="ER2" t="n">
-        <v>8.5154</v>
+        <v>10.3273</v>
       </c>
       <c r="ES2" t="n">
-        <v>9.9682</v>
+        <v>10.9766</v>
       </c>
       <c r="ET2" t="n">
-        <v>48.391</v>
+        <v>49.116</v>
       </c>
       <c r="EU2" t="n">
-        <v>-1.82</v>
+        <v>0.792</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.2043</v>
+        <v>1.3524</v>
       </c>
       <c r="EW2" t="n">
-        <v>47.3036</v>
+        <v>49.5649</v>
       </c>
       <c r="EX2" t="n">
-        <v>57.31</v>
+        <v>59.04</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2284,31 +2284,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>59.14</v>
+        <v>59.38</v>
       </c>
       <c r="FC2" t="n">
-        <v>29.98</v>
+        <v>34.9</v>
       </c>
       <c r="FD2" t="n">
-        <v>74.81999999999999</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="FE2" t="n">
-        <v>88.27</v>
+        <v>91.27</v>
       </c>
       <c r="FF2" t="n">
-        <v>48.28</v>
+        <v>49.47</v>
       </c>
       <c r="FG2" t="n">
-        <v>25.1804</v>
+        <v>25.2396</v>
       </c>
       <c r="FH2" t="n">
-        <v>69.511</v>
+        <v>70.574</v>
       </c>
       <c r="FI2" t="n">
-        <v>41.09</v>
+        <v>50.755</v>
       </c>
       <c r="FJ2" t="n">
-        <v>70.40000000000001</v>
+        <v>72.12</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,22 +2322,22 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>73.05</v>
+        <v>81.84999999999999</v>
       </c>
       <c r="FO2" t="n">
-        <v>70.01000000000001</v>
+        <v>73.19</v>
       </c>
       <c r="FP2" t="n">
-        <v>66.75</v>
+        <v>77.37</v>
       </c>
       <c r="FQ2" t="n">
-        <v>62.37</v>
+        <v>74.48999999999999</v>
       </c>
       <c r="FR2" t="n">
-        <v>83.54000000000001</v>
+        <v>94.7</v>
       </c>
       <c r="FS2" t="n">
-        <v>95.4545</v>
+        <v>100</v>
       </c>
       <c r="FT2" t="n">
         <v>5</v>
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>68.17700000000001</v>
+        <v>77.0005</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261023_203111</t>
+          <t>20261026_143220</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46318.85498938241</v>
+        <v>46321.6057876845</v>
       </c>
     </row>
   </sheetData>
@@ -2458,9 +2458,9 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="22" max="22"/>
     <col width="20" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="19" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46318.85498842593</v>
+        <v>46321.60578703704</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2663,50 +2663,50 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>10.77</v>
+        <v>10.82</v>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>1970</v>
+        <v>2051.2</v>
       </c>
       <c r="L2" t="n">
-        <v>1987.5</v>
+        <v>1960</v>
       </c>
       <c r="M2" t="n">
-        <v>2009.6</v>
+        <v>2058</v>
       </c>
       <c r="N2" t="n">
-        <v>1933.5</v>
+        <v>1951.6</v>
       </c>
       <c r="O2" t="n">
-        <v>1970</v>
+        <v>2051.2</v>
       </c>
       <c r="P2" t="n">
-        <v>1893589</v>
+        <v>1614484</v>
       </c>
       <c r="Q2" t="n">
-        <v>1970</v>
+        <v>2051.2</v>
       </c>
       <c r="R2" t="n">
-        <v>2188.17</v>
+        <v>2284.19</v>
       </c>
       <c r="S2" t="n">
-        <v>1860.91</v>
+        <v>1934.71</v>
       </c>
       <c r="T2" t="n">
-        <v>11.07461928934011</v>
+        <v>11.35871684867396</v>
       </c>
       <c r="U2" t="n">
-        <v>218.1700000000001</v>
+        <v>232.9900000000002</v>
       </c>
       <c r="V2" t="n">
-        <v>5.537563451776646</v>
+        <v>5.679114664586574</v>
       </c>
       <c r="W2" t="n">
-        <v>109.0899999999999</v>
+        <v>116.4899999999998</v>
       </c>
       <c r="X2" t="n">
-        <v>1.99990833256944</v>
+        <v>2.000085844278485</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>11.07461928934011</v>
+        <v>11.35871684867396</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.537563451776646</v>
+        <v>5.679114664586574</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02040733964618313</v>
+        <v>0.02044423465830534</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3239564737453765</v>
+        <v>0.324542163905541</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.0290133808847971</v>
+        <v>0.02900736645035623</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228670591851882</v>
+        <v>0.04228671425721302</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645463</v>
+        <v>0.1869493934347614</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.08</v>
+        <v>39.04</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-23 20:31:11.120117+05:30</t>
+          <t>2026-10-26 14:32:20.080876+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 11.074619289340106, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.9999083325694402}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 11.358716848673959, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000085844278485}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-26 16:46 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="19" customWidth="1" min="47" max="47"/>
+    <col width="18" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1862,7 +1862,7 @@
         <v>10.82</v>
       </c>
       <c r="R2" t="n">
-        <v>48.38</v>
+        <v>48.45</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1872,46 +1872,46 @@
         <v>1960</v>
       </c>
       <c r="V2" t="n">
-        <v>2058</v>
+        <v>2058.9</v>
       </c>
       <c r="W2" t="n">
         <v>1951.6</v>
       </c>
       <c r="X2" t="n">
-        <v>2051.2</v>
+        <v>2058.9</v>
       </c>
       <c r="Y2" t="n">
-        <v>2051.2</v>
+        <v>2058.9</v>
       </c>
       <c r="Z2" t="n">
-        <v>1614484</v>
+        <v>1858038</v>
       </c>
       <c r="AA2" t="n">
-        <v>1464313</v>
+        <v>1476491</v>
       </c>
       <c r="AB2" t="n">
-        <v>1.1</v>
+        <v>1.26</v>
       </c>
       <c r="AC2" t="n">
-        <v>4.12</v>
+        <v>4.51</v>
       </c>
       <c r="AD2" t="n">
         <v>-0.51</v>
       </c>
       <c r="AE2" t="n">
-        <v>106.4</v>
+        <v>107.3</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.19</v>
+        <v>5.21</v>
       </c>
       <c r="AG2" t="n">
-        <v>58.25</v>
+        <v>58.31</v>
       </c>
       <c r="AH2" t="n">
-        <v>58.25</v>
+        <v>58.31</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.84</v>
+        <v>2.83</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,50 +1920,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>1.5</v>
+        <v>1.86</v>
       </c>
       <c r="AM2" t="n">
-        <v>5.33</v>
+        <v>5.71</v>
       </c>
       <c r="AN2" t="n">
-        <v>43.77</v>
+        <v>44.31</v>
       </c>
       <c r="AO2" t="n">
-        <v>56.65</v>
+        <v>57.43</v>
       </c>
       <c r="AP2" t="n">
-        <v>0.72</v>
+        <v>1.09</v>
       </c>
       <c r="AQ2" t="n">
-        <v>28.1</v>
+        <v>28.58</v>
       </c>
       <c r="AR2" t="n">
-        <v>2051.2</v>
+        <v>2058.9</v>
       </c>
       <c r="AS2" t="n">
-        <v>2284.19</v>
+        <v>2292.14</v>
       </c>
       <c r="AT2" t="n">
-        <v>1934.71</v>
+        <v>1942.28</v>
       </c>
       <c r="AU2" t="n">
-        <v>2051.199951171875</v>
+        <v>2058.89990234375</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>11.36</v>
+        <v>11.33</v>
       </c>
       <c r="AY2" t="n">
-        <v>232.99</v>
+        <v>233.24</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.68</v>
+        <v>5.66</v>
       </c>
       <c r="BA2" t="n">
-        <v>116.49</v>
+        <v>116.62</v>
       </c>
       <c r="BB2" t="n">
         <v>2.06</v>
@@ -2020,10 +2020,10 @@
         <v>0.231</v>
       </c>
       <c r="BT2" t="n">
-        <v>1423.74</v>
+        <v>1424.03</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.66</v>
+        <v>-13.63</v>
       </c>
       <c r="BV2" t="n">
         <v>1.98</v>
@@ -2032,7 +2032,7 @@
         <v>2.06</v>
       </c>
       <c r="BX2" t="n">
-        <v>2.0001</v>
+        <v>2</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2082,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>96.92</v>
+        <v>97.34</v>
       </c>
       <c r="CO2" t="n">
-        <v>39.9</v>
+        <v>39.53</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2118,7 +2118,7 @@
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>11.3587</v>
+        <v>11.3284</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,58 +2127,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.7573</v>
+        <v>0.7553</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3787</v>
+        <v>0.3773</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1136</v>
+        <v>0.1133</v>
       </c>
       <c r="DF2" t="n">
+        <v>2.0018</v>
+      </c>
+      <c r="DG2" t="n">
+        <v>1.2259</v>
+      </c>
+      <c r="DH2" t="n">
+        <v>4.0035</v>
+      </c>
+      <c r="DI2" t="n">
+        <v>5.6642</v>
+      </c>
+      <c r="DJ2" t="n">
+        <v>41.61</v>
+      </c>
+      <c r="DK2" t="n">
+        <v>5.6642</v>
+      </c>
+      <c r="DL2" t="n">
         <v>2</v>
-      </c>
-      <c r="DG2" t="n">
-        <v>1.2292</v>
-      </c>
-      <c r="DH2" t="n">
-        <v>4</v>
-      </c>
-      <c r="DI2" t="n">
-        <v>5.6791</v>
-      </c>
-      <c r="DJ2" t="n">
-        <v>42.15</v>
-      </c>
-      <c r="DK2" t="n">
-        <v>5.6791</v>
-      </c>
-      <c r="DL2" t="n">
-        <v>2.0001</v>
       </c>
       <c r="DM2" t="n">
         <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>4</v>
+        <v>4.0035</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9997</v>
+        <v>2.0019</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.7042</v>
+        <v>0.7073</v>
       </c>
       <c r="DQ2" t="n">
-        <v>116.49</v>
+        <v>116.62</v>
       </c>
       <c r="DR2" t="n">
-        <v>59.36</v>
+        <v>73.58</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,16 +2187,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.2535</v>
+        <v>0.3852</v>
       </c>
       <c r="DX2" t="n">
-        <v>91.625</v>
+        <v>93.575</v>
       </c>
       <c r="DY2" t="n">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="DZ2" t="n">
-        <v>90.878</v>
+        <v>90.699</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2205,31 +2205,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>85.88</v>
+        <v>87.64</v>
       </c>
       <c r="ED2" t="n">
         <v>100</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.2535</v>
+        <v>0.3852</v>
       </c>
       <c r="EF2" t="n">
-        <v>1.1</v>
+        <v>1.26</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.0779</v>
+        <v>0.1179</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9995</v>
+        <v>4.003</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.008399999999999999</v>
+        <v>0.0128</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.5987</v>
+        <v>0.6011</v>
       </c>
       <c r="EK2" t="n">
-        <v>85.62</v>
+        <v>86.73999999999999</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2243,34 +2243,34 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>51.14</v>
+        <v>44.07</v>
       </c>
       <c r="EP2" t="n">
-        <v>5.5333</v>
+        <v>4.7684</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.119</v>
+        <v>0.1363</v>
       </c>
       <c r="ER2" t="n">
-        <v>10.3273</v>
+        <v>8.992100000000001</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.9766</v>
+        <v>10.8642</v>
       </c>
       <c r="ET2" t="n">
-        <v>49.116</v>
+        <v>46.847</v>
       </c>
       <c r="EU2" t="n">
-        <v>0.792</v>
+        <v>1.3734</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.3524</v>
+        <v>1.2522</v>
       </c>
       <c r="EW2" t="n">
-        <v>49.5649</v>
+        <v>42.8977</v>
       </c>
       <c r="EX2" t="n">
-        <v>59.04</v>
+        <v>58.53</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2287,28 +2287,28 @@
         <v>59.38</v>
       </c>
       <c r="FC2" t="n">
-        <v>34.9</v>
+        <v>34.42</v>
       </c>
       <c r="FD2" t="n">
         <v>74.29000000000001</v>
       </c>
       <c r="FE2" t="n">
-        <v>91.27</v>
+        <v>92.04000000000001</v>
       </c>
       <c r="FF2" t="n">
-        <v>49.47</v>
+        <v>49.03</v>
       </c>
       <c r="FG2" t="n">
-        <v>25.2396</v>
+        <v>25.4151</v>
       </c>
       <c r="FH2" t="n">
-        <v>70.574</v>
+        <v>70.598</v>
       </c>
       <c r="FI2" t="n">
-        <v>50.755</v>
+        <v>57.595</v>
       </c>
       <c r="FJ2" t="n">
-        <v>72.12</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,19 +2322,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>81.84999999999999</v>
+        <v>86.16</v>
       </c>
       <c r="FO2" t="n">
-        <v>73.19</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="FP2" t="n">
-        <v>77.37</v>
+        <v>83.27</v>
       </c>
       <c r="FQ2" t="n">
-        <v>74.48999999999999</v>
+        <v>81.25</v>
       </c>
       <c r="FR2" t="n">
-        <v>94.7</v>
+        <v>99.19</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2351,11 +2351,11 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>77.0005</v>
+        <v>81.3935</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Excellent</t>
         </is>
       </c>
       <c r="FY2" t="b">
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261026_143220</t>
+          <t>20261026_221645</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46321.6057876845</v>
+        <v>46321.928306788</v>
       </c>
     </row>
   </sheetData>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46321.60578703704</v>
+        <v>46321.92829861111</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2667,46 +2667,46 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>2051.2</v>
+        <v>2058.9</v>
       </c>
       <c r="L2" t="n">
         <v>1960</v>
       </c>
       <c r="M2" t="n">
-        <v>2058</v>
+        <v>2058.9</v>
       </c>
       <c r="N2" t="n">
         <v>1951.6</v>
       </c>
       <c r="O2" t="n">
-        <v>2051.2</v>
+        <v>2058.9</v>
       </c>
       <c r="P2" t="n">
-        <v>1614484</v>
+        <v>1858038</v>
       </c>
       <c r="Q2" t="n">
-        <v>2051.2</v>
+        <v>2058.9</v>
       </c>
       <c r="R2" t="n">
-        <v>2284.19</v>
+        <v>2292.14</v>
       </c>
       <c r="S2" t="n">
-        <v>1934.71</v>
+        <v>1942.28</v>
       </c>
       <c r="T2" t="n">
-        <v>11.35871684867396</v>
+        <v>11.32837923162853</v>
       </c>
       <c r="U2" t="n">
-        <v>232.9900000000002</v>
+        <v>233.2399999999998</v>
       </c>
       <c r="V2" t="n">
-        <v>5.679114664586574</v>
+        <v>5.664189615814275</v>
       </c>
       <c r="W2" t="n">
-        <v>116.4899999999998</v>
+        <v>116.6200000000001</v>
       </c>
       <c r="X2" t="n">
-        <v>2.000085844278485</v>
+        <v>1.999999999999996</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>11.35871684867396</v>
+        <v>11.32837923162853</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.679114664586574</v>
+        <v>5.664189615814275</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02044423465830534</v>
+        <v>0.02045507850895603</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.324542163905541</v>
+        <v>0.3247143046979973</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02900736645035623</v>
+        <v>0.02900729525746606</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228671425721302</v>
+        <v>0.04228669057350402</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347614</v>
+        <v>0.1869492979645463</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.04</v>
+        <v>39.02</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-26 14:32:20.080876+05:30</t>
+          <t>2026-10-26 22:16:45.741486+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 11.358716848673959, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000085844278485}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 11.328379231628528, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.999999999999996}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-27 09:05 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -1816,14 +1816,14 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="H2" t="n">
         <v>8.800000000000001</v>
@@ -1859,59 +1859,59 @@
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>10.82</v>
+        <v>10.86</v>
       </c>
       <c r="R2" t="n">
-        <v>48.45</v>
+        <v>48.69</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="n">
-        <v>1960</v>
+        <v>2075</v>
       </c>
       <c r="V2" t="n">
-        <v>2058.9</v>
+        <v>2137.7</v>
       </c>
       <c r="W2" t="n">
-        <v>1951.6</v>
+        <v>2067.4</v>
       </c>
       <c r="X2" t="n">
-        <v>2058.9</v>
+        <v>2131.1</v>
       </c>
       <c r="Y2" t="n">
-        <v>2058.9</v>
+        <v>2131.1</v>
       </c>
       <c r="Z2" t="n">
-        <v>1858038</v>
+        <v>2714843</v>
       </c>
       <c r="AA2" t="n">
-        <v>1476491</v>
+        <v>1540140</v>
       </c>
       <c r="AB2" t="n">
-        <v>1.26</v>
+        <v>1.76</v>
       </c>
       <c r="AC2" t="n">
-        <v>4.51</v>
+        <v>3.51</v>
       </c>
       <c r="AD2" t="n">
-        <v>-0.51</v>
+        <v>0.78</v>
       </c>
       <c r="AE2" t="n">
-        <v>107.3</v>
+        <v>70.3</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.21</v>
+        <v>3.3</v>
       </c>
       <c r="AG2" t="n">
-        <v>58.31</v>
+        <v>59.77</v>
       </c>
       <c r="AH2" t="n">
-        <v>58.31</v>
+        <v>59.77</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.83</v>
+        <v>2.8</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,53 +1920,53 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>1.86</v>
+        <v>5.11</v>
       </c>
       <c r="AM2" t="n">
-        <v>5.71</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="AN2" t="n">
-        <v>44.31</v>
+        <v>48.83</v>
       </c>
       <c r="AO2" t="n">
-        <v>57.43</v>
+        <v>63.94</v>
       </c>
       <c r="AP2" t="n">
-        <v>1.09</v>
+        <v>2.99</v>
       </c>
       <c r="AQ2" t="n">
-        <v>28.58</v>
+        <v>24.38</v>
       </c>
       <c r="AR2" t="n">
-        <v>2058.9</v>
+        <v>2131.1</v>
       </c>
       <c r="AS2" t="n">
-        <v>2292.14</v>
+        <v>2370.2</v>
       </c>
       <c r="AT2" t="n">
-        <v>1942.28</v>
+        <v>2011.55</v>
       </c>
       <c r="AU2" t="n">
-        <v>2058.89990234375</v>
+        <v>2131.10009765625</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>11.33</v>
+        <v>11.22</v>
       </c>
       <c r="AY2" t="n">
-        <v>233.24</v>
+        <v>239.1</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.66</v>
+        <v>5.61</v>
       </c>
       <c r="BA2" t="n">
-        <v>116.62</v>
+        <v>119.55</v>
       </c>
       <c r="BB2" t="n">
-        <v>2.06</v>
+        <v>2.07</v>
       </c>
       <c r="BC2" t="n">
         <v>213</v>
@@ -2008,7 +2008,7 @@
         <v>2.1</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.67</v>
+        <v>8.68</v>
       </c>
       <c r="BQ2" t="n">
         <v>-4.2</v>
@@ -2017,19 +2017,19 @@
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.231</v>
+        <v>0.232</v>
       </c>
       <c r="BT2" t="n">
-        <v>1424.03</v>
+        <v>1426.93</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.63</v>
+        <v>-13.34</v>
       </c>
       <c r="BV2" t="n">
         <v>1.98</v>
       </c>
       <c r="BW2" t="n">
-        <v>2.06</v>
+        <v>2.07</v>
       </c>
       <c r="BX2" t="n">
         <v>2</v>
@@ -2058,7 +2058,7 @@
         <v>49</v>
       </c>
       <c r="CF2" t="n">
-        <v>68.7</v>
+        <v>69</v>
       </c>
       <c r="CG2" t="n">
         <v>69.90000000000001</v>
@@ -2082,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>97.34</v>
+        <v>99.87</v>
       </c>
       <c r="CO2" t="n">
-        <v>39.53</v>
+        <v>43.92</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2109,7 +2109,7 @@
         <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>68.18181818181817</v>
+        <v>77.27272727272727</v>
       </c>
       <c r="CX2" t="n">
         <v>54.54545454545454</v>
@@ -2118,7 +2118,7 @@
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>11.3284</v>
+        <v>11.2196</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,58 +2127,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.7553</v>
+        <v>0.748</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3773</v>
+        <v>0.374</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1133</v>
+        <v>0.1122</v>
       </c>
       <c r="DF2" t="n">
-        <v>2.0018</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.2259</v>
+        <v>1.2185</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0035</v>
+        <v>4.0071</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.6642</v>
+        <v>5.6098</v>
       </c>
       <c r="DJ2" t="n">
-        <v>41.61</v>
+        <v>41.66</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.6642</v>
+        <v>5.6098</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
       </c>
       <c r="DM2" t="n">
+        <v>2.0036</v>
+      </c>
+      <c r="DN2" t="n">
+        <v>4.0071</v>
+      </c>
+      <c r="DO2" t="n">
         <v>2</v>
       </c>
-      <c r="DN2" t="n">
-        <v>4.0035</v>
-      </c>
-      <c r="DO2" t="n">
-        <v>2.0019</v>
-      </c>
       <c r="DP2" t="n">
-        <v>0.7073</v>
+        <v>0.7143</v>
       </c>
       <c r="DQ2" t="n">
-        <v>116.62</v>
+        <v>119.55</v>
       </c>
       <c r="DR2" t="n">
-        <v>73.58</v>
+        <v>52.62</v>
       </c>
       <c r="DS2" t="n">
         <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,16 +2187,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.3852</v>
+        <v>1.0679</v>
       </c>
       <c r="DX2" t="n">
-        <v>93.575</v>
+        <v>90.15000000000001</v>
       </c>
       <c r="DY2" t="n">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="DZ2" t="n">
-        <v>90.699</v>
+        <v>99.76600000000001</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2205,31 +2205,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>87.64</v>
+        <v>99.22</v>
       </c>
       <c r="ED2" t="n">
         <v>100</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.3852</v>
+        <v>1.0679</v>
       </c>
       <c r="EF2" t="n">
-        <v>1.26</v>
+        <v>1.76</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.1179</v>
+        <v>0.3247</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.003</v>
+        <v>4.007</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0128</v>
+        <v>0.0353</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6011</v>
+        <v>0.6062</v>
       </c>
       <c r="EK2" t="n">
-        <v>86.73999999999999</v>
+        <v>92.02</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2243,38 +2243,38 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>44.07</v>
+        <v>100</v>
       </c>
       <c r="EP2" t="n">
-        <v>4.7684</v>
+        <v>10.86</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.1363</v>
+        <v>0.1911</v>
       </c>
       <c r="ER2" t="n">
-        <v>8.992100000000001</v>
+        <v>6.375</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.8642</v>
+        <v>10.9632</v>
       </c>
       <c r="ET2" t="n">
-        <v>46.847</v>
+        <v>65.43899999999999</v>
       </c>
       <c r="EU2" t="n">
-        <v>1.3734</v>
+        <v>5.2624</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.2522</v>
+        <v>1.0145</v>
       </c>
       <c r="EW2" t="n">
-        <v>42.8977</v>
+        <v>99.87</v>
       </c>
       <c r="EX2" t="n">
-        <v>58.53</v>
+        <v>70.03</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Strong</t>
         </is>
       </c>
       <c r="EZ2" t="n">
@@ -2284,31 +2284,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>59.38</v>
+        <v>59.57</v>
       </c>
       <c r="FC2" t="n">
-        <v>34.42</v>
+        <v>32.99</v>
       </c>
       <c r="FD2" t="n">
-        <v>74.29000000000001</v>
+        <v>74.81999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>92.04000000000001</v>
+        <v>95.94499999999999</v>
       </c>
       <c r="FF2" t="n">
-        <v>49.03</v>
+        <v>56.975</v>
       </c>
       <c r="FG2" t="n">
-        <v>25.4151</v>
+        <v>26.2816</v>
       </c>
       <c r="FH2" t="n">
-        <v>70.598</v>
+        <v>73.752</v>
       </c>
       <c r="FI2" t="n">
-        <v>57.595</v>
+        <v>47.14</v>
       </c>
       <c r="FJ2" t="n">
-        <v>72.59999999999999</v>
+        <v>73.34999999999999</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,19 +2322,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>86.16</v>
+        <v>81.54000000000001</v>
       </c>
       <c r="FO2" t="n">
-        <v>72.93000000000001</v>
+        <v>72.73</v>
       </c>
       <c r="FP2" t="n">
-        <v>83.27</v>
+        <v>81.68000000000001</v>
       </c>
       <c r="FQ2" t="n">
-        <v>81.25</v>
+        <v>72.3</v>
       </c>
       <c r="FR2" t="n">
-        <v>99.19</v>
+        <v>97.47</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2351,11 +2351,11 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>81.3935</v>
+        <v>77.547</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
-          <t>Excellent</t>
+          <t>Strong</t>
         </is>
       </c>
       <c r="FY2" t="b">
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261026_221645</t>
+          <t>20261027_143543</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46321.928306788</v>
+        <v>46322.60814664064</v>
       </c>
     </row>
   </sheetData>
@@ -2458,9 +2458,9 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
     <col width="20" customWidth="1" min="23" max="23"/>
-    <col width="19" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46321.92829861111</v>
+        <v>46322.60813657408</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2663,50 +2663,50 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>10.82</v>
+        <v>10.86</v>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>2058.9</v>
+        <v>2131.1</v>
       </c>
       <c r="L2" t="n">
-        <v>1960</v>
+        <v>2075</v>
       </c>
       <c r="M2" t="n">
-        <v>2058.9</v>
+        <v>2137.7</v>
       </c>
       <c r="N2" t="n">
-        <v>1951.6</v>
+        <v>2067.4</v>
       </c>
       <c r="O2" t="n">
-        <v>2058.9</v>
+        <v>2131.1</v>
       </c>
       <c r="P2" t="n">
-        <v>1858038</v>
+        <v>2714843</v>
       </c>
       <c r="Q2" t="n">
-        <v>2058.9</v>
+        <v>2131.1</v>
       </c>
       <c r="R2" t="n">
-        <v>2292.14</v>
+        <v>2370.2</v>
       </c>
       <c r="S2" t="n">
-        <v>1942.28</v>
+        <v>2011.55</v>
       </c>
       <c r="T2" t="n">
-        <v>11.32837923162853</v>
+        <v>11.21955797475482</v>
       </c>
       <c r="U2" t="n">
-        <v>233.2399999999998</v>
+        <v>239.0999999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>5.664189615814275</v>
+        <v>5.609778987377409</v>
       </c>
       <c r="W2" t="n">
-        <v>116.6200000000001</v>
+        <v>119.55</v>
       </c>
       <c r="X2" t="n">
-        <v>1.999999999999996</v>
+        <v>2</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>11.32837923162853</v>
+        <v>11.21955797475482</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.664189615814275</v>
+        <v>5.609778987377409</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02045507850895603</v>
+        <v>0.02047672642086394</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3247143046979973</v>
+        <v>0.3250579546458702</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02900729525746606</v>
+        <v>0.02900127607683251</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228669057350402</v>
+        <v>0.04228670255513612</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645463</v>
+        <v>0.1869492979645462</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39.02</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-26 22:16:45.741486+05:30</t>
+          <t>2026-10-27 14:35:43.904538+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 11.328379231628528, 'average_current_return_pct': 0.0, 'average_risk_reward': 1.999999999999996}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 11.219557974754817, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-27 15:51 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="18" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -1862,7 +1862,7 @@
         <v>10.86</v>
       </c>
       <c r="R2" t="n">
-        <v>48.69</v>
+        <v>48.79</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1872,46 +1872,46 @@
         <v>2075</v>
       </c>
       <c r="V2" t="n">
-        <v>2137.7</v>
+        <v>2143.1</v>
       </c>
       <c r="W2" t="n">
         <v>2067.4</v>
       </c>
       <c r="X2" t="n">
-        <v>2131.1</v>
+        <v>2142</v>
       </c>
       <c r="Y2" t="n">
-        <v>2131.1</v>
+        <v>2142</v>
       </c>
       <c r="Z2" t="n">
-        <v>2714843</v>
+        <v>3116290</v>
       </c>
       <c r="AA2" t="n">
-        <v>1540140</v>
+        <v>1560213</v>
       </c>
       <c r="AB2" t="n">
-        <v>1.76</v>
+        <v>2</v>
       </c>
       <c r="AC2" t="n">
-        <v>3.51</v>
+        <v>4.04</v>
       </c>
       <c r="AD2" t="n">
         <v>0.78</v>
       </c>
       <c r="AE2" t="n">
-        <v>70.3</v>
+        <v>75.7</v>
       </c>
       <c r="AF2" t="n">
-        <v>3.3</v>
+        <v>3.53</v>
       </c>
       <c r="AG2" t="n">
-        <v>59.77</v>
+        <v>60.16</v>
       </c>
       <c r="AH2" t="n">
-        <v>59.77</v>
+        <v>60.16</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.8</v>
+        <v>2.81</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,50 +1920,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>5.11</v>
+        <v>5.62</v>
       </c>
       <c r="AM2" t="n">
-        <v>9.109999999999999</v>
+        <v>9.65</v>
       </c>
       <c r="AN2" t="n">
-        <v>48.83</v>
+        <v>49.59</v>
       </c>
       <c r="AO2" t="n">
-        <v>63.94</v>
+        <v>64.75</v>
       </c>
       <c r="AP2" t="n">
-        <v>2.99</v>
+        <v>3.52</v>
       </c>
       <c r="AQ2" t="n">
-        <v>24.38</v>
+        <v>25.01</v>
       </c>
       <c r="AR2" t="n">
-        <v>2131.1</v>
+        <v>2142</v>
       </c>
       <c r="AS2" t="n">
-        <v>2370.2</v>
+        <v>2382.64</v>
       </c>
       <c r="AT2" t="n">
-        <v>2011.55</v>
+        <v>2021.68</v>
       </c>
       <c r="AU2" t="n">
-        <v>2131.10009765625</v>
+        <v>2142</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>11.22</v>
+        <v>11.23</v>
       </c>
       <c r="AY2" t="n">
-        <v>239.1</v>
+        <v>240.64</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.61</v>
+        <v>5.62</v>
       </c>
       <c r="BA2" t="n">
-        <v>119.55</v>
+        <v>120.32</v>
       </c>
       <c r="BB2" t="n">
         <v>2.07</v>
@@ -2020,10 +2020,10 @@
         <v>0.232</v>
       </c>
       <c r="BT2" t="n">
-        <v>1426.93</v>
+        <v>1427.37</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.34</v>
+        <v>-13.3</v>
       </c>
       <c r="BV2" t="n">
         <v>1.98</v>
@@ -2082,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="CN2" t="n">
-        <v>99.87</v>
+        <v>100</v>
       </c>
       <c r="CO2" t="n">
-        <v>43.92</v>
+        <v>40.46</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2100,7 +2100,7 @@
         <v>100</v>
       </c>
       <c r="CT2" t="n">
-        <v>95.45454545454545</v>
+        <v>100</v>
       </c>
       <c r="CU2" t="n">
         <v>95.45454545454545</v>
@@ -2118,7 +2118,7 @@
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>11.2196</v>
+        <v>11.2344</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,58 +2127,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.748</v>
+        <v>0.7487</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.374</v>
+        <v>0.3747</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1122</v>
+        <v>0.1123</v>
       </c>
       <c r="DF2" t="n">
-        <v>2</v>
+        <v>1.9982</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.2185</v>
+        <v>1.2196</v>
       </c>
       <c r="DH2" t="n">
-        <v>4.0071</v>
+        <v>3.9964</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.6098</v>
+        <v>5.6172</v>
       </c>
       <c r="DJ2" t="n">
-        <v>41.66</v>
+        <v>42.05</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.6098</v>
+        <v>5.6172</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
       </c>
       <c r="DM2" t="n">
-        <v>2.0036</v>
+        <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>4.0071</v>
+        <v>3.9964</v>
       </c>
       <c r="DO2" t="n">
-        <v>2</v>
+        <v>1.9981</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.7143</v>
+        <v>0.7111</v>
       </c>
       <c r="DQ2" t="n">
-        <v>119.55</v>
+        <v>120.32</v>
       </c>
       <c r="DR2" t="n">
-        <v>52.62</v>
+        <v>42.76</v>
       </c>
       <c r="DS2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="DT2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,16 +2187,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.0679</v>
+        <v>1.2527</v>
       </c>
       <c r="DX2" t="n">
-        <v>90.15000000000001</v>
+        <v>88.125</v>
       </c>
       <c r="DY2" t="n">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="DZ2" t="n">
-        <v>99.76600000000001</v>
+        <v>99.988</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2205,31 +2205,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>99.22</v>
+        <v>99.95999999999999</v>
       </c>
       <c r="ED2" t="n">
-        <v>100</v>
+        <v>97.12</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.0679</v>
+        <v>1.2527</v>
       </c>
       <c r="EF2" t="n">
-        <v>1.76</v>
+        <v>2</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.3247</v>
+        <v>0.3823</v>
       </c>
       <c r="EH2" t="n">
-        <v>4.007</v>
+        <v>3.998</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0353</v>
+        <v>0.0415</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6062</v>
+        <v>0.6039</v>
       </c>
       <c r="EK2" t="n">
-        <v>92.02</v>
+        <v>91.51000000000001</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,28 +2249,28 @@
         <v>10.86</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.1911</v>
+        <v>0.2172</v>
       </c>
       <c r="ER2" t="n">
-        <v>6.375</v>
+        <v>5.615</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.9632</v>
+        <v>11.0367</v>
       </c>
       <c r="ET2" t="n">
-        <v>65.43899999999999</v>
+        <v>64.05500000000001</v>
       </c>
       <c r="EU2" t="n">
-        <v>5.2624</v>
+        <v>7.04</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.0145</v>
+        <v>0.9367</v>
       </c>
       <c r="EW2" t="n">
-        <v>99.87</v>
+        <v>100</v>
       </c>
       <c r="EX2" t="n">
-        <v>70.03</v>
+        <v>69.01000000000001</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2287,28 +2287,28 @@
         <v>59.57</v>
       </c>
       <c r="FC2" t="n">
-        <v>32.99</v>
+        <v>33.24</v>
       </c>
       <c r="FD2" t="n">
         <v>74.81999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>95.94499999999999</v>
+        <v>95.755</v>
       </c>
       <c r="FF2" t="n">
-        <v>56.975</v>
+        <v>54.735</v>
       </c>
       <c r="FG2" t="n">
-        <v>26.2816</v>
+        <v>26.2467</v>
       </c>
       <c r="FH2" t="n">
-        <v>73.752</v>
+        <v>73.587</v>
       </c>
       <c r="FI2" t="n">
-        <v>47.14</v>
+        <v>42.405</v>
       </c>
       <c r="FJ2" t="n">
-        <v>73.34999999999999</v>
+        <v>72.64</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,19 +2322,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>81.54000000000001</v>
+        <v>77.20999999999999</v>
       </c>
       <c r="FO2" t="n">
-        <v>72.73</v>
+        <v>72.94</v>
       </c>
       <c r="FP2" t="n">
-        <v>81.68000000000001</v>
+        <v>74.54000000000001</v>
       </c>
       <c r="FQ2" t="n">
-        <v>72.3</v>
+        <v>65.81999999999999</v>
       </c>
       <c r="FR2" t="n">
-        <v>97.47</v>
+        <v>92.01000000000001</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>77.547</v>
+        <v>73.25449999999999</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261027_143543</t>
+          <t>20261027_212138</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46322.60814664064</v>
+        <v>46322.89002405529</v>
       </c>
     </row>
   </sheetData>
@@ -2458,7 +2458,7 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="22" max="22"/>
     <col width="20" customWidth="1" min="23" max="23"/>
     <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46322.60813657408</v>
+        <v>46322.89002314815</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2667,43 +2667,43 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>2131.1</v>
+        <v>2142</v>
       </c>
       <c r="L2" t="n">
         <v>2075</v>
       </c>
       <c r="M2" t="n">
-        <v>2137.7</v>
+        <v>2143.1</v>
       </c>
       <c r="N2" t="n">
         <v>2067.4</v>
       </c>
       <c r="O2" t="n">
-        <v>2131.1</v>
+        <v>2142</v>
       </c>
       <c r="P2" t="n">
-        <v>2714843</v>
+        <v>3116290</v>
       </c>
       <c r="Q2" t="n">
-        <v>2131.1</v>
+        <v>2142</v>
       </c>
       <c r="R2" t="n">
-        <v>2370.2</v>
+        <v>2382.64</v>
       </c>
       <c r="S2" t="n">
-        <v>2011.55</v>
+        <v>2021.68</v>
       </c>
       <c r="T2" t="n">
-        <v>11.21955797475482</v>
+        <v>11.23436041083099</v>
       </c>
       <c r="U2" t="n">
-        <v>239.0999999999999</v>
+        <v>240.6399999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>5.609778987377409</v>
+        <v>5.617180205415496</v>
       </c>
       <c r="W2" t="n">
-        <v>119.55</v>
+        <v>120.3199999999999</v>
       </c>
       <c r="X2" t="n">
         <v>2</v>
@@ -2727,10 +2727,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>11.21955797475482</v>
+        <v>11.23436041083099</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.609778987377409</v>
+        <v>5.617180205415496</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02047672642086394</v>
+        <v>0.02048938366715312</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3250579546458702</v>
+        <v>0.3252588822016546</v>
       </c>
     </row>
     <row r="7">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228670255513612</v>
+        <v>0.04228670443788259</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645462</v>
+        <v>0.1869492979645463</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39</v>
+        <v>38.98</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-27 14:35:43.904538+05:30</t>
+          <t>2026-10-27 21:21:38.104398+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 11.219557974754817, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 11.234360410830993, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-28 09:46 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="18" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="17" customWidth="1" min="128" max="128"/>
+    <col width="19" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,14 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46322</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
+        <v>46323</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>46323</v>
+      </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="H2" t="n">
         <v>8.800000000000001</v>
@@ -1852,66 +1854,70 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="P2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q2" t="n">
         <v>10.86</v>
       </c>
       <c r="R2" t="n">
-        <v>48.79</v>
+        <v>48.5</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
       </c>
-      <c r="T2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>UPTREND</t>
+        </is>
+      </c>
       <c r="U2" t="n">
-        <v>2075</v>
+        <v>2142</v>
       </c>
       <c r="V2" t="n">
-        <v>2143.1</v>
+        <v>2198.8</v>
       </c>
       <c r="W2" t="n">
-        <v>2067.4</v>
+        <v>2131.7</v>
       </c>
       <c r="X2" t="n">
-        <v>2142</v>
+        <v>2181.9</v>
       </c>
       <c r="Y2" t="n">
-        <v>2142</v>
+        <v>2181.9</v>
       </c>
       <c r="Z2" t="n">
-        <v>3116290</v>
+        <v>2137249</v>
       </c>
       <c r="AA2" t="n">
-        <v>1560213</v>
+        <v>1619591</v>
       </c>
       <c r="AB2" t="n">
-        <v>2</v>
+        <v>1.32</v>
       </c>
       <c r="AC2" t="n">
-        <v>4.04</v>
+        <v>1.86</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.78</v>
+        <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>75.7</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="AF2" t="n">
-        <v>3.53</v>
+        <v>3.08</v>
       </c>
       <c r="AG2" t="n">
-        <v>60.16</v>
+        <v>60.66</v>
       </c>
       <c r="AH2" t="n">
-        <v>60.16</v>
+        <v>60.66</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.81</v>
+        <v>2.78</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1920,59 +1926,59 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>5.62</v>
+        <v>7.13</v>
       </c>
       <c r="AM2" t="n">
-        <v>9.65</v>
+        <v>11.25</v>
       </c>
       <c r="AN2" t="n">
-        <v>49.59</v>
+        <v>51.8</v>
       </c>
       <c r="AO2" t="n">
-        <v>64.75</v>
+        <v>67.63</v>
       </c>
       <c r="AP2" t="n">
-        <v>3.52</v>
+        <v>5.95</v>
       </c>
       <c r="AQ2" t="n">
-        <v>25.01</v>
+        <v>24.05</v>
       </c>
       <c r="AR2" t="n">
-        <v>2142</v>
+        <v>2181.9</v>
       </c>
       <c r="AS2" t="n">
-        <v>2382.64</v>
+        <v>2424.52</v>
       </c>
       <c r="AT2" t="n">
-        <v>2021.68</v>
+        <v>2060.59</v>
       </c>
       <c r="AU2" t="n">
-        <v>2142</v>
+        <v>2181.89990234375</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>11.23</v>
+        <v>11.12</v>
       </c>
       <c r="AY2" t="n">
-        <v>240.64</v>
+        <v>242.62</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.62</v>
+        <v>5.56</v>
       </c>
       <c r="BA2" t="n">
-        <v>120.32</v>
+        <v>121.31</v>
       </c>
       <c r="BB2" t="n">
         <v>2.07</v>
       </c>
       <c r="BC2" t="n">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="BD2" t="n">
-        <v>31.4</v>
+        <v>31.5</v>
       </c>
       <c r="BE2" t="n">
         <v>342</v>
@@ -1981,10 +1987,10 @@
         <v>50.4</v>
       </c>
       <c r="BG2" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.3</v>
+        <v>18.1</v>
       </c>
       <c r="BI2" t="n">
         <v>0</v>
@@ -2008,7 +2014,7 @@
         <v>2.1</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.68</v>
+        <v>8.69</v>
       </c>
       <c r="BQ2" t="n">
         <v>-4.2</v>
@@ -2020,10 +2026,10 @@
         <v>0.232</v>
       </c>
       <c r="BT2" t="n">
-        <v>1427.37</v>
+        <v>1428.97</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.3</v>
+        <v>-13.14</v>
       </c>
       <c r="BV2" t="n">
         <v>1.98</v>
@@ -2085,16 +2091,16 @@
         <v>100</v>
       </c>
       <c r="CO2" t="n">
-        <v>40.46</v>
+        <v>40.01</v>
       </c>
       <c r="CP2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CQ2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CR2" t="n">
-        <v>86.36363636363636</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="CS2" t="n">
         <v>100</v>
@@ -2103,22 +2109,22 @@
         <v>100</v>
       </c>
       <c r="CU2" t="n">
-        <v>95.45454545454545</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="CV2" t="n">
-        <v>86.36363636363636</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="CW2" t="n">
-        <v>77.27272727272727</v>
+        <v>76.19047619047619</v>
       </c>
       <c r="CX2" t="n">
-        <v>54.54545454545454</v>
+        <v>57.14285714285714</v>
       </c>
       <c r="CY2" t="n">
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>11.2344</v>
+        <v>11.1197</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2127,31 +2133,31 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.7487</v>
+        <v>0.7413</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3747</v>
+        <v>0.3707</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1123</v>
+        <v>0.1112</v>
       </c>
       <c r="DF2" t="n">
-        <v>1.9982</v>
+        <v>2</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.2196</v>
+        <v>1.2076</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9964</v>
+        <v>4</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.6172</v>
+        <v>5.5598</v>
       </c>
       <c r="DJ2" t="n">
-        <v>42.05</v>
+        <v>41</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.6172</v>
+        <v>5.5598</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
@@ -2160,25 +2166,25 @@
         <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9964</v>
+        <v>4</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9981</v>
+        <v>1.9997</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.7111</v>
+        <v>0.7194</v>
       </c>
       <c r="DQ2" t="n">
-        <v>120.32</v>
+        <v>121.31</v>
       </c>
       <c r="DR2" t="n">
-        <v>42.76</v>
+        <v>51.57</v>
       </c>
       <c r="DS2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2187,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>1.2527</v>
+        <v>2.1403</v>
       </c>
       <c r="DX2" t="n">
-        <v>88.125</v>
+        <v>80.92500000000001</v>
       </c>
       <c r="DY2" t="n">
-        <v>100</v>
+        <v>66</v>
       </c>
       <c r="DZ2" t="n">
-        <v>99.988</v>
+        <v>98.464</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2205,31 +2211,31 @@
         <v>10</v>
       </c>
       <c r="EC2" t="n">
-        <v>99.95999999999999</v>
+        <v>100</v>
       </c>
       <c r="ED2" t="n">
-        <v>97.12</v>
+        <v>94.91</v>
       </c>
       <c r="EE2" t="n">
-        <v>1.2527</v>
+        <v>2.1403</v>
       </c>
       <c r="EF2" t="n">
-        <v>2</v>
+        <v>1.32</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.3823</v>
+        <v>0.6462</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.998</v>
+        <v>3.9999</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0415</v>
+        <v>0.0702</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6039</v>
+        <v>0.6097</v>
       </c>
       <c r="EK2" t="n">
-        <v>91.51000000000001</v>
+        <v>91.63</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2243,34 +2249,34 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>100</v>
+        <v>84.64</v>
       </c>
       <c r="EP2" t="n">
-        <v>10.86</v>
+        <v>9.1919</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.2172</v>
+        <v>0.1434</v>
       </c>
       <c r="ER2" t="n">
-        <v>5.615</v>
+        <v>8.424200000000001</v>
       </c>
       <c r="ES2" t="n">
-        <v>11.0367</v>
+        <v>10.8466</v>
       </c>
       <c r="ET2" t="n">
-        <v>64.05500000000001</v>
+        <v>59.177</v>
       </c>
       <c r="EU2" t="n">
-        <v>7.04</v>
+        <v>7.854</v>
       </c>
       <c r="EV2" t="n">
-        <v>0.9367</v>
+        <v>1.1983</v>
       </c>
       <c r="EW2" t="n">
-        <v>100</v>
+        <v>84.64</v>
       </c>
       <c r="EX2" t="n">
-        <v>69.01000000000001</v>
+        <v>60.17</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2284,31 +2290,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>59.57</v>
+        <v>59.27</v>
       </c>
       <c r="FC2" t="n">
-        <v>33.24</v>
+        <v>31.13</v>
       </c>
       <c r="FD2" t="n">
-        <v>74.81999999999999</v>
+        <v>74.70999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>95.755</v>
+        <v>95.815</v>
       </c>
       <c r="FF2" t="n">
-        <v>54.735</v>
+        <v>50.09</v>
       </c>
       <c r="FG2" t="n">
-        <v>26.2467</v>
+        <v>26.455</v>
       </c>
       <c r="FH2" t="n">
-        <v>73.587</v>
+        <v>71.669</v>
       </c>
       <c r="FI2" t="n">
-        <v>42.405</v>
+        <v>46.285</v>
       </c>
       <c r="FJ2" t="n">
-        <v>72.64</v>
+        <v>71.69</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2322,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>77.20999999999999</v>
+        <v>81.3</v>
       </c>
       <c r="FO2" t="n">
-        <v>72.94</v>
+        <v>72.56999999999999</v>
       </c>
       <c r="FP2" t="n">
-        <v>74.54000000000001</v>
+        <v>77.81</v>
       </c>
       <c r="FQ2" t="n">
-        <v>65.81999999999999</v>
+        <v>73.28</v>
       </c>
       <c r="FR2" t="n">
-        <v>92.01000000000001</v>
+        <v>95.48</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2351,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>73.25449999999999</v>
+        <v>75.9635</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2416,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261027_212138</t>
+          <t>20261028_151613</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46322.89002405529</v>
+        <v>46323.63626676596</v>
       </c>
     </row>
   </sheetData>
@@ -2438,8 +2444,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -2458,7 +2464,7 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
     <col width="20" customWidth="1" min="23" max="23"/>
     <col width="13" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
@@ -2641,10 +2647,14 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46322.89002314815</v>
-      </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
+        <v>46323.63626157407</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>46323</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>46338</v>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>LAURUSLABS</t>
@@ -2665,45 +2675,49 @@
       <c r="I2" t="n">
         <v>10.86</v>
       </c>
-      <c r="J2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>UPTREND</t>
+        </is>
+      </c>
       <c r="K2" t="n">
+        <v>2181.9</v>
+      </c>
+      <c r="L2" t="n">
         <v>2142</v>
       </c>
-      <c r="L2" t="n">
-        <v>2075</v>
-      </c>
       <c r="M2" t="n">
-        <v>2143.1</v>
+        <v>2198.8</v>
       </c>
       <c r="N2" t="n">
-        <v>2067.4</v>
+        <v>2131.7</v>
       </c>
       <c r="O2" t="n">
-        <v>2142</v>
+        <v>2181.9</v>
       </c>
       <c r="P2" t="n">
-        <v>3116290</v>
+        <v>2137249</v>
       </c>
       <c r="Q2" t="n">
-        <v>2142</v>
+        <v>2181.9</v>
       </c>
       <c r="R2" t="n">
-        <v>2382.64</v>
+        <v>2424.52</v>
       </c>
       <c r="S2" t="n">
-        <v>2021.68</v>
+        <v>2060.59</v>
       </c>
       <c r="T2" t="n">
-        <v>11.23436041083099</v>
+        <v>11.11966634584536</v>
       </c>
       <c r="U2" t="n">
-        <v>240.6399999999999</v>
+        <v>242.6199999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>5.617180205415496</v>
+        <v>5.559833172922679</v>
       </c>
       <c r="W2" t="n">
-        <v>120.3199999999999</v>
+        <v>121.3099999999999</v>
       </c>
       <c r="X2" t="n">
         <v>2</v>
@@ -2727,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>11.23436041083099</v>
+        <v>11.11966634584536</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.617180205415496</v>
+        <v>5.559833172922679</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2805,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02048938366715312</v>
+        <v>0.02048376790538074</v>
       </c>
     </row>
     <row r="6">
@@ -2815,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3252588822016546</v>
+        <v>0.3251697347472232</v>
       </c>
     </row>
     <row r="7">
@@ -2865,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02900127607683251</v>
+        <v>0.02899525448839418</v>
       </c>
     </row>
     <row r="12">
@@ -2875,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228670443788259</v>
+        <v>0.0422867071950403</v>
       </c>
     </row>
     <row r="13">
@@ -2885,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645463</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -2905,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.98</v>
+        <v>38.99</v>
       </c>
     </row>
     <row r="16">
@@ -3184,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-27 21:21:38.104398+05:30</t>
+          <t>2026-10-28 15:16:13.465897+05:30</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 11.234360410830993, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 11.119666345845358, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-28 16:35 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -1864,7 +1864,7 @@
         <v>10.86</v>
       </c>
       <c r="R2" t="n">
-        <v>48.5</v>
+        <v>48.52</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1890,13 +1890,13 @@
         <v>2181.9</v>
       </c>
       <c r="Z2" t="n">
-        <v>2137249</v>
+        <v>2200547</v>
       </c>
       <c r="AA2" t="n">
-        <v>1619591</v>
+        <v>1622756</v>
       </c>
       <c r="AB2" t="n">
-        <v>1.32</v>
+        <v>1.36</v>
       </c>
       <c r="AC2" t="n">
         <v>1.86</v>
@@ -2026,7 +2026,7 @@
         <v>0.232</v>
       </c>
       <c r="BT2" t="n">
-        <v>1428.97</v>
+        <v>1428.98</v>
       </c>
       <c r="BU2" t="n">
         <v>-13.14</v>
@@ -2091,34 +2091,34 @@
         <v>100</v>
       </c>
       <c r="CO2" t="n">
-        <v>40.01</v>
+        <v>40.02</v>
       </c>
       <c r="CP2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CQ2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CR2" t="n">
-        <v>85.71428571428571</v>
+        <v>86.36363636363636</v>
       </c>
       <c r="CS2" t="n">
         <v>100</v>
       </c>
       <c r="CT2" t="n">
-        <v>100</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CU2" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="CV2" t="n">
-        <v>85.71428571428571</v>
+        <v>86.36363636363636</v>
       </c>
       <c r="CW2" t="n">
-        <v>76.19047619047619</v>
+        <v>77.27272727272727</v>
       </c>
       <c r="CX2" t="n">
-        <v>57.14285714285714</v>
+        <v>54.54545454545454</v>
       </c>
       <c r="CY2" t="n">
         <v>1</v>
@@ -2154,7 +2154,7 @@
         <v>5.5598</v>
       </c>
       <c r="DJ2" t="n">
-        <v>41</v>
+        <v>41.07</v>
       </c>
       <c r="DK2" t="n">
         <v>5.5598</v>
@@ -2178,13 +2178,13 @@
         <v>121.31</v>
       </c>
       <c r="DR2" t="n">
-        <v>51.57</v>
+        <v>54.88</v>
       </c>
       <c r="DS2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="DT2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2199,10 +2199,10 @@
         <v>80.92500000000001</v>
       </c>
       <c r="DY2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="DZ2" t="n">
-        <v>98.464</v>
+        <v>98.498</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2214,13 +2214,13 @@
         <v>100</v>
       </c>
       <c r="ED2" t="n">
-        <v>94.91</v>
+        <v>99.23999999999999</v>
       </c>
       <c r="EE2" t="n">
         <v>2.1403</v>
       </c>
       <c r="EF2" t="n">
-        <v>1.32</v>
+        <v>1.36</v>
       </c>
       <c r="EG2" t="n">
         <v>0.6462</v>
@@ -2235,7 +2235,7 @@
         <v>0.6097</v>
       </c>
       <c r="EK2" t="n">
-        <v>91.63</v>
+        <v>92.25</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2249,34 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>84.64</v>
+        <v>84.98</v>
       </c>
       <c r="EP2" t="n">
-        <v>9.1919</v>
+        <v>9.2288</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.1434</v>
+        <v>0.1477</v>
       </c>
       <c r="ER2" t="n">
-        <v>8.424200000000001</v>
+        <v>8.176500000000001</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.8466</v>
+        <v>10.8651</v>
       </c>
       <c r="ET2" t="n">
-        <v>59.177</v>
+        <v>59.373</v>
       </c>
       <c r="EU2" t="n">
-        <v>7.854</v>
+        <v>8.092000000000001</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.1983</v>
+        <v>1.178</v>
       </c>
       <c r="EW2" t="n">
-        <v>84.64</v>
+        <v>84.98</v>
       </c>
       <c r="EX2" t="n">
-        <v>60.17</v>
+        <v>60.98</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2290,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>59.27</v>
+        <v>59.57</v>
       </c>
       <c r="FC2" t="n">
-        <v>31.13</v>
+        <v>31.27</v>
       </c>
       <c r="FD2" t="n">
-        <v>74.70999999999999</v>
+        <v>74.81999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>95.815</v>
+        <v>96.125</v>
       </c>
       <c r="FF2" t="n">
-        <v>50.09</v>
+        <v>50.5</v>
       </c>
       <c r="FG2" t="n">
         <v>26.455</v>
       </c>
       <c r="FH2" t="n">
-        <v>71.669</v>
+        <v>71.98099999999999</v>
       </c>
       <c r="FI2" t="n">
-        <v>46.285</v>
+        <v>47.975</v>
       </c>
       <c r="FJ2" t="n">
-        <v>71.69</v>
+        <v>72.28</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>81.3</v>
+        <v>82.13</v>
       </c>
       <c r="FO2" t="n">
-        <v>72.56999999999999</v>
+        <v>72.54000000000001</v>
       </c>
       <c r="FP2" t="n">
-        <v>77.81</v>
+        <v>79.61</v>
       </c>
       <c r="FQ2" t="n">
-        <v>73.28</v>
+        <v>74.33</v>
       </c>
       <c r="FR2" t="n">
-        <v>95.48</v>
+        <v>95.84999999999999</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>75.9635</v>
+        <v>76.7735</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261028_151613</t>
+          <t>20261028_220543</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46323.63626676596</v>
+        <v>46323.92064266764</v>
       </c>
     </row>
   </sheetData>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46323.63626157407</v>
+        <v>46323.92063657408</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46323</v>
@@ -2696,7 +2696,7 @@
         <v>2181.9</v>
       </c>
       <c r="P2" t="n">
-        <v>2137249</v>
+        <v>2200547</v>
       </c>
       <c r="Q2" t="n">
         <v>2181.9</v>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02048376790538074</v>
+        <v>0.02048377260105075</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3251697347472232</v>
+        <v>0.3251698092886738</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02899525448839418</v>
+        <v>0.02899533758147449</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.0422867071950403</v>
+        <v>0.04228671424003135</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869493934347614</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-28 15:16:13.465897+05:30</t>
+          <t>2026-10-28 22:05:43.545047+05:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-29 10:04 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -641,7 +641,7 @@
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
     <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="18" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="18" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="19" customWidth="1" min="128" max="128"/>
+    <col width="17" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="H2" t="n">
         <v>8.800000000000001</v>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>STRONG BUY</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>10.86</v>
+        <v>10.93</v>
       </c>
       <c r="R2" t="n">
-        <v>48.52</v>
+        <v>48.74</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>2142</v>
+        <v>2190</v>
       </c>
       <c r="V2" t="n">
-        <v>2198.8</v>
+        <v>2244</v>
       </c>
       <c r="W2" t="n">
-        <v>2131.7</v>
+        <v>2166</v>
       </c>
       <c r="X2" t="n">
-        <v>2181.9</v>
+        <v>2244</v>
       </c>
       <c r="Y2" t="n">
-        <v>2181.9</v>
+        <v>2244</v>
       </c>
       <c r="Z2" t="n">
-        <v>2200547</v>
+        <v>2952155</v>
       </c>
       <c r="AA2" t="n">
-        <v>1622756</v>
+        <v>1648794</v>
       </c>
       <c r="AB2" t="n">
-        <v>1.36</v>
+        <v>1.79</v>
       </c>
       <c r="AC2" t="n">
-        <v>1.86</v>
+        <v>2.85</v>
       </c>
       <c r="AD2" t="n">
-        <v>0</v>
+        <v>0.37</v>
       </c>
       <c r="AE2" t="n">
-        <v>67.09999999999999</v>
+        <v>78</v>
       </c>
       <c r="AF2" t="n">
-        <v>3.08</v>
+        <v>3.48</v>
       </c>
       <c r="AG2" t="n">
-        <v>60.66</v>
+        <v>61.89</v>
       </c>
       <c r="AH2" t="n">
-        <v>60.66</v>
+        <v>61.89</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.78</v>
+        <v>2.76</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,50 +1926,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>7.13</v>
+        <v>9.470000000000001</v>
       </c>
       <c r="AM2" t="n">
-        <v>11.25</v>
+        <v>13.91</v>
       </c>
       <c r="AN2" t="n">
-        <v>51.8</v>
+        <v>55.51</v>
       </c>
       <c r="AO2" t="n">
-        <v>67.63</v>
+        <v>71.53</v>
       </c>
       <c r="AP2" t="n">
-        <v>5.95</v>
+        <v>10.17</v>
       </c>
       <c r="AQ2" t="n">
-        <v>24.05</v>
+        <v>25.98</v>
       </c>
       <c r="AR2" t="n">
-        <v>2181.9</v>
+        <v>2244</v>
       </c>
       <c r="AS2" t="n">
-        <v>2424.52</v>
+        <v>2491.58</v>
       </c>
       <c r="AT2" t="n">
-        <v>2060.59</v>
+        <v>2120.21</v>
       </c>
       <c r="AU2" t="n">
-        <v>2181.89990234375</v>
+        <v>2244</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>11.12</v>
+        <v>11.03</v>
       </c>
       <c r="AY2" t="n">
-        <v>242.62</v>
+        <v>247.58</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.56</v>
+        <v>5.52</v>
       </c>
       <c r="BA2" t="n">
-        <v>121.31</v>
+        <v>123.79</v>
       </c>
       <c r="BB2" t="n">
         <v>2.07</v>
@@ -1984,13 +1984,13 @@
         <v>342</v>
       </c>
       <c r="BF2" t="n">
-        <v>50.4</v>
+        <v>50.3</v>
       </c>
       <c r="BG2" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.1</v>
+        <v>18.2</v>
       </c>
       <c r="BI2" t="n">
         <v>0</v>
@@ -2005,16 +2005,16 @@
         <v>0</v>
       </c>
       <c r="BM2" t="n">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="BN2" t="n">
-        <v>48.9</v>
+        <v>49</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.1</v>
+        <v>2.11</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.69</v>
+        <v>8.68</v>
       </c>
       <c r="BQ2" t="n">
         <v>-4.2</v>
@@ -2023,13 +2023,13 @@
         <v>9.1</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.232</v>
+        <v>0.233</v>
       </c>
       <c r="BT2" t="n">
-        <v>1428.98</v>
+        <v>1433.28</v>
       </c>
       <c r="BU2" t="n">
-        <v>-13.14</v>
+        <v>-12.71</v>
       </c>
       <c r="BV2" t="n">
         <v>1.98</v>
@@ -2047,7 +2047,7 @@
         <v>8</v>
       </c>
       <c r="CA2" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="CB2" t="n">
         <v>0</v>
@@ -2058,7 +2058,7 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>42</v>
+        <v>42.2</v>
       </c>
       <c r="CE2" t="n">
         <v>49</v>
@@ -2067,7 +2067,7 @@
         <v>69</v>
       </c>
       <c r="CG2" t="n">
-        <v>69.90000000000001</v>
+        <v>70</v>
       </c>
       <c r="CH2" t="n">
         <v>100</v>
@@ -2091,7 +2091,7 @@
         <v>100</v>
       </c>
       <c r="CO2" t="n">
-        <v>40.02</v>
+        <v>44.98</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2124,7 +2124,7 @@
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>11.1197</v>
+        <v>11.033</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,31 +2133,31 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.7413</v>
+        <v>0.7353</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.3707</v>
+        <v>0.368</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1112</v>
+        <v>0.1103</v>
       </c>
       <c r="DF2" t="n">
-        <v>2</v>
+        <v>1.9982</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.2076</v>
+        <v>1.2056</v>
       </c>
       <c r="DH2" t="n">
-        <v>4</v>
+        <v>3.9964</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.5598</v>
+        <v>5.5165</v>
       </c>
       <c r="DJ2" t="n">
-        <v>41.07</v>
+        <v>42.74</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.5598</v>
+        <v>5.5165</v>
       </c>
       <c r="DL2" t="n">
         <v>2</v>
@@ -2166,25 +2166,25 @@
         <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>4</v>
+        <v>3.9964</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9997</v>
+        <v>1.9981</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.7194</v>
+        <v>0.724</v>
       </c>
       <c r="DQ2" t="n">
-        <v>121.31</v>
+        <v>123.79</v>
       </c>
       <c r="DR2" t="n">
-        <v>54.88</v>
+        <v>38.96</v>
       </c>
       <c r="DS2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="DT2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>2.1403</v>
+        <v>3.6848</v>
       </c>
       <c r="DX2" t="n">
-        <v>80.92500000000001</v>
+        <v>71.175</v>
       </c>
       <c r="DY2" t="n">
-        <v>68</v>
+        <v>89.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>98.498</v>
+        <v>100</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2214,28 +2214,28 @@
         <v>100</v>
       </c>
       <c r="ED2" t="n">
-        <v>99.23999999999999</v>
+        <v>60.01</v>
       </c>
       <c r="EE2" t="n">
-        <v>2.1403</v>
+        <v>3.6848</v>
       </c>
       <c r="EF2" t="n">
-        <v>1.36</v>
+        <v>1.79</v>
       </c>
       <c r="EG2" t="n">
-        <v>0.6462</v>
+        <v>1.1116</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9999</v>
+        <v>3.9975</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.0702</v>
+        <v>0.1215</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6097</v>
+        <v>0.6131</v>
       </c>
       <c r="EK2" t="n">
-        <v>92.25</v>
+        <v>83.52</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
@@ -2249,34 +2249,34 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>84.98</v>
+        <v>100</v>
       </c>
       <c r="EP2" t="n">
-        <v>9.2288</v>
+        <v>10.93</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.1477</v>
+        <v>0.1956</v>
       </c>
       <c r="ER2" t="n">
-        <v>8.176500000000001</v>
+        <v>6.162</v>
       </c>
       <c r="ES2" t="n">
-        <v>10.8651</v>
+        <v>11.367</v>
       </c>
       <c r="ET2" t="n">
-        <v>59.373</v>
+        <v>65.965</v>
       </c>
       <c r="EU2" t="n">
-        <v>8.092000000000001</v>
+        <v>18.2043</v>
       </c>
       <c r="EV2" t="n">
-        <v>1.178</v>
+        <v>0.9892</v>
       </c>
       <c r="EW2" t="n">
-        <v>84.98</v>
+        <v>100</v>
       </c>
       <c r="EX2" t="n">
-        <v>60.98</v>
+        <v>70.95999999999999</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2290,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>59.57</v>
+        <v>59.91</v>
       </c>
       <c r="FC2" t="n">
-        <v>31.27</v>
+        <v>32.32</v>
       </c>
       <c r="FD2" t="n">
         <v>74.81999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>96.125</v>
+        <v>91.76000000000001</v>
       </c>
       <c r="FF2" t="n">
-        <v>50.5</v>
+        <v>57.97</v>
       </c>
       <c r="FG2" t="n">
-        <v>26.455</v>
+        <v>26.5957</v>
       </c>
       <c r="FH2" t="n">
-        <v>71.98099999999999</v>
+        <v>74.14700000000001</v>
       </c>
       <c r="FI2" t="n">
-        <v>47.975</v>
+        <v>40.85</v>
       </c>
       <c r="FJ2" t="n">
-        <v>72.28</v>
+        <v>72.59</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>82.13</v>
+        <v>77.48999999999999</v>
       </c>
       <c r="FO2" t="n">
-        <v>72.54000000000001</v>
+        <v>73.3</v>
       </c>
       <c r="FP2" t="n">
-        <v>79.61</v>
+        <v>75.59</v>
       </c>
       <c r="FQ2" t="n">
-        <v>74.33</v>
+        <v>66.23</v>
       </c>
       <c r="FR2" t="n">
-        <v>95.84999999999999</v>
+        <v>91.17</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>76.7735</v>
+        <v>72.358</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261028_220543</t>
+          <t>20261029_153437</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46323.92064266764</v>
+        <v>46324.64904221162</v>
       </c>
     </row>
   </sheetData>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46323.92063657408</v>
+        <v>46324.64903935185</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46338</v>
+        <v>46339</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>10.86</v>
+        <v>10.93</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,43 +2681,43 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>2181.9</v>
+        <v>2244</v>
       </c>
       <c r="L2" t="n">
-        <v>2142</v>
+        <v>2190</v>
       </c>
       <c r="M2" t="n">
-        <v>2198.8</v>
+        <v>2244</v>
       </c>
       <c r="N2" t="n">
-        <v>2131.7</v>
+        <v>2166</v>
       </c>
       <c r="O2" t="n">
-        <v>2181.9</v>
+        <v>2244</v>
       </c>
       <c r="P2" t="n">
-        <v>2200547</v>
+        <v>2952155</v>
       </c>
       <c r="Q2" t="n">
-        <v>2181.9</v>
+        <v>2244</v>
       </c>
       <c r="R2" t="n">
-        <v>2424.52</v>
+        <v>2491.58</v>
       </c>
       <c r="S2" t="n">
-        <v>2060.59</v>
+        <v>2120.21</v>
       </c>
       <c r="T2" t="n">
-        <v>11.11966634584536</v>
+        <v>11.03297682709447</v>
       </c>
       <c r="U2" t="n">
-        <v>242.6199999999999</v>
+        <v>247.5799999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>5.559833172922679</v>
+        <v>5.516488413547235</v>
       </c>
       <c r="W2" t="n">
-        <v>121.3099999999999</v>
+        <v>123.79</v>
       </c>
       <c r="X2" t="n">
         <v>2</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>11.11966634584536</v>
+        <v>11.03297682709447</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.559833172922679</v>
+        <v>5.516488413547235</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02048377260105075</v>
+        <v>0.02049208033240395</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3251698092886738</v>
+        <v>0.325301690435392</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02899533758147449</v>
+        <v>0.02898932314703362</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228671424003135</v>
+        <v>0.04228669940338745</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347614</v>
+        <v>0.1869492979645463</v>
       </c>
     </row>
     <row r="14">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.99</v>
+        <v>38.98</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-28 22:05:43.545047+05:30</t>
+          <t>2026-10-29 15:34:37.283100+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 11.119666345845358, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 11.03297682709447, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-29 16:53 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -1864,7 +1864,7 @@
         <v>10.93</v>
       </c>
       <c r="R2" t="n">
-        <v>48.74</v>
+        <v>48.73</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1890,13 +1890,13 @@
         <v>2244</v>
       </c>
       <c r="Z2" t="n">
-        <v>2952155</v>
+        <v>2898447</v>
       </c>
       <c r="AA2" t="n">
-        <v>1648794</v>
+        <v>1646109</v>
       </c>
       <c r="AB2" t="n">
-        <v>1.79</v>
+        <v>1.76</v>
       </c>
       <c r="AC2" t="n">
         <v>2.85</v>
@@ -2026,7 +2026,7 @@
         <v>0.233</v>
       </c>
       <c r="BT2" t="n">
-        <v>1433.28</v>
+        <v>1433.27</v>
       </c>
       <c r="BU2" t="n">
         <v>-12.71</v>
@@ -2091,7 +2091,7 @@
         <v>100</v>
       </c>
       <c r="CO2" t="n">
-        <v>44.98</v>
+        <v>44.85</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2181,10 +2181,10 @@
         <v>38.96</v>
       </c>
       <c r="DS2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="DT2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2199,7 +2199,7 @@
         <v>71.175</v>
       </c>
       <c r="DY2" t="n">
-        <v>89.5</v>
+        <v>88</v>
       </c>
       <c r="DZ2" t="n">
         <v>100</v>
@@ -2220,7 +2220,7 @@
         <v>3.6848</v>
       </c>
       <c r="EF2" t="n">
-        <v>1.79</v>
+        <v>1.76</v>
       </c>
       <c r="EG2" t="n">
         <v>1.1116</v>
@@ -2255,28 +2255,28 @@
         <v>10.93</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.1956</v>
+        <v>0.1924</v>
       </c>
       <c r="ER2" t="n">
-        <v>6.162</v>
+        <v>6.267</v>
       </c>
       <c r="ES2" t="n">
         <v>11.367</v>
       </c>
       <c r="ET2" t="n">
-        <v>65.965</v>
+        <v>65.913</v>
       </c>
       <c r="EU2" t="n">
-        <v>18.2043</v>
+        <v>17.8992</v>
       </c>
       <c r="EV2" t="n">
-        <v>0.9892</v>
+        <v>1</v>
       </c>
       <c r="EW2" t="n">
         <v>100</v>
       </c>
       <c r="EX2" t="n">
-        <v>70.95999999999999</v>
+        <v>70.94</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2302,19 +2302,19 @@
         <v>91.76000000000001</v>
       </c>
       <c r="FF2" t="n">
-        <v>57.97</v>
+        <v>57.895</v>
       </c>
       <c r="FG2" t="n">
         <v>26.5957</v>
       </c>
       <c r="FH2" t="n">
-        <v>74.14700000000001</v>
+        <v>74.143</v>
       </c>
       <c r="FI2" t="n">
         <v>40.85</v>
       </c>
       <c r="FJ2" t="n">
-        <v>72.59</v>
+        <v>72.58</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2334,13 +2334,13 @@
         <v>73.3</v>
       </c>
       <c r="FP2" t="n">
-        <v>75.59</v>
+        <v>75.56999999999999</v>
       </c>
       <c r="FQ2" t="n">
         <v>66.23</v>
       </c>
       <c r="FR2" t="n">
-        <v>91.17</v>
+        <v>91.15000000000001</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>72.358</v>
+        <v>72.346</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261029_153437</t>
+          <t>20261029_222351</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46324.64904221162</v>
+        <v>46324.9332344645</v>
       </c>
     </row>
   </sheetData>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46324.64903935185</v>
+        <v>46324.93322916667</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46324</v>
@@ -2696,7 +2696,7 @@
         <v>2244</v>
       </c>
       <c r="P2" t="n">
-        <v>2952155</v>
+        <v>2898447</v>
       </c>
       <c r="Q2" t="n">
         <v>2244</v>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02049208033240395</v>
+        <v>0.02049208169301076</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.325301690435392</v>
+        <v>0.3253017120343555</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02898932314703362</v>
+        <v>0.0289892238899152</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228669940338745</v>
+        <v>0.04228669803315287</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869492979645463</v>
+        <v>0.1869493934347616</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:34:37.283100+05:30</t>
+          <t>2026-10-29 22:23:51.483854+05:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-30 10:07 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -722,7 +722,7 @@
     <col width="17" customWidth="1" min="125" max="125"/>
     <col width="16" customWidth="1" min="126" max="126"/>
     <col width="22" customWidth="1" min="127" max="127"/>
-    <col width="17" customWidth="1" min="128" max="128"/>
+    <col width="20" customWidth="1" min="128" max="128"/>
     <col width="19" customWidth="1" min="129" max="129"/>
     <col width="18" customWidth="1" min="130" max="130"/>
     <col width="16" customWidth="1" min="131" max="131"/>
@@ -1816,16 +1816,16 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>43101</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="H2" t="n">
         <v>8.800000000000001</v>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1861,10 +1861,10 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>10.93</v>
+        <v>11.08</v>
       </c>
       <c r="R2" t="n">
-        <v>48.73</v>
+        <v>49.02</v>
       </c>
       <c r="S2" t="n">
         <v>1</v>
@@ -1875,49 +1875,49 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>2190</v>
+        <v>2246.6</v>
       </c>
       <c r="V2" t="n">
-        <v>2244</v>
+        <v>2405.5</v>
       </c>
       <c r="W2" t="n">
-        <v>2166</v>
+        <v>2206.1</v>
       </c>
       <c r="X2" t="n">
-        <v>2244</v>
+        <v>2405.5</v>
       </c>
       <c r="Y2" t="n">
-        <v>2244</v>
+        <v>2405.5</v>
       </c>
       <c r="Z2" t="n">
-        <v>2898447</v>
+        <v>7909825</v>
       </c>
       <c r="AA2" t="n">
-        <v>1646109</v>
+        <v>1971821</v>
       </c>
       <c r="AB2" t="n">
-        <v>1.76</v>
+        <v>4.01</v>
       </c>
       <c r="AC2" t="n">
-        <v>2.85</v>
+        <v>7.2</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.37</v>
+        <v>0.12</v>
       </c>
       <c r="AE2" t="n">
-        <v>78</v>
+        <v>199.4</v>
       </c>
       <c r="AF2" t="n">
-        <v>3.48</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="AG2" t="n">
-        <v>61.89</v>
+        <v>71.72</v>
       </c>
       <c r="AH2" t="n">
-        <v>61.89</v>
+        <v>71.72</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.76</v>
+        <v>2.98</v>
       </c>
       <c r="AJ2" t="b">
         <v>1</v>
@@ -1926,50 +1926,50 @@
         <v>1</v>
       </c>
       <c r="AL2" t="n">
-        <v>9.470000000000001</v>
+        <v>16.14</v>
       </c>
       <c r="AM2" t="n">
-        <v>13.91</v>
+        <v>21.38</v>
       </c>
       <c r="AN2" t="n">
-        <v>55.51</v>
+        <v>65.97</v>
       </c>
       <c r="AO2" t="n">
-        <v>71.53</v>
+        <v>78.70999999999999</v>
       </c>
       <c r="AP2" t="n">
-        <v>10.17</v>
+        <v>19.17</v>
       </c>
       <c r="AQ2" t="n">
-        <v>25.98</v>
+        <v>35.04</v>
       </c>
       <c r="AR2" t="n">
-        <v>2244</v>
+        <v>2405.5</v>
       </c>
       <c r="AS2" t="n">
-        <v>2491.58</v>
+        <v>2692.37</v>
       </c>
       <c r="AT2" t="n">
-        <v>2120.21</v>
+        <v>2262.07</v>
       </c>
       <c r="AU2" t="n">
-        <v>2244</v>
+        <v>2405.5</v>
       </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>15</v>
       </c>
       <c r="AX2" t="n">
-        <v>11.03</v>
+        <v>11.93</v>
       </c>
       <c r="AY2" t="n">
-        <v>247.58</v>
+        <v>286.87</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5.52</v>
+        <v>5.96</v>
       </c>
       <c r="BA2" t="n">
-        <v>123.79</v>
+        <v>143.43</v>
       </c>
       <c r="BB2" t="n">
         <v>2.07</v>
@@ -1978,19 +1978,19 @@
         <v>214</v>
       </c>
       <c r="BD2" t="n">
-        <v>31.5</v>
+        <v>31.4</v>
       </c>
       <c r="BE2" t="n">
         <v>342</v>
       </c>
       <c r="BF2" t="n">
-        <v>50.3</v>
+        <v>50.2</v>
       </c>
       <c r="BG2" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="BH2" t="n">
-        <v>18.2</v>
+        <v>18.4</v>
       </c>
       <c r="BI2" t="n">
         <v>0</v>
@@ -2005,40 +2005,40 @@
         <v>0</v>
       </c>
       <c r="BM2" t="n">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="BN2" t="n">
         <v>49</v>
       </c>
       <c r="BO2" t="n">
-        <v>2.11</v>
+        <v>2.13</v>
       </c>
       <c r="BP2" t="n">
-        <v>8.68</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="BQ2" t="n">
         <v>-4.2</v>
       </c>
       <c r="BR2" t="n">
-        <v>9.1</v>
+        <v>9</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.233</v>
+        <v>0.236</v>
       </c>
       <c r="BT2" t="n">
-        <v>1433.27</v>
+        <v>1451.16</v>
       </c>
       <c r="BU2" t="n">
-        <v>-12.71</v>
+        <v>-11.74</v>
       </c>
       <c r="BV2" t="n">
-        <v>1.98</v>
+        <v>2</v>
       </c>
       <c r="BW2" t="n">
         <v>2.07</v>
       </c>
       <c r="BX2" t="n">
-        <v>2</v>
+        <v>2.0001</v>
       </c>
       <c r="BY2" t="n">
         <v>-80.69</v>
@@ -2058,10 +2058,10 @@
         </is>
       </c>
       <c r="CD2" t="n">
-        <v>42.2</v>
+        <v>42.6</v>
       </c>
       <c r="CE2" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="CF2" t="n">
         <v>69</v>
@@ -2091,7 +2091,7 @@
         <v>100</v>
       </c>
       <c r="CO2" t="n">
-        <v>44.85</v>
+        <v>48.33</v>
       </c>
       <c r="CP2" t="n">
         <v>95.45454545454545</v>
@@ -2106,16 +2106,16 @@
         <v>100</v>
       </c>
       <c r="CT2" t="n">
-        <v>95.45454545454545</v>
+        <v>100</v>
       </c>
       <c r="CU2" t="n">
         <v>95.45454545454545</v>
       </c>
       <c r="CV2" t="n">
-        <v>86.36363636363636</v>
+        <v>93.18181818181817</v>
       </c>
       <c r="CW2" t="n">
-        <v>77.27272727272727</v>
+        <v>81.81818181818183</v>
       </c>
       <c r="CX2" t="n">
         <v>54.54545454545454</v>
@@ -2124,7 +2124,7 @@
         <v>1</v>
       </c>
       <c r="CZ2" t="n">
-        <v>11.033</v>
+        <v>11.9256</v>
       </c>
       <c r="DA2" t="n">
         <v>0</v>
@@ -2133,58 +2133,58 @@
         <v>0</v>
       </c>
       <c r="DC2" t="n">
-        <v>0.7353</v>
+        <v>0.7953</v>
       </c>
       <c r="DD2" t="n">
-        <v>0.368</v>
+        <v>0.3973</v>
       </c>
       <c r="DE2" t="n">
-        <v>0.1103</v>
+        <v>0.1193</v>
       </c>
       <c r="DF2" t="n">
-        <v>1.9982</v>
+        <v>2.0017</v>
       </c>
       <c r="DG2" t="n">
-        <v>1.2056</v>
+        <v>1.3218</v>
       </c>
       <c r="DH2" t="n">
-        <v>3.9964</v>
+        <v>4.0034</v>
       </c>
       <c r="DI2" t="n">
-        <v>5.5165</v>
+        <v>5.9626</v>
       </c>
       <c r="DJ2" t="n">
-        <v>42.74</v>
+        <v>54.4</v>
       </c>
       <c r="DK2" t="n">
-        <v>5.5165</v>
+        <v>5.9626</v>
       </c>
       <c r="DL2" t="n">
-        <v>2</v>
+        <v>2.0001</v>
       </c>
       <c r="DM2" t="n">
         <v>2</v>
       </c>
       <c r="DN2" t="n">
-        <v>3.9964</v>
+        <v>4.0034</v>
       </c>
       <c r="DO2" t="n">
-        <v>1.9981</v>
+        <v>2.0018</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.724</v>
+        <v>0.6717</v>
       </c>
       <c r="DQ2" t="n">
-        <v>123.79</v>
+        <v>143.43</v>
       </c>
       <c r="DR2" t="n">
-        <v>38.96</v>
+        <v>68.64</v>
       </c>
       <c r="DS2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="DT2" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="DU2" t="n">
         <v>2</v>
@@ -2193,16 +2193,16 @@
         <v>100</v>
       </c>
       <c r="DW2" t="n">
-        <v>3.6848</v>
+        <v>6.4329</v>
       </c>
       <c r="DX2" t="n">
-        <v>71.175</v>
+        <v>53.22500000000002</v>
       </c>
       <c r="DY2" t="n">
-        <v>88</v>
+        <v>200.5</v>
       </c>
       <c r="DZ2" t="n">
-        <v>100</v>
+        <v>93.94199999999999</v>
       </c>
       <c r="EA2" t="n">
         <v>5</v>
@@ -2214,32 +2214,32 @@
         <v>100</v>
       </c>
       <c r="ED2" t="n">
-        <v>60.01</v>
+        <v>48.13</v>
       </c>
       <c r="EE2" t="n">
-        <v>3.6848</v>
+        <v>6.4329</v>
       </c>
       <c r="EF2" t="n">
-        <v>1.76</v>
+        <v>4.01</v>
       </c>
       <c r="EG2" t="n">
-        <v>1.1116</v>
+        <v>2.124</v>
       </c>
       <c r="EH2" t="n">
-        <v>3.9975</v>
+        <v>4.0019</v>
       </c>
       <c r="EI2" t="n">
-        <v>0.1215</v>
+        <v>0.2353</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.6131</v>
+        <v>0.575</v>
       </c>
       <c r="EK2" t="n">
-        <v>83.52</v>
+        <v>79.51000000000001</v>
       </c>
       <c r="EL2" t="inlineStr">
         <is>
-          <t>Excellent</t>
+          <t>Strong</t>
         </is>
       </c>
       <c r="EM2" t="n">
@@ -2249,34 +2249,34 @@
         <v>10</v>
       </c>
       <c r="EO2" t="n">
-        <v>100</v>
+        <v>39.42</v>
       </c>
       <c r="EP2" t="n">
-        <v>10.93</v>
+        <v>4.3677</v>
       </c>
       <c r="EQ2" t="n">
-        <v>0.1924</v>
+        <v>0.4443</v>
       </c>
       <c r="ER2" t="n">
-        <v>6.267</v>
+        <v>2.9751</v>
       </c>
       <c r="ES2" t="n">
-        <v>11.367</v>
+        <v>13.6683</v>
       </c>
       <c r="ET2" t="n">
-        <v>65.913</v>
+        <v>49.344</v>
       </c>
       <c r="EU2" t="n">
-        <v>17.8992</v>
+        <v>76.8717</v>
       </c>
       <c r="EV2" t="n">
-        <v>1</v>
+        <v>0.5948</v>
       </c>
       <c r="EW2" t="n">
-        <v>100</v>
+        <v>39.42</v>
       </c>
       <c r="EX2" t="n">
-        <v>70.94</v>
+        <v>71.65000000000001</v>
       </c>
       <c r="EY2" t="inlineStr">
         <is>
@@ -2290,31 +2290,31 @@
         <v>10</v>
       </c>
       <c r="FB2" t="n">
-        <v>59.91</v>
+        <v>60.62</v>
       </c>
       <c r="FC2" t="n">
-        <v>32.32</v>
+        <v>45.38</v>
       </c>
       <c r="FD2" t="n">
         <v>74.81999999999999</v>
       </c>
       <c r="FE2" t="n">
-        <v>91.76000000000001</v>
+        <v>89.755</v>
       </c>
       <c r="FF2" t="n">
-        <v>57.895</v>
+        <v>59.99</v>
       </c>
       <c r="FG2" t="n">
-        <v>26.5957</v>
+        <v>25.1256</v>
       </c>
       <c r="FH2" t="n">
-        <v>74.143</v>
+        <v>74.64</v>
       </c>
       <c r="FI2" t="n">
-        <v>40.85</v>
+        <v>61.52</v>
       </c>
       <c r="FJ2" t="n">
-        <v>72.58</v>
+        <v>76.39</v>
       </c>
       <c r="FK2" t="inlineStr">
         <is>
@@ -2328,19 +2328,19 @@
         <v>10</v>
       </c>
       <c r="FN2" t="n">
-        <v>77.48999999999999</v>
+        <v>86.04000000000001</v>
       </c>
       <c r="FO2" t="n">
-        <v>73.3</v>
+        <v>79.11</v>
       </c>
       <c r="FP2" t="n">
-        <v>75.56999999999999</v>
+        <v>84.73</v>
       </c>
       <c r="FQ2" t="n">
-        <v>66.23</v>
+        <v>79.06</v>
       </c>
       <c r="FR2" t="n">
-        <v>91.15000000000001</v>
+        <v>97.77</v>
       </c>
       <c r="FS2" t="n">
         <v>100</v>
@@ -2357,11 +2357,11 @@
         </is>
       </c>
       <c r="FW2" t="n">
-        <v>72.346</v>
+        <v>82.619</v>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Excellent</t>
         </is>
       </c>
       <c r="FY2" t="b">
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261029_222351</t>
+          <t>20261030_153734</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46324.9332344645</v>
+        <v>46325.65109852684</v>
       </c>
     </row>
   </sheetData>
@@ -2466,7 +2466,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
     <col width="20" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="19" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
@@ -2647,13 +2647,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46324.93322916667</v>
+        <v>46325.65108796296</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46339</v>
+        <v>46340</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>10.93</v>
+        <v>11.08</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2681,46 +2681,46 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>2244</v>
+        <v>2405.5</v>
       </c>
       <c r="L2" t="n">
-        <v>2190</v>
+        <v>2246.6</v>
       </c>
       <c r="M2" t="n">
-        <v>2244</v>
+        <v>2405.5</v>
       </c>
       <c r="N2" t="n">
-        <v>2166</v>
+        <v>2206.1</v>
       </c>
       <c r="O2" t="n">
-        <v>2244</v>
+        <v>2405.5</v>
       </c>
       <c r="P2" t="n">
-        <v>2898447</v>
+        <v>7909825</v>
       </c>
       <c r="Q2" t="n">
-        <v>2244</v>
+        <v>2405.5</v>
       </c>
       <c r="R2" t="n">
-        <v>2491.58</v>
+        <v>2692.37</v>
       </c>
       <c r="S2" t="n">
-        <v>2120.21</v>
+        <v>2262.07</v>
       </c>
       <c r="T2" t="n">
-        <v>11.03297682709447</v>
+        <v>11.92558719600914</v>
       </c>
       <c r="U2" t="n">
-        <v>247.5799999999999</v>
+        <v>286.8699999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>5.516488413547235</v>
+        <v>5.962585741010178</v>
       </c>
       <c r="W2" t="n">
-        <v>123.79</v>
+        <v>143.4299999999998</v>
       </c>
       <c r="X2" t="n">
-        <v>2</v>
+        <v>2.000069720421113</v>
       </c>
       <c r="Y2" t="n">
         <v>15</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>11.03297682709447</v>
+        <v>11.92558719600914</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.516488413547235</v>
+        <v>5.962585741010178</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02049208169301076</v>
+        <v>0.02063986472767657</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3253017120343555</v>
+        <v>0.3276476949806765</v>
       </c>
     </row>
     <row r="7">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.0289892238899152</v>
+        <v>0.02898330871259274</v>
       </c>
     </row>
     <row r="12">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228669803315287</v>
+        <v>0.04228671623812318</v>
       </c>
     </row>
     <row r="13">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38.98</v>
+        <v>38.79</v>
       </c>
     </row>
     <row r="16">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-29 22:23:51.483854+05:30</t>
+          <t>2026-10-30 15:37:34.932335+05:30</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 11.03297682709447, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.0}</t>
+          <t>{'active_trades': 1, 'target_hits': 0, 'stop_losses': 0, 'time_exits': 0, 'average_expected_return_pct': 11.925587196009142, 'average_current_return_pct': 0.0, 'average_risk_reward': 2.000069720421113}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update scanner reports (2026-10-30 16:41 UTC)
</commit_message>
<xml_diff>
--- a/scanner_monitor/reports/latest/Portfolio_Report.xlsx
+++ b/scanner_monitor/reports/latest/Portfolio_Report.xlsx
@@ -2422,11 +2422,11 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t>20261030_153734</t>
+          <t>20261030_221112</t>
         </is>
       </c>
       <c r="GR2" s="2" t="n">
-        <v>46325.65109852684</v>
+        <v>46325.92444930257</v>
       </c>
     </row>
   </sheetData>
@@ -2647,7 +2647,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46325.65108796296</v>
+        <v>46325.92444444444</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46325</v>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02063986472767657</v>
+        <v>0.02063986296596309</v>
       </c>
     </row>
     <row r="6">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3276476949806765</v>
+        <v>0.3276476670143419</v>
       </c>
     </row>
     <row r="7">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04228671623812318</v>
+        <v>0.04228670650262135</v>
       </c>
     </row>
     <row r="13">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1869493934347616</v>
+        <v>0.1869493934347614</v>
       </c>
     </row>
     <row r="14">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-30 15:37:34.932335+05:30</t>
+          <t>2026-10-30 22:11:12.454439+05:30</t>
         </is>
       </c>
     </row>

</xml_diff>